<commit_message>
Complexes : 10 fiches ajoutées d'après le cours de référence, M027 retirée
Conjugaison, argument, propriétés de e^{iθ}, interprétation géométrique,
X² = α, propriétés des arguments, définition du module, inverse et produit nul,
compléments sur le module, linéarisation.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N461"/>
+  <dimension ref="A1:N471"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2337,8 +2337,16 @@
         <v>20</v>
       </c>
       <c r="L28" s="12" t="inlineStr"/>
-      <c r="M28" s="14" t="n"/>
-      <c r="N28" s="14" t="n"/>
+      <c r="M28" s="14" t="inlineStr">
+        <is>
+          <t>Passer en rouge</t>
+        </is>
+      </c>
+      <c r="N28" s="14" t="inlineStr">
+        <is>
+          <t>Retirée : absente du Cours BCPST « Les complexes » 2024 et non citée dans le programme.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
@@ -27470,10 +27478,610 @@
       <c r="M461" s="14" t="n"/>
       <c r="N461" s="14" t="n"/>
     </row>
+    <row r="462">
+      <c r="A462" s="9" t="inlineStr">
+        <is>
+          <t>M461</t>
+        </is>
+      </c>
+      <c r="B462" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C462" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D462" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 4 – Nombres complexes</t>
+        </is>
+      </c>
+      <c r="E462" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F462" s="9" t="inlineStr">
+        <is>
+          <t>Propriétés de la conjugaison</t>
+        </is>
+      </c>
+      <c r="G462" s="9" t="inlineStr">
+        <is>
+          <t>Soient $z$ et $z'$ deux nombres complexes et $n\in\mathbb N$.</t>
+        </is>
+      </c>
+      <c r="H462" s="10" t="inlineStr">
+        <is>
+          <t>Donner les propriétés de la conjugaison : conjugué d'une somme, d'un produit, d'un inverse, d'une puissance, et de $\bar z$.</t>
+        </is>
+      </c>
+      <c r="I462" s="9" t="inlineStr">
+        <is>
+          <t>$\overline{z+z'}=\bar z+\overline{z'}$ ; $\overline{zz'}=\bar z\,\overline{z'}$ ; si $z\neq0$, $\overline{\left(\frac1z\right)}=\frac1{\bar z}$ ; $\overline{z^n}=\bar z^{\,n}$ ; $\overline{\bar z}=z$.</t>
+        </is>
+      </c>
+      <c r="J462" s="9" t="inlineStr">
+        <is>
+          <t>« Conjugué d'un nombre complexe. Interprétation géométrique. Propriétés de la conjugaison. »</t>
+        </is>
+      </c>
+      <c r="K462" s="9" t="n"/>
+      <c r="L462" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le Cours BCPST « Les complexes » 2024</t>
+        </is>
+      </c>
+      <c r="M462" s="11" t="n"/>
+      <c r="N462" s="11" t="n"/>
+    </row>
+    <row r="463">
+      <c r="A463" s="9" t="inlineStr">
+        <is>
+          <t>M462</t>
+        </is>
+      </c>
+      <c r="B463" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C463" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D463" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 4 – Nombres complexes</t>
+        </is>
+      </c>
+      <c r="E463" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F463" s="9" t="inlineStr">
+        <is>
+          <t>Argument d'un nombre complexe non nul</t>
+        </is>
+      </c>
+      <c r="G463" s="9" t="inlineStr">
+        <is>
+          <t>Soit $z$ un nombre complexe non nul.</t>
+        </is>
+      </c>
+      <c r="H463" s="10" t="inlineStr">
+        <is>
+          <t>Définir un argument de $z$ et l'argument principal de $z$.</t>
+        </is>
+      </c>
+      <c r="I463" s="9" t="inlineStr">
+        <is>
+          <t>Si $z=\rho e^{i\theta}$ avec $\rho&gt;0$ et $\theta\in\mathbb R$, $\theta$ est un argument de $z$ ; on note $\arg z\equiv\theta\ [2\pi]$. L'argument principal est l'unique argument appartenant à $]-\pi,\pi]$. Le nombre $0$ n'a pas d'argument.</t>
+        </is>
+      </c>
+      <c r="J463" s="9" t="inlineStr">
+        <is>
+          <t>« Arguments d'un nombre complexe non nul. On met en évidence quelques choix usuels d'intervalles permettant de définir l'argument. »</t>
+        </is>
+      </c>
+      <c r="K463" s="9" t="n"/>
+      <c r="L463" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le Cours BCPST « Les complexes » 2024</t>
+        </is>
+      </c>
+      <c r="M463" s="11" t="n"/>
+      <c r="N463" s="11" t="n"/>
+    </row>
+    <row r="464">
+      <c r="A464" s="9" t="inlineStr">
+        <is>
+          <t>M463</t>
+        </is>
+      </c>
+      <c r="B464" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C464" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D464" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 4 – Nombres complexes</t>
+        </is>
+      </c>
+      <c r="E464" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F464" s="9" t="inlineStr">
+        <is>
+          <t>Propriétés de $e^{i\theta}$</t>
+        </is>
+      </c>
+      <c r="G464" s="9" t="inlineStr">
+        <is>
+          <t>Soient $\alpha$, $\beta$, $\theta$ des réels et $n\in\mathbb Z$.</t>
+        </is>
+      </c>
+      <c r="H464" s="10" t="inlineStr">
+        <is>
+          <t>Donner les propriétés de $e^{i\theta}$ : module, conjugué, exponentielle d'une somme, puissance.</t>
+        </is>
+      </c>
+      <c r="I464" s="9" t="inlineStr">
+        <is>
+          <t>$|e^{i\theta}|=1$ ; $\overline{e^{i\theta}}=e^{-i\theta}$ ; $e^{i(\alpha+\beta)}=e^{i\alpha}e^{i\beta}$ ; $(e^{i\theta})^n=e^{in\theta}$.</t>
+        </is>
+      </c>
+      <c r="J464" s="9" t="inlineStr">
+        <is>
+          <t>« Notation e^{iθ}. Propriétés |e^{iθ}| = 1, e^{i(α+β)} = e^{iα} × e^{iβ}, conjugué de e^{iθ} = e^{−iθ}, (e^{iθ})^n = e^{inθ} »</t>
+        </is>
+      </c>
+      <c r="K464" s="9" t="n"/>
+      <c r="L464" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le Cours BCPST « Les complexes » 2024</t>
+        </is>
+      </c>
+      <c r="M464" s="11" t="n"/>
+      <c r="N464" s="11" t="n"/>
+    </row>
+    <row r="465">
+      <c r="A465" s="9" t="inlineStr">
+        <is>
+          <t>M464</t>
+        </is>
+      </c>
+      <c r="B465" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C465" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D465" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 4 – Nombres complexes</t>
+        </is>
+      </c>
+      <c r="E465" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F465" s="9" t="inlineStr">
+        <is>
+          <t>Interprétation géométrique des complexes</t>
+        </is>
+      </c>
+      <c r="G465" s="9" t="inlineStr">
+        <is>
+          <t>Le plan est muni d'un repère orthonormé direct $(O;\vec u,\vec v)$. Soient $M$, $A$, $B$ des points d'affixes $z$, $z_A$, $z_B$.</t>
+        </is>
+      </c>
+      <c r="H465" s="10" t="inlineStr">
+        <is>
+          <t>Donner l'interprétation géométrique de l'affixe de $\overrightarrow{AB}$, de la somme de deux complexes, de $|z|$, de $\bar z$ et de $-z$.</t>
+        </is>
+      </c>
+      <c r="I465" s="9" t="inlineStr">
+        <is>
+          <t>L'affixe de $\overrightarrow{AB}$ est $z_B-z_A$ ; la somme des affixes de deux vecteurs est l'affixe de leur somme ; $|z|=OM$ et $|z_B-z_A|=AB$ ; le point d'affixe $\bar z$ est le symétrique de $M$ par rapport à l'axe des abscisses ; celui d'affixe $-z$ est le symétrique de $M$ par rapport à $O$.</t>
+        </is>
+      </c>
+      <c r="J465" s="9" t="inlineStr">
+        <is>
+          <t>« Représentation géométrique d'un nombre complexe. Affixe d'un point, d'un vecteur. Interprétation géométrique de la somme » ; conjugué et module : « Interprétation géométrique ». Les problèmes de géométrie par les complexes ne sont pas un objectif.</t>
+        </is>
+      </c>
+      <c r="K465" s="9" t="n"/>
+      <c r="L465" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le Cours BCPST « Les complexes » 2024</t>
+        </is>
+      </c>
+      <c r="M465" s="11" t="n"/>
+      <c r="N465" s="11" t="n"/>
+    </row>
+    <row r="466">
+      <c r="A466" s="9" t="inlineStr">
+        <is>
+          <t>M465</t>
+        </is>
+      </c>
+      <c r="B466" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C466" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D466" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 4 – Nombres complexes</t>
+        </is>
+      </c>
+      <c r="E466" s="9" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+      <c r="F466" s="9" t="inlineStr">
+        <is>
+          <t>Résolution de $X^2=\alpha$ avec $\alpha\in\mathbb C$</t>
+        </is>
+      </c>
+      <c r="G466" s="9" t="inlineStr">
+        <is>
+          <t>Soient $\alpha=a+ib$ ($a,b$ réels) et l'équation $X^2=\alpha$ d'inconnue $X=x+iy$ ($x,y$ réels).</t>
+        </is>
+      </c>
+      <c r="H466" s="10" t="inlineStr">
+        <is>
+          <t>Donner la méthode de résolution de $X^2=\alpha$.</t>
+        </is>
+      </c>
+      <c r="I466" s="9" t="inlineStr">
+        <is>
+          <t>On utilise $X^2=\alpha$ et $|X|^2=|\alpha|$ : $x^2-y^2=a$, $2xy=b$, $x^2+y^2=\sqrt{a^2+b^2}$. On en tire $x^2$ et $y^2$, puis le signe de $xy$ (celui de $b$) donne deux solutions opposées. Variante : si $\alpha=re^{i\varphi}$ avec $r&gt;0$, les solutions sont $\pm\sqrt r\,e^{i\varphi/2}$.</t>
+        </is>
+      </c>
+      <c r="J466" s="9" t="inlineStr">
+        <is>
+          <t>« Résolution de l'équation x² = a avec a ∈ C. […] cette équation doit pouvoir être traitée algébriquement ou en la retranscrivant trigonométriquement »</t>
+        </is>
+      </c>
+      <c r="K466" s="9" t="n"/>
+      <c r="L466" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le Cours BCPST « Les complexes » 2024</t>
+        </is>
+      </c>
+      <c r="M466" s="11" t="n"/>
+      <c r="N466" s="11" t="n"/>
+    </row>
+    <row r="467">
+      <c r="A467" s="9" t="inlineStr">
+        <is>
+          <t>M466</t>
+        </is>
+      </c>
+      <c r="B467" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C467" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D467" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 4 – Nombres complexes</t>
+        </is>
+      </c>
+      <c r="E467" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F467" s="9" t="inlineStr">
+        <is>
+          <t>Propriétés des arguments</t>
+        </is>
+      </c>
+      <c r="G467" s="9" t="inlineStr">
+        <is>
+          <t>Soient $z$ et $z'$ deux nombres complexes non nuls et $n\in\mathbb Z$.</t>
+        </is>
+      </c>
+      <c r="H467" s="10" t="inlineStr">
+        <is>
+          <t>Donner un argument de $zz'$, $z^n$, $\frac1z$, $\frac z{z'}$ et $\bar z$ en fonction de $\arg z$ et $\arg z'$.</t>
+        </is>
+      </c>
+      <c r="I467" s="9" t="inlineStr">
+        <is>
+          <t>Modulo $2\pi$ : $\arg(zz')\equiv\arg z+\arg z'$ ; $\arg(z^n)\equiv n\arg z$ ; $\arg\frac1z\equiv-\arg z$ ; $\arg\frac z{z'}\equiv\arg z-\arg z'$ ; $\arg\bar z\equiv-\arg z$.</t>
+        </is>
+      </c>
+      <c r="J467" s="9" t="inlineStr">
+        <is>
+          <t>Conséquence directe des propriétés de e^{iθ} et de « Arguments d'un nombre complexe non nul ».</t>
+        </is>
+      </c>
+      <c r="K467" s="9" t="n"/>
+      <c r="L467" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le Cours BCPST « Les complexes » 2024</t>
+        </is>
+      </c>
+      <c r="M467" s="11" t="n"/>
+      <c r="N467" s="11" t="n"/>
+    </row>
+    <row r="468">
+      <c r="A468" s="9" t="inlineStr">
+        <is>
+          <t>M467</t>
+        </is>
+      </c>
+      <c r="B468" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C468" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D468" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 4 – Nombres complexes</t>
+        </is>
+      </c>
+      <c r="E468" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F468" s="9" t="inlineStr">
+        <is>
+          <t>Module d'un nombre complexe – Définition</t>
+        </is>
+      </c>
+      <c r="G468" s="9" t="inlineStr">
+        <is>
+          <t>Soit $z=a+ib$ un nombre complexe ($a,b$ réels).</t>
+        </is>
+      </c>
+      <c r="H468" s="10" t="inlineStr">
+        <is>
+          <t>Définir le module $|z|$.</t>
+        </is>
+      </c>
+      <c r="I468" s="9" t="inlineStr">
+        <is>
+          <t>$|z|=\sqrt{a^2+b^2}=\sqrt{z\bar z}$. Si $M$ a pour affixe $z$, $|z|=OM$.</t>
+        </is>
+      </c>
+      <c r="J468" s="9" t="inlineStr">
+        <is>
+          <t>« Module d'un nombre complexe. […] on choisit la formulation adéquate : |z| = √(z z̄) ou |a + ib| = √(a² + b²). »</t>
+        </is>
+      </c>
+      <c r="K468" s="9" t="n"/>
+      <c r="L468" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le Cours BCPST « Les complexes » 2024</t>
+        </is>
+      </c>
+      <c r="M468" s="11" t="n"/>
+      <c r="N468" s="11" t="n"/>
+    </row>
+    <row r="469">
+      <c r="A469" s="9" t="inlineStr">
+        <is>
+          <t>M468</t>
+        </is>
+      </c>
+      <c r="B469" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C469" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D469" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 4 – Nombres complexes</t>
+        </is>
+      </c>
+      <c r="E469" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F469" s="9" t="inlineStr">
+        <is>
+          <t>Inverse – Produit nul</t>
+        </is>
+      </c>
+      <c r="G469" s="9" t="inlineStr">
+        <is>
+          <t>Soient $z$ et $z'$ deux nombres complexes.</t>
+        </is>
+      </c>
+      <c r="H469" s="10" t="inlineStr">
+        <is>
+          <t>Donner la forme algébrique de l'inverse de $z=a+ib\neq0$ ($a,b$ réels) et énoncer la règle du produit nul.</t>
+        </is>
+      </c>
+      <c r="I469" s="9" t="inlineStr">
+        <is>
+          <t>$\dfrac1z=\dfrac{\bar z}{|z|^2}=\dfrac{a-ib}{a^2+b^2}$ ; $zz'=0\iff z=0$ ou $z'=0$.</t>
+        </is>
+      </c>
+      <c r="J469" s="9" t="inlineStr">
+        <is>
+          <t>« Nombres complexes. Écriture algébrique. »</t>
+        </is>
+      </c>
+      <c r="K469" s="9" t="n"/>
+      <c r="L469" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le Cours BCPST « Les complexes » 2024</t>
+        </is>
+      </c>
+      <c r="M469" s="11" t="n"/>
+      <c r="N469" s="11" t="n"/>
+    </row>
+    <row r="470">
+      <c r="A470" s="9" t="inlineStr">
+        <is>
+          <t>M469</t>
+        </is>
+      </c>
+      <c r="B470" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C470" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D470" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 4 – Nombres complexes</t>
+        </is>
+      </c>
+      <c r="E470" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F470" s="9" t="inlineStr">
+        <is>
+          <t>Module – Compléments</t>
+        </is>
+      </c>
+      <c r="G470" s="9" t="inlineStr">
+        <is>
+          <t>Soient $z$, $z_1$, $z_2$ des nombres complexes et $n\in\mathbb N$.</t>
+        </is>
+      </c>
+      <c r="H470" s="10" t="inlineStr">
+        <is>
+          <t>Donner $|z^n|$, comparer $|z|$, $|\bar z|$ et $|-z|$, caractériser $|z|=0$, et minorer $|z_1+z_2|$.</t>
+        </is>
+      </c>
+      <c r="I470" s="9" t="inlineStr">
+        <is>
+          <t>$|z^n|=|z|^n$ ; $|\bar z|=|-z|=|z|$ ; $|z|=0\iff z=0$ ; $\big||z_1|-|z_2|\big|\le|z_1+z_2|$.</t>
+        </is>
+      </c>
+      <c r="J470" s="9" t="inlineStr">
+        <is>
+          <t>« Propriétés du module : multiplicativité, inégalité triangulaire. »</t>
+        </is>
+      </c>
+      <c r="K470" s="9" t="n"/>
+      <c r="L470" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le Cours BCPST « Les complexes » 2024</t>
+        </is>
+      </c>
+      <c r="M470" s="11" t="n"/>
+      <c r="N470" s="11" t="n"/>
+    </row>
+    <row r="471">
+      <c r="A471" s="9" t="inlineStr">
+        <is>
+          <t>M470</t>
+        </is>
+      </c>
+      <c r="B471" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C471" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D471" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 4 – Nombres complexes</t>
+        </is>
+      </c>
+      <c r="E471" s="9" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+      <c r="F471" s="9" t="inlineStr">
+        <is>
+          <t>Linéarisation de $\cos^px\,\sin^qx$</t>
+        </is>
+      </c>
+      <c r="G471" s="9" t="inlineStr">
+        <is>
+          <t>Soient $x$ un réel et $p$, $q$ des entiers naturels.</t>
+        </is>
+      </c>
+      <c r="H471" s="10" t="inlineStr">
+        <is>
+          <t>Donner la méthode pour linéariser $\cos^px\,\sin^qx$.</t>
+        </is>
+      </c>
+      <c r="I471" s="9" t="inlineStr">
+        <is>
+          <t>Remplacer $\cos x$ et $\sin x$ par les formules d'Euler, développer (binôme de Newton), puis regrouper $e^{ikx}$ et $e^{-ikx}$ en $2\cos(kx)$ ou $2i\sin(kx)$. On obtient une combinaison linéaire de $\cos(kx)$ et $\sin(kx)$.</t>
+        </is>
+      </c>
+      <c r="J471" s="9" t="inlineStr">
+        <is>
+          <t>« Linéarisation de cos^p(x) sin^q(x). À chaque fois que le recours à la formule d'Euler sera nécessaire pour linéariser ou développer des formules, l'énoncé devra l'indiquer. »</t>
+        </is>
+      </c>
+      <c r="K471" s="9" t="n"/>
+      <c r="L471" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le Cours BCPST « Les complexes » 2024</t>
+        </is>
+      </c>
+      <c r="M471" s="11" t="n"/>
+      <c r="N471" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M461" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M471" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -30685,6 +31293,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
@@ -30709,7 +31318,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$461,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$471,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -30724,7 +31333,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$461,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$471,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -30739,7 +31348,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$461,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$471,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -30758,6 +31367,7 @@
         <v/>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="25" t="inlineStr">
         <is>
@@ -30765,10 +31375,11 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$461)</f>
+        <f>COUNTA(Fiches!$M$2:$M$471)</f>
         <v/>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="18" t="inlineStr">
         <is>
@@ -30810,15 +31421,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A13,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A13,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A13,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A13,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A13,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A13,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -30833,15 +31444,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A14,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A14,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A14,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A14,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A14,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A14,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -30856,15 +31467,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A15,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A15,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A15,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A15,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A15,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A15,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -30879,15 +31490,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A16,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A16,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A16,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A16,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A16,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A16,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -30902,15 +31513,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A17,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A17,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A17,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A17,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A17,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A17,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -30925,15 +31536,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A18,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A18,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A18,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A18,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A18,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A18,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -30948,15 +31559,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A19,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A19,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A19,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A19,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A19,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A19,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -30971,15 +31582,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A20,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A20,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A20,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A20,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A20,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A20,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -30994,15 +31605,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A21,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A21,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A21,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A21,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A21,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A21,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -31017,15 +31628,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A22,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A22,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A22,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A22,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A22,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A22,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -31040,15 +31651,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A23,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A23,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A23,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A23,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A23,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A23,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -31063,15 +31674,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A24,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A24,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A24,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A24,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A24,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A24,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -31086,15 +31697,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A25,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A25,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A25,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A25,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A25,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A25,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -31109,15 +31720,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A26,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A26,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A26,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A26,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A26,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A26,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -31132,15 +31743,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A27,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A27,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A27,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A27,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A27,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A27,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -31155,15 +31766,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A28,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A28,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A28,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A28,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A28,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A28,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -31178,15 +31789,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A29,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A29,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A29,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A29,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A29,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A29,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -31201,15 +31812,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A30,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A30,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A30,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A30,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A30,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A30,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -31224,15 +31835,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A31,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A31,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A31,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A31,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A31,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A31,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -31247,15 +31858,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A32,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A32,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A32,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A32,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A32,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A32,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -31270,15 +31881,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A33,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A33,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A33,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A33,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A33,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A33,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -31293,15 +31904,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A34,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A34,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A34,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A34,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A34,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A34,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -31316,15 +31927,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A35,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A35,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A35,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A35,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A35,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A35,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -31339,15 +31950,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A36,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A36,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A36,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A36,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A36,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A36,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -31362,15 +31973,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A37,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A37,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A37,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A37,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A37,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A37,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -31385,15 +31996,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A38,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A38,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A38,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A38,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A38,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A38,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -31408,15 +32019,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A39,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A39,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A39,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A39,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A39,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A39,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -31431,15 +32042,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A40,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A40,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A40,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A40,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A40,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A40,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -31454,15 +32065,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A41,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A41,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A41,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A41,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A41,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A41,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -31477,15 +32088,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A42,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A42,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A42,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A42,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A42,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A42,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -31500,15 +32111,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A43,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A43,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A43,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A43,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A43,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A43,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -31523,15 +32134,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A44,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A44,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A44,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A44,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A44,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A44,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -31546,15 +32157,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A45,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A45,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A45,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A45,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A45,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A45,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -31569,15 +32180,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A46,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A46,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A46,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A46,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A46,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A46,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -31592,15 +32203,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A47,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A47,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A47,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A47,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A47,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A47,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -31615,15 +32226,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A48,Fiches!$B$2:$B$461,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A48,Fiches!$B$2:$B$471,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A48,Fiches!$B$2:$B$461,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A48,Fiches!$B$2:$B$471,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$461,$A48,Fiches!$B$2:$B$461,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$471,$A48,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Applications : 8 fiches ajoutées d'après le cours de référence
Définition et égalité, composée et identité, propriétés de la composition,
caractérisations injection/surjection, bijection, réciproque, composée
d'injections/surjections/bijections, stricte monotonie ⇒ injectivité.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N471"/>
+  <dimension ref="A1:N479"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -28078,10 +28078,490 @@
       <c r="M471" s="11" t="n"/>
       <c r="N471" s="11" t="n"/>
     </row>
+    <row r="472">
+      <c r="A472" s="9" t="inlineStr">
+        <is>
+          <t>M471</t>
+        </is>
+      </c>
+      <c r="B472" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C472" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D472" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 6 – Vocabulaire des applications</t>
+        </is>
+      </c>
+      <c r="E472" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F472" s="9" t="inlineStr">
+        <is>
+          <t>Application – Définition et égalité</t>
+        </is>
+      </c>
+      <c r="G472" s="9" t="inlineStr">
+        <is>
+          <t>Soient $E$ et $F$ deux ensembles.</t>
+        </is>
+      </c>
+      <c r="H472" s="10" t="inlineStr">
+        <is>
+          <t>Définir une application $f:E\to F$, puis l'égalité de deux applications.</t>
+        </is>
+      </c>
+      <c r="I472" s="9" t="inlineStr">
+        <is>
+          <t>Une application $f:E\to F$ associe à chaque élément $x$ de $E$ (ensemble de départ) un unique élément $f(x)$ de $F$ (ensemble d'arrivée). Deux applications sont égales si elles ont le même ensemble de départ, le même ensemble d'arrivée, et $f(x)=g(x)$ pour tout $x$ de l'ensemble de départ.</t>
+        </is>
+      </c>
+      <c r="J472" s="9" t="inlineStr">
+        <is>
+          <t>« Application d'un ensemble de départ dans un ensemble d'arrivée. »</t>
+        </is>
+      </c>
+      <c r="K472" s="9" t="n"/>
+      <c r="L472" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Applications » 2024</t>
+        </is>
+      </c>
+      <c r="M472" s="11" t="n"/>
+      <c r="N472" s="11" t="n"/>
+    </row>
+    <row r="473">
+      <c r="A473" s="9" t="inlineStr">
+        <is>
+          <t>M472</t>
+        </is>
+      </c>
+      <c r="B473" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C473" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D473" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 6 – Vocabulaire des applications</t>
+        </is>
+      </c>
+      <c r="E473" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F473" s="9" t="inlineStr">
+        <is>
+          <t>Composée – Application identité</t>
+        </is>
+      </c>
+      <c r="G473" s="9" t="inlineStr">
+        <is>
+          <t>Soient $f:E\to F$ et $g:F\to G$ deux applications.</t>
+        </is>
+      </c>
+      <c r="H473" s="10" t="inlineStr">
+        <is>
+          <t>Définir la composée $g\circ f$ et l'application identité $\mathrm{Id}_E$.</t>
+        </is>
+      </c>
+      <c r="I473" s="9" t="inlineStr">
+        <is>
+          <t>$g\circ f:E\to G$, $x\mapsto g(f(x))$ ; $\mathrm{Id}_E:E\to E$, $x\mapsto x$.</t>
+        </is>
+      </c>
+      <c r="J473" s="9" t="inlineStr">
+        <is>
+          <t>« Composition. »</t>
+        </is>
+      </c>
+      <c r="K473" s="9" t="n"/>
+      <c r="L473" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Applications » 2024</t>
+        </is>
+      </c>
+      <c r="M473" s="11" t="n"/>
+      <c r="N473" s="11" t="n"/>
+    </row>
+    <row r="474">
+      <c r="A474" s="9" t="inlineStr">
+        <is>
+          <t>M473</t>
+        </is>
+      </c>
+      <c r="B474" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C474" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D474" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 6 – Vocabulaire des applications</t>
+        </is>
+      </c>
+      <c r="E474" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F474" s="9" t="inlineStr">
+        <is>
+          <t>Composition – Propriétés</t>
+        </is>
+      </c>
+      <c r="G474" s="9" t="inlineStr">
+        <is>
+          <t>Soient $f:E\to F$, $g:F\to G$ et $h:G\to H$ des applications.</t>
+        </is>
+      </c>
+      <c r="H474" s="10" t="inlineStr">
+        <is>
+          <t>Donner les propriétés de la composition : composition par l'identité, associativité, commutativité.</t>
+        </is>
+      </c>
+      <c r="I474" s="9" t="inlineStr">
+        <is>
+          <t>$\mathrm{Id}_F\circ f=f\circ\mathrm{Id}_E=f$ ; $h\circ(g\circ f)=(h\circ g)\circ f$ (associativité). La composition n'est pas commutative : en général $f\circ g\neq g\circ f$, même quand les deux existent.</t>
+        </is>
+      </c>
+      <c r="J474" s="9" t="inlineStr">
+        <is>
+          <t>« Composition. On étudie quelques exemples fournis par des fonctions de R dans R que l'on compose de diverses manières. »</t>
+        </is>
+      </c>
+      <c r="K474" s="9" t="n"/>
+      <c r="L474" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Applications » 2024</t>
+        </is>
+      </c>
+      <c r="M474" s="11" t="n"/>
+      <c r="N474" s="11" t="n"/>
+    </row>
+    <row r="475">
+      <c r="A475" s="9" t="inlineStr">
+        <is>
+          <t>M474</t>
+        </is>
+      </c>
+      <c r="B475" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C475" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D475" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 6 – Vocabulaire des applications</t>
+        </is>
+      </c>
+      <c r="E475" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F475" s="9" t="inlineStr">
+        <is>
+          <t>Injection, surjection – Caractérisations</t>
+        </is>
+      </c>
+      <c r="G475" s="9" t="inlineStr">
+        <is>
+          <t>Soit $f:E\to F$ une application.</t>
+        </is>
+      </c>
+      <c r="H475" s="10" t="inlineStr">
+        <is>
+          <t>Caractériser l'injectivité et la surjectivité de $f$ par les antécédents et par l'équation $y=f(x)$.</t>
+        </is>
+      </c>
+      <c r="I475" s="9" t="inlineStr">
+        <is>
+          <t>$f$ injective $\iff$ tout élément de $F$ a au plus un antécédent $\iff$ pour tout $y\in F$, l'équation $y=f(x)$ a au plus une solution dans $E$ $\iff$ ($x\neq x'\Rightarrow f(x)\neq f(x')$). $f$ surjective $\iff$ tout élément de $F$ a au moins un antécédent $\iff$ $f(E)=F$.</t>
+        </is>
+      </c>
+      <c r="J475" s="9" t="inlineStr">
+        <is>
+          <t>« Injection, surjection, bijection »</t>
+        </is>
+      </c>
+      <c r="K475" s="9" t="n"/>
+      <c r="L475" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Applications » 2024</t>
+        </is>
+      </c>
+      <c r="M475" s="11" t="n"/>
+      <c r="N475" s="11" t="n"/>
+    </row>
+    <row r="476">
+      <c r="A476" s="9" t="inlineStr">
+        <is>
+          <t>M475</t>
+        </is>
+      </c>
+      <c r="B476" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C476" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D476" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 6 – Vocabulaire des applications</t>
+        </is>
+      </c>
+      <c r="E476" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F476" s="9" t="inlineStr">
+        <is>
+          <t>Application bijective</t>
+        </is>
+      </c>
+      <c r="G476" s="9" t="inlineStr">
+        <is>
+          <t>Soit $f:E\to F$ une application.</t>
+        </is>
+      </c>
+      <c r="H476" s="10" t="inlineStr">
+        <is>
+          <t>Définir : $f$ est bijective, et donner deux caractérisations.</t>
+        </is>
+      </c>
+      <c r="I476" s="9" t="inlineStr">
+        <is>
+          <t>$\forall y\in F,\ \exists!\,x\in E,\ y=f(x)$. De façon équivalente : $f$ est injective et surjective ; tout élément de $F$ a exactement un antécédent par $f$.</t>
+        </is>
+      </c>
+      <c r="J476" s="9" t="inlineStr">
+        <is>
+          <t>« Injection, surjection, bijection »</t>
+        </is>
+      </c>
+      <c r="K476" s="9" t="n"/>
+      <c r="L476" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Applications » 2024</t>
+        </is>
+      </c>
+      <c r="M476" s="11" t="n"/>
+      <c r="N476" s="11" t="n"/>
+    </row>
+    <row r="477">
+      <c r="A477" s="9" t="inlineStr">
+        <is>
+          <t>M476</t>
+        </is>
+      </c>
+      <c r="B477" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C477" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D477" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 6 – Vocabulaire des applications</t>
+        </is>
+      </c>
+      <c r="E477" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F477" s="9" t="inlineStr">
+        <is>
+          <t>Application réciproque</t>
+        </is>
+      </c>
+      <c r="G477" s="9" t="inlineStr">
+        <is>
+          <t>Soit $f:E\to F$ une application bijective.</t>
+        </is>
+      </c>
+      <c r="H477" s="10" t="inlineStr">
+        <is>
+          <t>Définir l'application réciproque $f^{-1}$ et donner ses propriétés.</t>
+        </is>
+      </c>
+      <c r="I477" s="9" t="inlineStr">
+        <is>
+          <t>$f^{-1}:F\to E$ associe à $y$ son unique antécédent par $f$ : $y=f(x)\iff x=f^{-1}(y)$. On a $f\circ f^{-1}=\mathrm{Id}_F$ et $f^{-1}\circ f=\mathrm{Id}_E$ ; $f^{-1}$ est bijective et $(f^{-1})^{-1}=f$. Pour une bijection entre parties de $\mathbb R$, les graphes de $f$ et $f^{-1}$ sont symétriques par rapport à la droite $y=x$.</t>
+        </is>
+      </c>
+      <c r="J477" s="9" t="inlineStr">
+        <is>
+          <t>« application réciproque » ; « une bijection et sa réciproque ont des graphes symétriques l'un de l'autre par rapport à la première bissectrice. »</t>
+        </is>
+      </c>
+      <c r="K477" s="9" t="n"/>
+      <c r="L477" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Applications » 2024</t>
+        </is>
+      </c>
+      <c r="M477" s="11" t="n"/>
+      <c r="N477" s="11" t="n"/>
+    </row>
+    <row r="478">
+      <c r="A478" s="9" t="inlineStr">
+        <is>
+          <t>M477</t>
+        </is>
+      </c>
+      <c r="B478" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C478" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D478" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 6 – Vocabulaire des applications</t>
+        </is>
+      </c>
+      <c r="E478" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F478" s="9" t="inlineStr">
+        <is>
+          <t>Composée d’injections, de surjections, de bijections</t>
+        </is>
+      </c>
+      <c r="G478" s="9" t="inlineStr">
+        <is>
+          <t>Soient $f:E\to F$ et $g:F\to G$ deux applications.</t>
+        </is>
+      </c>
+      <c r="H478" s="10" t="inlineStr">
+        <is>
+          <t>Que dire de $g\circ f$ si $f$ et $g$ sont injectives ? surjectives ? bijectives ?</t>
+        </is>
+      </c>
+      <c r="I478" s="9" t="inlineStr">
+        <is>
+          <t>Injectives $\Rightarrow g\circ f$ injective ; surjectives $\Rightarrow g\circ f$ surjective ; bijectives $\Rightarrow g\circ f$ bijective et $(g\circ f)^{-1}=f^{-1}\circ g^{-1}$. Les réciproques sont fausses.</t>
+        </is>
+      </c>
+      <c r="J478" s="9" t="inlineStr">
+        <is>
+          <t>« Composée de deux bijections, réciproque de la composée. »</t>
+        </is>
+      </c>
+      <c r="K478" s="9" t="n"/>
+      <c r="L478" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Applications » 2024</t>
+        </is>
+      </c>
+      <c r="M478" s="11" t="n"/>
+      <c r="N478" s="11" t="n"/>
+    </row>
+    <row r="479">
+      <c r="A479" s="9" t="inlineStr">
+        <is>
+          <t>M478</t>
+        </is>
+      </c>
+      <c r="B479" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C479" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D479" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 6 – Vocabulaire des applications</t>
+        </is>
+      </c>
+      <c r="E479" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F479" s="9" t="inlineStr">
+        <is>
+          <t>Stricte monotonie et injectivité</t>
+        </is>
+      </c>
+      <c r="G479" s="9" t="inlineStr">
+        <is>
+          <t>Soient $A$ une partie de $\mathbb R$ et $f:A\to\mathbb R$.</t>
+        </is>
+      </c>
+      <c r="H479" s="10" t="inlineStr">
+        <is>
+          <t>Donner une condition suffisante d'injectivité de $f$ portant sur sa monotonie.</t>
+        </is>
+      </c>
+      <c r="I479" s="9" t="inlineStr">
+        <is>
+          <t>Si $f$ est strictement monotone sur $A$, alors $f$ est injective.</t>
+        </is>
+      </c>
+      <c r="J479" s="9" t="inlineStr">
+        <is>
+          <t>« on illustre les notions présentées par des exemples issus majoritairement de fonctions de R dans R. »</t>
+        </is>
+      </c>
+      <c r="K479" s="9" t="n"/>
+      <c r="L479" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Applications » 2024</t>
+        </is>
+      </c>
+      <c r="M479" s="11" t="n"/>
+      <c r="N479" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M471" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M479" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -31318,7 +31798,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$471,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$479,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -31333,7 +31813,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$471,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$479,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -31348,7 +31828,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$471,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$479,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -31375,7 +31855,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$471)</f>
+        <f>COUNTA(Fiches!$M$2:$M$479)</f>
         <v/>
       </c>
     </row>
@@ -31421,15 +31901,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A13,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A13,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A13,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A13,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A13,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A13,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -31444,15 +31924,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A14,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A14,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A14,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A14,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A14,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A14,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -31467,15 +31947,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A15,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A15,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A15,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A15,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A15,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A15,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -31490,15 +31970,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A16,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A16,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A16,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A16,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A16,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A16,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -31513,15 +31993,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A17,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A17,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A17,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A17,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A17,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A17,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -31536,15 +32016,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A18,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A18,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A18,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A18,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A18,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A18,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -31559,15 +32039,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A19,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A19,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A19,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A19,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A19,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A19,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -31582,15 +32062,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A20,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A20,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A20,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A20,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A20,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A20,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -31605,15 +32085,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A21,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A21,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A21,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A21,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A21,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A21,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -31628,15 +32108,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A22,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A22,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A22,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A22,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A22,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A22,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -31651,15 +32131,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A23,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A23,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A23,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A23,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A23,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A23,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -31674,15 +32154,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A24,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A24,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A24,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A24,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A24,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A24,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -31697,15 +32177,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A25,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A25,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A25,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A25,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A25,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A25,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -31720,15 +32200,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A26,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A26,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A26,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A26,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A26,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A26,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -31743,15 +32223,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A27,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A27,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A27,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A27,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A27,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A27,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -31766,15 +32246,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A28,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A28,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A28,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A28,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A28,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A28,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -31789,15 +32269,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A29,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A29,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A29,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A29,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A29,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A29,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -31812,15 +32292,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A30,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A30,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A30,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A30,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A30,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A30,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -31835,15 +32315,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A31,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A31,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A31,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A31,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A31,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A31,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -31858,15 +32338,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A32,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A32,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A32,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A32,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A32,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A32,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -31881,15 +32361,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A33,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A33,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A33,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A33,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A33,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A33,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -31904,15 +32384,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A34,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A34,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A34,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A34,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A34,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A34,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -31927,15 +32407,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A35,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A35,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A35,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A35,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A35,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A35,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -31950,15 +32430,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A36,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A36,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A36,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A36,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A36,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A36,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -31973,15 +32453,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A37,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A37,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A37,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A37,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A37,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A37,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -31996,15 +32476,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A38,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A38,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A38,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A38,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A38,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A38,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -32019,15 +32499,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A39,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A39,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A39,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A39,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A39,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A39,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -32042,15 +32522,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A40,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A40,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A40,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A40,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A40,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A40,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -32065,15 +32545,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A41,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A41,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A41,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A41,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A41,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A41,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -32088,15 +32568,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A42,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A42,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A42,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A42,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A42,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A42,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -32111,15 +32591,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A43,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A43,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A43,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A43,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A43,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A43,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -32134,15 +32614,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A44,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A44,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A44,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A44,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A44,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A44,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -32157,15 +32637,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A45,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A45,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A45,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A45,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A45,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A45,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -32180,15 +32660,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A46,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A46,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A46,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A46,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A46,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A46,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -32203,15 +32683,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A47,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A47,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A47,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A47,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A47,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A47,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -32226,15 +32706,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A48,Fiches!$B$2:$B$471,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A48,Fiches!$B$2:$B$479,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A48,Fiches!$B$2:$B$471,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A48,Fiches!$B$2:$B$479,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$471,$A48,Fiches!$B$2:$B$471,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$479,$A48,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Équations différentielles : 7 fiches ajoutées, M076 complétée, M072 retirée
D'après le cours de référence : homogène à coefficient constant, cas a et f
constants, superposition, vocabulaire et structure des solutions à l'ordre 2,
solutions particulières usuelles (orange : forme donnée par l'énoncé).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N479"/>
+  <dimension ref="A1:N486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4939,8 +4939,16 @@
         <v>40</v>
       </c>
       <c r="L73" s="12" t="inlineStr"/>
-      <c r="M73" s="14" t="n"/>
-      <c r="N73" s="14" t="n"/>
+      <c r="M73" s="14" t="inlineStr">
+        <is>
+          <t>Passer en rouge</t>
+        </is>
+      </c>
+      <c r="N73" s="14" t="inlineStr">
+        <is>
+          <t>Retirée : absente du cours « Équations différentielles linéaires » 2024 ; le programme ne cite que la primitive de t ↦ e^{iωt}.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
@@ -5159,7 +5167,7 @@
       </c>
       <c r="I77" s="9" t="inlineStr">
         <is>
-          <t>1) Résoudre l'équation homogène : $y=\lambda y_0$. 2) Chercher une solution particulière par variation de la constante ($y=\lambda(x)y_0(x)$).</t>
+          <t>1) Résoudre l'équation homogène : $y=\lambda y_0$ (avec $y_0=e^{-A}$, $A$ primitive de $\beta$). 2) Chercher une solution particulière par variation de la constante : $y=\lambda(x)e^{-A(x)}$ est solution si et seulement si $\lambda'(x)=\gamma(x)e^{A(x)}$, donc $\lambda$ est une primitive de $\gamma e^{A}$. 3) Additionner.</t>
         </is>
       </c>
       <c r="J77" s="9" t="inlineStr">
@@ -28558,10 +28566,430 @@
       <c r="M479" s="11" t="n"/>
       <c r="N479" s="11" t="n"/>
     </row>
+    <row r="480">
+      <c r="A480" s="9" t="inlineStr">
+        <is>
+          <t>M479</t>
+        </is>
+      </c>
+      <c r="B480" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C480" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D480" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 4 – Équations différentielles linéaires</t>
+        </is>
+      </c>
+      <c r="E480" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F480" s="9" t="inlineStr">
+        <is>
+          <t>EDL1 homogène à coefficient constant</t>
+        </is>
+      </c>
+      <c r="G480" s="9" t="inlineStr">
+        <is>
+          <t>Soient $a\in\mathbb R$ et l'équation homogène $(H)$ : $y'+ay=0$.</t>
+        </is>
+      </c>
+      <c r="H480" s="10" t="inlineStr">
+        <is>
+          <t>Donner les solutions de $(H)$ sur $\mathbb R$.</t>
+        </is>
+      </c>
+      <c r="I480" s="9" t="inlineStr">
+        <is>
+          <t>Les fonctions $x\mapsto Ce^{-ax}$, $C\in\mathbb R$.</t>
+        </is>
+      </c>
+      <c r="J480" s="9" t="inlineStr">
+        <is>
+          <t>« résolution de l'équation homogène associée, cas particulier où a est constante »</t>
+        </is>
+      </c>
+      <c r="K480" s="9" t="n"/>
+      <c r="L480" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Équations différentielles linéaires » 2024</t>
+        </is>
+      </c>
+      <c r="M480" s="11" t="n"/>
+      <c r="N480" s="11" t="n"/>
+    </row>
+    <row r="481">
+      <c r="A481" s="9" t="inlineStr">
+        <is>
+          <t>M480</t>
+        </is>
+      </c>
+      <c r="B481" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C481" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D481" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 4 – Équations différentielles linéaires</t>
+        </is>
+      </c>
+      <c r="E481" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F481" s="9" t="inlineStr">
+        <is>
+          <t>EDL1 à coefficient et second membre constants</t>
+        </is>
+      </c>
+      <c r="G481" s="9" t="inlineStr">
+        <is>
+          <t>Soient $a\neq0$ et $b$ deux réels, et l'équation $(E)$ : $y'+ay=b$.</t>
+        </is>
+      </c>
+      <c r="H481" s="10" t="inlineStr">
+        <is>
+          <t>Donner une solution particulière puis toutes les solutions de $(E)$ sur $\mathbb R$.</t>
+        </is>
+      </c>
+      <c r="I481" s="9" t="inlineStr">
+        <is>
+          <t>La fonction constante $x\mapsto\frac ba$ est solution ; les solutions sont $x\mapsto\frac ba+Ce^{-ax}$, $C\in\mathbb R$.</t>
+        </is>
+      </c>
+      <c r="J481" s="9" t="inlineStr">
+        <is>
+          <t>« cas particulier où a et f sont constantes »</t>
+        </is>
+      </c>
+      <c r="K481" s="9" t="n"/>
+      <c r="L481" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Équations différentielles linéaires » 2024</t>
+        </is>
+      </c>
+      <c r="M481" s="11" t="n"/>
+      <c r="N481" s="11" t="n"/>
+    </row>
+    <row r="482">
+      <c r="A482" s="9" t="inlineStr">
+        <is>
+          <t>M481</t>
+        </is>
+      </c>
+      <c r="B482" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C482" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D482" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 4 – Équations différentielles linéaires</t>
+        </is>
+      </c>
+      <c r="E482" s="9" t="inlineStr">
+        <is>
+          <t>Théorème</t>
+        </is>
+      </c>
+      <c r="F482" s="9" t="inlineStr">
+        <is>
+          <t>Principe de superposition</t>
+        </is>
+      </c>
+      <c r="G482" s="9" t="inlineStr">
+        <is>
+          <t>Soient $a$, $b_1$, $b_2$ des fonctions continues sur un intervalle $I$ (ou $a$, $b$ réels pour l'ordre 2).</t>
+        </is>
+      </c>
+      <c r="H482" s="10" t="inlineStr">
+        <is>
+          <t>Énoncer le principe de superposition pour une équation différentielle linéaire.</t>
+        </is>
+      </c>
+      <c r="I482" s="9" t="inlineStr">
+        <is>
+          <t>Si $f_1$ est solution de $y'+a(x)y=b_1(x)$ et $f_2$ de $y'+a(x)y=b_2(x)$, alors $f_1+f_2$ est solution de $y'+a(x)y=b_1(x)+b_2(x)$. De même à l'ordre 2 : si $f_i$ est solution de $y''+ay'+by=b_i(x)$, alors $f_1+f_2$ est solution de $y''+ay'+by=b_1(x)+b_2(x)$ (et pour $n$ seconds membres).</t>
+        </is>
+      </c>
+      <c r="J482" s="9" t="inlineStr">
+        <is>
+          <t>« principe de superposition » (premier et second ordre)</t>
+        </is>
+      </c>
+      <c r="K482" s="9" t="n"/>
+      <c r="L482" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Équations différentielles linéaires » 2024</t>
+        </is>
+      </c>
+      <c r="M482" s="11" t="n"/>
+      <c r="N482" s="11" t="n"/>
+    </row>
+    <row r="483">
+      <c r="A483" s="9" t="inlineStr">
+        <is>
+          <t>M482</t>
+        </is>
+      </c>
+      <c r="B483" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C483" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D483" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 4 – Équations différentielles linéaires</t>
+        </is>
+      </c>
+      <c r="E483" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F483" s="9" t="inlineStr">
+        <is>
+          <t>EDL2 à coefficients constants – Vocabulaire</t>
+        </is>
+      </c>
+      <c r="G483" s="9" t="inlineStr">
+        <is>
+          <t>Soient $\alpha\neq0$, $\beta$, $\gamma$ des réels, $\delta$ continue sur un intervalle $I$, et $(E)$ : $\alpha y''+\beta y'+\gamma y=\delta(x)$.</t>
+        </is>
+      </c>
+      <c r="H483" s="10" t="inlineStr">
+        <is>
+          <t>Définir une solution de $(E)$ sur $I$, l'équation homogène associée et l'équation caractéristique.</t>
+        </is>
+      </c>
+      <c r="I483" s="9" t="inlineStr">
+        <is>
+          <t>$f$ est solution sur $I$ si $f$ est deux fois dérivable et $\alpha f''(x)+\beta f'(x)+\gamma f(x)=\delta(x)$ pour tout $x\in I$. Équation homogène associée : $\alpha y''+\beta y'+\gamma y=0$. Équation caractéristique : $\alpha r^2+\beta r+\gamma=0$ (obtenue en cherchant des solutions $x\mapsto e^{rx}$).</t>
+        </is>
+      </c>
+      <c r="J483" s="9" t="inlineStr">
+        <is>
+          <t>« Résolution de ay″ + by′ + cy = f(t) […] La résolution de l'équation homogène se fera à l'aide de l'équation caractéristique. »</t>
+        </is>
+      </c>
+      <c r="K483" s="9" t="n"/>
+      <c r="L483" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Équations différentielles linéaires » 2024</t>
+        </is>
+      </c>
+      <c r="M483" s="11" t="n"/>
+      <c r="N483" s="11" t="n"/>
+    </row>
+    <row r="484">
+      <c r="A484" s="9" t="inlineStr">
+        <is>
+          <t>M483</t>
+        </is>
+      </c>
+      <c r="B484" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C484" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D484" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 4 – Équations différentielles linéaires</t>
+        </is>
+      </c>
+      <c r="E484" s="9" t="inlineStr">
+        <is>
+          <t>Théorème</t>
+        </is>
+      </c>
+      <c r="F484" s="9" t="inlineStr">
+        <is>
+          <t>EDL2 – Structure des solutions</t>
+        </is>
+      </c>
+      <c r="G484" s="9" t="inlineStr">
+        <is>
+          <t>Soient $a$, $b$ des réels, $c$ continue sur un intervalle $I$, et $(E)$ : $y''+ay'+by=c(x)$.</t>
+        </is>
+      </c>
+      <c r="H484" s="10" t="inlineStr">
+        <is>
+          <t>Donner la forme de la solution générale de $(E)$ et la méthode pratique de résolution.</t>
+        </is>
+      </c>
+      <c r="I484" s="9" t="inlineStr">
+        <is>
+          <t>Si $f_0$ est une solution particulière de $(E)$, les solutions de $(E)$ sont les $f_0+\varphi$, où $\varphi$ parcourt les solutions de l'équation homogène. Méthode : résoudre l'homogène (équation caractéristique), trouver une solution particulière, additionner.</t>
+        </is>
+      </c>
+      <c r="J484" s="9" t="inlineStr">
+        <is>
+          <t>« résolution de l'équation homogène associée, principe de superposition, détermination d'une solution particulière »</t>
+        </is>
+      </c>
+      <c r="K484" s="9" t="n"/>
+      <c r="L484" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Équations différentielles linéaires » 2024</t>
+        </is>
+      </c>
+      <c r="M484" s="11" t="n"/>
+      <c r="N484" s="11" t="n"/>
+    </row>
+    <row r="485">
+      <c r="A485" s="9" t="inlineStr">
+        <is>
+          <t>M484</t>
+        </is>
+      </c>
+      <c r="B485" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C485" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D485" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 4 – Équations différentielles linéaires</t>
+        </is>
+      </c>
+      <c r="E485" s="9" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+      <c r="F485" s="9" t="inlineStr">
+        <is>
+          <t>EDL1 à coefficient constant – Solutions particulières usuelles</t>
+        </is>
+      </c>
+      <c r="G485" s="9" t="inlineStr">
+        <is>
+          <t>Soient $a\neq0$ un réel, $m$ un réel, $P$ un polynôme, et l'équation $y'+ay=g(x)$.</t>
+        </is>
+      </c>
+      <c r="H485" s="10" t="inlineStr">
+        <is>
+          <t>Quelle forme de solution particulière chercher si $g(x)=P(x)$ ? $P(x)e^{mx}$ ? $P(x)\cos(mx)$ ?</t>
+        </is>
+      </c>
+      <c r="I485" s="9" t="inlineStr">
+        <is>
+          <t>$g=P$ : un polynôme de même degré que $P$. $g=Pe^{mx}$ : $Q(x)e^{mx}$ avec $\deg Q=\deg P$ si $m\neq-a$, et $xQ(x)e^{mx}$ si $m=-a$. $g=P\cos(mx)$ ($m\neq0$) : $Q_1(x)\cos(mx)+Q_2(x)\sin(mx)$ avec $\deg Q_1=\deg Q_2=\deg P$.</t>
+        </is>
+      </c>
+      <c r="J485" s="9" t="inlineStr">
+        <is>
+          <t>Programme : « Pour toute autre équation différentielle du premier ordre, une méthode de résolution doit être fournie. » La forme est donc normalement donnée par l'énoncé.</t>
+        </is>
+      </c>
+      <c r="K485" s="9" t="n"/>
+      <c r="L485" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Équations différentielles linéaires » 2024</t>
+        </is>
+      </c>
+      <c r="M485" s="11" t="n"/>
+      <c r="N485" s="11" t="n"/>
+    </row>
+    <row r="486">
+      <c r="A486" s="9" t="inlineStr">
+        <is>
+          <t>M485</t>
+        </is>
+      </c>
+      <c r="B486" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C486" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D486" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 4 – Équations différentielles linéaires</t>
+        </is>
+      </c>
+      <c r="E486" s="9" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+      <c r="F486" s="9" t="inlineStr">
+        <is>
+          <t>EDL2 – Solutions particulières (polynôme, cosinus)</t>
+        </is>
+      </c>
+      <c r="G486" s="9" t="inlineStr">
+        <is>
+          <t>Soient $a$, $b$ des réels, $m\neq0$ un réel, $P$ un polynôme, et $(E)$ : $y''+ay'+by=g(x)$.</t>
+        </is>
+      </c>
+      <c r="H486" s="10" t="inlineStr">
+        <is>
+          <t>Quelle forme de solution particulière chercher si $g(x)=P(x)$ ? si $g(x)=P(x)\cos(mx)$ ?</t>
+        </is>
+      </c>
+      <c r="I486" s="9" t="inlineStr">
+        <is>
+          <t>$g=P$ et $b\neq0$ : un polynôme de même degré que $P$ (si $b=0$ et $a\neq0$ : degré $\deg P+1$). $g=P\cos(mx)$ : $Q_1(x)\cos(mx)+Q_2(x)\sin(mx)$ avec $\deg Q_i=\deg P$ si $im$ n'est pas racine de l'équation caractéristique, et $x\big(Q_1(x)\cos(mx)+Q_2(x)\sin(mx)\big)$ si $im$ est racine.</t>
+        </is>
+      </c>
+      <c r="J486" s="9" t="inlineStr">
+        <is>
+          <t>Programme : « La forme d'une solution particulière est donnée sauf lorsque f est une fonction constante. »</t>
+        </is>
+      </c>
+      <c r="K486" s="9" t="n"/>
+      <c r="L486" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Équations différentielles linéaires » 2024</t>
+        </is>
+      </c>
+      <c r="M486" s="11" t="n"/>
+      <c r="N486" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M479" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M486" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -31798,7 +32226,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$479,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$486,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -31813,7 +32241,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$479,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$486,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -31828,7 +32256,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$479,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$486,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -31855,7 +32283,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$479)</f>
+        <f>COUNTA(Fiches!$M$2:$M$486)</f>
         <v/>
       </c>
     </row>
@@ -31901,15 +32329,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A13,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A13,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A13,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A13,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A13,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A13,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -31924,15 +32352,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A14,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A14,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A14,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A14,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A14,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A14,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -31947,15 +32375,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A15,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A15,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A15,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A15,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A15,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A15,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -31970,15 +32398,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A16,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A16,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A16,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A16,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A16,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A16,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -31993,15 +32421,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A17,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A17,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A17,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A17,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A17,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A17,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -32016,15 +32444,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A18,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A18,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A18,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A18,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A18,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A18,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -32039,15 +32467,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A19,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A19,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A19,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A19,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A19,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A19,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -32062,15 +32490,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A20,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A20,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A20,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A20,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A20,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A20,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -32085,15 +32513,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A21,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A21,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A21,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A21,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A21,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A21,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -32108,15 +32536,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A22,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A22,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A22,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A22,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A22,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A22,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -32131,15 +32559,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A23,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A23,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A23,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A23,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A23,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A23,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -32154,15 +32582,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A24,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A24,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A24,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A24,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A24,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A24,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -32177,15 +32605,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A25,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A25,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A25,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A25,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A25,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A25,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -32200,15 +32628,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A26,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A26,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A26,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A26,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A26,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A26,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -32223,15 +32651,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A27,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A27,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A27,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A27,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A27,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A27,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -32246,15 +32674,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A28,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A28,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A28,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A28,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A28,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A28,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -32269,15 +32697,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A29,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A29,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A29,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A29,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A29,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A29,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -32292,15 +32720,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A30,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A30,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A30,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A30,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A30,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A30,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -32315,15 +32743,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A31,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A31,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A31,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A31,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A31,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A31,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -32338,15 +32766,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A32,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A32,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A32,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A32,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A32,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A32,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -32361,15 +32789,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A33,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A33,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A33,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A33,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A33,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A33,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -32384,15 +32812,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A34,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A34,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A34,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A34,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A34,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A34,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -32407,15 +32835,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A35,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A35,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A35,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A35,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A35,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A35,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -32430,15 +32858,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A36,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A36,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A36,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A36,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A36,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A36,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -32453,15 +32881,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A37,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A37,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A37,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A37,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A37,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A37,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -32476,15 +32904,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A38,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A38,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A38,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A38,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A38,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A38,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -32499,15 +32927,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A39,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A39,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A39,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A39,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A39,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A39,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -32522,15 +32950,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A40,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A40,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A40,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A40,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A40,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A40,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -32545,15 +32973,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A41,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A41,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A41,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A41,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A41,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A41,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -32568,15 +32996,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A42,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A42,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A42,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A42,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A42,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A42,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -32591,15 +33019,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A43,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A43,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A43,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A43,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A43,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A43,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -32614,15 +33042,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A44,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A44,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A44,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A44,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A44,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A44,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -32637,15 +33065,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A45,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A45,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A45,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A45,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A45,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A45,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -32660,15 +33088,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A46,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A46,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A46,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A46,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A46,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A46,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -32683,15 +33111,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A47,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A47,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A47,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A47,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A47,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A47,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -32706,15 +33134,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A48,Fiches!$B$2:$B$479,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A48,Fiches!$B$2:$B$486,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A48,Fiches!$B$2:$B$479,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A48,Fiches!$B$2:$B$486,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$479,$A48,Fiches!$B$2:$B$479,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$486,$A48,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Fonctions usuelles : 18 fiches ajoutées d'après le cours de référence
Vocabulaire (ensemble de définition, monotonie, parité, périodicité, bornée,
fonctions associées) et fonctions usuelles (ln, exp, a^b, a^x, x^α, log,
puissances entières, racine, sin/cos, tan, valeur absolue).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N486"/>
+  <dimension ref="A1:N504"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -28986,10 +28986,1090 @@
       <c r="M486" s="11" t="n"/>
       <c r="N486" s="11" t="n"/>
     </row>
+    <row r="487">
+      <c r="A487" s="9" t="inlineStr">
+        <is>
+          <t>M486</t>
+        </is>
+      </c>
+      <c r="B487" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C487" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D487" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E487" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F487" s="9" t="inlineStr">
+        <is>
+          <t>Ensemble de définition</t>
+        </is>
+      </c>
+      <c r="G487" s="9" t="inlineStr">
+        <is>
+          <t>Soit $f(x)$ une expression dépendant d'une variable réelle $x$.</t>
+        </is>
+      </c>
+      <c r="H487" s="10" t="inlineStr">
+        <is>
+          <t>Définir l'ensemble de définition $D_f$ de $f$.</t>
+        </is>
+      </c>
+      <c r="I487" s="9" t="inlineStr">
+        <is>
+          <t>$D_f$ est l'ensemble des réels $x$ pour lesquels $f(x)$ existe. Attention : $f$ (la fonction) et $f(x)$ (un nombre) sont deux objets différents.</t>
+        </is>
+      </c>
+      <c r="J487" s="9" t="inlineStr">
+        <is>
+          <t>« Ensemble de définition. »</t>
+        </is>
+      </c>
+      <c r="K487" s="9" t="n"/>
+      <c r="L487" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les fonctions usuelles » 2024</t>
+        </is>
+      </c>
+      <c r="M487" s="11" t="n"/>
+      <c r="N487" s="11" t="n"/>
+    </row>
+    <row r="488">
+      <c r="A488" s="9" t="inlineStr">
+        <is>
+          <t>M487</t>
+        </is>
+      </c>
+      <c r="B488" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C488" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D488" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E488" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F488" s="9" t="inlineStr">
+        <is>
+          <t>Fonction monotone – Définitions</t>
+        </is>
+      </c>
+      <c r="G488" s="9" t="inlineStr">
+        <is>
+          <t>Soit $f$ une fonction définie sur une partie $I$ de $\mathbb R$.</t>
+        </is>
+      </c>
+      <c r="H488" s="10" t="inlineStr">
+        <is>
+          <t>Définir : $f$ est croissante, strictement croissante, monotone, strictement monotone sur $I$.</t>
+        </is>
+      </c>
+      <c r="I488" s="9" t="inlineStr">
+        <is>
+          <t>Croissante : $\forall(x,y)\in I^2,\ x&lt;y\Rightarrow f(x)\le f(y)$ ; strictement croissante : $x&lt;y\Rightarrow f(x)&lt;f(y)$ (de même pour décroissante avec $\ge$ et $&gt;$). Monotone : croissante ou décroissante ; strictement monotone : strictement croissante ou strictement décroissante.</t>
+        </is>
+      </c>
+      <c r="J488" s="9" t="inlineStr">
+        <is>
+          <t>« Monotonie. »</t>
+        </is>
+      </c>
+      <c r="K488" s="9" t="n"/>
+      <c r="L488" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les fonctions usuelles » 2024</t>
+        </is>
+      </c>
+      <c r="M488" s="11" t="n"/>
+      <c r="N488" s="11" t="n"/>
+    </row>
+    <row r="489">
+      <c r="A489" s="9" t="inlineStr">
+        <is>
+          <t>M488</t>
+        </is>
+      </c>
+      <c r="B489" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C489" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D489" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E489" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F489" s="9" t="inlineStr">
+        <is>
+          <t>Fonction paire, fonction impaire</t>
+        </is>
+      </c>
+      <c r="G489" s="9" t="inlineStr">
+        <is>
+          <t>Soit $f$ une fonction définie sur une partie $I$ de $\mathbb R$.</t>
+        </is>
+      </c>
+      <c r="H489" s="10" t="inlineStr">
+        <is>
+          <t>Définir : $f$ est paire, $f$ est impaire, et donner l'interprétation graphique.</t>
+        </is>
+      </c>
+      <c r="I489" s="9" t="inlineStr">
+        <is>
+          <t>Dans les deux cas $I$ est symétrique : $\forall x\in I,\ -x\in I$. Paire : $f(-x)=f(x)$ pour tout $x\in I$, courbe symétrique par rapport à l'axe des ordonnées. Impaire : $f(-x)=-f(x)$, courbe symétrique par rapport à l'origine.</t>
+        </is>
+      </c>
+      <c r="J489" s="9" t="inlineStr">
+        <is>
+          <t>« Parité, périodicité. Interprétation géométrique de ces propriétés. »</t>
+        </is>
+      </c>
+      <c r="K489" s="9" t="n"/>
+      <c r="L489" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les fonctions usuelles » 2024</t>
+        </is>
+      </c>
+      <c r="M489" s="11" t="n"/>
+      <c r="N489" s="11" t="n"/>
+    </row>
+    <row r="490">
+      <c r="A490" s="9" t="inlineStr">
+        <is>
+          <t>M489</t>
+        </is>
+      </c>
+      <c r="B490" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C490" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D490" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E490" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F490" s="9" t="inlineStr">
+        <is>
+          <t>Fonction périodique</t>
+        </is>
+      </c>
+      <c r="G490" s="9" t="inlineStr">
+        <is>
+          <t>Soient $f$ une fonction définie sur une partie $I$ de $\mathbb R$ et $T&gt;0$.</t>
+        </is>
+      </c>
+      <c r="H490" s="10" t="inlineStr">
+        <is>
+          <t>Définir : $f$ est $T$-périodique, et donner l'interprétation graphique.</t>
+        </is>
+      </c>
+      <c r="I490" s="9" t="inlineStr">
+        <is>
+          <t>Pour tout $x\in I$, $x+T\in I$ et $f(x+T)=f(x)$. La courbe est invariante par la translation de vecteur $T\vec\imath$ : on l'étudie sur un intervalle de longueur $T$.</t>
+        </is>
+      </c>
+      <c r="J490" s="9" t="inlineStr">
+        <is>
+          <t>« Parité, périodicité. Interprétation géométrique de ces propriétés. »</t>
+        </is>
+      </c>
+      <c r="K490" s="9" t="n"/>
+      <c r="L490" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les fonctions usuelles » 2024</t>
+        </is>
+      </c>
+      <c r="M490" s="11" t="n"/>
+      <c r="N490" s="11" t="n"/>
+    </row>
+    <row r="491">
+      <c r="A491" s="9" t="inlineStr">
+        <is>
+          <t>M490</t>
+        </is>
+      </c>
+      <c r="B491" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C491" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D491" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E491" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F491" s="9" t="inlineStr">
+        <is>
+          <t>Fonction bornée – Caractérisation</t>
+        </is>
+      </c>
+      <c r="G491" s="9" t="inlineStr">
+        <is>
+          <t>Soit $f$ une fonction définie sur une partie $I$ de $\mathbb R$.</t>
+        </is>
+      </c>
+      <c r="H491" s="10" t="inlineStr">
+        <is>
+          <t>Caractériser à l'aide de $|f|$ le fait que $f$ est bornée sur $I$.</t>
+        </is>
+      </c>
+      <c r="I491" s="9" t="inlineStr">
+        <is>
+          <t>$f$ est bornée sur $I$ si et seulement si $\exists C\in\mathbb R,\ \forall x\in I,\ |f(x)|\le C$.</t>
+        </is>
+      </c>
+      <c r="J491" s="9" t="inlineStr">
+        <is>
+          <t>« Fonctions majorées, minorées, bornées. »</t>
+        </is>
+      </c>
+      <c r="K491" s="9" t="n"/>
+      <c r="L491" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les fonctions usuelles » 2024</t>
+        </is>
+      </c>
+      <c r="M491" s="11" t="n"/>
+      <c r="N491" s="11" t="n"/>
+    </row>
+    <row r="492">
+      <c r="A492" s="9" t="inlineStr">
+        <is>
+          <t>M491</t>
+        </is>
+      </c>
+      <c r="B492" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C492" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D492" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E492" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F492" s="9" t="inlineStr">
+        <is>
+          <t>Graphes des fonctions associées</t>
+        </is>
+      </c>
+      <c r="G492" s="9" t="inlineStr">
+        <is>
+          <t>Soient $f$ une fonction, $\mathcal C$ sa courbe et $a$ un réel non nul.</t>
+        </is>
+      </c>
+      <c r="H492" s="10" t="inlineStr">
+        <is>
+          <t>Comment obtenir à partir de $\mathcal C$ les courbes de $x\mapsto f(x)+a$, $f(x+a)$, $af(x)$, $f(ax)$ et $f(a-x)$ ?</t>
+        </is>
+      </c>
+      <c r="I492" s="9" t="inlineStr">
+        <is>
+          <t>$f(x)+a$ : translation de vecteur $a\vec\jmath$. $f(x+a)$ : translation de vecteur $-a\vec\imath$. $af(x)$ : ordonnées multipliées par $a$. $f(ax)$ : abscisses divisées par $a$. $f(a-x)$ : symétrie par rapport à la droite $x=\frac a2$.</t>
+        </is>
+      </c>
+      <c r="J492" s="9" t="inlineStr">
+        <is>
+          <t>« Graphes des fonctions x ↦ f(x) + a, x ↦ f(a − x), x ↦ f(ax), x ↦ af(x). »</t>
+        </is>
+      </c>
+      <c r="K492" s="9" t="n"/>
+      <c r="L492" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les fonctions usuelles » 2024</t>
+        </is>
+      </c>
+      <c r="M492" s="11" t="n"/>
+      <c r="N492" s="11" t="n"/>
+    </row>
+    <row r="493">
+      <c r="A493" s="9" t="inlineStr">
+        <is>
+          <t>M492</t>
+        </is>
+      </c>
+      <c r="B493" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C493" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D493" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E493" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F493" s="9" t="inlineStr">
+        <is>
+          <t>Logarithme népérien – Propriétés algébriques</t>
+        </is>
+      </c>
+      <c r="G493" s="9" t="inlineStr">
+        <is>
+          <t>Soient $a$ et $b$ deux réels strictement positifs et $n\in\mathbb Z$.</t>
+        </is>
+      </c>
+      <c r="H493" s="10" t="inlineStr">
+        <is>
+          <t>Donner les propriétés algébriques de $\ln$.</t>
+        </is>
+      </c>
+      <c r="I493" s="9" t="inlineStr">
+        <is>
+          <t>$\ln1=0$ ; $\ln(ab)=\ln a+\ln b$ ; $\ln\frac ab=\ln a-\ln b$ ; $\ln\frac1a=-\ln a$ ; $\ln(a^n)=n\ln a$ ; $\ln\sqrt a=\frac12\ln a$.</t>
+        </is>
+      </c>
+      <c r="J493" s="9" t="inlineStr">
+        <is>
+          <t>« Fonctions exponentielle et logarithme népérien (ln). » ; la maîtrise attendue porte sur « les principales propriétés ».</t>
+        </is>
+      </c>
+      <c r="K493" s="9" t="n"/>
+      <c r="L493" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les fonctions usuelles » 2024</t>
+        </is>
+      </c>
+      <c r="M493" s="11" t="n"/>
+      <c r="N493" s="11" t="n"/>
+    </row>
+    <row r="494">
+      <c r="A494" s="9" t="inlineStr">
+        <is>
+          <t>M493</t>
+        </is>
+      </c>
+      <c r="B494" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C494" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D494" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E494" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F494" s="9" t="inlineStr">
+        <is>
+          <t>Logarithme népérien – Étude</t>
+        </is>
+      </c>
+      <c r="G494" s="9" t="inlineStr">
+        <is>
+          <t>On considère la fonction $\ln$.</t>
+        </is>
+      </c>
+      <c r="H494" s="10" t="inlineStr">
+        <is>
+          <t>Donner l'ensemble de définition, la dérivée, les variations et les limites de $\ln$.</t>
+        </is>
+      </c>
+      <c r="I494" s="9" t="inlineStr">
+        <is>
+          <t>$\ln$ est définie et dérivable sur $]0,+\infty[$, $\ln'(x)=\frac1x$ ; strictement croissante ; $\lim_{0^+}\ln=-\infty$, $\lim_{+\infty}\ln=+\infty$ ; $\ln e=1$ ; courbe concave.</t>
+        </is>
+      </c>
+      <c r="J494" s="9" t="inlineStr">
+        <is>
+          <t>« Pour chaque fonction, la maitrise attendue concerne la définition, les principales propriétés, la formule de dérivation (avec son domaine de validité) et la courbe représentative. »</t>
+        </is>
+      </c>
+      <c r="K494" s="9" t="n"/>
+      <c r="L494" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les fonctions usuelles » 2024</t>
+        </is>
+      </c>
+      <c r="M494" s="11" t="n"/>
+      <c r="N494" s="11" t="n"/>
+    </row>
+    <row r="495">
+      <c r="A495" s="9" t="inlineStr">
+        <is>
+          <t>M494</t>
+        </is>
+      </c>
+      <c r="B495" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C495" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D495" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E495" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F495" s="9" t="inlineStr">
+        <is>
+          <t>Exponentielle – Propriétés et étude</t>
+        </is>
+      </c>
+      <c r="G495" s="9" t="inlineStr">
+        <is>
+          <t>Soient $a$ et $b$ deux réels et $n\in\mathbb Z$.</t>
+        </is>
+      </c>
+      <c r="H495" s="10" t="inlineStr">
+        <is>
+          <t>Donner les propriétés algébriques de $\exp$, puis sa dérivée, ses variations et ses limites.</t>
+        </is>
+      </c>
+      <c r="I495" s="9" t="inlineStr">
+        <is>
+          <t>$e^{a+b}=e^ae^b$ ; $e^{-a}=\frac1{e^a}$ ; $(e^a)^n=e^{na}$ ; $\ln(e^a)=a$ et $e^{\ln x}=x$ pour $x&gt;0$. $\exp$ est définie et dérivable sur $\mathbb R$, $\exp'=\exp$, strictement croissante, à valeurs dans $]0,+\infty[$ ; $\lim_{-\infty}\exp=0$, $\lim_{+\infty}\exp=+\infty$ ; courbe convexe.</t>
+        </is>
+      </c>
+      <c r="J495" s="9" t="inlineStr">
+        <is>
+          <t>« Fonctions exponentielle et logarithme népérien (ln). »</t>
+        </is>
+      </c>
+      <c r="K495" s="9" t="n"/>
+      <c r="L495" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les fonctions usuelles » 2024</t>
+        </is>
+      </c>
+      <c r="M495" s="11" t="n"/>
+      <c r="N495" s="11" t="n"/>
+    </row>
+    <row r="496">
+      <c r="A496" s="9" t="inlineStr">
+        <is>
+          <t>M495</t>
+        </is>
+      </c>
+      <c r="B496" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C496" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D496" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E496" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F496" s="9" t="inlineStr">
+        <is>
+          <t>Notation $a^b$ et règles de calcul</t>
+        </is>
+      </c>
+      <c r="G496" s="9" t="inlineStr">
+        <is>
+          <t>Soient $a$, $a'$ deux réels strictement positifs et $b$, $c$ deux réels.</t>
+        </is>
+      </c>
+      <c r="H496" s="10" t="inlineStr">
+        <is>
+          <t>Définir $a^b$ et donner les règles de calcul sur les puissances réelles.</t>
+        </is>
+      </c>
+      <c r="I496" s="9" t="inlineStr">
+        <is>
+          <t>$a^b=e^{b\ln a}$. $a^{b+c}=a^ba^c$ ; $a^{-b}=\frac1{a^b}$ ; $(a^b)^c=a^{bc}$ ; $(aa')^b=a^ba'^b$ ; $\ln(a^b)=b\ln a$.</t>
+        </is>
+      </c>
+      <c r="J496" s="9" t="inlineStr">
+        <is>
+          <t>« Notation a^b. On généralise les propriétés évoquées dans Outils 2. »</t>
+        </is>
+      </c>
+      <c r="K496" s="9" t="n"/>
+      <c r="L496" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les fonctions usuelles » 2024</t>
+        </is>
+      </c>
+      <c r="M496" s="11" t="n"/>
+      <c r="N496" s="11" t="n"/>
+    </row>
+    <row r="497">
+      <c r="A497" s="9" t="inlineStr">
+        <is>
+          <t>M496</t>
+        </is>
+      </c>
+      <c r="B497" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C497" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D497" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E497" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F497" s="9" t="inlineStr">
+        <is>
+          <t>Exponentielle de base $a$</t>
+        </is>
+      </c>
+      <c r="G497" s="9" t="inlineStr">
+        <is>
+          <t>Soit $a$ un réel strictement positif.</t>
+        </is>
+      </c>
+      <c r="H497" s="10" t="inlineStr">
+        <is>
+          <t>Donner l'ensemble de définition, l'expression, la dérivée et les variations de $x\mapsto a^x$.</t>
+        </is>
+      </c>
+      <c r="I497" s="9" t="inlineStr">
+        <is>
+          <t>$x\mapsto a^x=e^{x\ln a}$ est définie et dérivable sur $\mathbb R$, de dérivée $x\mapsto\ln(a)\,a^x$. Strictement croissante si $a&gt;1$, strictement décroissante si $0&lt;a&lt;1$, constante égale à $1$ si $a=1$.</t>
+        </is>
+      </c>
+      <c r="J497" s="9" t="inlineStr">
+        <is>
+          <t>« Fonctions exponentielles : x ↦ a^x avec a ∈ R*+. »</t>
+        </is>
+      </c>
+      <c r="K497" s="9" t="n"/>
+      <c r="L497" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les fonctions usuelles » 2024</t>
+        </is>
+      </c>
+      <c r="M497" s="11" t="n"/>
+      <c r="N497" s="11" t="n"/>
+    </row>
+    <row r="498">
+      <c r="A498" s="9" t="inlineStr">
+        <is>
+          <t>M497</t>
+        </is>
+      </c>
+      <c r="B498" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C498" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D498" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E498" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F498" s="9" t="inlineStr">
+        <is>
+          <t>Fonction puissance $x\mapsto x^\alpha$ ($\alpha$ réel)</t>
+        </is>
+      </c>
+      <c r="G498" s="9" t="inlineStr">
+        <is>
+          <t>Soit $\alpha\in\mathbb R\setminus\mathbb Z$.</t>
+        </is>
+      </c>
+      <c r="H498" s="10" t="inlineStr">
+        <is>
+          <t>Donner l'ensemble de définition, l'expression, la dérivée, les variations et la limite en $0^+$ de $x\mapsto x^\alpha$.</t>
+        </is>
+      </c>
+      <c r="I498" s="9" t="inlineStr">
+        <is>
+          <t>Définie et dérivable sur $]0,+\infty[$ par $x^\alpha=e^{\alpha\ln x}$ ; dérivée $\alpha x^{\alpha-1}$. Si $\alpha&gt;0$ : strictement croissante, $\lim_{0^+}x^\alpha=0$, $\lim_{+\infty}x^\alpha=+\infty$. Si $\alpha&lt;0$ : strictement décroissante, $\lim_{0^+}x^\alpha=+\infty$, $\lim_{+\infty}x^\alpha=0$.</t>
+        </is>
+      </c>
+      <c r="J498" s="9" t="inlineStr">
+        <is>
+          <t>« Fonctions puissances : x ↦ x^α avec α ∈ R \ Z ; x ↦ x^α est définie sur R*+. »</t>
+        </is>
+      </c>
+      <c r="K498" s="9" t="n"/>
+      <c r="L498" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les fonctions usuelles » 2024</t>
+        </is>
+      </c>
+      <c r="M498" s="11" t="n"/>
+      <c r="N498" s="11" t="n"/>
+    </row>
+    <row r="499">
+      <c r="A499" s="9" t="inlineStr">
+        <is>
+          <t>M498</t>
+        </is>
+      </c>
+      <c r="B499" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C499" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D499" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E499" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F499" s="9" t="inlineStr">
+        <is>
+          <t>Logarithme décimal</t>
+        </is>
+      </c>
+      <c r="G499" s="9" t="inlineStr">
+        <is>
+          <t>Soit $x$ un réel strictement positif.</t>
+        </is>
+      </c>
+      <c r="H499" s="10" t="inlineStr">
+        <is>
+          <t>Définir $\log x$ et donner ses propriétés principales.</t>
+        </is>
+      </c>
+      <c r="I499" s="9" t="inlineStr">
+        <is>
+          <t>$\log x=\dfrac{\ln x}{\ln10}$. $\log(10^n)=n$ ; $\log(ab)=\log a+\log b$ ; $\log$ est dérivable sur $]0,+\infty[$ de dérivée $\frac1{x\ln10}$, strictement croissante.</t>
+        </is>
+      </c>
+      <c r="J499" s="9" t="inlineStr">
+        <is>
+          <t>« Fonction logarithme décimal (log). Les logarithmes dans une base différente de e et 10 sont hors programme. »</t>
+        </is>
+      </c>
+      <c r="K499" s="9" t="n"/>
+      <c r="L499" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les fonctions usuelles » 2024</t>
+        </is>
+      </c>
+      <c r="M499" s="11" t="n"/>
+      <c r="N499" s="11" t="n"/>
+    </row>
+    <row r="500">
+      <c r="A500" s="9" t="inlineStr">
+        <is>
+          <t>M499</t>
+        </is>
+      </c>
+      <c r="B500" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C500" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D500" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E500" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F500" s="9" t="inlineStr">
+        <is>
+          <t>Fonctions puissances d’exposant entier</t>
+        </is>
+      </c>
+      <c r="G500" s="9" t="inlineStr">
+        <is>
+          <t>Soit $n\in\mathbb N^*$.</t>
+        </is>
+      </c>
+      <c r="H500" s="10" t="inlineStr">
+        <is>
+          <t>Donner l'ensemble de définition, la parité et la dérivée de $x\mapsto x^n$ et de $x\mapsto\frac1{x^n}$.</t>
+        </is>
+      </c>
+      <c r="I500" s="9" t="inlineStr">
+        <is>
+          <t>$x\mapsto x^n$ : définie sur $\mathbb R$, de même parité que $n$, dérivée $nx^{n-1}$. $x\mapsto\frac1{x^n}=x^{-n}$ : définie sur $\mathbb R^*$, de même parité que $n$, dérivée $-\dfrac n{x^{n+1}}$.</t>
+        </is>
+      </c>
+      <c r="J500" s="9" t="inlineStr">
+        <is>
+          <t>« Fonctions puissances d'exposant entier (dans Z) »</t>
+        </is>
+      </c>
+      <c r="K500" s="9" t="n"/>
+      <c r="L500" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les fonctions usuelles » 2024</t>
+        </is>
+      </c>
+      <c r="M500" s="11" t="n"/>
+      <c r="N500" s="11" t="n"/>
+    </row>
+    <row r="501">
+      <c r="A501" s="9" t="inlineStr">
+        <is>
+          <t>M500</t>
+        </is>
+      </c>
+      <c r="B501" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C501" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D501" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E501" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F501" s="9" t="inlineStr">
+        <is>
+          <t>Fonction racine carrée</t>
+        </is>
+      </c>
+      <c r="G501" s="9" t="inlineStr">
+        <is>
+          <t>Soient $x$ et $y$ deux réels positifs, et $t$ un réel.</t>
+        </is>
+      </c>
+      <c r="H501" s="10" t="inlineStr">
+        <is>
+          <t>Donner l'ensemble de définition, la dérivée (avec son domaine) et les propriétés de calcul de $\sqrt{\ }$.</t>
+        </is>
+      </c>
+      <c r="I501" s="9" t="inlineStr">
+        <is>
+          <t>Définie sur $[0,+\infty[$, dérivable sur $]0,+\infty[$ seulement, de dérivée $\frac1{2\sqrt x}$ ; strictement croissante. $\sqrt{xy}=\sqrt x\sqrt y$ ; $\sqrt{t^2}=|t|$.</t>
+        </is>
+      </c>
+      <c r="J501" s="9" t="inlineStr">
+        <is>
+          <t>« Fonction racine carrée. » ; Outils 2 : « √(x²) = |x|, √(xy) = √x √y »</t>
+        </is>
+      </c>
+      <c r="K501" s="9" t="n"/>
+      <c r="L501" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les fonctions usuelles » 2024</t>
+        </is>
+      </c>
+      <c r="M501" s="11" t="n"/>
+      <c r="N501" s="11" t="n"/>
+    </row>
+    <row r="502">
+      <c r="A502" s="9" t="inlineStr">
+        <is>
+          <t>M501</t>
+        </is>
+      </c>
+      <c r="B502" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C502" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D502" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E502" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F502" s="9" t="inlineStr">
+        <is>
+          <t>Fonctions sinus et cosinus</t>
+        </is>
+      </c>
+      <c r="G502" s="9" t="inlineStr">
+        <is>
+          <t>On considère les fonctions $\sin$ et $\cos$ sur $\mathbb R$.</t>
+        </is>
+      </c>
+      <c r="H502" s="10" t="inlineStr">
+        <is>
+          <t>Donner la période, la parité et les dérivées de $\sin$ et $\cos$.</t>
+        </is>
+      </c>
+      <c r="I502" s="9" t="inlineStr">
+        <is>
+          <t>$\sin$ et $\cos$ sont $2\pi$-périodiques ; $\sin$ est impaire, $\cos$ est paire ; $\sin'=\cos$ et $\cos'=-\sin$ ; à valeurs dans $[-1,1]$.</t>
+        </is>
+      </c>
+      <c r="J502" s="9" t="inlineStr">
+        <is>
+          <t>« Fonctions circulaires : sin, cos et tan. »</t>
+        </is>
+      </c>
+      <c r="K502" s="9" t="n"/>
+      <c r="L502" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les fonctions usuelles » 2024</t>
+        </is>
+      </c>
+      <c r="M502" s="11" t="n"/>
+      <c r="N502" s="11" t="n"/>
+    </row>
+    <row r="503">
+      <c r="A503" s="9" t="inlineStr">
+        <is>
+          <t>M502</t>
+        </is>
+      </c>
+      <c r="B503" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C503" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D503" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E503" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F503" s="9" t="inlineStr">
+        <is>
+          <t>Fonction tangente</t>
+        </is>
+      </c>
+      <c r="G503" s="9" t="inlineStr">
+        <is>
+          <t>On considère la fonction $\tan=\dfrac{\sin}{\cos}$.</t>
+        </is>
+      </c>
+      <c r="H503" s="10" t="inlineStr">
+        <is>
+          <t>Donner l'ensemble de définition, la période, la parité et la dérivée de $\tan$.</t>
+        </is>
+      </c>
+      <c r="I503" s="9" t="inlineStr">
+        <is>
+          <t>Définie sur $\mathbb R\setminus\{\frac\pi2+k\pi,\ k\in\mathbb Z\}$ ; $\pi$-périodique ; impaire ; $\tan'=1+\tan^2=\dfrac1{\cos^2}$ ; strictement croissante sur $\left]-\frac\pi2,\frac\pi2\right[$.</t>
+        </is>
+      </c>
+      <c r="J503" s="9" t="inlineStr">
+        <is>
+          <t>« Fonctions circulaires : sin, cos et tan. Formule tan′ = 1 + tan² = 1/cos². »</t>
+        </is>
+      </c>
+      <c r="K503" s="9" t="n"/>
+      <c r="L503" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les fonctions usuelles » 2024</t>
+        </is>
+      </c>
+      <c r="M503" s="11" t="n"/>
+      <c r="N503" s="11" t="n"/>
+    </row>
+    <row r="504">
+      <c r="A504" s="9" t="inlineStr">
+        <is>
+          <t>M503</t>
+        </is>
+      </c>
+      <c r="B504" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C504" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D504" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 2 – Nombres réels</t>
+        </is>
+      </c>
+      <c r="E504" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F504" s="9" t="inlineStr">
+        <is>
+          <t>Valeur absolue</t>
+        </is>
+      </c>
+      <c r="G504" s="9" t="inlineStr">
+        <is>
+          <t>Soient $x$, $y$, $a$ des réels et $r\ge0$.</t>
+        </is>
+      </c>
+      <c r="H504" s="10" t="inlineStr">
+        <is>
+          <t>Définir $|x|$ et donner ses propriétés, dont l'interprétation en termes de distance.</t>
+        </is>
+      </c>
+      <c r="I504" s="9" t="inlineStr">
+        <is>
+          <t>$|x|=\max(x,-x)$ ; $|xy|=|x||y|$ ; $|x+y|\le|x|+|y|$ ; $|x-a|$ est la distance de $x$ à $a$, donc $|x-a|\le r\iff a-r\le x\le a+r$.</t>
+        </is>
+      </c>
+      <c r="J504" s="9" t="inlineStr">
+        <is>
+          <t>« Valeur absolue. Interprétation de la valeur absolue en termes de distance. »</t>
+        </is>
+      </c>
+      <c r="K504" s="9" t="n"/>
+      <c r="L504" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les fonctions usuelles » 2024</t>
+        </is>
+      </c>
+      <c r="M504" s="11" t="n"/>
+      <c r="N504" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M486" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -32226,7 +33306,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$486,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$504,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -32241,7 +33321,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$486,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$504,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -32256,7 +33336,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$486,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$504,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -32283,7 +33363,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$486)</f>
+        <f>COUNTA(Fiches!$M$2:$M$504)</f>
         <v/>
       </c>
     </row>
@@ -32329,15 +33409,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A13,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A13,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A13,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A13,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A13,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A13,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -32352,15 +33432,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A14,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A14,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A14,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A14,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A14,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A14,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -32375,15 +33455,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A15,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A15,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A15,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A15,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A15,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A15,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -32398,15 +33478,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A16,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A16,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A16,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A16,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A16,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A16,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -32421,15 +33501,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A17,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A17,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A17,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A17,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A17,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A17,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -32444,15 +33524,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A18,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A18,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A18,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A18,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A18,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A18,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -32467,15 +33547,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A19,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A19,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A19,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A19,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A19,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A19,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -32490,15 +33570,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A20,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A20,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A20,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A20,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A20,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A20,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -32513,15 +33593,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A21,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A21,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A21,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A21,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A21,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A21,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -32536,15 +33616,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A22,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A22,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A22,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A22,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A22,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A22,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -32559,15 +33639,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A23,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A23,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A23,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A23,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A23,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A23,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -32582,15 +33662,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A24,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A24,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A24,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A24,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A24,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A24,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -32605,15 +33685,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A25,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A25,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A25,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A25,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A25,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A25,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -32628,15 +33708,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A26,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A26,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A26,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A26,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A26,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A26,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -32651,15 +33731,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A27,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A27,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A27,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A27,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A27,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A27,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -32674,15 +33754,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A28,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A28,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A28,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A28,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A28,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A28,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -32697,15 +33777,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A29,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A29,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A29,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A29,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A29,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A29,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -32720,15 +33800,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A30,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A30,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A30,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A30,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A30,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A30,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -32743,15 +33823,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A31,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A31,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A31,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A31,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A31,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A31,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -32766,15 +33846,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A32,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A32,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A32,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A32,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A32,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A32,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -32789,15 +33869,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A33,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A33,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A33,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A33,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A33,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A33,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -32812,15 +33892,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A34,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A34,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A34,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A34,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A34,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A34,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -32835,15 +33915,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A35,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A35,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A35,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A35,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A35,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A35,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -32858,15 +33938,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A36,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A36,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A36,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A36,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A36,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A36,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -32881,15 +33961,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A37,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A37,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A37,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A37,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A37,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A37,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -32904,15 +33984,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A38,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A38,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A38,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A38,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A38,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A38,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -32927,15 +34007,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A39,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A39,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A39,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A39,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A39,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A39,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -32950,15 +34030,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A40,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A40,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A40,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A40,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A40,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A40,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -32973,15 +34053,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A41,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A41,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A41,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A41,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A41,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A41,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -32996,15 +34076,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A42,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A42,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A42,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A42,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A42,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A42,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -33019,15 +34099,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A43,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A43,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A43,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A43,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A43,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A43,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -33042,15 +34122,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A44,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A44,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A44,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A44,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A44,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A44,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -33065,15 +34145,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A45,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A45,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A45,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A45,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A45,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A45,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -33088,15 +34168,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A46,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A46,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A46,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A46,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A46,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A46,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -33111,15 +34191,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A47,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A47,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A47,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A47,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A47,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A47,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -33134,15 +34214,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A48,Fiches!$B$2:$B$486,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A48,Fiches!$B$2:$B$504,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A48,Fiches!$B$2:$B$486,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A48,Fiches!$B$2:$B$504,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$486,$A48,Fiches!$B$2:$B$486,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$504,$A48,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Géométrie : 5 fiches ajoutées, 6 retirées d'après le cours de référence
Ajouts : déterminant, projeté d'un vecteur, produit scalaire et cosinus,
Pythagore (équivalence), reconnaître un cercle. Retraits : cercle paramétrique,
orientation, angle orienté, angles de droites et de plans.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N504"/>
+  <dimension ref="A1:N509"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8133,8 +8133,16 @@
         <v>59</v>
       </c>
       <c r="L128" s="12" t="inlineStr"/>
-      <c r="M128" s="14" t="n"/>
-      <c r="N128" s="14" t="n"/>
+      <c r="M128" s="14" t="inlineStr">
+        <is>
+          <t>Passer en rouge</t>
+        </is>
+      </c>
+      <c r="N128" s="14" t="inlineStr">
+        <is>
+          <t>Retirée : absente du cours « Géométrie » 2024 et du programme.</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="12" t="inlineStr">
@@ -8191,8 +8199,16 @@
         <v>59</v>
       </c>
       <c r="L129" s="12" t="inlineStr"/>
-      <c r="M129" s="14" t="n"/>
-      <c r="N129" s="14" t="n"/>
+      <c r="M129" s="14" t="inlineStr">
+        <is>
+          <t>Passer en rouge</t>
+        </is>
+      </c>
+      <c r="N129" s="14" t="inlineStr">
+        <is>
+          <t>Retirée : absente du cours « Géométrie » 2024 ; programme : « Aucun développement sur la notion d'angle orienté n'est un attendu ».</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="12" t="inlineStr">
@@ -8249,8 +8265,16 @@
         <v>59</v>
       </c>
       <c r="L130" s="12" t="inlineStr"/>
-      <c r="M130" s="14" t="n"/>
-      <c r="N130" s="14" t="n"/>
+      <c r="M130" s="14" t="inlineStr">
+        <is>
+          <t>Passer en rouge</t>
+        </is>
+      </c>
+      <c r="N130" s="14" t="inlineStr">
+        <is>
+          <t>Retirée : absente du cours « Géométrie » 2024 ; programme : « Aucun développement sur la notion d'angle orienté n'est un attendu ».</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="15" t="inlineStr">
@@ -8415,8 +8439,16 @@
         <v>60</v>
       </c>
       <c r="L133" s="12" t="inlineStr"/>
-      <c r="M133" s="14" t="n"/>
-      <c r="N133" s="14" t="n"/>
+      <c r="M133" s="14" t="inlineStr">
+        <is>
+          <t>Passer en rouge</t>
+        </is>
+      </c>
+      <c r="N133" s="14" t="inlineStr">
+        <is>
+          <t>Retirée : absente du cours « Géométrie » 2024 et du programme.</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="9" t="inlineStr">
@@ -10151,8 +10183,16 @@
         <v>69</v>
       </c>
       <c r="L163" s="12" t="inlineStr"/>
-      <c r="M163" s="14" t="n"/>
-      <c r="N163" s="14" t="n"/>
+      <c r="M163" s="14" t="inlineStr">
+        <is>
+          <t>Passer en rouge</t>
+        </is>
+      </c>
+      <c r="N163" s="14" t="inlineStr">
+        <is>
+          <t>Retirée : absente du cours « Géométrie » 2024 et du programme.</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="12" t="inlineStr">
@@ -10213,8 +10253,16 @@
           <t>Titre de l'ouvrage : « Angle de deux droites du plan » (coquille)</t>
         </is>
       </c>
-      <c r="M164" s="14" t="n"/>
-      <c r="N164" s="14" t="n"/>
+      <c r="M164" s="14" t="inlineStr">
+        <is>
+          <t>Passer en rouge</t>
+        </is>
+      </c>
+      <c r="N164" s="14" t="inlineStr">
+        <is>
+          <t>Retirée : absente du cours « Géométrie » 2024 et du programme.</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="9" t="inlineStr">
@@ -30066,10 +30114,310 @@
       <c r="M504" s="11" t="n"/>
       <c r="N504" s="11" t="n"/>
     </row>
+    <row r="505">
+      <c r="A505" s="9" t="inlineStr">
+        <is>
+          <t>M504</t>
+        </is>
+      </c>
+      <c r="B505" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C505" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D505" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Géométrie 1</t>
+        </is>
+      </c>
+      <c r="E505" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F505" s="9" t="inlineStr">
+        <is>
+          <t>Déterminant de deux vecteurs du plan</t>
+        </is>
+      </c>
+      <c r="G505" s="9" t="inlineStr">
+        <is>
+          <t>Le plan est muni d'une base orthonormée. Soient $\vec u(x,y)$, $\vec v(x',y')$, $\vec w$ trois vecteurs et $\alpha$, $\beta$ deux réels.</t>
+        </is>
+      </c>
+      <c r="H505" s="10" t="inlineStr">
+        <is>
+          <t>Définir $\det(\vec u,\vec v)$, donner ses propriétés et son lien avec la colinéarité.</t>
+        </is>
+      </c>
+      <c r="I505" s="9" t="inlineStr">
+        <is>
+          <t>$\det(\vec u,\vec v)=xy'-yx'$. Antisymétrie : $\det(\vec v,\vec u)=-\det(\vec u,\vec v)$ ; linéarité par rapport à chaque vecteur : $\det(\alpha\vec u+\beta\vec v,\vec w)=\alpha\det(\vec u,\vec w)+\beta\det(\vec v,\vec w)$. $\vec u$ et $\vec v$ sont colinéaires $\iff\det(\vec u,\vec v)=0$.</t>
+        </is>
+      </c>
+      <c r="J505" s="9" t="inlineStr">
+        <is>
+          <t>« déterminant de deux vecteurs dans le plan définis à l'aide de leurs coordonnées. Caractérisation de la colinéarité de deux vecteurs du plan par l'annulation du déterminant. »</t>
+        </is>
+      </c>
+      <c r="K505" s="9" t="n"/>
+      <c r="L505" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Géométrie » 2024</t>
+        </is>
+      </c>
+      <c r="M505" s="11" t="n"/>
+      <c r="N505" s="11" t="n"/>
+    </row>
+    <row r="506">
+      <c r="A506" s="9" t="inlineStr">
+        <is>
+          <t>M505</t>
+        </is>
+      </c>
+      <c r="B506" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C506" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D506" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Géométrie 1</t>
+        </is>
+      </c>
+      <c r="E506" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F506" s="9" t="inlineStr">
+        <is>
+          <t>Projeté orthogonal d'un vecteur sur un vecteur</t>
+        </is>
+      </c>
+      <c r="G506" s="9" t="inlineStr">
+        <is>
+          <t>Soient $\vec u$ et $\vec v$ deux vecteurs, avec $\vec v\neq\vec0$.</t>
+        </is>
+      </c>
+      <c r="H506" s="10" t="inlineStr">
+        <is>
+          <t>Définir le projeté orthogonal $\vec w$ de $\vec u$ sur $\vec v$ et l'exprimer.</t>
+        </is>
+      </c>
+      <c r="I506" s="9" t="inlineStr">
+        <is>
+          <t>C'est l'unique vecteur $\vec w$ colinéaire à $\vec v$ tel que $\vec u-\vec w$ soit orthogonal à $\vec v$ : $\vec w=\dfrac{\vec u\cdot\vec v}{\|\vec v\|^2}\,\vec v$. On a $|\vec u\cdot\vec v|=\|\vec w\|\,\|\vec v\|$.</t>
+        </is>
+      </c>
+      <c r="J506" s="9" t="inlineStr">
+        <is>
+          <t>« On pourra aborder la définition de projection orthogonale d'un vecteur sur une droite en lien avec les applications en physique. » (facultatif)</t>
+        </is>
+      </c>
+      <c r="K506" s="9" t="n"/>
+      <c r="L506" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Géométrie » 2024</t>
+        </is>
+      </c>
+      <c r="M506" s="11" t="n"/>
+      <c r="N506" s="11" t="n"/>
+    </row>
+    <row r="507">
+      <c r="A507" s="9" t="inlineStr">
+        <is>
+          <t>M506</t>
+        </is>
+      </c>
+      <c r="B507" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C507" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D507" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Géométrie 1</t>
+        </is>
+      </c>
+      <c r="E507" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F507" s="9" t="inlineStr">
+        <is>
+          <t>Produit scalaire et cosinus</t>
+        </is>
+      </c>
+      <c r="G507" s="9" t="inlineStr">
+        <is>
+          <t>Soient $\vec u$ et $\vec v$ deux vecteurs non nuls formant un angle géométrique $\theta$.</t>
+        </is>
+      </c>
+      <c r="H507" s="10" t="inlineStr">
+        <is>
+          <t>Exprimer $\vec u\cdot\vec v$ à l'aide de $\theta$, puis dans le cas où $\vec u$ et $\vec v$ sont colinéaires.</t>
+        </is>
+      </c>
+      <c r="I507" s="9" t="inlineStr">
+        <is>
+          <t>$\vec u\cdot\vec v=\|\vec u\|\,\|\vec v\|\cos\theta$. Si $\vec u=\alpha\vec v$ : $\vec u\cdot\vec v=\|\vec u\|\,\|\vec v\|$ si $\alpha\ge0$, et $-\|\vec u\|\,\|\vec v\|$ si $\alpha\le0$.</t>
+        </is>
+      </c>
+      <c r="J507" s="9" t="inlineStr">
+        <is>
+          <t>« Formulation du produit scalaire à l'aide du cosinus de l'angle formé entre deux vecteurs non nuls. »</t>
+        </is>
+      </c>
+      <c r="K507" s="9" t="n"/>
+      <c r="L507" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Géométrie » 2024</t>
+        </is>
+      </c>
+      <c r="M507" s="11" t="n"/>
+      <c r="N507" s="11" t="n"/>
+    </row>
+    <row r="508">
+      <c r="A508" s="9" t="inlineStr">
+        <is>
+          <t>M507</t>
+        </is>
+      </c>
+      <c r="B508" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C508" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D508" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Géométrie 1</t>
+        </is>
+      </c>
+      <c r="E508" s="9" t="inlineStr">
+        <is>
+          <t>Théorème</t>
+        </is>
+      </c>
+      <c r="F508" s="9" t="inlineStr">
+        <is>
+          <t>Théorème de Pythagore (plan et espace)</t>
+        </is>
+      </c>
+      <c r="G508" s="9" t="inlineStr">
+        <is>
+          <t>Soient $\vec u$ et $\vec v$ deux vecteurs du plan ou de l'espace.</t>
+        </is>
+      </c>
+      <c r="H508" s="10" t="inlineStr">
+        <is>
+          <t>Énoncer le théorème de Pythagore sous forme d'équivalence.</t>
+        </is>
+      </c>
+      <c r="I508" s="9" t="inlineStr">
+        <is>
+          <t>$\vec u$ et $\vec v$ sont orthogonaux $\iff\|\vec u+\vec v\|^2=\|\vec u\|^2+\|\vec v\|^2$ (car $\|\vec u+\vec v\|^2=\|\vec u\|^2+2\,\vec u\cdot\vec v+\|\vec v\|^2$).</t>
+        </is>
+      </c>
+      <c r="J508" s="9" t="inlineStr">
+        <is>
+          <t>« Caractérisation de l'orthogonalité de deux vecteurs par le produit scalaire. Lien avec la norme. »</t>
+        </is>
+      </c>
+      <c r="K508" s="9" t="n"/>
+      <c r="L508" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Géométrie » 2024</t>
+        </is>
+      </c>
+      <c r="M508" s="11" t="n"/>
+      <c r="N508" s="11" t="n"/>
+    </row>
+    <row r="509">
+      <c r="A509" s="9" t="inlineStr">
+        <is>
+          <t>M508</t>
+        </is>
+      </c>
+      <c r="B509" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C509" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D509" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Géométrie 1</t>
+        </is>
+      </c>
+      <c r="E509" s="9" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+      <c r="F509" s="9" t="inlineStr">
+        <is>
+          <t>Reconnaître un cercle</t>
+        </is>
+      </c>
+      <c r="G509" s="9" t="inlineStr">
+        <is>
+          <t>Le plan est muni d'un repère orthonormé. Soient $a$, $b$, $c$ des réels et $\mathcal E$ : $x^2+ax+y^2+by=c$.</t>
+        </is>
+      </c>
+      <c r="H509" s="10" t="inlineStr">
+        <is>
+          <t>Comment reconnaître si $\mathcal E$ est un cercle et trouver son centre et son rayon ?</t>
+        </is>
+      </c>
+      <c r="I509" s="9" t="inlineStr">
+        <is>
+          <t>Mettre sous forme canonique : $\left(x+\frac a2\right)^2+\left(y+\frac b2\right)^2=c+\frac{a^2+b^2}4=k$. Si $k&gt;0$, c'est le cercle de centre $\Omega\left(-\frac a2,-\frac b2\right)$ et de rayon $\sqrt k$ ; si $k=0$, c'est le point $\Omega$ ; si $k&lt;0$, l'ensemble est vide.</t>
+        </is>
+      </c>
+      <c r="J509" s="9" t="inlineStr">
+        <is>
+          <t>« Équation cartésienne d'un cercle défini par son centre et son rayon. »</t>
+        </is>
+      </c>
+      <c r="K509" s="9" t="n"/>
+      <c r="L509" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Géométrie » 2024</t>
+        </is>
+      </c>
+      <c r="M509" s="11" t="n"/>
+      <c r="N509" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M509" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -33306,7 +33654,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$504,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$509,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -33321,7 +33669,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$504,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$509,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -33336,7 +33684,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$504,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$509,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -33363,7 +33711,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$504)</f>
+        <f>COUNTA(Fiches!$M$2:$M$509)</f>
         <v/>
       </c>
     </row>
@@ -33409,15 +33757,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A13,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A13,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A13,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A13,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A13,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A13,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -33432,15 +33780,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A14,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A14,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A14,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A14,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A14,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A14,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -33455,15 +33803,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A15,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A15,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A15,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A15,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A15,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A15,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -33478,15 +33826,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A16,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A16,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A16,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A16,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A16,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A16,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -33501,15 +33849,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A17,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A17,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A17,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A17,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A17,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A17,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -33524,15 +33872,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A18,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A18,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A18,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A18,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A18,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A18,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -33547,15 +33895,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A19,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A19,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A19,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A19,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A19,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A19,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -33570,15 +33918,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A20,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A20,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A20,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A20,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A20,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A20,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -33593,15 +33941,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A21,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A21,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A21,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A21,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A21,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A21,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -33616,15 +33964,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A22,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A22,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A22,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A22,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A22,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A22,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -33639,15 +33987,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A23,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A23,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A23,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A23,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A23,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A23,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -33662,15 +34010,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A24,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A24,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A24,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A24,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A24,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A24,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -33685,15 +34033,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A25,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A25,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A25,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A25,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A25,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A25,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -33708,15 +34056,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A26,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A26,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A26,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A26,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A26,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A26,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -33731,15 +34079,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A27,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A27,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A27,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A27,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A27,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A27,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -33754,15 +34102,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A28,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A28,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A28,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A28,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A28,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A28,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -33777,15 +34125,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A29,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A29,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A29,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A29,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A29,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A29,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -33800,15 +34148,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A30,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A30,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A30,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A30,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A30,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A30,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -33823,15 +34171,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A31,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A31,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A31,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A31,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A31,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A31,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -33846,15 +34194,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A32,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A32,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A32,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A32,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A32,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A32,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -33869,15 +34217,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A33,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A33,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A33,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A33,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A33,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A33,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -33892,15 +34240,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A34,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A34,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A34,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A34,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A34,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A34,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -33915,15 +34263,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A35,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A35,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A35,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A35,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A35,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A35,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -33938,15 +34286,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A36,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A36,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A36,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A36,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A36,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A36,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -33961,15 +34309,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A37,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A37,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A37,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A37,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A37,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A37,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -33984,15 +34332,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A38,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A38,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A38,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A38,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A38,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A38,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -34007,15 +34355,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A39,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A39,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A39,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A39,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A39,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A39,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -34030,15 +34378,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A40,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A40,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A40,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A40,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A40,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A40,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -34053,15 +34401,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A41,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A41,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A41,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A41,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A41,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A41,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -34076,15 +34424,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A42,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A42,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A42,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A42,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A42,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A42,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -34099,15 +34447,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A43,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A43,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A43,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A43,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A43,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A43,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -34122,15 +34470,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A44,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A44,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A44,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A44,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A44,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A44,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -34145,15 +34493,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A45,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A45,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A45,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A45,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A45,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A45,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -34168,15 +34516,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A46,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A46,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A46,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A46,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A46,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A46,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -34191,15 +34539,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A47,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A47,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A47,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A47,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A47,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A47,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -34214,15 +34562,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A48,Fiches!$B$2:$B$504,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A48,Fiches!$B$2:$B$509,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A48,Fiches!$B$2:$B$504,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A48,Fiches!$B$2:$B$509,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$504,$A48,Fiches!$B$2:$B$504,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$509,$A48,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Matrices : 12 fiches ajoutées, définition du rang alignée sur le programme
Vocabulaire, transposée, identité, puissances, précautions du produit,
inversibilité (définition, règles, 2×2, méthode, AX = Y), diagonales,
triangulaires. Rang défini comme nombre de pivots.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N509"/>
+  <dimension ref="A1:N521"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6331,7 +6331,7 @@
       </c>
       <c r="I97" s="9" t="inlineStr">
         <is>
-          <t>Le rang de $M\in\mathcal M_{n,p}(\mathbb K)$ est le rang de l'application linéaire canoniquement associée (= rang de la famille de ses colonnes).</t>
+          <t>Le rang de $M$ est le nombre de pivots obtenus en appliquant la méthode du pivot de Gauss à $M$ (c'est aussi le rang de la famille de ses colonnes).</t>
         </is>
       </c>
       <c r="J97" s="9" t="inlineStr">
@@ -30414,10 +30414,730 @@
       <c r="M509" s="11" t="n"/>
       <c r="N509" s="11" t="n"/>
     </row>
+    <row r="510">
+      <c r="A510" s="9" t="inlineStr">
+        <is>
+          <t>M509</t>
+        </is>
+      </c>
+      <c r="B510" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C510" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D510" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre linéaire 2 – Matrices</t>
+        </is>
+      </c>
+      <c r="E510" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F510" s="9" t="inlineStr">
+        <is>
+          <t>Matrices – Vocabulaire</t>
+        </is>
+      </c>
+      <c r="G510" s="9" t="inlineStr">
+        <is>
+          <t>Soient $n,p\in\mathbb N^*$ et $\mathbb K=\mathbb R$ ou $\mathbb C$.</t>
+        </is>
+      </c>
+      <c r="H510" s="10" t="inlineStr">
+        <is>
+          <t>Définir $\mathcal M_{n,p}(\mathbb K)$, la matrice nulle, une matrice carrée, ligne, colonne, et l'égalité de deux matrices.</t>
+        </is>
+      </c>
+      <c r="I510" s="9" t="inlineStr">
+        <is>
+          <t>$\mathcal M_{n,p}(\mathbb K)$ : matrices à $n$ lignes et $p$ colonnes à coefficients dans $\mathbb K$. Matrice nulle $0_{n,p}$ : tous les coefficients nuls. Carrée : $n=p$, ensemble $\mathcal M_n(\mathbb K)$. Colonne : taille $(n,1)$ ; ligne : taille $(1,p)$. Deux matrices sont égales si elles ont la même taille et les mêmes coefficients.</t>
+        </is>
+      </c>
+      <c r="J510" s="9" t="inlineStr">
+        <is>
+          <t>« Matrices : définition, vocabulaire. Matrice nulle. Matrices carrées, matrices lignes, colonnes. »</t>
+        </is>
+      </c>
+      <c r="K510" s="9" t="n"/>
+      <c r="L510" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les matrices » 2024</t>
+        </is>
+      </c>
+      <c r="M510" s="11" t="n"/>
+      <c r="N510" s="11" t="n"/>
+    </row>
+    <row r="511">
+      <c r="A511" s="9" t="inlineStr">
+        <is>
+          <t>M510</t>
+        </is>
+      </c>
+      <c r="B511" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C511" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D511" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre linéaire 2 – Matrices</t>
+        </is>
+      </c>
+      <c r="E511" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F511" s="9" t="inlineStr">
+        <is>
+          <t>Transposée d'une matrice – Définition</t>
+        </is>
+      </c>
+      <c r="G511" s="9" t="inlineStr">
+        <is>
+          <t>Soit $A=(a_{i,j})\in\mathcal M_{n,p}(\mathbb K)$.</t>
+        </is>
+      </c>
+      <c r="H511" s="10" t="inlineStr">
+        <is>
+          <t>Définir la transposée $A^T$.</t>
+        </is>
+      </c>
+      <c r="I511" s="9" t="inlineStr">
+        <is>
+          <t>$A^T=(b_{i,j})\in\mathcal M_{p,n}(\mathbb K)$ avec $b_{i,j}=a_{j,i}$ : les lignes de $A$ deviennent les colonnes de $A^T$.</t>
+        </is>
+      </c>
+      <c r="J511" s="9" t="inlineStr">
+        <is>
+          <t>« Transposée d'une matrice M, notée M^T. »</t>
+        </is>
+      </c>
+      <c r="K511" s="9" t="n"/>
+      <c r="L511" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les matrices » 2024</t>
+        </is>
+      </c>
+      <c r="M511" s="11" t="n"/>
+      <c r="N511" s="11" t="n"/>
+    </row>
+    <row r="512">
+      <c r="A512" s="9" t="inlineStr">
+        <is>
+          <t>M511</t>
+        </is>
+      </c>
+      <c r="B512" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C512" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D512" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre linéaire 2 – Matrices</t>
+        </is>
+      </c>
+      <c r="E512" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F512" s="9" t="inlineStr">
+        <is>
+          <t>Matrice identité</t>
+        </is>
+      </c>
+      <c r="G512" s="9" t="inlineStr">
+        <is>
+          <t>Soient $n,p\in\mathbb N^*$ et $A\in\mathcal M_{n,p}(\mathbb K)$.</t>
+        </is>
+      </c>
+      <c r="H512" s="10" t="inlineStr">
+        <is>
+          <t>Définir la matrice identité $I_n$ et donner son rôle dans le produit.</t>
+        </is>
+      </c>
+      <c r="I512" s="9" t="inlineStr">
+        <is>
+          <t>$I_n\in\mathcal M_n(\mathbb K)$ a des $1$ sur la diagonale et des $0$ ailleurs. $I_nA=AI_p=A$.</t>
+        </is>
+      </c>
+      <c r="J512" s="9" t="inlineStr">
+        <is>
+          <t>« Matrice identité. »</t>
+        </is>
+      </c>
+      <c r="K512" s="9" t="n"/>
+      <c r="L512" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les matrices » 2024</t>
+        </is>
+      </c>
+      <c r="M512" s="11" t="n"/>
+      <c r="N512" s="11" t="n"/>
+    </row>
+    <row r="513">
+      <c r="A513" s="9" t="inlineStr">
+        <is>
+          <t>M512</t>
+        </is>
+      </c>
+      <c r="B513" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C513" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D513" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre linéaire 2 – Matrices</t>
+        </is>
+      </c>
+      <c r="E513" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F513" s="9" t="inlineStr">
+        <is>
+          <t>Puissances d'une matrice carrée</t>
+        </is>
+      </c>
+      <c r="G513" s="9" t="inlineStr">
+        <is>
+          <t>Soient $A,B\in\mathcal M_n(\mathbb K)$ et $p,q\in\mathbb N$.</t>
+        </is>
+      </c>
+      <c r="H513" s="10" t="inlineStr">
+        <is>
+          <t>Définir $A^p$ et donner les règles de calcul sur les puissances.</t>
+        </is>
+      </c>
+      <c r="I513" s="9" t="inlineStr">
+        <is>
+          <t>$A^0=I_n$ et $A^{p+1}=A\times A^p=A^p\times A$. $A^{p+q}=A^pA^q$ ; $(A^p)^q=A^{pq}$ ; $(A^p)^T=(A^T)^p$. Si $AB=BA$ : $(AB)^p=A^pB^p$ (faux en général sinon).</t>
+        </is>
+      </c>
+      <c r="J513" s="9" t="inlineStr">
+        <is>
+          <t>« Opérations sur les matrices […] Propriétés de ces opérations. »</t>
+        </is>
+      </c>
+      <c r="K513" s="9" t="n"/>
+      <c r="L513" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les matrices » 2024</t>
+        </is>
+      </c>
+      <c r="M513" s="11" t="n"/>
+      <c r="N513" s="11" t="n"/>
+    </row>
+    <row r="514">
+      <c r="A514" s="9" t="inlineStr">
+        <is>
+          <t>M513</t>
+        </is>
+      </c>
+      <c r="B514" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C514" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D514" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre linéaire 2 – Matrices</t>
+        </is>
+      </c>
+      <c r="E514" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F514" s="9" t="inlineStr">
+        <is>
+          <t>Produit matriciel – Précautions</t>
+        </is>
+      </c>
+      <c r="G514" s="9" t="inlineStr">
+        <is>
+          <t>Soient $A\in\mathcal M_{n,p}(\mathbb K)$ et $B$, $C$ des matrices.</t>
+        </is>
+      </c>
+      <c r="H514" s="10" t="inlineStr">
+        <is>
+          <t>À quelle condition $AB$ est-il défini ? Quels réflexes du calcul sur les réels sont faux pour les matrices ?</t>
+        </is>
+      </c>
+      <c r="I514" s="9" t="inlineStr">
+        <is>
+          <t>$AB$ est défini si le nombre de colonnes de $A$ égale le nombre de lignes de $B$. En général $AB\neq BA$ ; on peut avoir $AB=0$ avec $A\neq0$ et $B\neq0$ ; $AB=AC$ n'entraîne pas $B=C$ (sauf si $A$ est inversible).</t>
+        </is>
+      </c>
+      <c r="J514" s="9" t="inlineStr">
+        <is>
+          <t>Introduction du chapitre : « mettre en place le calcul sur les matrices avec ses analogies et différences vis-à-vis du calcul sur les nombres réels et complexes ».</t>
+        </is>
+      </c>
+      <c r="K514" s="9" t="n"/>
+      <c r="L514" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les matrices » 2024</t>
+        </is>
+      </c>
+      <c r="M514" s="11" t="n"/>
+      <c r="N514" s="11" t="n"/>
+    </row>
+    <row r="515">
+      <c r="A515" s="9" t="inlineStr">
+        <is>
+          <t>M514</t>
+        </is>
+      </c>
+      <c r="B515" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C515" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D515" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre linéaire 2 – Matrices</t>
+        </is>
+      </c>
+      <c r="E515" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F515" s="9" t="inlineStr">
+        <is>
+          <t>Matrice inversible – Définition</t>
+        </is>
+      </c>
+      <c r="G515" s="9" t="inlineStr">
+        <is>
+          <t>Soit $A\in\mathcal M_n(\mathbb K)$.</t>
+        </is>
+      </c>
+      <c r="H515" s="10" t="inlineStr">
+        <is>
+          <t>Définir : $A$ est inversible, et son inverse.</t>
+        </is>
+      </c>
+      <c r="I515" s="9" t="inlineStr">
+        <is>
+          <t>$A$ est inversible s'il existe $B\in\mathcal M_n(\mathbb K)$ telle que $AB=BA=I_n$. Cette matrice est unique, notée $A^{-1}$. L'ensemble des matrices inversibles est noté $GL_n(\mathbb K)$.</t>
+        </is>
+      </c>
+      <c r="J515" s="9" t="inlineStr">
+        <is>
+          <t>« Matrices carrées inversibles, matrice inverse »</t>
+        </is>
+      </c>
+      <c r="K515" s="9" t="n"/>
+      <c r="L515" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les matrices » 2024</t>
+        </is>
+      </c>
+      <c r="M515" s="11" t="n"/>
+      <c r="N515" s="11" t="n"/>
+    </row>
+    <row r="516">
+      <c r="A516" s="9" t="inlineStr">
+        <is>
+          <t>M515</t>
+        </is>
+      </c>
+      <c r="B516" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C516" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D516" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre linéaire 2 – Matrices</t>
+        </is>
+      </c>
+      <c r="E516" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F516" s="9" t="inlineStr">
+        <is>
+          <t>Inverse – Règles de calcul</t>
+        </is>
+      </c>
+      <c r="G516" s="9" t="inlineStr">
+        <is>
+          <t>Soient $A,B\in GL_n(\mathbb K)$, $\lambda\in\mathbb K^*$, $p\in\mathbb N$, et $M,N\in\mathcal M_n(\mathbb K)$.</t>
+        </is>
+      </c>
+      <c r="H516" s="10" t="inlineStr">
+        <is>
+          <t>Donner l'inverse de $AB$, $\lambda A$, $A^{-1}$, $A^p$ et $A^T$, et la règle de simplification par une matrice inversible.</t>
+        </is>
+      </c>
+      <c r="I516" s="9" t="inlineStr">
+        <is>
+          <t>$(AB)^{-1}=B^{-1}A^{-1}$ ; $(\lambda A)^{-1}=\frac1\lambda A^{-1}$ ; $(A^{-1})^{-1}=A$ ; $(A^p)^{-1}=(A^{-1})^p$ ; $(A^T)^{-1}=(A^{-1})^T$. $AM=AN\iff M=N$ et $MA=NA\iff M=N$.</t>
+        </is>
+      </c>
+      <c r="J516" s="9" t="inlineStr">
+        <is>
+          <t>« inverse d'un produit, inverse de la transposée d'une matrice carrée inversible. »</t>
+        </is>
+      </c>
+      <c r="K516" s="9" t="n"/>
+      <c r="L516" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les matrices » 2024</t>
+        </is>
+      </c>
+      <c r="M516" s="11" t="n"/>
+      <c r="N516" s="11" t="n"/>
+    </row>
+    <row r="517">
+      <c r="A517" s="9" t="inlineStr">
+        <is>
+          <t>M516</t>
+        </is>
+      </c>
+      <c r="B517" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C517" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D517" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre linéaire 2 – Matrices</t>
+        </is>
+      </c>
+      <c r="E517" s="9" t="inlineStr">
+        <is>
+          <t>Théorème</t>
+        </is>
+      </c>
+      <c r="F517" s="9" t="inlineStr">
+        <is>
+          <t>Matrices 2×2 : déterminant et inverse</t>
+        </is>
+      </c>
+      <c r="G517" s="9" t="inlineStr">
+        <is>
+          <t>Soient $a,b,c,d\in\mathbb K$ et $A=\begin{pmatrix}a&amp;b\\c&amp;d\end{pmatrix}$.</t>
+        </is>
+      </c>
+      <c r="H517" s="10" t="inlineStr">
+        <is>
+          <t>Donner une caractérisation de l'inversibilité de $A$ et l'expression de $A^{-1}$.</t>
+        </is>
+      </c>
+      <c r="I517" s="9" t="inlineStr">
+        <is>
+          <t>$\det A=ad-bc$. $A$ est inversible si et seulement si $ad-bc\neq0$, et alors $A^{-1}=\dfrac1{ad-bc}\begin{pmatrix}d&amp;-b\\-c&amp;a\end{pmatrix}$.</t>
+        </is>
+      </c>
+      <c r="J517" s="9" t="inlineStr">
+        <is>
+          <t>« Déterminant des matrices 2 × 2 et caractérisation des matrices 2 × 2 inversibles. »</t>
+        </is>
+      </c>
+      <c r="K517" s="9" t="n"/>
+      <c r="L517" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les matrices » 2024</t>
+        </is>
+      </c>
+      <c r="M517" s="11" t="n"/>
+      <c r="N517" s="11" t="n"/>
+    </row>
+    <row r="518">
+      <c r="A518" s="9" t="inlineStr">
+        <is>
+          <t>M517</t>
+        </is>
+      </c>
+      <c r="B518" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C518" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D518" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre linéaire 2 – Matrices</t>
+        </is>
+      </c>
+      <c r="E518" s="9" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+      <c r="F518" s="9" t="inlineStr">
+        <is>
+          <t>Recherche pratique de l'inverse</t>
+        </is>
+      </c>
+      <c r="G518" s="9" t="inlineStr">
+        <is>
+          <t>Soit $A\in\mathcal M_n(\mathbb K)$.</t>
+        </is>
+      </c>
+      <c r="H518" s="10" t="inlineStr">
+        <is>
+          <t>Donner une méthode pour savoir si $A$ est inversible et calculer $A^{-1}$.</t>
+        </is>
+      </c>
+      <c r="I518" s="9" t="inlineStr">
+        <is>
+          <t>Résoudre le système $AX=Y$ d'inconnue $X$ pour $Y$ quelconque (pivot de Gauss). Si l'on obtient une unique solution $X=BY$ pour tout $Y$, alors $A$ est inversible et $A^{-1}=B$ ; sinon $A$ n'est pas inversible. Autre piste : une relation polynomiale, par exemple $A^2-3A=-2I_n$ donne $A\cdot\frac{3I_n-A}2=I_n$.</t>
+        </is>
+      </c>
+      <c r="J518" s="9" t="inlineStr">
+        <is>
+          <t>« Recherche pratique de l'inverse d'une matrice. L'inversion peut se ramener à la résolution de systèmes linéaires. »</t>
+        </is>
+      </c>
+      <c r="K518" s="9" t="n"/>
+      <c r="L518" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les matrices » 2024</t>
+        </is>
+      </c>
+      <c r="M518" s="11" t="n"/>
+      <c r="N518" s="11" t="n"/>
+    </row>
+    <row r="519">
+      <c r="A519" s="9" t="inlineStr">
+        <is>
+          <t>M518</t>
+        </is>
+      </c>
+      <c r="B519" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C519" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D519" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre linéaire 2 – Matrices</t>
+        </is>
+      </c>
+      <c r="E519" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F519" s="9" t="inlineStr">
+        <is>
+          <t>Système linéaire et matrice inversible</t>
+        </is>
+      </c>
+      <c r="G519" s="9" t="inlineStr">
+        <is>
+          <t>Soient $A\in\mathcal M_n(\mathbb K)$ et $Y\in\mathcal M_{n,1}(\mathbb K)$, et le système $AX=Y$.</t>
+        </is>
+      </c>
+      <c r="H519" s="10" t="inlineStr">
+        <is>
+          <t>Que dire du système $AX=Y$ si $A$ est inversible ?</t>
+        </is>
+      </c>
+      <c r="I519" s="9" t="inlineStr">
+        <is>
+          <t>Il admet une unique solution : $X=A^{-1}Y$.</t>
+        </is>
+      </c>
+      <c r="J519" s="9" t="inlineStr">
+        <is>
+          <t>« Expression matricielle formelle, X = A⁻¹Y, de la solution d'un système linéaire AX = Y lorsque la matrice carrée A qui lui est associée est inversible. »</t>
+        </is>
+      </c>
+      <c r="K519" s="9" t="n"/>
+      <c r="L519" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les matrices » 2024</t>
+        </is>
+      </c>
+      <c r="M519" s="11" t="n"/>
+      <c r="N519" s="11" t="n"/>
+    </row>
+    <row r="520">
+      <c r="A520" s="9" t="inlineStr">
+        <is>
+          <t>M519</t>
+        </is>
+      </c>
+      <c r="B520" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C520" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D520" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre linéaire 2 – Matrices</t>
+        </is>
+      </c>
+      <c r="E520" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F520" s="9" t="inlineStr">
+        <is>
+          <t>Matrices diagonales</t>
+        </is>
+      </c>
+      <c r="G520" s="9" t="inlineStr">
+        <is>
+          <t>Soient $a_1,\dots,a_n,b_1,\dots,b_n\in\mathbb K$ et $k\in\mathbb N$.</t>
+        </is>
+      </c>
+      <c r="H520" s="10" t="inlineStr">
+        <is>
+          <t>Définir une matrice diagonale et donner le produit, les puissances et l'inverse de matrices diagonales.</t>
+        </is>
+      </c>
+      <c r="I520" s="9" t="inlineStr">
+        <is>
+          <t>Diagonale : $a_{i,j}=0$ pour $i\neq j$ ; on note $\mathrm{Diag}(a_1,\dots,a_n)$. $\mathrm{Diag}(a_i)\,\mathrm{Diag}(b_i)=\mathrm{Diag}(a_ib_i)$ ; $\mathrm{Diag}(a_i)^k=\mathrm{Diag}(a_i^k)$ ; si tous les $a_i\neq0$, elle est inversible et $\mathrm{Diag}(a_i)^{-1}=\mathrm{Diag}(a_i^{-1})$.</t>
+        </is>
+      </c>
+      <c r="J520" s="9" t="inlineStr">
+        <is>
+          <t>« Matrices triangulaires, diagonales. […] Produit de matrices diagonales. »</t>
+        </is>
+      </c>
+      <c r="K520" s="9" t="n"/>
+      <c r="L520" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les matrices » 2024</t>
+        </is>
+      </c>
+      <c r="M520" s="11" t="n"/>
+      <c r="N520" s="11" t="n"/>
+    </row>
+    <row r="521">
+      <c r="A521" s="9" t="inlineStr">
+        <is>
+          <t>M520</t>
+        </is>
+      </c>
+      <c r="B521" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C521" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D521" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre linéaire 2 – Matrices</t>
+        </is>
+      </c>
+      <c r="E521" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F521" s="9" t="inlineStr">
+        <is>
+          <t>Matrices triangulaires</t>
+        </is>
+      </c>
+      <c r="G521" s="9" t="inlineStr">
+        <is>
+          <t>Soit $A=(a_{i,j})\in\mathcal M_n(\mathbb K)$.</t>
+        </is>
+      </c>
+      <c r="H521" s="10" t="inlineStr">
+        <is>
+          <t>Définir une matrice triangulaire supérieure (inférieure) et donner ses propriétés : produit, inversibilité.</t>
+        </is>
+      </c>
+      <c r="I521" s="9" t="inlineStr">
+        <is>
+          <t>Triangulaire supérieure : $a_{i,j}=0$ pour $i&gt;j$ (inférieure : pour $i&lt;j$). Un produit de triangulaires supérieures est triangulaire supérieure, de coefficients diagonaux les produits des coefficients diagonaux. Une matrice triangulaire est inversible si et seulement si ses coefficients diagonaux sont tous non nuls.</t>
+        </is>
+      </c>
+      <c r="J521" s="9" t="inlineStr">
+        <is>
+          <t>« Matrices triangulaires, diagonales. »</t>
+        </is>
+      </c>
+      <c r="K521" s="9" t="n"/>
+      <c r="L521" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les matrices » 2024</t>
+        </is>
+      </c>
+      <c r="M521" s="11" t="n"/>
+      <c r="N521" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M509" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M521" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -33654,7 +34374,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$509,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$521,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -33669,7 +34389,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$509,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$521,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -33684,7 +34404,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$509,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$521,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -33711,7 +34431,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$509)</f>
+        <f>COUNTA(Fiches!$M$2:$M$521)</f>
         <v/>
       </c>
     </row>
@@ -33757,15 +34477,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A13,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A13,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A13,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A13,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A13,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A13,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -33780,15 +34500,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A14,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A14,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A14,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A14,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A14,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A14,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -33803,15 +34523,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A15,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A15,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A15,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A15,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A15,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A15,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -33826,15 +34546,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A16,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A16,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A16,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A16,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A16,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A16,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -33849,15 +34569,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A17,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A17,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A17,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A17,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A17,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A17,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -33872,15 +34592,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A18,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A18,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A18,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A18,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A18,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A18,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -33895,15 +34615,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A19,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A19,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A19,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A19,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A19,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A19,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -33918,15 +34638,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A20,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A20,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A20,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A20,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A20,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A20,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -33941,15 +34661,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A21,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A21,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A21,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A21,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A21,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A21,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -33964,15 +34684,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A22,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A22,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A22,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A22,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A22,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A22,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -33987,15 +34707,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A23,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A23,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A23,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A23,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A23,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A23,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -34010,15 +34730,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A24,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A24,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A24,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A24,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A24,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A24,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -34033,15 +34753,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A25,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A25,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A25,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A25,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A25,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A25,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -34056,15 +34776,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A26,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A26,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A26,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A26,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A26,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A26,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -34079,15 +34799,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A27,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A27,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A27,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A27,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A27,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A27,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -34102,15 +34822,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A28,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A28,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A28,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A28,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A28,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A28,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -34125,15 +34845,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A29,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A29,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A29,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A29,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A29,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A29,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -34148,15 +34868,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A30,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A30,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A30,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A30,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A30,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A30,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -34171,15 +34891,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A31,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A31,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A31,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A31,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A31,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A31,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -34194,15 +34914,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A32,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A32,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A32,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A32,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A32,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A32,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -34217,15 +34937,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A33,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A33,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A33,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A33,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A33,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A33,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -34240,15 +34960,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A34,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A34,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A34,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A34,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A34,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A34,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -34263,15 +34983,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A35,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A35,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A35,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A35,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A35,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A35,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -34286,15 +35006,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A36,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A36,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A36,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A36,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A36,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A36,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -34309,15 +35029,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A37,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A37,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A37,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A37,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A37,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A37,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -34332,15 +35052,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A38,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A38,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A38,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A38,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A38,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A38,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -34355,15 +35075,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A39,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A39,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A39,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A39,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A39,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A39,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -34378,15 +35098,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A40,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A40,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A40,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A40,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A40,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A40,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -34401,15 +35121,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A41,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A41,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A41,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A41,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A41,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A41,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -34424,15 +35144,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A42,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A42,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A42,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A42,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A42,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A42,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -34447,15 +35167,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A43,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A43,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A43,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A43,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A43,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A43,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -34470,15 +35190,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A44,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A44,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A44,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A44,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A44,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A44,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -34493,15 +35213,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A45,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A45,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A45,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A45,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A45,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A45,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -34516,15 +35236,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A46,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A46,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A46,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A46,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A46,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A46,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -34539,15 +35259,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A47,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A47,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A47,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A47,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A47,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A47,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -34562,15 +35282,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A48,Fiches!$B$2:$B$509,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A48,Fiches!$B$2:$B$521,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A48,Fiches!$B$2:$B$509,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A48,Fiches!$B$2:$B$521,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$509,$A48,Fiches!$B$2:$B$509,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$521,$A48,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Polynômes : 10 fiches ajoutées, M319 complétée, M320 retirée
Unicité des coefficients, vocabulaire, opérations, dérivée, racine et
factorisation, nombre de racines, n racines distinctes, racine multiple et
dérivée, degré impair, racines conjuguées (2e année).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N521"/>
+  <dimension ref="A1:N531"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -19277,7 +19277,7 @@
       </c>
       <c r="I320" s="9" t="inlineStr">
         <is>
-          <t>$a$ est racine de multiplicité $m$ de $P$ si $(X-a)^m$ divise $P$ et $(X-a)^{m+1}$ ne divise pas $P$ (multiplicité 0 si $a$ n'est pas racine).</t>
+          <t>$a$ est racine de multiplicité $m$ de $P$ si $(X-a)^m$ divise $P$ et $(X-a)^{m+1}$ ne divise pas $P$ ; de façon équivalente, $P=(X-a)^mR$ avec $R(a)\neq0$. Multiplicité 1 : racine simple ; 2 : double.</t>
         </is>
       </c>
       <c r="J320" s="9" t="inlineStr">
@@ -19347,8 +19347,16 @@
         <v>4</v>
       </c>
       <c r="L321" s="12" t="inlineStr"/>
-      <c r="M321" s="14" t="n"/>
-      <c r="N321" s="14" t="n"/>
+      <c r="M321" s="14" t="inlineStr">
+        <is>
+          <t>Passer en rouge</t>
+        </is>
+      </c>
+      <c r="N321" s="14" t="inlineStr">
+        <is>
+          <t>Retirée : le mot « scindé » n'est ni dans le cours « Les polynômes » 2024 ni dans le programme.</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" s="9" t="inlineStr">
@@ -31134,10 +31142,610 @@
       <c r="M521" s="11" t="n"/>
       <c r="N521" s="11" t="n"/>
     </row>
+    <row r="522">
+      <c r="A522" s="9" t="inlineStr">
+        <is>
+          <t>M521</t>
+        </is>
+      </c>
+      <c r="B522" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C522" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D522" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre – Polynômes réels</t>
+        </is>
+      </c>
+      <c r="E522" s="9" t="inlineStr">
+        <is>
+          <t>Théorème</t>
+        </is>
+      </c>
+      <c r="F522" s="9" t="inlineStr">
+        <is>
+          <t>Unicité des coefficients</t>
+        </is>
+      </c>
+      <c r="G522" s="9" t="inlineStr">
+        <is>
+          <t>Soient $P:x\mapsto\sum_{k=0}^na_kx^k$ et $Q:x\mapsto\sum_{k=0}^nb_kx^k$ deux polynômes.</t>
+        </is>
+      </c>
+      <c r="H522" s="10" t="inlineStr">
+        <is>
+          <t>À quelle condition $P$ est-il le polynôme nul ? À quelle condition $P=Q$ ?</t>
+        </is>
+      </c>
+      <c r="I522" s="9" t="inlineStr">
+        <is>
+          <t>$P$ est nul si et seulement si tous ses coefficients sont nuls : $a_0=\dots=a_n=0$. Par conséquent $P=Q$ si et seulement si $a_k=b_k$ pour tout $k$ (on peut identifier les coefficients).</t>
+        </is>
+      </c>
+      <c r="J522" s="9" t="inlineStr">
+        <is>
+          <t>« Unicité de l'écriture des polynômes : un polynôme à coefficients dans R est nul si et seulement si tous ses coefficients sont nuls. »</t>
+        </is>
+      </c>
+      <c r="K522" s="9" t="n"/>
+      <c r="L522" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les polynômes » 2024</t>
+        </is>
+      </c>
+      <c r="M522" s="11" t="n"/>
+      <c r="N522" s="11" t="n"/>
+    </row>
+    <row r="523">
+      <c r="A523" s="9" t="inlineStr">
+        <is>
+          <t>M522</t>
+        </is>
+      </c>
+      <c r="B523" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C523" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D523" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre – Polynômes réels</t>
+        </is>
+      </c>
+      <c r="E523" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F523" s="9" t="inlineStr">
+        <is>
+          <t>Coefficient dominant – Vocabulaire</t>
+        </is>
+      </c>
+      <c r="G523" s="9" t="inlineStr">
+        <is>
+          <t>Soit $P:x\mapsto\sum_{k=0}^na_kx^k$ un polynôme non nul avec $a_n\neq0$.</t>
+        </is>
+      </c>
+      <c r="H523" s="10" t="inlineStr">
+        <is>
+          <t>Définir le degré, le coefficient dominant, le terme dominant, le coefficient constant, un polynôme unitaire. Quel est le degré du polynôme nul ?</t>
+        </is>
+      </c>
+      <c r="I523" s="9" t="inlineStr">
+        <is>
+          <t>$\deg P=n$ ; coefficient dominant $a_n$ ; terme dominant $a_nx^n$ ; coefficient constant $a_0=P(0)$ ; $P$ est unitaire si $a_n=1$. Par convention, le polynôme nul est de degré $-\infty$. En 2e année : $\mathbb K_n[X]$ désigne les polynômes de degré $\le n$.</t>
+        </is>
+      </c>
+      <c r="J523" s="9" t="inlineStr">
+        <is>
+          <t>« Coefficient dominant. Degré d'un polynôme. On convient que le polynôme nul est de degré −∞. »</t>
+        </is>
+      </c>
+      <c r="K523" s="9" t="n"/>
+      <c r="L523" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les polynômes » 2024</t>
+        </is>
+      </c>
+      <c r="M523" s="11" t="n"/>
+      <c r="N523" s="11" t="n"/>
+    </row>
+    <row r="524">
+      <c r="A524" s="9" t="inlineStr">
+        <is>
+          <t>M523</t>
+        </is>
+      </c>
+      <c r="B524" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C524" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D524" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre – Polynômes réels</t>
+        </is>
+      </c>
+      <c r="E524" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F524" s="9" t="inlineStr">
+        <is>
+          <t>Opérations sur les polynômes</t>
+        </is>
+      </c>
+      <c r="G524" s="9" t="inlineStr">
+        <is>
+          <t>Soient $P$ et $Q$ deux polynômes non nuls et $\lambda$ un réel.</t>
+        </is>
+      </c>
+      <c r="H524" s="10" t="inlineStr">
+        <is>
+          <t>Que dire de $\lambda P+Q$, $PQ$ et $P\circ Q$ ? Donner le coefficient dominant de $PQ$.</t>
+        </is>
+      </c>
+      <c r="I524" s="9" t="inlineStr">
+        <is>
+          <t>Ce sont des polynômes. Le coefficient dominant (resp. terme dominant) de $PQ$ est le produit des coefficients (resp. termes) dominants de $P$ et $Q$ ; en particulier $PQ\neq0$. Coefficients du produit : $c_k=\sum_{i+j=k}a_ib_j$.</t>
+        </is>
+      </c>
+      <c r="J524" s="9" t="inlineStr">
+        <is>
+          <t>« Les opérations usuelles (combinaison linéaire, produit, composée) sur les polynômes fournissent des polynômes. »</t>
+        </is>
+      </c>
+      <c r="K524" s="9" t="n"/>
+      <c r="L524" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les polynômes » 2024</t>
+        </is>
+      </c>
+      <c r="M524" s="11" t="n"/>
+      <c r="N524" s="11" t="n"/>
+    </row>
+    <row r="525">
+      <c r="A525" s="9" t="inlineStr">
+        <is>
+          <t>M524</t>
+        </is>
+      </c>
+      <c r="B525" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C525" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D525" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre – Polynômes réels</t>
+        </is>
+      </c>
+      <c r="E525" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F525" s="9" t="inlineStr">
+        <is>
+          <t>Polynôme dérivé – Propriétés</t>
+        </is>
+      </c>
+      <c r="G525" s="9" t="inlineStr">
+        <is>
+          <t>Soient $P$ et $Q$ deux polynômes et $\lambda$ un réel.</t>
+        </is>
+      </c>
+      <c r="H525" s="10" t="inlineStr">
+        <is>
+          <t>Donner le degré de $P'$ et les règles de dérivation de $P+Q$, $\lambda P$ et $PQ$.</t>
+        </is>
+      </c>
+      <c r="I525" s="9" t="inlineStr">
+        <is>
+          <t>Si $\deg P\ge1$, $\deg P'=\deg P-1$ ; si $P$ est constant, $P'=0$. $(P+Q)'=P'+Q'$ ; $(\lambda P)'=\lambda P'$ ; $(PQ)'=P'Q+PQ'$. Si $k&gt;\deg P$, $P^{(k)}=0$.</t>
+        </is>
+      </c>
+      <c r="J525" s="9" t="inlineStr">
+        <is>
+          <t>« Polynôme dérivé. Degré du polynôme dérivé. »</t>
+        </is>
+      </c>
+      <c r="K525" s="9" t="n"/>
+      <c r="L525" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les polynômes » 2024</t>
+        </is>
+      </c>
+      <c r="M525" s="11" t="n"/>
+      <c r="N525" s="11" t="n"/>
+    </row>
+    <row r="526">
+      <c r="A526" s="9" t="inlineStr">
+        <is>
+          <t>M525</t>
+        </is>
+      </c>
+      <c r="B526" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C526" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D526" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre – Polynômes réels</t>
+        </is>
+      </c>
+      <c r="E526" s="9" t="inlineStr">
+        <is>
+          <t>Théorème</t>
+        </is>
+      </c>
+      <c r="F526" s="9" t="inlineStr">
+        <is>
+          <t>Racine et factorisation</t>
+        </is>
+      </c>
+      <c r="G526" s="9" t="inlineStr">
+        <is>
+          <t>Soient $P$ un polynôme et $\alpha$ un réel.</t>
+        </is>
+      </c>
+      <c r="H526" s="10" t="inlineStr">
+        <is>
+          <t>Caractériser par une factorisation le fait que $\alpha$ est racine de $P$, puis généraliser à plusieurs racines.</t>
+        </is>
+      </c>
+      <c r="I526" s="9" t="inlineStr">
+        <is>
+          <t>$P(\alpha)=0\iff$ il existe un polynôme $Q$ tel que $P(x)=(x-\alpha)Q(x)$ pour tout $x$. Si $\alpha_1,\dots,\alpha_k$ sont des racines deux à deux distinctes de $P$, alors $P(x)=(x-\alpha_1)\cdots(x-\alpha_k)Q(x)$ avec $Q$ polynôme.</t>
+        </is>
+      </c>
+      <c r="J526" s="9" t="inlineStr">
+        <is>
+          <t>« Un nombre réel α ∈ R est racine d'un polynôme P si et seulement s'il existe un polynôme Q tel que P(x) = (x − α)Q(x) […] Généralisation à plusieurs racines distinctes. »</t>
+        </is>
+      </c>
+      <c r="K526" s="9" t="n"/>
+      <c r="L526" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les polynômes » 2024</t>
+        </is>
+      </c>
+      <c r="M526" s="11" t="n"/>
+      <c r="N526" s="11" t="n"/>
+    </row>
+    <row r="527">
+      <c r="A527" s="9" t="inlineStr">
+        <is>
+          <t>M526</t>
+        </is>
+      </c>
+      <c r="B527" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C527" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D527" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre – Polynômes réels</t>
+        </is>
+      </c>
+      <c r="E527" s="9" t="inlineStr">
+        <is>
+          <t>Théorème</t>
+        </is>
+      </c>
+      <c r="F527" s="9" t="inlineStr">
+        <is>
+          <t>Nombre de racines et degré</t>
+        </is>
+      </c>
+      <c r="G527" s="9" t="inlineStr">
+        <is>
+          <t>Soient $n\in\mathbb N$ et $P$, $Q$ deux polynômes.</t>
+        </is>
+      </c>
+      <c r="H527" s="10" t="inlineStr">
+        <is>
+          <t>Majorer le nombre de racines d'un polynôme non nul et en donner les conséquences.</t>
+        </is>
+      </c>
+      <c r="I527" s="9" t="inlineStr">
+        <is>
+          <t>Un polynôme non nul de degré $n$ a au plus $n$ racines distinctes. Donc : si $\deg P\le n$ et $P$ a au moins $n+1$ racines distinctes, $P=0$ ; si $P$ a une infinité de racines, $P=0$ ; si $P$ et $Q$ coïncident en une infinité de points, $P=Q$.</t>
+        </is>
+      </c>
+      <c r="J527" s="9" t="inlineStr">
+        <is>
+          <t>« Le nombre de racines distinctes d'un polynôme non nul est majoré par son degré. »</t>
+        </is>
+      </c>
+      <c r="K527" s="9" t="n"/>
+      <c r="L527" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les polynômes » 2024</t>
+        </is>
+      </c>
+      <c r="M527" s="11" t="n"/>
+      <c r="N527" s="11" t="n"/>
+    </row>
+    <row r="528">
+      <c r="A528" s="9" t="inlineStr">
+        <is>
+          <t>M527</t>
+        </is>
+      </c>
+      <c r="B528" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C528" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D528" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre – Polynômes réels</t>
+        </is>
+      </c>
+      <c r="E528" s="9" t="inlineStr">
+        <is>
+          <t>Théorème</t>
+        </is>
+      </c>
+      <c r="F528" s="9" t="inlineStr">
+        <is>
+          <t>Polynôme de degré n à n racines distinctes</t>
+        </is>
+      </c>
+      <c r="G528" s="9" t="inlineStr">
+        <is>
+          <t>Soit $P$ un polynôme de degré $n\ge1$, de coefficient dominant $a_n$, ayant $n$ racines distinctes $\alpha_1,\dots,\alpha_n$.</t>
+        </is>
+      </c>
+      <c r="H528" s="10" t="inlineStr">
+        <is>
+          <t>Donner la forme factorisée de $P$.</t>
+        </is>
+      </c>
+      <c r="I528" s="9" t="inlineStr">
+        <is>
+          <t>$P(x)=a_n(x-\alpha_1)\cdots(x-\alpha_n)$ pour tout $x$, et ce sont ses seules racines.</t>
+        </is>
+      </c>
+      <c r="J528" s="9" t="inlineStr">
+        <is>
+          <t>« Un polynôme de degré n ∈ N* possédant n racines distinctes s'écrit sous la forme P : x ↦ a_n(x − α1)···(x − αn). »</t>
+        </is>
+      </c>
+      <c r="K528" s="9" t="n"/>
+      <c r="L528" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les polynômes » 2024</t>
+        </is>
+      </c>
+      <c r="M528" s="11" t="n"/>
+      <c r="N528" s="11" t="n"/>
+    </row>
+    <row r="529">
+      <c r="A529" s="9" t="inlineStr">
+        <is>
+          <t>M528</t>
+        </is>
+      </c>
+      <c r="B529" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C529" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D529" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre – Polynômes réels</t>
+        </is>
+      </c>
+      <c r="E529" s="9" t="inlineStr">
+        <is>
+          <t>Théorème</t>
+        </is>
+      </c>
+      <c r="F529" s="9" t="inlineStr">
+        <is>
+          <t>Racine multiple et dérivée</t>
+        </is>
+      </c>
+      <c r="G529" s="9" t="inlineStr">
+        <is>
+          <t>Soient $P$ un polynôme et $\alpha$ une racine de $P$.</t>
+        </is>
+      </c>
+      <c r="H529" s="10" t="inlineStr">
+        <is>
+          <t>Caractériser à l'aide de $P'$ le fait que $\alpha$ est racine multiple de $P$.</t>
+        </is>
+      </c>
+      <c r="I529" s="9" t="inlineStr">
+        <is>
+          <t>$\alpha$ est racine multiple de $P$ si et seulement si $P(\alpha)=P'(\alpha)=0$. Ainsi $\alpha$ est racine simple si et seulement si $P(\alpha)=0$ et $P'(\alpha)\neq0$.</t>
+        </is>
+      </c>
+      <c r="J529" s="9" t="inlineStr">
+        <is>
+          <t>« Une racine α d'un polynôme P est une racine multiple si et seulement si P′(α) = 0. »</t>
+        </is>
+      </c>
+      <c r="K529" s="9" t="n"/>
+      <c r="L529" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les polynômes » 2024</t>
+        </is>
+      </c>
+      <c r="M529" s="11" t="n"/>
+      <c r="N529" s="11" t="n"/>
+    </row>
+    <row r="530">
+      <c r="A530" s="9" t="inlineStr">
+        <is>
+          <t>M529</t>
+        </is>
+      </c>
+      <c r="B530" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C530" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D530" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre – Polynômes réels</t>
+        </is>
+      </c>
+      <c r="E530" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F530" s="9" t="inlineStr">
+        <is>
+          <t>Polynôme de degré impair</t>
+        </is>
+      </c>
+      <c r="G530" s="9" t="inlineStr">
+        <is>
+          <t>Soit $P$ un polynôme à coefficients réels de degré impair.</t>
+        </is>
+      </c>
+      <c r="H530" s="10" t="inlineStr">
+        <is>
+          <t>Que peut-on dire des racines réelles de $P$ ?</t>
+        </is>
+      </c>
+      <c r="I530" s="9" t="inlineStr">
+        <is>
+          <t>$P$ admet au moins une racine réelle (théorème des valeurs intermédiaires : $P$ tend vers $+\infty$ d'un côté et $-\infty$ de l'autre).</t>
+        </is>
+      </c>
+      <c r="J530" s="9" t="inlineStr">
+        <is>
+          <t>« Tout polynôme de degré impair a au moins une racine réelle. »</t>
+        </is>
+      </c>
+      <c r="K530" s="9" t="n"/>
+      <c r="L530" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les polynômes » 2024</t>
+        </is>
+      </c>
+      <c r="M530" s="11" t="n"/>
+      <c r="N530" s="11" t="n"/>
+    </row>
+    <row r="531">
+      <c r="A531" s="9" t="inlineStr">
+        <is>
+          <t>M530</t>
+        </is>
+      </c>
+      <c r="B531" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C531" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2</t>
+        </is>
+      </c>
+      <c r="D531" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2 · Algèbre – Polynômes</t>
+        </is>
+      </c>
+      <c r="E531" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F531" s="9" t="inlineStr">
+        <is>
+          <t>Racines complexes d’un polynôme réel</t>
+        </is>
+      </c>
+      <c r="G531" s="9" t="inlineStr">
+        <is>
+          <t>Soient $P$ un polynôme à coefficients réels et $\alpha\in\mathbb C$.</t>
+        </is>
+      </c>
+      <c r="H531" s="10" t="inlineStr">
+        <is>
+          <t>Si $\alpha$ est racine de $P$, que dire de $\bar\alpha$ ?</t>
+        </is>
+      </c>
+      <c r="I531" s="9" t="inlineStr">
+        <is>
+          <t>$\bar\alpha$ est aussi racine de $P$, car $P(\bar\alpha)=\overline{P(\alpha)}=0$ ; les racines non réelles vont par paires conjuguées.</t>
+        </is>
+      </c>
+      <c r="J531" s="9" t="inlineStr">
+        <is>
+          <t>« Cas des polynômes réels : si α est racine, ᾱ est aussi racine. »</t>
+        </is>
+      </c>
+      <c r="K531" s="9" t="n"/>
+      <c r="L531" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Les polynômes » 2024</t>
+        </is>
+      </c>
+      <c r="M531" s="11" t="n"/>
+      <c r="N531" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M521" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M531" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -34374,7 +34982,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$521,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$531,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -34389,7 +34997,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$521,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$531,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -34404,7 +35012,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$521,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$531,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -34431,7 +35039,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$521)</f>
+        <f>COUNTA(Fiches!$M$2:$M$531)</f>
         <v/>
       </c>
     </row>
@@ -34477,15 +35085,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A13,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A13,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A13,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A13,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A13,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A13,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -34500,15 +35108,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A14,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A14,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A14,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A14,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A14,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A14,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -34523,15 +35131,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A15,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A15,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A15,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A15,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A15,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A15,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -34546,15 +35154,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A16,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A16,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A16,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A16,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A16,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A16,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -34569,15 +35177,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A17,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A17,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A17,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A17,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A17,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A17,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -34592,15 +35200,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A18,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A18,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A18,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A18,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A18,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A18,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -34615,15 +35223,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A19,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A19,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A19,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A19,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A19,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A19,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -34638,15 +35246,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A20,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A20,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A20,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A20,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A20,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A20,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -34661,15 +35269,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A21,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A21,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A21,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A21,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A21,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A21,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -34684,15 +35292,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A22,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A22,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A22,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A22,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A22,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A22,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -34707,15 +35315,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A23,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A23,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A23,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A23,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A23,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A23,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -34730,15 +35338,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A24,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A24,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A24,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A24,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A24,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A24,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -34753,15 +35361,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A25,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A25,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A25,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A25,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A25,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A25,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -34776,15 +35384,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A26,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A26,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A26,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A26,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A26,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A26,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -34799,15 +35407,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A27,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A27,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A27,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A27,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A27,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A27,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -34822,15 +35430,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A28,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A28,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A28,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A28,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A28,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A28,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -34845,15 +35453,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A29,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A29,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A29,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A29,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A29,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A29,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -34868,15 +35476,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A30,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A30,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A30,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A30,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A30,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A30,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -34891,15 +35499,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A31,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A31,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A31,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A31,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A31,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A31,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -34914,15 +35522,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A32,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A32,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A32,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A32,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A32,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A32,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -34937,15 +35545,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A33,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A33,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A33,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A33,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A33,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A33,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -34960,15 +35568,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A34,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A34,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A34,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A34,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A34,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A34,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -34983,15 +35591,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A35,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A35,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A35,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A35,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A35,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A35,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -35006,15 +35614,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A36,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A36,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A36,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A36,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A36,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A36,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -35029,15 +35637,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A37,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A37,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A37,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A37,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A37,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A37,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -35052,15 +35660,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A38,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A38,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A38,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A38,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A38,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A38,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -35075,15 +35683,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A39,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A39,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A39,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A39,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A39,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A39,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -35098,15 +35706,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A40,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A40,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A40,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A40,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A40,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A40,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -35121,15 +35729,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A41,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A41,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A41,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A41,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A41,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A41,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -35144,15 +35752,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A42,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A42,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A42,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A42,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A42,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A42,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -35167,15 +35775,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A43,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A43,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A43,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A43,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A43,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A43,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -35190,15 +35798,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A44,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A44,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A44,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A44,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A44,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A44,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -35213,15 +35821,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A45,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A45,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A45,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A45,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A45,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A45,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -35236,15 +35844,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A46,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A46,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A46,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A46,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A46,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A46,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -35259,15 +35867,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A47,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A47,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A47,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A47,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A47,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A47,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -35282,15 +35890,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A48,Fiches!$B$2:$B$521,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A48,Fiches!$B$2:$B$531,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A48,Fiches!$B$2:$B$521,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A48,Fiches!$B$2:$B$531,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$521,$A48,Fiches!$B$2:$B$521,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$531,$A48,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Compléments : 10 fiches pour couvrir tout le contenu des cours de référence
Re/Im, opérations et composée de fonctions, norme et distance, matrices
élémentaires, produit par colonnes, antisymétriques, polynômes pairs/impairs,
divisibilité, a^n − b^n ; M484 complétée. Hors programme du cours : orange.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N531"/>
+  <dimension ref="A1:N541"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -28960,12 +28960,12 @@
       </c>
       <c r="H485" s="10" t="inlineStr">
         <is>
-          <t>Quelle forme de solution particulière chercher si $g(x)=P(x)$ ? $P(x)e^{mx}$ ? $P(x)\cos(mx)$ ?</t>
+          <t>Quelle forme de solution particulière chercher si $g(x)=P(x)$ ? $P(x)e^{mx}$ ? $P(x)\cos(mx)$ ? $\cos(mx)e^{\alpha x}$ ?</t>
         </is>
       </c>
       <c r="I485" s="9" t="inlineStr">
         <is>
-          <t>$g=P$ : un polynôme de même degré que $P$. $g=Pe^{mx}$ : $Q(x)e^{mx}$ avec $\deg Q=\deg P$ si $m\neq-a$, et $xQ(x)e^{mx}$ si $m=-a$. $g=P\cos(mx)$ ($m\neq0$) : $Q_1(x)\cos(mx)+Q_2(x)\sin(mx)$ avec $\deg Q_1=\deg Q_2=\deg P$.</t>
+          <t>$g=P$ : un polynôme de même degré que $P$. $g=Pe^{mx}$ : $Q(x)e^{mx}$ avec $\deg Q=\deg P$ si $m\neq-a$, et $xQ(x)e^{mx}$ si $m=-a$. $g=P\cos(mx)$ ($m\neq0$) : $Q_1(x)\cos(mx)+Q_2(x)\sin(mx)$ avec $\deg Q_1=\deg Q_2=\deg P$. $g=\cos(mx)e^{\alpha x}$ : $(\lambda\cos(mx)+\mu\sin(mx))e^{\alpha x}$.</t>
         </is>
       </c>
       <c r="J485" s="9" t="inlineStr">
@@ -31741,11 +31741,611 @@
       </c>
       <c r="M531" s="11" t="n"/>
       <c r="N531" s="11" t="n"/>
+    </row>
+    <row r="532">
+      <c r="A532" s="9" t="inlineStr">
+        <is>
+          <t>M532</t>
+        </is>
+      </c>
+      <c r="B532" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C532" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D532" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 4 – Nombres complexes</t>
+        </is>
+      </c>
+      <c r="E532" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F532" s="9" t="inlineStr">
+        <is>
+          <t>Parties réelle et imaginaire – Propriétés</t>
+        </is>
+      </c>
+      <c r="G532" s="9" t="inlineStr">
+        <is>
+          <t>Soient $z,z_1,\dots,z_n$ des nombres complexes et $\lambda$ un réel.</t>
+        </is>
+      </c>
+      <c r="H532" s="10" t="inlineStr">
+        <is>
+          <t>Donner les propriétés de $\mathrm{Re}$ et $\mathrm{Im}$ : somme, produit par un réel, comparaison avec le module.</t>
+        </is>
+      </c>
+      <c r="I532" s="9" t="inlineStr">
+        <is>
+          <t>$\mathrm{Re}(z_1+\dots+z_n)=\mathrm{Re}(z_1)+\dots+\mathrm{Re}(z_n)$ et de même pour $\mathrm{Im}$ ; $\mathrm{Re}(\lambda z)=\lambda\mathrm{Re}(z)$ et $\mathrm{Im}(\lambda z)=\lambda\mathrm{Im}(z)$ ($\lambda$ réel) ; $|\mathrm{Re}(z)|\le|z|$ et $|\mathrm{Im}(z)|\le|z|$.</t>
+        </is>
+      </c>
+      <c r="J532" s="9" t="inlineStr">
+        <is>
+          <t>« Propriétés élémentaires de Re et Im. »</t>
+        </is>
+      </c>
+      <c r="K532" s="9" t="n"/>
+      <c r="L532" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST 2024 (compléments)</t>
+        </is>
+      </c>
+      <c r="M532" s="11" t="n"/>
+      <c r="N532" s="11" t="n"/>
+    </row>
+    <row r="533">
+      <c r="A533" s="9" t="inlineStr">
+        <is>
+          <t>M533</t>
+        </is>
+      </c>
+      <c r="B533" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C533" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D533" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E533" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F533" s="9" t="inlineStr">
+        <is>
+          <t>Opérations sur les fonctions</t>
+        </is>
+      </c>
+      <c r="G533" s="9" t="inlineStr">
+        <is>
+          <t>Soient $f,g:I\to\mathbb R$ deux fonctions et $\lambda$ un réel.</t>
+        </is>
+      </c>
+      <c r="H533" s="10" t="inlineStr">
+        <is>
+          <t>Définir $\lambda f$, $f+g$, $fg$, $\frac1f$ et la relation $f\le g$.</t>
+        </is>
+      </c>
+      <c r="I533" s="9" t="inlineStr">
+        <is>
+          <t>$(\lambda f)(x)=\lambda f(x)$ ; $(f+g)(x)=f(x)+g(x)$ ; $(fg)(x)=f(x)g(x)$ ; $\frac1f$ est définie sur $J=\{x\in I,\ f(x)\neq0\}$ par $\left(\frac1f\right)(x)=\frac1{f(x)}$ ; $f\le g\iff\forall x\in I,\ f(x)\le g(x)$.</t>
+        </is>
+      </c>
+      <c r="J533" s="9" t="inlineStr">
+        <is>
+          <t>« Opérations algébriques sur les fonctions. »</t>
+        </is>
+      </c>
+      <c r="K533" s="9" t="n"/>
+      <c r="L533" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST 2024 (compléments)</t>
+        </is>
+      </c>
+      <c r="M533" s="11" t="n"/>
+      <c r="N533" s="11" t="n"/>
+    </row>
+    <row r="534">
+      <c r="A534" s="9" t="inlineStr">
+        <is>
+          <t>M534</t>
+        </is>
+      </c>
+      <c r="B534" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C534" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D534" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E534" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F534" s="9" t="inlineStr">
+        <is>
+          <t>Composée de deux fonctions numériques</t>
+        </is>
+      </c>
+      <c r="G534" s="9" t="inlineStr">
+        <is>
+          <t>Soient $f:I\to\mathbb R$ à valeurs dans $J$ et $g:J\to\mathbb R$.</t>
+        </is>
+      </c>
+      <c r="H534" s="10" t="inlineStr">
+        <is>
+          <t>Définir $g\circ f$ et préciser la condition d'existence.</t>
+        </is>
+      </c>
+      <c r="I534" s="9" t="inlineStr">
+        <is>
+          <t>$g\circ f:I\to\mathbb R$, $x\mapsto g(f(x))$. Il faut que $f$ prenne ses valeurs dans l'ensemble de définition de $g$. $g\circ f$ peut exister sans que $f\circ g$ existe, et en général $g\circ f\neq f\circ g$.</t>
+        </is>
+      </c>
+      <c r="J534" s="9" t="inlineStr">
+        <is>
+          <t>« Composition de fonctions. »</t>
+        </is>
+      </c>
+      <c r="K534" s="9" t="n"/>
+      <c r="L534" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST 2024 (compléments)</t>
+        </is>
+      </c>
+      <c r="M534" s="11" t="n"/>
+      <c r="N534" s="11" t="n"/>
+    </row>
+    <row r="535">
+      <c r="A535" s="9" t="inlineStr">
+        <is>
+          <t>M535</t>
+        </is>
+      </c>
+      <c r="B535" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C535" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D535" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Géométrie 1</t>
+        </is>
+      </c>
+      <c r="E535" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F535" s="9" t="inlineStr">
+        <is>
+          <t>Norme et distance</t>
+        </is>
+      </c>
+      <c r="G535" s="9" t="inlineStr">
+        <is>
+          <t>Soient $\vec u$, $\vec v$ deux vecteurs du plan ou de l'espace, $\alpha$ un réel, $A$ et $B$ deux points.</t>
+        </is>
+      </c>
+      <c r="H535" s="10" t="inlineStr">
+        <is>
+          <t>Donner les propriétés de la norme, la distance $AB$ et la définition d'un vecteur normé.</t>
+        </is>
+      </c>
+      <c r="I535" s="9" t="inlineStr">
+        <is>
+          <t>$\|\alpha\vec u\|=|\alpha|\,\|\vec u\|$ ; $\|\vec u+\vec v\|\le\|\vec u\|+\|\vec v\|$ ; $\|\vec u\|\ge0$ et $\|\vec u\|=0\iff\vec u=\vec0$. $AB=\|\overrightarrow{AB}\|$. $\vec u$ est normé (unitaire) si $\|\vec u\|=1$.</t>
+        </is>
+      </c>
+      <c r="J535" s="9" t="inlineStr">
+        <is>
+          <t>« Lien avec la norme. »</t>
+        </is>
+      </c>
+      <c r="K535" s="9" t="n"/>
+      <c r="L535" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST 2024 (compléments)</t>
+        </is>
+      </c>
+      <c r="M535" s="11" t="n"/>
+      <c r="N535" s="11" t="n"/>
+    </row>
+    <row r="536">
+      <c r="A536" s="9" t="inlineStr">
+        <is>
+          <t>M536</t>
+        </is>
+      </c>
+      <c r="B536" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C536" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D536" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre linéaire 2 – Matrices</t>
+        </is>
+      </c>
+      <c r="E536" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F536" s="9" t="inlineStr">
+        <is>
+          <t>Matrices élémentaires</t>
+        </is>
+      </c>
+      <c r="G536" s="9" t="inlineStr">
+        <is>
+          <t>Soient $n,p\in\mathbb N^*$ et $A=(a_{i,j})\in\mathcal M_{n,p}(\mathbb K)$.</t>
+        </is>
+      </c>
+      <c r="H536" s="10" t="inlineStr">
+        <is>
+          <t>Définir les matrices élémentaires $E_{i,j}$ et écrire $A$ à l'aide de ces matrices.</t>
+        </is>
+      </c>
+      <c r="I536" s="9" t="inlineStr">
+        <is>
+          <t>$E_{i,j}$ est la matrice de $\mathcal M_{n,p}(\mathbb K)$ dont le seul coefficient non nul vaut $1$, en position $(i,j)$. $A=\displaystyle\sum_{\substack{1\le i\le n\\1\le j\le p}}a_{i,j}E_{i,j}$.</t>
+        </is>
+      </c>
+      <c r="J536" s="9" t="inlineStr">
+        <is>
+          <t>Programme muet ; dans le cours de référence.</t>
+        </is>
+      </c>
+      <c r="K536" s="9" t="n"/>
+      <c r="L536" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST 2024 (compléments)</t>
+        </is>
+      </c>
+      <c r="M536" s="11" t="n"/>
+      <c r="N536" s="11" t="n"/>
+    </row>
+    <row r="537">
+      <c r="A537" s="9" t="inlineStr">
+        <is>
+          <t>M537</t>
+        </is>
+      </c>
+      <c r="B537" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C537" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D537" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre linéaire 2 – Matrices</t>
+        </is>
+      </c>
+      <c r="E537" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F537" s="9" t="inlineStr">
+        <is>
+          <t>Produit matriciel par colonnes et par lignes</t>
+        </is>
+      </c>
+      <c r="G537" s="9" t="inlineStr">
+        <is>
+          <t>Soient $A$ une matrice, $C_1,\dots,C_p$ ses colonnes, $L_1,\dots,L_n$ ses lignes, et $x_1,\dots,x_p$ des scalaires.</t>
+        </is>
+      </c>
+      <c r="H537" s="10" t="inlineStr">
+        <is>
+          <t>Interpréter les produits $A\begin{pmatrix}x_1\\\vdots\\x_p\end{pmatrix}$, $AB$ en colonnes et $BA$ en lignes.</t>
+        </is>
+      </c>
+      <c r="I537" s="9" t="inlineStr">
+        <is>
+          <t>$A\begin{pmatrix}x_1\\\vdots\\x_p\end{pmatrix}=x_1C_1+\dots+x_pC_p$ (combinaison des colonnes). Les colonnes de $BA$ sont les $BC_j$ ; les lignes de $AB$ sont les $L_iB$. Une ligne nulle dans $A$ donne une ligne nulle dans $AB$ ; une colonne nulle dans $B$ donne une colonne nulle dans $AB$.</t>
+        </is>
+      </c>
+      <c r="J537" s="9" t="inlineStr">
+        <is>
+          <t>Programme muet ; dans le cours de référence.</t>
+        </is>
+      </c>
+      <c r="K537" s="9" t="n"/>
+      <c r="L537" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST 2024 (compléments)</t>
+        </is>
+      </c>
+      <c r="M537" s="11" t="n"/>
+      <c r="N537" s="11" t="n"/>
+    </row>
+    <row r="538">
+      <c r="A538" s="9" t="inlineStr">
+        <is>
+          <t>M538</t>
+        </is>
+      </c>
+      <c r="B538" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C538" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D538" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre linéaire 2 – Matrices</t>
+        </is>
+      </c>
+      <c r="E538" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F538" s="9" t="inlineStr">
+        <is>
+          <t>Matrices antisymétriques</t>
+        </is>
+      </c>
+      <c r="G538" s="9" t="inlineStr">
+        <is>
+          <t>Soit $A\in\mathcal M_n(\mathbb K)$.</t>
+        </is>
+      </c>
+      <c r="H538" s="10" t="inlineStr">
+        <is>
+          <t>Définir : $A$ est antisymétrique.</t>
+        </is>
+      </c>
+      <c r="I538" s="9" t="inlineStr">
+        <is>
+          <t>$A^T=-A$ ; ensemble noté $\mathcal A_n(\mathbb K)$. Toute matrice carrée s'écrit de façon unique comme somme d'une matrice symétrique et d'une matrice antisymétrique : $M=\frac{M+M^T}2+\frac{M-M^T}2$.</t>
+        </is>
+      </c>
+      <c r="J538" s="9" t="inlineStr">
+        <is>
+          <t>Le programme ne cite que les matrices symétriques ; dans le cours de référence.</t>
+        </is>
+      </c>
+      <c r="K538" s="9" t="n"/>
+      <c r="L538" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST 2024 (compléments)</t>
+        </is>
+      </c>
+      <c r="M538" s="11" t="n"/>
+      <c r="N538" s="11" t="n"/>
+    </row>
+    <row r="539">
+      <c r="A539" s="9" t="inlineStr">
+        <is>
+          <t>M539</t>
+        </is>
+      </c>
+      <c r="B539" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C539" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D539" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre – Polynômes réels</t>
+        </is>
+      </c>
+      <c r="E539" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F539" s="9" t="inlineStr">
+        <is>
+          <t>Polynômes pairs et impairs</t>
+        </is>
+      </c>
+      <c r="G539" s="9" t="inlineStr">
+        <is>
+          <t>Soit $P$ un polynôme.</t>
+        </is>
+      </c>
+      <c r="H539" s="10" t="inlineStr">
+        <is>
+          <t>Caractériser par ses coefficients le fait que $P$ est pair, impair.</t>
+        </is>
+      </c>
+      <c r="I539" s="9" t="inlineStr">
+        <is>
+          <t>$P$ est pair ($P(-x)=P(x)$) si et seulement s'il ne comporte que des puissances paires : $P=\sum a_ix^{2i}$. $P$ est impair si et seulement s'il ne comporte que des puissances impaires : $P=\sum a_ix^{2i+1}$.</t>
+        </is>
+      </c>
+      <c r="J539" s="9" t="inlineStr">
+        <is>
+          <t>Programme muet ; dans le cours de référence.</t>
+        </is>
+      </c>
+      <c r="K539" s="9" t="n"/>
+      <c r="L539" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST 2024 (compléments)</t>
+        </is>
+      </c>
+      <c r="M539" s="11" t="n"/>
+      <c r="N539" s="11" t="n"/>
+    </row>
+    <row r="540">
+      <c r="A540" s="9" t="inlineStr">
+        <is>
+          <t>M540</t>
+        </is>
+      </c>
+      <c r="B540" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C540" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D540" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre – Polynômes réels</t>
+        </is>
+      </c>
+      <c r="E540" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F540" s="9" t="inlineStr">
+        <is>
+          <t>Divisibilité de polynômes</t>
+        </is>
+      </c>
+      <c r="G540" s="9" t="inlineStr">
+        <is>
+          <t>Soient $P$ et $Q$ deux polynômes avec $Q\neq0$.</t>
+        </is>
+      </c>
+      <c r="H540" s="10" t="inlineStr">
+        <is>
+          <t>Définir : $Q$ divise $P$, et comparer alors les degrés.</t>
+        </is>
+      </c>
+      <c r="I540" s="9" t="inlineStr">
+        <is>
+          <t>$Q$ divise $P$ (ou $P$ est un multiple de $Q$) s'il existe un polynôme $R$ tel que $P=QR$. Si de plus $P\neq0$, alors $\deg Q\le\deg P$.</t>
+        </is>
+      </c>
+      <c r="J540" s="9" t="inlineStr">
+        <is>
+          <t>Programme : division euclidienne hors programme, mais « P(x) = (x − α)Q(x) » utilise la divisibilité ; dans le cours de référence.</t>
+        </is>
+      </c>
+      <c r="K540" s="9" t="n"/>
+      <c r="L540" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST 2024 (compléments)</t>
+        </is>
+      </c>
+      <c r="M540" s="11" t="n"/>
+      <c r="N540" s="11" t="n"/>
+    </row>
+    <row r="541">
+      <c r="A541" s="9" t="inlineStr">
+        <is>
+          <t>M541</t>
+        </is>
+      </c>
+      <c r="B541" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C541" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D541" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Algèbre – Polynômes réels</t>
+        </is>
+      </c>
+      <c r="E541" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F541" s="9" t="inlineStr">
+        <is>
+          <t>Factorisation de $a^n-b^n$</t>
+        </is>
+      </c>
+      <c r="G541" s="9" t="inlineStr">
+        <is>
+          <t>Soient $a$, $b$ deux nombres complexes et $n\in\mathbb N^*$.</t>
+        </is>
+      </c>
+      <c r="H541" s="10" t="inlineStr">
+        <is>
+          <t>Factoriser $a^n-b^n$.</t>
+        </is>
+      </c>
+      <c r="I541" s="9" t="inlineStr">
+        <is>
+          <t>$a^n-b^n=(a-b)\displaystyle\sum_{k=0}^{n-1}a^kb^{n-1-k}=(a-b)(a^{n-1}+a^{n-2}b+\dots+b^{n-1})$. De même pour deux polynômes $P^n-Q^n$.</t>
+        </is>
+      </c>
+      <c r="J541" s="9" t="inlineStr">
+        <is>
+          <t>Outils 5 – Méthodes de calcul ; dans le cours de référence (Polynômes).</t>
+        </is>
+      </c>
+      <c r="K541" s="9" t="n"/>
+      <c r="L541" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST 2024 (compléments)</t>
+        </is>
+      </c>
+      <c r="M541" s="11" t="n"/>
+      <c r="N541" s="11" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M531" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M541" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -34982,7 +35582,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$531,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$541,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -34997,7 +35597,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$531,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$541,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -35012,7 +35612,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$531,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$541,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -35039,7 +35639,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$531)</f>
+        <f>COUNTA(Fiches!$M$2:$M$541)</f>
         <v/>
       </c>
     </row>
@@ -35085,15 +35685,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A13,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A13,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A13,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A13,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A13,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A13,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -35108,15 +35708,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A14,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A14,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A14,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A14,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A14,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A14,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -35131,15 +35731,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A15,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A15,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A15,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A15,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A15,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A15,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -35154,15 +35754,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A16,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A16,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A16,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A16,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A16,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A16,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -35177,15 +35777,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A17,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A17,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A17,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A17,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A17,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A17,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -35200,15 +35800,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A18,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A18,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A18,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A18,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A18,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A18,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -35223,15 +35823,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A19,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A19,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A19,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A19,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A19,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A19,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -35246,15 +35846,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A20,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A20,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A20,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A20,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A20,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A20,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -35269,15 +35869,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A21,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A21,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A21,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A21,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A21,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A21,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -35292,15 +35892,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A22,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A22,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A22,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A22,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A22,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A22,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -35315,15 +35915,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A23,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A23,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A23,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A23,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A23,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A23,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -35338,15 +35938,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A24,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A24,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A24,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A24,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A24,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A24,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -35361,15 +35961,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A25,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A25,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A25,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A25,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A25,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A25,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -35384,15 +35984,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A26,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A26,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A26,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A26,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A26,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A26,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -35407,15 +36007,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A27,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A27,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A27,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A27,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A27,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A27,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -35430,15 +36030,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A28,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A28,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A28,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A28,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A28,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A28,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -35453,15 +36053,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A29,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A29,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A29,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A29,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A29,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A29,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -35476,15 +36076,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A30,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A30,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A30,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A30,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A30,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A30,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -35499,15 +36099,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A31,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A31,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A31,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A31,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A31,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A31,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -35522,15 +36122,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A32,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A32,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A32,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A32,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A32,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A32,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -35545,15 +36145,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A33,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A33,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A33,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A33,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A33,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A33,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -35568,15 +36168,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A34,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A34,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A34,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A34,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A34,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A34,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -35591,15 +36191,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A35,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A35,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A35,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A35,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A35,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A35,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -35614,15 +36214,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A36,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A36,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A36,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A36,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A36,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A36,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -35637,15 +36237,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A37,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A37,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A37,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A37,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A37,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A37,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -35660,15 +36260,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A38,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A38,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A38,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A38,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A38,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A38,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -35683,15 +36283,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A39,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A39,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A39,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A39,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A39,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A39,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -35706,15 +36306,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A40,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A40,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A40,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A40,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A40,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A40,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -35729,15 +36329,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A41,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A41,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A41,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A41,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A41,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A41,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -35752,15 +36352,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A42,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A42,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A42,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A42,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A42,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A42,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -35775,15 +36375,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A43,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A43,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A43,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A43,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A43,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A43,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -35798,15 +36398,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A44,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A44,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A44,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A44,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A44,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A44,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -35821,15 +36421,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A45,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A45,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A45,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A45,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A45,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A45,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -35844,15 +36444,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A46,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A46,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A46,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A46,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A46,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A46,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -35867,15 +36467,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A47,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A47,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A47,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A47,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A47,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A47,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -35890,15 +36490,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A48,Fiches!$B$2:$B$531,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A48,Fiches!$B$2:$B$541,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A48,Fiches!$B$2:$B$531,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A48,Fiches!$B$2:$B$541,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$531,$A48,Fiches!$B$2:$B$531,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$541,$A48,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Suites : 6 fiches ajoutées, M172 et M183 complétées
Unicité et conséquences de la convergence, limites de référence, croissances
comparées, bornée × limite nulle, équivalent d'un polynôme en n,
u_{n+1} = f(u_n) avec f croissante (orange).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N541"/>
+  <dimension ref="A1:N547"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -10771,7 +10771,7 @@
       </c>
       <c r="I173" s="9" t="inlineStr">
         <is>
-          <t>Limite d'une somme, d'un produit, d'un produit par un réel, d'un quotient, sauf formes indéterminées $\infty-\infty$, $0\times\infty$, $\frac00$, $\frac\infty\infty$.</t>
+          <t>Limite d'une somme, d'un produit, d'un produit par un réel, d'un quotient, sauf formes indéterminées $\infty-\infty$, $0\times\infty$, $\frac00$, $\frac\infty\infty$. Inverse : si $u_n\to l\neq0$, $\frac1{u_n}\to\frac1l$ ; si $u_n\to\pm\infty$, $\frac1{u_n}\to0$ ; si $u_n\to0$ avec $u_n&gt;0$ (resp. $&lt;0$), $\frac1{u_n}\to+\infty$ (resp. $-\infty$).</t>
         </is>
       </c>
       <c r="J173" s="9" t="inlineStr">
@@ -11404,12 +11404,12 @@
       </c>
       <c r="H184" s="10" t="inlineStr">
         <is>
-          <t>Définir : $(u_n)$ est croissante, décroissante.</t>
+          <t>Définir : $(u_n)$ est croissante, strictement croissante, décroissante, monotone, strictement monotone.</t>
         </is>
       </c>
       <c r="I184" s="9" t="inlineStr">
         <is>
-          <t>$(u_n)$ est croissante si $\forall n,\ u_n\le u_{n+1}$ ; décroissante si $\forall n,\ u_n\ge u_{n+1}$.</t>
+          <t>Croissante : $\forall n,\ u_{n+1}\ge u_n$ ; strictement croissante : $u_{n+1}&gt;u_n$ ; décroissante : $u_{n+1}\le u_n$ ; strictement décroissante : $u_{n+1}&lt;u_n$. Monotone : croissante ou décroissante ; strictement monotone : strictement croissante ou strictement décroissante.</t>
         </is>
       </c>
       <c r="J184" s="9" t="inlineStr">
@@ -32342,10 +32342,370 @@
       <c r="M541" s="11" t="n"/>
       <c r="N541" s="11" t="n"/>
     </row>
+    <row r="542">
+      <c r="A542" s="9" t="inlineStr">
+        <is>
+          <t>M542</t>
+        </is>
+      </c>
+      <c r="B542" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C542" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D542" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 5 – Suites réelles</t>
+        </is>
+      </c>
+      <c r="E542" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F542" s="9" t="inlineStr">
+        <is>
+          <t>Convergence – Unicité et conséquences</t>
+        </is>
+      </c>
+      <c r="G542" s="9" t="inlineStr">
+        <is>
+          <t>Soient $(u_n)$ une suite réelle et $l$ un réel.</t>
+        </is>
+      </c>
+      <c r="H542" s="10" t="inlineStr">
+        <is>
+          <t>Que dire de la limite d'une suite si elle existe ? D'une suite convergente ? Caractériser $u_n\to l$ à l'aide de $|u_n-l|$.</t>
+        </is>
+      </c>
+      <c r="I542" s="9" t="inlineStr">
+        <is>
+          <t>Si une suite a une limite, celle-ci est unique ; on la note $\lim_{n\to+\infty}u_n$. Une suite est convergente si elle tend vers un réel, divergente sinon (limite infinie ou pas de limite). Toute suite convergente est bornée (réciproque fausse). $u_n\to l\iff|u_n-l|\to0$ ; en particulier $u_n\to0\iff|u_n|\to0$.</t>
+        </is>
+      </c>
+      <c r="J542" s="9" t="inlineStr">
+        <is>
+          <t>« Convergence, divergence. Limite infinie. »</t>
+        </is>
+      </c>
+      <c r="K542" s="9" t="n"/>
+      <c r="L542" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Suites : comportement asymptotique » 2025</t>
+        </is>
+      </c>
+      <c r="M542" s="11" t="n"/>
+      <c r="N542" s="11" t="n"/>
+    </row>
+    <row r="543">
+      <c r="A543" s="9" t="inlineStr">
+        <is>
+          <t>M543</t>
+        </is>
+      </c>
+      <c r="B543" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C543" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D543" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 5 – Suites réelles</t>
+        </is>
+      </c>
+      <c r="E543" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F543" s="9" t="inlineStr">
+        <is>
+          <t>Limites de référence</t>
+        </is>
+      </c>
+      <c r="G543" s="9" t="inlineStr">
+        <is>
+          <t>Soient $a$ un réel, $\alpha&gt;0$ et $q$ un réel.</t>
+        </is>
+      </c>
+      <c r="H543" s="10" t="inlineStr">
+        <is>
+          <t>Donner les limites de $\frac1{n^\alpha}$, $n^\alpha$, $\ln n$, $\frac1{(\ln n)^\alpha}$, $e^n$ et $q^n$ selon $q$.</t>
+        </is>
+      </c>
+      <c r="I543" s="9" t="inlineStr">
+        <is>
+          <t>$\frac1{n^\alpha}\to0$ ; $n^\alpha\to+\infty$ (dont $\sqrt n$) ; $(\ln n)^\alpha\to+\infty$ et $\frac1{(\ln n)^\alpha}\to0$ ; $e^n\to+\infty$. $q^n\to0$ si $|q|&lt;1$ ; $q^n=1$ si $q=1$ ; $q^n\to+\infty$ si $q&gt;1$ ; pas de limite si $q\le-1$.</t>
+        </is>
+      </c>
+      <c r="J543" s="9" t="inlineStr">
+        <is>
+          <t>« Opérations sur les limites. » ; limites usuelles des classes antérieures.</t>
+        </is>
+      </c>
+      <c r="K543" s="9" t="n"/>
+      <c r="L543" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Suites : comportement asymptotique » 2025</t>
+        </is>
+      </c>
+      <c r="M543" s="11" t="n"/>
+      <c r="N543" s="11" t="n"/>
+    </row>
+    <row r="544">
+      <c r="A544" s="9" t="inlineStr">
+        <is>
+          <t>M544</t>
+        </is>
+      </c>
+      <c r="B544" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C544" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D544" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 5 – Suites réelles</t>
+        </is>
+      </c>
+      <c r="E544" s="9" t="inlineStr">
+        <is>
+          <t>Théorème</t>
+        </is>
+      </c>
+      <c r="F544" s="9" t="inlineStr">
+        <is>
+          <t>Croissances comparées (suites)</t>
+        </is>
+      </c>
+      <c r="G544" s="9" t="inlineStr">
+        <is>
+          <t>Soient $\alpha\in\mathbb R$, $\beta&gt;0$ et $a&gt;1$.</t>
+        </is>
+      </c>
+      <c r="H544" s="10" t="inlineStr">
+        <is>
+          <t>Donner les croissances comparées entre $(\ln n)^\alpha$, $n^\beta$, $a^n$ et $n!$.</t>
+        </is>
+      </c>
+      <c r="I544" s="9" t="inlineStr">
+        <is>
+          <t>$\dfrac{(\ln n)^\alpha}{n^\beta}\to0$ ; $\dfrac{n^\alpha}{a^n}\to0$ ; $\dfrac{n^\alpha}{n!}\to0$ ; $\dfrac{a^n}{n!}\to0$ (pour tout réel $a$). Ordre : $(\ln n)^\alpha\ll n^\beta\ll a^n\ll n!$.</t>
+        </is>
+      </c>
+      <c r="J544" s="9" t="inlineStr">
+        <is>
+          <t>« Croissances comparées entre les suites factorielle, puissance (n^α avec α &gt; 0), géométriques (a^n avec a &gt; 1). »</t>
+        </is>
+      </c>
+      <c r="K544" s="9" t="n"/>
+      <c r="L544" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Suites : comportement asymptotique » 2025</t>
+        </is>
+      </c>
+      <c r="M544" s="11" t="n"/>
+      <c r="N544" s="11" t="n"/>
+    </row>
+    <row r="545">
+      <c r="A545" s="9" t="inlineStr">
+        <is>
+          <t>M545</t>
+        </is>
+      </c>
+      <c r="B545" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C545" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D545" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 5 – Suites réelles</t>
+        </is>
+      </c>
+      <c r="E545" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F545" s="9" t="inlineStr">
+        <is>
+          <t>Suite bornée fois suite de limite nulle</t>
+        </is>
+      </c>
+      <c r="G545" s="9" t="inlineStr">
+        <is>
+          <t>Soient $(u_n)$ une suite bornée et $(v_n)$ une suite de limite nulle.</t>
+        </is>
+      </c>
+      <c r="H545" s="10" t="inlineStr">
+        <is>
+          <t>Que dire de $(u_nv_n)$ ?</t>
+        </is>
+      </c>
+      <c r="I545" s="9" t="inlineStr">
+        <is>
+          <t>$u_nv_n\to0$ : si $|u_n|\le M$, alors $0\le|u_nv_n|\le M|v_n|\to0$ (gendarmes). Exemple : $\frac{\cos n}n\to0$.</t>
+        </is>
+      </c>
+      <c r="J545" s="9" t="inlineStr">
+        <is>
+          <t>« Théorème d'encadrement, dit « des gendarmes » »</t>
+        </is>
+      </c>
+      <c r="K545" s="9" t="n"/>
+      <c r="L545" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Suites : comportement asymptotique » 2025</t>
+        </is>
+      </c>
+      <c r="M545" s="11" t="n"/>
+      <c r="N545" s="11" t="n"/>
+    </row>
+    <row r="546">
+      <c r="A546" s="9" t="inlineStr">
+        <is>
+          <t>M546</t>
+        </is>
+      </c>
+      <c r="B546" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C546" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D546" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 5 – Suites réelles</t>
+        </is>
+      </c>
+      <c r="E546" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F546" s="9" t="inlineStr">
+        <is>
+          <t>Équivalent d'un polynôme en $n$</t>
+        </is>
+      </c>
+      <c r="G546" s="9" t="inlineStr">
+        <is>
+          <t>Soit $P(x)=a_px^p+\dots+a_0$ un polynôme de degré $p$ ($a_p\neq0$).</t>
+        </is>
+      </c>
+      <c r="H546" s="10" t="inlineStr">
+        <is>
+          <t>Donner un équivalent simple de $P(n)$ quand $n\to+\infty$, et de même pour un quotient de polynômes.</t>
+        </is>
+      </c>
+      <c r="I546" s="9" t="inlineStr">
+        <is>
+          <t>$P(n)\sim a_pn^p$ (le terme de plus haut degré). Pour un quotient : $\dfrac{P(n)}{Q(n)}\sim\dfrac{a_pn^p}{b_qn^q}$ (quotient des termes dominants).</t>
+        </is>
+      </c>
+      <c r="J546" s="9" t="inlineStr">
+        <is>
+          <t>« Utilisation des équivalents pour la recherche de limites. »</t>
+        </is>
+      </c>
+      <c r="K546" s="9" t="n"/>
+      <c r="L546" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Suites : comportement asymptotique » 2025</t>
+        </is>
+      </c>
+      <c r="M546" s="11" t="n"/>
+      <c r="N546" s="11" t="n"/>
+    </row>
+    <row r="547">
+      <c r="A547" s="9" t="inlineStr">
+        <is>
+          <t>M547</t>
+        </is>
+      </c>
+      <c r="B547" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C547" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D547" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 5 – Suites réelles</t>
+        </is>
+      </c>
+      <c r="E547" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F547" s="9" t="inlineStr">
+        <is>
+          <t>Suite $u_{n+1}=f(u_n)$ avec $f$ croissante</t>
+        </is>
+      </c>
+      <c r="G547" s="9" t="inlineStr">
+        <is>
+          <t>Soient $f$ une fonction croissante sur un intervalle $I$ stable par $f$, et $(u_n)$ définie par $u_0\in I$ et $u_{n+1}=f(u_n)$.</t>
+        </is>
+      </c>
+      <c r="H547" s="10" t="inlineStr">
+        <is>
+          <t>Que dire de la monotonie de $(u_n)$ ?</t>
+        </is>
+      </c>
+      <c r="I547" s="9" t="inlineStr">
+        <is>
+          <t>$(u_n)$ est monotone : croissante si $u_1\ge u_0$, décroissante si $u_1\le u_0$ (récurrence : $u_{n+1}-u_n$ garde le signe de $u_1-u_0$). Si de plus $f$ est continue et $u_n\to l\in I$, alors $f(l)=l$.</t>
+        </is>
+      </c>
+      <c r="J547" s="9" t="inlineStr">
+        <is>
+          <t>Programme : « Aucun théorème général relatif à ce type de suites n'est exigible des étudiants. »</t>
+        </is>
+      </c>
+      <c r="K547" s="9" t="n"/>
+      <c r="L547" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours BCPST « Suites : comportement asymptotique » 2025</t>
+        </is>
+      </c>
+      <c r="M547" s="11" t="n"/>
+      <c r="N547" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M541" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M547" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -35582,7 +35942,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$541,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$547,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -35597,7 +35957,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$541,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$547,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -35612,7 +35972,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$541,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$547,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -35639,7 +35999,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$541)</f>
+        <f>COUNTA(Fiches!$M$2:$M$547)</f>
         <v/>
       </c>
     </row>
@@ -35685,15 +36045,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A13,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A13,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A13,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A13,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A13,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A13,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -35708,15 +36068,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A14,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A14,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A14,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A14,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A14,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A14,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -35731,15 +36091,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A15,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A15,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A15,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A15,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A15,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A15,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -35754,15 +36114,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A16,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A16,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A16,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A16,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A16,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A16,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -35777,15 +36137,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A17,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A17,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A17,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A17,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A17,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A17,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -35800,15 +36160,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A18,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A18,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A18,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A18,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A18,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A18,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -35823,15 +36183,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A19,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A19,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A19,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A19,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A19,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A19,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -35846,15 +36206,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A20,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A20,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A20,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A20,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A20,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A20,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -35869,15 +36229,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A21,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A21,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A21,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A21,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A21,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A21,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -35892,15 +36252,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A22,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A22,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A22,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A22,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A22,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A22,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -35915,15 +36275,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A23,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A23,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A23,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A23,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A23,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A23,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -35938,15 +36298,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A24,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A24,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A24,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A24,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A24,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A24,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -35961,15 +36321,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A25,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A25,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A25,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A25,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A25,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A25,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -35984,15 +36344,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A26,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A26,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A26,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A26,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A26,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A26,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -36007,15 +36367,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A27,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A27,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A27,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A27,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A27,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A27,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -36030,15 +36390,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A28,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A28,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A28,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A28,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A28,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A28,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -36053,15 +36413,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A29,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A29,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A29,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A29,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A29,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A29,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -36076,15 +36436,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A30,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A30,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A30,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A30,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A30,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A30,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -36099,15 +36459,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A31,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A31,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A31,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A31,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A31,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A31,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -36122,15 +36482,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A32,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A32,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A32,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A32,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A32,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A32,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -36145,15 +36505,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A33,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A33,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A33,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A33,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A33,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A33,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -36168,15 +36528,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A34,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A34,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A34,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A34,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A34,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A34,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -36191,15 +36551,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A35,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A35,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A35,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A35,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A35,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A35,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -36214,15 +36574,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A36,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A36,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A36,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A36,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A36,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A36,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -36237,15 +36597,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A37,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A37,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A37,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A37,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A37,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A37,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -36260,15 +36620,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A38,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A38,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A38,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A38,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A38,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A38,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -36283,15 +36643,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A39,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A39,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A39,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A39,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A39,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A39,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -36306,15 +36666,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A40,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A40,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A40,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A40,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A40,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A40,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -36329,15 +36689,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A41,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A41,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A41,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A41,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A41,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A41,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -36352,15 +36712,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A42,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A42,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A42,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A42,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A42,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A42,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -36375,15 +36735,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A43,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A43,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A43,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A43,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A43,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A43,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -36398,15 +36758,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A44,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A44,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A44,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A44,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A44,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A44,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -36421,15 +36781,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A45,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A45,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A45,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A45,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A45,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A45,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -36444,15 +36804,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A46,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A46,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A46,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A46,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A46,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A46,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -36467,15 +36827,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A47,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A47,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A47,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A47,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A47,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A47,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -36490,15 +36850,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A48,Fiches!$B$2:$B$541,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A48,Fiches!$B$2:$B$547,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A48,Fiches!$B$2:$B$541,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A48,Fiches!$B$2:$B$547,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$541,$A48,Fiches!$B$2:$B$541,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$547,$A48,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Dérivation : intégration du cours (Cⁿ, opérations, notations, réciproque)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N547"/>
+  <dimension ref="A1:N551"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -13671,8 +13671,16 @@
           <t>Titre de l'ouvrage : « Reste intégral »</t>
         </is>
       </c>
-      <c r="M223" s="14" t="n"/>
-      <c r="N223" s="14" t="n"/>
+      <c r="M223" s="14" t="inlineStr">
+        <is>
+          <t>Passer en rouge</t>
+        </is>
+      </c>
+      <c r="N223" s="14" t="inlineStr">
+        <is>
+          <t>Taylor avec reste intégral absent du cours ; programme : formule de Taylor (polynômes) et Taylor-Lagrange hors programme.</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="12" t="inlineStr">
@@ -13702,22 +13710,22 @@
       </c>
       <c r="F224" s="12" t="inlineStr">
         <is>
-          <t>Difféomorphisme – Définition</t>
+          <t>Réciproque d’une fonction de classe Cⁿ</t>
         </is>
       </c>
       <c r="G224" s="12" t="inlineStr">
         <is>
-          <t>Soient $I$, $J$ deux intervalles, $f:I\to J$ et $k\ge1$.</t>
+          <t>Soient $I$ un intervalle, $n\ge1$ et $f$ de classe $\mathcal C^n$ sur $I$.</t>
         </is>
       </c>
       <c r="H224" s="13" t="inlineStr">
         <is>
-          <t>Définir : $f$ est un $\mathcal C^k$-difféomorphisme.</t>
+          <t>Si $f'&gt;0$ sur $I$, que peut-on dire de $f$ et de sa réciproque ?</t>
         </is>
       </c>
       <c r="I224" s="12" t="inlineStr">
         <is>
-          <t>$f:I\to J$ est un $\mathcal C^k$-difféomorphisme si $f$ est de classe $\mathcal C^k$, bijective, et $f^{-1}$ de classe $\mathcal C^k$.</t>
+          <t>$f$ est une bijection de $I$ sur l'intervalle $J=f(I)$ et $f^{-1}$ est de classe $\mathcal C^n$ sur $J$ (on dit que $f$ est un $\mathcal C^n$-difféomorphisme de $I$ sur $J$). Idem si $f'&lt;0$.</t>
         </is>
       </c>
       <c r="J224" s="12" t="inlineStr">
@@ -13775,12 +13783,12 @@
       </c>
       <c r="I225" s="9" t="inlineStr">
         <is>
-          <t>Sur un intervalle : $f$ croissante $\iff f'\ge0$ (décroissante $\iff f'\le0$) ; si $f'&gt;0$ (resp. $&lt;0$), $f$ est strictement croissante (resp. décroissante).</t>
+          <t>Sur un intervalle : $f$ croissante $\iff f'\ge0$ (décroissante $\iff f'\le0$) ; $f$ constante $\iff f'=0$. Si $f$ est continue sur $I$ et $f'&gt;0$ sauf peut-être en un nombre fini de points, $f$ est strictement croissante (idem avec $&lt;0$ et décroissante).</t>
         </is>
       </c>
       <c r="J225" s="9" t="inlineStr">
         <is>
-          <t>« Caractérisation des fonctions croissantes (au sens large) par la positivité de leur dérivée … Cas des fonctions strictement croissantes. »</t>
+          <t>Programme Analyse 7 : « Une fonction continue définie sur un intervalle et dont, sauf peut-être en un nombre fini de points, la dérivée existe et est strictement positive, est strictement croissante. » ; « Cas des fonctions constantes ».</t>
         </is>
       </c>
       <c r="K225" s="9" t="n">
@@ -32702,10 +32710,250 @@
       <c r="M547" s="11" t="n"/>
       <c r="N547" s="11" t="n"/>
     </row>
+    <row r="548">
+      <c r="A548" s="9" t="inlineStr">
+        <is>
+          <t>M548</t>
+        </is>
+      </c>
+      <c r="B548" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C548" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D548" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 7 – Dérivation</t>
+        </is>
+      </c>
+      <c r="E548" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F548" s="9" t="inlineStr">
+        <is>
+          <t>Dérivées successives – notations</t>
+        </is>
+      </c>
+      <c r="G548" s="9" t="inlineStr">
+        <is>
+          <t>Soient $f$ définie sur un intervalle $I$ et $n\in\mathbb N$.</t>
+        </is>
+      </c>
+      <c r="H548" s="10" t="inlineStr">
+        <is>
+          <t>Comment définit-on la dérivée $n$-ième de $f$ ? Quelles notations ? Que signifie « $f$ de classe $\mathcal C^\infty$ » ?</t>
+        </is>
+      </c>
+      <c r="I548" s="9" t="inlineStr">
+        <is>
+          <t>$f^{(0)}=f$ et, si $f^{(n)}$ est dérivable sur $I$, $f^{(n+1)}=\big(f^{(n)}\big)'$. Notations : $f'=\dfrac{df}{dx}$, $f''=\dfrac{d^2f}{dx^2}$, $f^{(n)}=\dfrac{d^nf}{dx^n}$. $f$ est de classe $\mathcal C^\infty$ si elle est de classe $\mathcal C^n$ pour tout $n\in\mathbb N$ (indéfiniment dérivable).</t>
+        </is>
+      </c>
+      <c r="J548" s="9" t="inlineStr">
+        <is>
+          <t>Programme Analyse 7 : « Notations $f'$ et $\frac{df}{dx}$ » ; « Fonctions de classe $\mathcal C^n$, de classe $\mathcal C^\infty$ ».</t>
+        </is>
+      </c>
+      <c r="K548" s="9" t="n"/>
+      <c r="L548" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Dérivabilité »</t>
+        </is>
+      </c>
+      <c r="M548" s="11" t="n"/>
+      <c r="N548" s="11" t="n"/>
+    </row>
+    <row r="549">
+      <c r="A549" s="9" t="inlineStr">
+        <is>
+          <t>M549</t>
+        </is>
+      </c>
+      <c r="B549" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C549" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D549" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 7 – Dérivation</t>
+        </is>
+      </c>
+      <c r="E549" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F549" s="9" t="inlineStr">
+        <is>
+          <t>Opérations sur les fonctions de classe Cⁿ</t>
+        </is>
+      </c>
+      <c r="G549" s="9" t="inlineStr">
+        <is>
+          <t>Soient $f$, $g$ de classe $\mathcal C^n$ sur un intervalle $I$ et $a,b\in\mathbb R$.</t>
+        </is>
+      </c>
+      <c r="H549" s="10" t="inlineStr">
+        <is>
+          <t>Quelles opérations conservent la classe $\mathcal C^n$ ? Que vaut $(af+bg)^{(n)}$ ?</t>
+        </is>
+      </c>
+      <c r="I549" s="9" t="inlineStr">
+        <is>
+          <t>$af+bg$ et $fg$ sont $\mathcal C^n$ sur $I$, avec $(af+bg)^{(n)}=af^{(n)}+bg^{(n)}$ ; $\dfrac fg$ est $\mathcal C^n$ si $g$ ne s'annule pas ; si $f(I)\subset J$ et $g$ est $\mathcal C^n$ sur $J$, $g\circ f$ est $\mathcal C^n$ sur $I$. Les fonctions usuelles sont $\mathcal C^\infty$ sur leur domaine de dérivabilité.</t>
+        </is>
+      </c>
+      <c r="J549" s="9" t="inlineStr">
+        <is>
+          <t>Programme Analyse 7 : « Une combinaison linéaire, le produit et la composée de deux fonctions de classe $\mathcal C^n$ est de classe $\mathcal C^n$ ». Quotient : programme muet.</t>
+        </is>
+      </c>
+      <c r="K549" s="9" t="n"/>
+      <c r="L549" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Dérivabilité »</t>
+        </is>
+      </c>
+      <c r="M549" s="11" t="n"/>
+      <c r="N549" s="11" t="n"/>
+    </row>
+    <row r="550">
+      <c r="A550" s="9" t="inlineStr">
+        <is>
+          <t>M550</t>
+        </is>
+      </c>
+      <c r="B550" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C550" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D550" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 7 – Dérivation</t>
+        </is>
+      </c>
+      <c r="E550" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F550" s="9" t="inlineStr">
+        <is>
+          <t>Dérivées n-ièmes de cos et sin</t>
+        </is>
+      </c>
+      <c r="G550" s="9" t="inlineStr">
+        <is>
+          <t>Soient $n\in\mathbb N$ et $x\in\mathbb R$.</t>
+        </is>
+      </c>
+      <c r="H550" s="10" t="inlineStr">
+        <is>
+          <t>Que valent $\cos^{(n)}(x)$ et $\sin^{(n)}(x)$ ?</t>
+        </is>
+      </c>
+      <c r="I550" s="9" t="inlineStr">
+        <is>
+          <t>$\cos^{(n)}(x)=\cos\!\left(x+\dfrac{n\pi}2\right)$ et $\sin^{(n)}(x)=\sin\!\left(x+\dfrac{n\pi}2\right)$ (preuve par récurrence) ; $\cos$ et $\sin$ sont $\mathcal C^\infty$ sur $\mathbb R$.</t>
+        </is>
+      </c>
+      <c r="J550" s="9" t="inlineStr">
+        <is>
+          <t>Exemple du cours ; le programme ne cite pas ces formules.</t>
+        </is>
+      </c>
+      <c r="K550" s="9" t="n"/>
+      <c r="L550" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Dérivabilité »</t>
+        </is>
+      </c>
+      <c r="M550" s="11" t="n"/>
+      <c r="N550" s="11" t="n"/>
+    </row>
+    <row r="551">
+      <c r="A551" s="9" t="inlineStr">
+        <is>
+          <t>M551</t>
+        </is>
+      </c>
+      <c r="B551" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C551" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D551" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 7 – Dérivation</t>
+        </is>
+      </c>
+      <c r="E551" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F551" s="9" t="inlineStr">
+        <is>
+          <t>Différentielle en un point</t>
+        </is>
+      </c>
+      <c r="G551" s="9" t="inlineStr">
+        <is>
+          <t>Soit $f$ dérivable en $x_0$.</t>
+        </is>
+      </c>
+      <c r="H551" s="10" t="inlineStr">
+        <is>
+          <t>Qu'appelle-t-on différentielle de $f$ en $x_0$ ?</t>
+        </is>
+      </c>
+      <c r="I551" s="9" t="inlineStr">
+        <is>
+          <t>L'application linéaire $df_{x_0}:\mathbb R\to\mathbb R,\ h\mapsto h\,f'(x_0)$ ; on a $f(x_0+h)=f(x_0)+df_{x_0}(h)+o(h)$.</t>
+        </is>
+      </c>
+      <c r="J551" s="9" t="inlineStr">
+        <is>
+          <t>Remarque du cours ; notion absente du programme de mathématiques (utile en physique-chimie).</t>
+        </is>
+      </c>
+      <c r="K551" s="9" t="n"/>
+      <c r="L551" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Dérivabilité »</t>
+        </is>
+      </c>
+      <c r="M551" s="11" t="n"/>
+      <c r="N551" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M547" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M551" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -35942,7 +36190,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$547,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$551,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -35957,7 +36205,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$547,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$551,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -35972,7 +36220,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$547,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$551,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -35999,7 +36247,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$547)</f>
+        <f>COUNTA(Fiches!$M$2:$M$551)</f>
         <v/>
       </c>
     </row>
@@ -36045,15 +36293,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A13,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A13,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A13,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A13,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A13,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A13,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -36068,15 +36316,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A14,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A14,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A14,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A14,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A14,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A14,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -36091,15 +36339,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A15,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A15,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A15,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A15,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A15,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A15,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -36114,15 +36362,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A16,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A16,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A16,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A16,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A16,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A16,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -36137,15 +36385,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A17,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A17,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A17,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A17,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A17,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A17,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -36160,15 +36408,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A18,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A18,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A18,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A18,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A18,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A18,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -36183,15 +36431,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A19,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A19,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A19,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A19,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A19,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A19,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -36206,15 +36454,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A20,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A20,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A20,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A20,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A20,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A20,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -36229,15 +36477,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A21,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A21,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A21,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A21,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A21,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A21,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -36252,15 +36500,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A22,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A22,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A22,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A22,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A22,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A22,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -36275,15 +36523,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A23,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A23,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A23,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A23,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A23,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A23,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -36298,15 +36546,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A24,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A24,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A24,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A24,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A24,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A24,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -36321,15 +36569,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A25,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A25,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A25,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A25,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A25,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A25,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -36344,15 +36592,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A26,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A26,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A26,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A26,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A26,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A26,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -36367,15 +36615,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A27,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A27,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A27,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A27,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A27,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A27,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -36390,15 +36638,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A28,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A28,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A28,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A28,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A28,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A28,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -36413,15 +36661,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A29,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A29,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A29,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A29,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A29,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A29,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -36436,15 +36684,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A30,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A30,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A30,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A30,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A30,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A30,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -36459,15 +36707,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A31,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A31,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A31,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A31,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A31,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A31,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -36482,15 +36730,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A32,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A32,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A32,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A32,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A32,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A32,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -36505,15 +36753,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A33,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A33,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A33,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A33,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A33,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A33,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -36528,15 +36776,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A34,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A34,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A34,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A34,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A34,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A34,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -36551,15 +36799,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A35,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A35,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A35,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A35,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A35,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A35,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -36574,15 +36822,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A36,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A36,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A36,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A36,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A36,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A36,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -36597,15 +36845,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A37,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A37,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A37,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A37,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A37,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A37,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -36620,15 +36868,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A38,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A38,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A38,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A38,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A38,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A38,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -36643,15 +36891,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A39,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A39,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A39,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A39,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A39,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A39,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -36666,15 +36914,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A40,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A40,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A40,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A40,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A40,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A40,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -36689,15 +36937,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A41,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A41,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A41,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A41,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A41,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A41,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -36712,15 +36960,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A42,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A42,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A42,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A42,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A42,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A42,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -36735,15 +36983,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A43,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A43,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A43,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A43,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A43,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A43,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -36758,15 +37006,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A44,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A44,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A44,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A44,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A44,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A44,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -36781,15 +37029,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A45,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A45,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A45,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A45,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A45,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A45,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -36804,15 +37052,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A46,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A46,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A46,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A46,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A46,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A46,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -36827,15 +37075,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A47,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A47,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A47,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A47,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A47,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A47,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -36850,15 +37098,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A48,Fiches!$B$2:$B$547,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A48,Fiches!$B$2:$B$551,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A48,Fiches!$B$2:$B$547,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A48,Fiches!$B$2:$B$551,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$547,$A48,Fiches!$B$2:$B$547,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$551,$A48,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Dénombrement : intégration du cours (cardinal, union disjointe, injections/surjections)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N551"/>
+  <dimension ref="A1:N555"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3718,22 +3718,22 @@
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>Lemme des bergers (partition)</t>
+          <t>Cardinal d’une union disjointe</t>
         </is>
       </c>
       <c r="G52" s="9" t="inlineStr">
         <is>
-          <t>Soient $\Omega$ un ensemble fini et $(A_1,\dots,A_n)$ un système complet (partition) de $\Omega$.</t>
+          <t>Soient $E_1,\dots,E_n$ des ensembles finis deux à deux disjoints.</t>
         </is>
       </c>
       <c r="H52" s="10" t="inlineStr">
         <is>
-          <t>Exprimer $\mathrm{Card}\,\Omega$ à l'aide des $A_i$ (lemme des bergers).</t>
+          <t>Que vaut $\mathrm{card}(E_1\cup\dots\cup E_n)$ ? Cas d'une partition de $\Omega$ ?</t>
         </is>
       </c>
       <c r="I52" s="9" t="inlineStr">
         <is>
-          <t>$\mathrm{Card}\,\Omega=\sum_{i=1}^n\mathrm{Card}A_i$.</t>
+          <t>$\mathrm{card}(E_1\cup\dots\cup E_n)=\sum_{i=1}^n\mathrm{card}\,E_i$ (pour deux : $\mathrm{card}(A\cup B)=\mathrm{card}\,A+\mathrm{card}\,B$ si $A\cap B=\varnothing$). Si $(A_1,\dots,A_n)$ est une partition de $\Omega$ : $\mathrm{card}\,\Omega=\sum_i\mathrm{card}\,A_i$.</t>
         </is>
       </c>
       <c r="J52" s="9" t="inlineStr">
@@ -32950,10 +32950,250 @@
       <c r="M551" s="11" t="n"/>
       <c r="N551" s="11" t="n"/>
     </row>
+    <row r="552">
+      <c r="A552" s="9" t="inlineStr">
+        <is>
+          <t>M552</t>
+        </is>
+      </c>
+      <c r="B552" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C552" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D552" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 7 – Dénombrement</t>
+        </is>
+      </c>
+      <c r="E552" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F552" s="9" t="inlineStr">
+        <is>
+          <t>Cardinal d’un ensemble fini</t>
+        </is>
+      </c>
+      <c r="G552" s="9" t="inlineStr">
+        <is>
+          <t>Soit $E$ un ensemble fini.</t>
+        </is>
+      </c>
+      <c r="H552" s="10" t="inlineStr">
+        <is>
+          <t>Qu'est-ce que le cardinal de $E$ ? Quelles notations ? Quel lien avec les bijections ?</t>
+        </is>
+      </c>
+      <c r="I552" s="9" t="inlineStr">
+        <is>
+          <t>$\mathrm{card}(E)$ (ou $\#E$) est le nombre d'éléments de $E$, avec $\mathrm{card}(\varnothing)=0$. $\mathrm{card}(E)=n\ge1$ ssi il existe une bijection de $E$ sur $[\![1,n]\!]$ ; deux ensembles finis sont en bijection ssi ils ont le même cardinal.</t>
+        </is>
+      </c>
+      <c r="J552" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 7 : « Cardinal, notation card(E) ou #E. » ; « deux ensembles en bijection ont même cardinal ».</t>
+        </is>
+      </c>
+      <c r="K552" s="9" t="n"/>
+      <c r="L552" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Dénombrement »</t>
+        </is>
+      </c>
+      <c r="M552" s="11" t="n"/>
+      <c r="N552" s="11" t="n"/>
+    </row>
+    <row r="553">
+      <c r="A553" s="9" t="inlineStr">
+        <is>
+          <t>M553</t>
+        </is>
+      </c>
+      <c r="B553" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C553" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D553" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 7 – Dénombrement</t>
+        </is>
+      </c>
+      <c r="E553" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F553" s="9" t="inlineStr">
+        <is>
+          <t>Cardinal d’un intervalle d’entiers</t>
+        </is>
+      </c>
+      <c r="G553" s="9" t="inlineStr">
+        <is>
+          <t>Soient $p\le q$ deux entiers.</t>
+        </is>
+      </c>
+      <c r="H553" s="10" t="inlineStr">
+        <is>
+          <t>Combien l'ensemble $[\![p,q]\!]$ a-t-il d'éléments ?</t>
+        </is>
+      </c>
+      <c r="I553" s="9" t="inlineStr">
+        <is>
+          <t>$\mathrm{card}\,[\![p,q]\!]=q-p+1$.</t>
+        </is>
+      </c>
+      <c r="J553" s="9" t="inlineStr">
+        <is>
+          <t>Remarque du cours ; non citée par le programme.</t>
+        </is>
+      </c>
+      <c r="K553" s="9" t="n"/>
+      <c r="L553" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Dénombrement »</t>
+        </is>
+      </c>
+      <c r="M553" s="11" t="n"/>
+      <c r="N553" s="11" t="n"/>
+    </row>
+    <row r="554">
+      <c r="A554" s="9" t="inlineStr">
+        <is>
+          <t>M554</t>
+        </is>
+      </c>
+      <c r="B554" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C554" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D554" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 7 – Dénombrement</t>
+        </is>
+      </c>
+      <c r="E554" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F554" s="9" t="inlineStr">
+        <is>
+          <t>Cardinal d’une partie et du complémentaire</t>
+        </is>
+      </c>
+      <c r="G554" s="9" t="inlineStr">
+        <is>
+          <t>Soient $E$ un ensemble fini et $A\subset E$.</t>
+        </is>
+      </c>
+      <c r="H554" s="10" t="inlineStr">
+        <is>
+          <t>Que peut-on dire de $\mathrm{card}\,A$ ? Que vaut $\mathrm{card}\,\bar A$ ?</t>
+        </is>
+      </c>
+      <c r="I554" s="9" t="inlineStr">
+        <is>
+          <t>$A$ est fini et $\mathrm{card}\,A\le\mathrm{card}\,E$, avec égalité ssi $A=E$. $\mathrm{card}\,\bar A=\mathrm{card}\,E-\mathrm{card}\,A$ (où $\bar A=E\setminus A$).</t>
+        </is>
+      </c>
+      <c r="J554" s="9" t="inlineStr">
+        <is>
+          <t>Cours ; le complémentaire découle du cardinal d'une union disjointe (programme), l'inégalité n'est pas citée.</t>
+        </is>
+      </c>
+      <c r="K554" s="9" t="n"/>
+      <c r="L554" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Dénombrement »</t>
+        </is>
+      </c>
+      <c r="M554" s="11" t="n"/>
+      <c r="N554" s="11" t="n"/>
+    </row>
+    <row r="555">
+      <c r="A555" s="9" t="inlineStr">
+        <is>
+          <t>M555</t>
+        </is>
+      </c>
+      <c r="B555" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C555" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D555" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 7 – Dénombrement</t>
+        </is>
+      </c>
+      <c r="E555" s="9" t="inlineStr">
+        <is>
+          <t>Théorème</t>
+        </is>
+      </c>
+      <c r="F555" s="9" t="inlineStr">
+        <is>
+          <t>Injections, surjections et cardinaux</t>
+        </is>
+      </c>
+      <c r="G555" s="9" t="inlineStr">
+        <is>
+          <t>Soient $E$, $F$ deux ensembles finis et $f:E\to F$.</t>
+        </is>
+      </c>
+      <c r="H555" s="10" t="inlineStr">
+        <is>
+          <t>Que déduit-on sur les cardinaux si $f$ est injective ? surjective ? Et si $\mathrm{card}\,E=\mathrm{card}\,F$ ?</t>
+        </is>
+      </c>
+      <c r="I555" s="9" t="inlineStr">
+        <is>
+          <t>Si $f$ est injective, $\mathrm{card}\,E\le\mathrm{card}\,F$ ; si $f$ est surjective, $\mathrm{card}\,E\ge\mathrm{card}\,F$. Si $\mathrm{card}\,E=\mathrm{card}\,F$ : $f$ bijective $\iff$ $f$ injective $\iff$ $f$ surjective.</t>
+        </is>
+      </c>
+      <c r="J555" s="9" t="inlineStr">
+        <is>
+          <t>Théorème du cours ; le programme ne le cite pas (il ne parle que des bijections).</t>
+        </is>
+      </c>
+      <c r="K555" s="9" t="n"/>
+      <c r="L555" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Dénombrement »</t>
+        </is>
+      </c>
+      <c r="M555" s="11" t="n"/>
+      <c r="N555" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M551" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M555" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -36190,7 +36430,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$551,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$555,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -36205,7 +36445,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$551,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$555,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -36220,7 +36460,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$551,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$555,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -36247,7 +36487,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$551)</f>
+        <f>COUNTA(Fiches!$M$2:$M$555)</f>
         <v/>
       </c>
     </row>
@@ -36293,15 +36533,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A13,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A13,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A13,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A13,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A13,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A13,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -36316,15 +36556,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A14,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A14,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A14,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A14,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A14,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A14,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -36339,15 +36579,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A15,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A15,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A15,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A15,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A15,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A15,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -36362,15 +36602,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A16,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A16,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A16,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A16,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A16,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A16,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -36385,15 +36625,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A17,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A17,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A17,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A17,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A17,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A17,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -36408,15 +36648,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A18,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A18,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A18,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A18,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A18,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A18,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -36431,15 +36671,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A19,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A19,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A19,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A19,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A19,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A19,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -36454,15 +36694,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A20,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A20,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A20,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A20,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A20,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A20,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -36477,15 +36717,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A21,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A21,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A21,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A21,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A21,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A21,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -36500,15 +36740,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A22,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A22,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A22,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A22,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A22,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A22,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -36523,15 +36763,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A23,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A23,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A23,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A23,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A23,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A23,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -36546,15 +36786,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A24,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A24,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A24,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A24,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A24,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A24,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -36569,15 +36809,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A25,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A25,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A25,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A25,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A25,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A25,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -36592,15 +36832,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A26,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A26,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A26,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A26,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A26,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A26,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -36615,15 +36855,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A27,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A27,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A27,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A27,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A27,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A27,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -36638,15 +36878,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A28,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A28,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A28,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A28,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A28,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A28,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -36661,15 +36901,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A29,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A29,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A29,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A29,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A29,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A29,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -36684,15 +36924,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A30,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A30,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A30,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A30,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A30,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A30,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -36707,15 +36947,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A31,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A31,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A31,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A31,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A31,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A31,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -36730,15 +36970,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A32,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A32,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A32,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A32,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A32,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A32,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -36753,15 +36993,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A33,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A33,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A33,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A33,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A33,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A33,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -36776,15 +37016,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A34,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A34,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A34,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A34,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A34,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A34,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -36799,15 +37039,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A35,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A35,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A35,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A35,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A35,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A35,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -36822,15 +37062,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A36,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A36,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A36,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A36,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A36,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A36,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -36845,15 +37085,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A37,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A37,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A37,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A37,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A37,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A37,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -36868,15 +37108,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A38,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A38,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A38,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A38,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A38,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A38,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -36891,15 +37131,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A39,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A39,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A39,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A39,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A39,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A39,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -36914,15 +37154,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A40,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A40,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A40,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A40,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A40,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A40,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -36937,15 +37177,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A41,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A41,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A41,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A41,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A41,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A41,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -36960,15 +37200,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A42,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A42,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A42,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A42,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A42,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A42,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -36983,15 +37223,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A43,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A43,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A43,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A43,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A43,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A43,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -37006,15 +37246,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A44,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A44,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A44,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A44,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A44,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A44,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -37029,15 +37269,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A45,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A45,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A45,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A45,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A45,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A45,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -37052,15 +37292,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A46,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A46,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A46,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A46,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A46,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A46,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -37075,15 +37315,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A47,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A47,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A47,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A47,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A47,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A47,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -37098,15 +37338,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A48,Fiches!$B$2:$B$551,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A48,Fiches!$B$2:$B$555,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A48,Fiches!$B$2:$B$551,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A48,Fiches!$B$2:$B$555,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$551,$A48,Fiches!$B$2:$B$551,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$555,$A48,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Espaces vectoriels : intégration du cours (coordonnées, base canonique, matrices, rang)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N555"/>
+  <dimension ref="A1:N561"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -20127,7 +20127,7 @@
       </c>
       <c r="I335" s="9" t="inlineStr">
         <is>
-          <t>$\mathrm{rg}(x_1,\dots,x_n)=\dim\mathrm{Vect}(x_1,\dots,x_n)$.</t>
+          <t>$\mathrm{rg}(x_1,\dots,x_n)=\dim\mathrm{Vect}(x_1,\dots,x_n)$. Il se calcule comme le rang de la matrice des coordonnées de la famille dans n'importe quelle base (méthode du pivot).</t>
         </is>
       </c>
       <c r="J335" s="9" t="inlineStr">
@@ -20417,7 +20417,7 @@
       </c>
       <c r="I340" s="9" t="inlineStr">
         <is>
-          <t>$E$ est de dimension finie s'il admet une famille génératrice finie. Alors $E$ admet une base, toutes ses bases sont finies et ont le même cardinal, noté $\dim E$.</t>
+          <t>$E$ est de dimension finie s'il admet une famille génératrice finie. Alors $E$ admet une base, toutes ses bases sont finies et ont le même cardinal, noté $\dim E$. Par convention, $\dim\{0_E\}=0$ (base vide).</t>
         </is>
       </c>
       <c r="J340" s="9" t="inlineStr">
@@ -20464,22 +20464,22 @@
       </c>
       <c r="F341" s="9" t="inlineStr">
         <is>
-          <t>Propriétés des familles libres et des familles génératrices</t>
+          <t>Familles libres en dimension finie</t>
         </is>
       </c>
       <c r="G341" s="9" t="inlineStr">
         <is>
-          <t>Soit $E$ un espace vectoriel de dimension $n$.</t>
+          <t>Soit $E$ un espace vectoriel de dimension $n\ge1$ et $\mathcal F$ une famille libre de $E$.</t>
         </is>
       </c>
       <c r="H341" s="10" t="inlineStr">
         <is>
-          <t>Que dire du nombre d'éléments d'une famille libre ? d'une famille génératrice ?</t>
+          <t>Que peut-on dire d'une famille libre $\mathcal F$ de $E$ (complétion, nombre de vecteurs, cas de $n$ vecteurs) ?</t>
         </is>
       </c>
       <c r="I341" s="9" t="inlineStr">
         <is>
-          <t>Si $\dim E=n$ : toute famille libre a au plus $n$ éléments, toute famille génératrice au moins $n$ éléments.</t>
+          <t>$\mathcal F$ peut être complétée en une base de $E$ ; $\mathcal F$ a au plus $n$ vecteurs ; si $\mathcal F$ a exactement $n$ vecteurs, c'est une base.</t>
         </is>
       </c>
       <c r="J341" s="9" t="inlineStr">
@@ -33190,10 +33190,370 @@
       <c r="M555" s="11" t="n"/>
       <c r="N555" s="11" t="n"/>
     </row>
+    <row r="556">
+      <c r="A556" s="9" t="inlineStr">
+        <is>
+          <t>M556</t>
+        </is>
+      </c>
+      <c r="B556" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C556" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2</t>
+        </is>
+      </c>
+      <c r="D556" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2 · Algèbre linéaire 1 – Espaces vectoriels</t>
+        </is>
+      </c>
+      <c r="E556" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F556" s="9" t="inlineStr">
+        <is>
+          <t>Coordonnées dans une base</t>
+        </is>
+      </c>
+      <c r="G556" s="9" t="inlineStr">
+        <is>
+          <t>Soient $E$ un espace vectoriel et $\mathcal B=(e_1,\dots,e_p)$ une base de $E$.</t>
+        </is>
+      </c>
+      <c r="H556" s="10" t="inlineStr">
+        <is>
+          <t>Que sont les coordonnées d'un vecteur $x\in E$ dans $\mathcal B$ ? Pourquoi sont-elles bien définies ?</t>
+        </is>
+      </c>
+      <c r="I556" s="9" t="inlineStr">
+        <is>
+          <t>Pour tout $x\in E$, il existe un unique $(x_1,\dots,x_p)\in\mathbb K^p$ tel que $x=\sum_{i=1}^p x_ie_i$ : ce sont les coordonnées de $x$ dans $\mathcal B$. Existence : $\mathcal B$ est génératrice ; unicité : $\mathcal B$ est libre. Réciproquement, si tout $x$ s'écrit de façon unique ainsi, $(e_i)$ est une base.</t>
+        </is>
+      </c>
+      <c r="J556" s="9" t="inlineStr">
+        <is>
+          <t>Programme BCPST1 AL3 et BCPST2 AL1 : « Coordonnées d'un vecteur par rapport à une base. »</t>
+        </is>
+      </c>
+      <c r="K556" s="9" t="n"/>
+      <c r="L556" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Espaces vectoriels » (Kⁿ)</t>
+        </is>
+      </c>
+      <c r="M556" s="11" t="n"/>
+      <c r="N556" s="11" t="n"/>
+    </row>
+    <row r="557">
+      <c r="A557" s="9" t="inlineStr">
+        <is>
+          <t>M557</t>
+        </is>
+      </c>
+      <c r="B557" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C557" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2</t>
+        </is>
+      </c>
+      <c r="D557" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2 · Algèbre linéaire 1 – Espaces vectoriels</t>
+        </is>
+      </c>
+      <c r="E557" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F557" s="9" t="inlineStr">
+        <is>
+          <t>Base canonique de Kⁿ</t>
+        </is>
+      </c>
+      <c r="G557" s="9" t="inlineStr">
+        <is>
+          <t>Soit $n\in\mathbb N^*$.</t>
+        </is>
+      </c>
+      <c r="H557" s="10" t="inlineStr">
+        <is>
+          <t>Quelle est la base canonique de $\mathbb K^n$ ? Quelles sont les coordonnées de $(x_1,\dots,x_n)$ dans cette base ?</t>
+        </is>
+      </c>
+      <c r="I557" s="9" t="inlineStr">
+        <is>
+          <t>$(e_1,\dots,e_n)$ avec $e_i=(0,\dots,0,1,0,\dots,0)$ (1 en $i$-ème position). Comme $(x_1,\dots,x_n)=\sum_i x_ie_i$, ses coordonnées sont $(x_1,\dots,x_n)$ ; $\dim\mathbb K^n=n$.</t>
+        </is>
+      </c>
+      <c r="J557" s="9" t="inlineStr">
+        <is>
+          <t>Programme BCPST1 AL3 : « Base canonique de $\mathbb K^n$. »</t>
+        </is>
+      </c>
+      <c r="K557" s="9" t="n"/>
+      <c r="L557" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Espaces vectoriels » (Kⁿ)</t>
+        </is>
+      </c>
+      <c r="M557" s="11" t="n"/>
+      <c r="N557" s="11" t="n"/>
+    </row>
+    <row r="558">
+      <c r="A558" s="9" t="inlineStr">
+        <is>
+          <t>M558</t>
+        </is>
+      </c>
+      <c r="B558" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C558" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2</t>
+        </is>
+      </c>
+      <c r="D558" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2 · Algèbre linéaire 1 – Espaces vectoriels</t>
+        </is>
+      </c>
+      <c r="E558" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F558" s="9" t="inlineStr">
+        <is>
+          <t>Matrice d’un vecteur, d’une famille dans une base</t>
+        </is>
+      </c>
+      <c r="G558" s="9" t="inlineStr">
+        <is>
+          <t>Soient $\mathcal B$ une base de $E$ ($\dim E=p$) et $(u_1,\dots,u_q)$ une famille de vecteurs de $E$.</t>
+        </is>
+      </c>
+      <c r="H558" s="10" t="inlineStr">
+        <is>
+          <t>Que sont $\mathrm{mat}_{\mathcal B}(u)$ et $\mathrm{mat}_{\mathcal B}(u_1,\dots,u_q)$ ? Comment se comportent-elles avec $+$ et $\lambda\cdot$ ?</t>
+        </is>
+      </c>
+      <c r="I558" s="9" t="inlineStr">
+        <is>
+          <t>$\mathrm{mat}_{\mathcal B}(u)$ est la matrice colonne des coordonnées de $u$ ; $\mathrm{mat}_{\mathcal B}(u_1,\dots,u_q)\in\mathcal M_{p,q}(\mathbb K)$ a pour $j$-ème colonne les coordonnées de $u_j$. $\mathrm{mat}_{\mathcal B}(u+v)=\mathrm{mat}_{\mathcal B}(u)+\mathrm{mat}_{\mathcal B}(v)$, $\mathrm{mat}_{\mathcal B}(\lambda u)=\lambda\,\mathrm{mat}_{\mathcal B}(u)$ ; $\mathrm{mat}_{\mathcal B}(\mathcal B)=I_p$.</t>
+        </is>
+      </c>
+      <c r="J558" s="9" t="inlineStr">
+        <is>
+          <t>Programme BCPST2 AL1 : « Matrice des coordonnées d'une famille finie de vecteurs dans une base » ; BCPST1 AL3 : « matrice colonne associée au vecteur ».</t>
+        </is>
+      </c>
+      <c r="K558" s="9" t="n"/>
+      <c r="L558" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Espaces vectoriels » (Kⁿ)</t>
+        </is>
+      </c>
+      <c r="M558" s="11" t="n"/>
+      <c r="N558" s="11" t="n"/>
+    </row>
+    <row r="559">
+      <c r="A559" s="9" t="inlineStr">
+        <is>
+          <t>M559</t>
+        </is>
+      </c>
+      <c r="B559" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C559" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2</t>
+        </is>
+      </c>
+      <c r="D559" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2 · Algèbre linéaire 1 – Espaces vectoriels</t>
+        </is>
+      </c>
+      <c r="E559" s="9" t="inlineStr">
+        <is>
+          <t>Théorème</t>
+        </is>
+      </c>
+      <c r="F559" s="9" t="inlineStr">
+        <is>
+          <t>Familles génératrices en dimension finie</t>
+        </is>
+      </c>
+      <c r="G559" s="9" t="inlineStr">
+        <is>
+          <t>Soit $E$ un espace vectoriel de dimension $p\ge1$ et $\mathcal F$ une famille génératrice de $E$.</t>
+        </is>
+      </c>
+      <c r="H559" s="10" t="inlineStr">
+        <is>
+          <t>Que peut-on dire de $\mathcal F$ (base extraite, nombre de vecteurs, cas de $p$ vecteurs) ?</t>
+        </is>
+      </c>
+      <c r="I559" s="9" t="inlineStr">
+        <is>
+          <t>On peut extraire de $\mathcal F$ une base de $E$ ; $\mathcal F$ a au moins $p$ vecteurs ; si $\mathcal F$ a exactement $p$ vecteurs, c'est une base.</t>
+        </is>
+      </c>
+      <c r="J559" s="9" t="inlineStr">
+        <is>
+          <t>Programme : « De toute famille génératrice on peut extraire une base. Toute famille génératrice a au moins p éléments. Une famille génératrice ayant p éléments est une base. »</t>
+        </is>
+      </c>
+      <c r="K559" s="9" t="n"/>
+      <c r="L559" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Espaces vectoriels » (Kⁿ)</t>
+        </is>
+      </c>
+      <c r="M559" s="11" t="n"/>
+      <c r="N559" s="11" t="n"/>
+    </row>
+    <row r="560">
+      <c r="A560" s="9" t="inlineStr">
+        <is>
+          <t>M560</t>
+        </is>
+      </c>
+      <c r="B560" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C560" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2</t>
+        </is>
+      </c>
+      <c r="D560" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2 · Algèbre linéaire 1 – Espaces vectoriels</t>
+        </is>
+      </c>
+      <c r="E560" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F560" s="9" t="inlineStr">
+        <is>
+          <t>Familles liées et colinéarité</t>
+        </is>
+      </c>
+      <c r="G560" s="9" t="inlineStr">
+        <is>
+          <t>Soit $(u_1,\dots,u_p)$ une famille de vecteurs, $p\ge2$.</t>
+        </is>
+      </c>
+      <c r="H560" s="10" t="inlineStr">
+        <is>
+          <t>Caractériser le fait que $(u_1,\dots,u_p)$ soit liée. Cas de deux vecteurs ?</t>
+        </is>
+      </c>
+      <c r="I560" s="9" t="inlineStr">
+        <is>
+          <t>$(u_1,\dots,u_p)$ est liée ssi l'un au moins des $u_i$ est combinaison linéaire des $p-1$ autres. En particulier, $(u,v)$ est liée ssi $u$ et $v$ sont colinéaires. Toute famille contenant une famille liée est liée.</t>
+        </is>
+      </c>
+      <c r="J560" s="9" t="inlineStr">
+        <is>
+          <t>Théorème et propriétés du cours ; le programme définit seulement les familles libres et liées.</t>
+        </is>
+      </c>
+      <c r="K560" s="9" t="n"/>
+      <c r="L560" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Espaces vectoriels » (Kⁿ)</t>
+        </is>
+      </c>
+      <c r="M560" s="11" t="n"/>
+      <c r="N560" s="11" t="n"/>
+    </row>
+    <row r="561">
+      <c r="A561" s="9" t="inlineStr">
+        <is>
+          <t>M561</t>
+        </is>
+      </c>
+      <c r="B561" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C561" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2</t>
+        </is>
+      </c>
+      <c r="D561" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2 · Algèbre linéaire 1 – Espaces vectoriels</t>
+        </is>
+      </c>
+      <c r="E561" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F561" s="9" t="inlineStr">
+        <is>
+          <t>Rang d’une famille – propriétés</t>
+        </is>
+      </c>
+      <c r="G561" s="9" t="inlineStr">
+        <is>
+          <t>Soit $(u_1,\dots,u_p)$ une famille de vecteurs d'un espace $E$ de dimension $n$.</t>
+        </is>
+      </c>
+      <c r="H561" s="10" t="inlineStr">
+        <is>
+          <t>Majorer $\mathrm{rg}(u_1,\dots,u_p)$. Quand vaut-il $p$ ? Quand vaut-il $n$ ?</t>
+        </is>
+      </c>
+      <c r="I561" s="9" t="inlineStr">
+        <is>
+          <t>$\mathrm{rg}(u_1,\dots,u_p)\le\min(n,p)$ ; $\mathrm{rg}=p\iff$ la famille est libre ; $\mathrm{rg}=n\iff$ la famille est génératrice de $E$.</t>
+        </is>
+      </c>
+      <c r="J561" s="9" t="inlineStr">
+        <is>
+          <t>Propriété du cours ; conséquence directe des théorèmes de dimension, non citée telle quelle par le programme.</t>
+        </is>
+      </c>
+      <c r="K561" s="9" t="n"/>
+      <c r="L561" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Espaces vectoriels » (Kⁿ)</t>
+        </is>
+      </c>
+      <c r="M561" s="11" t="n"/>
+      <c r="N561" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M555" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M561" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -36430,7 +36790,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$555,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$561,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -36445,7 +36805,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$555,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$561,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -36460,7 +36820,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$555,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$561,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -36487,7 +36847,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$555)</f>
+        <f>COUNTA(Fiches!$M$2:$M$561)</f>
         <v/>
       </c>
     </row>
@@ -36533,15 +36893,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A13,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A13,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A13,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A13,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A13,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A13,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -36556,15 +36916,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A14,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A14,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A14,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A14,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A14,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A14,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -36579,15 +36939,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A15,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A15,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A15,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A15,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A15,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A15,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -36602,15 +36962,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A16,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A16,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A16,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A16,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A16,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A16,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -36625,15 +36985,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A17,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A17,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A17,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A17,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A17,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A17,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -36648,15 +37008,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A18,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A18,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A18,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A18,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A18,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A18,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -36671,15 +37031,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A19,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A19,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A19,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A19,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A19,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A19,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -36694,15 +37054,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A20,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A20,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A20,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A20,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A20,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A20,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -36717,15 +37077,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A21,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A21,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A21,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A21,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A21,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A21,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -36740,15 +37100,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A22,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A22,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A22,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A22,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A22,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A22,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -36763,15 +37123,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A23,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A23,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A23,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A23,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A23,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A23,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -36786,15 +37146,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A24,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A24,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A24,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A24,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A24,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A24,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -36809,15 +37169,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A25,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A25,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A25,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A25,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A25,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A25,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -36832,15 +37192,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A26,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A26,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A26,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A26,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A26,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A26,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -36855,15 +37215,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A27,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A27,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A27,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A27,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A27,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A27,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -36878,15 +37238,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A28,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A28,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A28,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A28,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A28,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A28,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -36901,15 +37261,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A29,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A29,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A29,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A29,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A29,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A29,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -36924,15 +37284,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A30,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A30,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A30,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A30,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A30,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A30,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -36947,15 +37307,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A31,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A31,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A31,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A31,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A31,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A31,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -36970,15 +37330,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A32,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A32,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A32,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A32,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A32,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A32,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -36993,15 +37353,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A33,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A33,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A33,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A33,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A33,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A33,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -37016,15 +37376,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A34,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A34,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A34,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A34,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A34,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A34,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -37039,15 +37399,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A35,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A35,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A35,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A35,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A35,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A35,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -37062,15 +37422,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A36,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A36,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A36,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A36,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A36,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A36,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -37085,15 +37445,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A37,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A37,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A37,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A37,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A37,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A37,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -37108,15 +37468,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A38,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A38,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A38,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A38,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A38,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A38,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -37131,15 +37491,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A39,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A39,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A39,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A39,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A39,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A39,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -37154,15 +37514,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A40,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A40,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A40,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A40,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A40,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A40,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -37177,15 +37537,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A41,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A41,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A41,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A41,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A41,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A41,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -37200,15 +37560,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A42,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A42,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A42,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A42,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A42,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A42,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -37223,15 +37583,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A43,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A43,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A43,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A43,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A43,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A43,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -37246,15 +37606,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A44,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A44,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A44,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A44,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A44,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A44,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -37269,15 +37629,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A45,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A45,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A45,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A45,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A45,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A45,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -37292,15 +37652,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A46,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A46,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A46,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A46,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A46,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A46,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -37315,15 +37675,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A47,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A47,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A47,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A47,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A47,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A47,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -37338,15 +37698,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A48,Fiches!$B$2:$B$555,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A48,Fiches!$B$2:$B$561,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A48,Fiches!$B$2:$B$555,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A48,Fiches!$B$2:$B$561,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$555,$A48,Fiches!$B$2:$B$555,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$561,$A48,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Fonctions de deux variables : intégration du cours (surface, petites variations, gradient, plan tangent)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N561"/>
+  <dimension ref="A1:N566"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -33550,10 +33550,310 @@
       <c r="M561" s="11" t="n"/>
       <c r="N561" s="11" t="n"/>
     </row>
+    <row r="562">
+      <c r="A562" s="9" t="inlineStr">
+        <is>
+          <t>M562</t>
+        </is>
+      </c>
+      <c r="B562" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C562" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D562" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 10 – Fonctions de deux variables</t>
+        </is>
+      </c>
+      <c r="E562" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F562" s="9" t="inlineStr">
+        <is>
+          <t>Surface représentative, sections et lignes de niveau</t>
+        </is>
+      </c>
+      <c r="G562" s="9" t="inlineStr">
+        <is>
+          <t>Soit $f$ une fonction de deux variables définie sur $D\subset\mathbb R^2$ et $(x_0,y_0)\in D$.</t>
+        </is>
+      </c>
+      <c r="H562" s="10" t="inlineStr">
+        <is>
+          <t>Qu'est-ce que la surface représentative de $f$ ? À quoi correspondent graphiquement les fonctions partielles en $(x_0,y_0)$ et les lignes de niveau ?</t>
+        </is>
+      </c>
+      <c r="I562" s="9" t="inlineStr">
+        <is>
+          <t>Surface : ensemble des points $(x,y,f(x,y))$ de $\mathbb R^3$, $(x,y)\in D$. La fonction partielle $x\mapsto f(x,y_0)$ décrit la section de la surface par le plan $y=y_0$ (et $\frac{\partial f}{\partial x}(x_0,y_0)$ est la pente de sa tangente) ; de même $y\mapsto f(x_0,y)$ et le plan $x=x_0$. La ligne de niveau $k$ est $\{(x,y)\in D,\ f(x,y)=k\}$ (comme les courbes de niveau d'une carte).</t>
+        </is>
+      </c>
+      <c r="J562" s="9" t="inlineStr">
+        <is>
+          <t>Programme Analyse 10 : « Surface représentative d'une fonction de deux variables, courbes ou lignes de niveau. On souligne le lien entre fonctions partielles et certaines sections de cette surface. »</t>
+        </is>
+      </c>
+      <c r="K562" s="9" t="n"/>
+      <c r="L562" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Fonctions de plusieurs variables »</t>
+        </is>
+      </c>
+      <c r="M562" s="11" t="n"/>
+      <c r="N562" s="11" t="n"/>
+    </row>
+    <row r="563">
+      <c r="A563" s="9" t="inlineStr">
+        <is>
+          <t>M563</t>
+        </is>
+      </c>
+      <c r="B563" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C563" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D563" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 10 – Fonctions de deux variables</t>
+        </is>
+      </c>
+      <c r="E563" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F563" s="9" t="inlineStr">
+        <is>
+          <t>Petites variations d’une fonction de deux variables</t>
+        </is>
+      </c>
+      <c r="G563" s="9" t="inlineStr">
+        <is>
+          <t>Soient $f$ de classe $\mathcal C^1$ sur un pavé ouvert et $(x_0,y_0)$ un point de ce pavé.</t>
+        </is>
+      </c>
+      <c r="H563" s="10" t="inlineStr">
+        <is>
+          <t>Comment évaluer la variation $\Delta f$ de $f$ due à de petites variations $\Delta x$, $\Delta y$ des variables ?</t>
+        </is>
+      </c>
+      <c r="I563" s="9" t="inlineStr">
+        <is>
+          <t>$\Delta f=f(x_0+\Delta x,y_0+\Delta y)-f(x_0,y_0)\approx\dfrac{\partial f}{\partial x}(x_0,y_0)\,\Delta x+\dfrac{\partial f}{\partial y}(x_0,y_0)\,\Delta y=\overrightarrow{\mathrm{grad}}f(x_0,y_0)\cdot(\Delta x,\Delta y)$.</t>
+        </is>
+      </c>
+      <c r="J563" s="9" t="inlineStr">
+        <is>
+          <t>Programme Analyse 10 : « Utilisation des dérivées partielles premières pour évaluer une petite variation de la valeur d'une fonction de classe $\mathcal C^1$ découlant de petites variations sur les variables. »</t>
+        </is>
+      </c>
+      <c r="K563" s="9" t="n"/>
+      <c r="L563" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Fonctions de plusieurs variables »</t>
+        </is>
+      </c>
+      <c r="M563" s="11" t="n"/>
+      <c r="N563" s="11" t="n"/>
+    </row>
+    <row r="564">
+      <c r="A564" s="9" t="inlineStr">
+        <is>
+          <t>M564</t>
+        </is>
+      </c>
+      <c r="B564" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C564" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D564" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 10 – Fonctions de deux variables</t>
+        </is>
+      </c>
+      <c r="E564" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F564" s="9" t="inlineStr">
+        <is>
+          <t>Interprétation graphique du gradient</t>
+        </is>
+      </c>
+      <c r="G564" s="9" t="inlineStr">
+        <is>
+          <t>Soient $f$ de classe $\mathcal C^1$ sur un pavé ouvert de $\mathbb R^2$ et $(x_0,y_0)$ un point où $\overrightarrow{\mathrm{grad}}f\neq\vec 0$.</t>
+        </is>
+      </c>
+      <c r="H564" s="10" t="inlineStr">
+        <is>
+          <t>Que représente géométriquement $\overrightarrow{\mathrm{grad}}f(x_0,y_0)$ ?</t>
+        </is>
+      </c>
+      <c r="I564" s="9" t="inlineStr">
+        <is>
+          <t>Il est orthogonal à la ligne de niveau de $f$ passant par $(x_0,y_0)$ et indique la direction dans laquelle $f$ croît le plus vite ; sa norme mesure la « pente ». Se déplacer orthogonalement au gradient, c'est suivre la ligne de niveau.</t>
+        </is>
+      </c>
+      <c r="J564" s="9" t="inlineStr">
+        <is>
+          <t>Programme Analyse 10 : « On pourra donner sans démonstration l'interprétation graphique du gradient. »</t>
+        </is>
+      </c>
+      <c r="K564" s="9" t="n"/>
+      <c r="L564" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Fonctions de plusieurs variables »</t>
+        </is>
+      </c>
+      <c r="M564" s="11" t="n"/>
+      <c r="N564" s="11" t="n"/>
+    </row>
+    <row r="565">
+      <c r="A565" s="9" t="inlineStr">
+        <is>
+          <t>M565</t>
+        </is>
+      </c>
+      <c r="B565" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C565" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D565" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 10 – Fonctions de deux variables</t>
+        </is>
+      </c>
+      <c r="E565" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F565" s="9" t="inlineStr">
+        <is>
+          <t>Plan tangent à une surface</t>
+        </is>
+      </c>
+      <c r="G565" s="9" t="inlineStr">
+        <is>
+          <t>Soient $f$ de classe $\mathcal C^1$ sur un pavé ouvert de $\mathbb R^2$ et $(x_0,y_0)$ un point de ce pavé.</t>
+        </is>
+      </c>
+      <c r="H565" s="10" t="inlineStr">
+        <is>
+          <t>Donner l'équation du plan tangent à la surface $z=f(x,y)$ au point $(x_0,y_0,f(x_0,y_0))$, et deux vecteurs directeurs.</t>
+        </is>
+      </c>
+      <c r="I565" s="9" t="inlineStr">
+        <is>
+          <t>$z=f(x_0,y_0)+(x-x_0)\dfrac{\partial f}{\partial x}(x_0,y_0)+(y-y_0)\dfrac{\partial f}{\partial y}(x_0,y_0)$ ; vecteurs directeurs $\left(1,0,\frac{\partial f}{\partial x}(x_0,y_0)\right)$ et $\left(0,1,\frac{\partial f}{\partial y}(x_0,y_0)\right)$.</t>
+        </is>
+      </c>
+      <c r="J565" s="9" t="inlineStr">
+        <is>
+          <t>Cours ; le programme ne mentionne pas le plan tangent (seulement les petites variations).</t>
+        </is>
+      </c>
+      <c r="K565" s="9" t="n"/>
+      <c r="L565" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Fonctions de plusieurs variables »</t>
+        </is>
+      </c>
+      <c r="M565" s="11" t="n"/>
+      <c r="N565" s="11" t="n"/>
+    </row>
+    <row r="566">
+      <c r="A566" s="9" t="inlineStr">
+        <is>
+          <t>M566</t>
+        </is>
+      </c>
+      <c r="B566" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C566" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D566" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 10 – Fonctions de deux variables</t>
+        </is>
+      </c>
+      <c r="E566" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F566" s="9" t="inlineStr">
+        <is>
+          <t>Opérations sur les fonctions de classe C¹ (deux variables)</t>
+        </is>
+      </c>
+      <c r="G566" s="9" t="inlineStr">
+        <is>
+          <t>Soient $f$, $g$ des fonctions de deux variables sur un pavé ouvert $P$.</t>
+        </is>
+      </c>
+      <c r="H566" s="10" t="inlineStr">
+        <is>
+          <t>Quelles opérations donnent des fonctions de classe $\mathcal C^1$ sur $P$ ?</t>
+        </is>
+      </c>
+      <c r="I566" s="9" t="inlineStr">
+        <is>
+          <t>Les fonctions polynomiales en $(x,y)$ sont $\mathcal C^1$ ; si $f$ et $g$ sont $\mathcal C^1$ : combinaisons linéaires, produit, quotient $f/g$ (si $g$ ne s'annule pas sur $P$) ; si $\varphi$ est $\mathcal C^1$ sur un intervalle contenant $f(P)$, $\varphi\circ f$ est $\mathcal C^1$ (théorèmes admis).</t>
+        </is>
+      </c>
+      <c r="J566" s="9" t="inlineStr">
+        <is>
+          <t>Cours (admis) ; le programme précise qu'on ne demandera jamais de montrer qu'une fonction est $\mathcal C^1$.</t>
+        </is>
+      </c>
+      <c r="K566" s="9" t="n"/>
+      <c r="L566" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Fonctions de plusieurs variables »</t>
+        </is>
+      </c>
+      <c r="M566" s="11" t="n"/>
+      <c r="N566" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M561" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M566" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -36790,7 +37090,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$561,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$566,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -36805,7 +37105,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$561,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$566,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -36820,7 +37120,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$561,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$566,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -36847,7 +37147,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$561)</f>
+        <f>COUNTA(Fiches!$M$2:$M$566)</f>
         <v/>
       </c>
     </row>
@@ -36893,15 +37193,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A13,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A13,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A13,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A13,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A13,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A13,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -36916,15 +37216,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A14,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A14,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A14,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A14,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A14,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A14,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -36939,15 +37239,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A15,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A15,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A15,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A15,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A15,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A15,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -36962,15 +37262,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A16,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A16,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A16,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A16,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A16,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A16,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -36985,15 +37285,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A17,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A17,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A17,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A17,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A17,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A17,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -37008,15 +37308,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A18,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A18,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A18,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A18,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A18,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A18,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -37031,15 +37331,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A19,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A19,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A19,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A19,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A19,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A19,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -37054,15 +37354,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A20,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A20,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A20,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A20,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A20,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A20,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -37077,15 +37377,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A21,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A21,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A21,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A21,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A21,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A21,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -37100,15 +37400,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A22,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A22,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A22,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A22,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A22,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A22,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -37123,15 +37423,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A23,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A23,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A23,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A23,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A23,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A23,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -37146,15 +37446,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A24,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A24,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A24,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A24,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A24,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A24,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -37169,15 +37469,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A25,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A25,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A25,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A25,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A25,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A25,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -37192,15 +37492,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A26,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A26,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A26,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A26,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A26,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A26,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -37215,15 +37515,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A27,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A27,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A27,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A27,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A27,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A27,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -37238,15 +37538,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A28,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A28,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A28,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A28,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A28,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A28,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -37261,15 +37561,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A29,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A29,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A29,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A29,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A29,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A29,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -37284,15 +37584,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A30,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A30,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A30,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A30,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A30,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A30,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -37307,15 +37607,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A31,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A31,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A31,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A31,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A31,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A31,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -37330,15 +37630,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A32,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A32,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A32,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A32,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A32,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A32,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -37353,15 +37653,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A33,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A33,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A33,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A33,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A33,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A33,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -37376,15 +37676,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A34,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A34,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A34,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A34,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A34,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A34,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -37399,15 +37699,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A35,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A35,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A35,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A35,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A35,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A35,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -37422,15 +37722,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A36,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A36,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A36,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A36,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A36,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A36,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -37445,15 +37745,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A37,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A37,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A37,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A37,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A37,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A37,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -37468,15 +37768,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A38,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A38,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A38,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A38,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A38,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A38,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -37491,15 +37791,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A39,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A39,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A39,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A39,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A39,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A39,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -37514,15 +37814,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A40,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A40,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A40,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A40,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A40,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A40,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -37537,15 +37837,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A41,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A41,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A41,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A41,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A41,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A41,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -37560,15 +37860,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A42,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A42,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A42,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A42,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A42,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A42,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -37583,15 +37883,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A43,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A43,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A43,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A43,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A43,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A43,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -37606,15 +37906,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A44,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A44,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A44,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A44,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A44,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A44,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -37629,15 +37929,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A45,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A45,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A45,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A45,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A45,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A45,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -37652,15 +37952,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A46,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A46,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A46,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A46,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A46,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A46,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -37675,15 +37975,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A47,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A47,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A47,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A47,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A47,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A47,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -37698,15 +37998,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A48,Fiches!$B$2:$B$561,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A48,Fiches!$B$2:$B$566,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A48,Fiches!$B$2:$B$561,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A48,Fiches!$B$2:$B$566,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$561,$A48,Fiches!$B$2:$B$561,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$566,$A48,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Intégration : intégration du cours (valeur moyenne, aires, parité/périodicité, primitives composées)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N566"/>
+  <dimension ref="A1:N569"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -14131,7 +14131,7 @@
       </c>
       <c r="I231" s="9" t="inlineStr">
         <is>
-          <t>Une fonction continue sur un intervalle admet des primitives ; deux primitives diffèrent d'une constante.</t>
+          <t>Une fonction continue sur un intervalle admet des primitives ; si $F$ en est une, les primitives de $f$ sont les $F+k$, $k\in\mathbb R$. Pour $x_0\in I$ et $y_0\in\mathbb R$, il existe une unique primitive valant $y_0$ en $x_0$.</t>
         </is>
       </c>
       <c r="J231" s="9" t="inlineStr">
@@ -14414,7 +14414,7 @@
       </c>
       <c r="F236" s="9" t="inlineStr">
         <is>
-          <t>Sommes de Riemann (« Théorème de la valeur moyenne »)</t>
+          <t>Sommes de Riemann</t>
         </is>
       </c>
       <c r="G236" s="9" t="inlineStr">
@@ -14429,7 +14429,7 @@
       </c>
       <c r="I236" s="9" t="inlineStr">
         <is>
-          <t>Si $f$ est continue sur $[a,b]$ : $\dfrac1{b-a}\int_a^bf(t)\,dt=\lim_{n\to\infty}\dfrac1n\sum_{k=0}^{n-1}f\!\left(a+k\frac{b-a}n\right)$.</t>
+          <t>Si $f$ est continue sur $[a,b]$ : $\displaystyle\int_a^bf(t)\,dt=\lim_{n\to\infty}\frac{b-a}n\sum_{k=0}^{n-1}f\!\left(a+k\frac{b-a}n\right)=\lim_{n\to\infty}\frac{b-a}n\sum_{k=1}^{n}f\!\left(a+k\frac{b-a}n\right)$. Sur $[0,1]$ : $\int_0^1f=\lim\frac1n\sum_{k=0}^{n-1}f\!\left(\frac kn\right)$.</t>
         </is>
       </c>
       <c r="J236" s="9" t="inlineStr">
@@ -33850,10 +33850,190 @@
       <c r="M566" s="11" t="n"/>
       <c r="N566" s="11" t="n"/>
     </row>
+    <row r="567">
+      <c r="A567" s="9" t="inlineStr">
+        <is>
+          <t>M567</t>
+        </is>
+      </c>
+      <c r="B567" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C567" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D567" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 8 – Intégration sur un segment</t>
+        </is>
+      </c>
+      <c r="E567" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F567" s="9" t="inlineStr">
+        <is>
+          <t>Valeur moyenne et encadrement d’une intégrale</t>
+        </is>
+      </c>
+      <c r="G567" s="9" t="inlineStr">
+        <is>
+          <t>Soient $a&lt;b$ et $f$ continue sur $[a,b]$.</t>
+        </is>
+      </c>
+      <c r="H567" s="10" t="inlineStr">
+        <is>
+          <t>Définir la valeur moyenne de $f$ sur $[a,b]$. Comment encadrer $\int_a^bf$ si $m\le f\le M$ sur $[a,b]$ ?</t>
+        </is>
+      </c>
+      <c r="I567" s="9" t="inlineStr">
+        <is>
+          <t>$\mu=\dfrac1{b-a}\displaystyle\int_a^bf(t)\,dt$ ; c'est une valeur atteinte par $f$ sur $[a,b]$. Si $m\le f\le M$ : $m(b-a)\le\displaystyle\int_a^bf(t)\,dt\le M(b-a)$, donc $m\le\mu\le M$.</t>
+        </is>
+      </c>
+      <c r="J567" s="9" t="inlineStr">
+        <is>
+          <t>Programme Analyse 8 : « Encadrement de l'intégrale à partir d'un encadrement de la fonction » ; « Valeur moyenne d'une fonction continue sur un segment. La valeur moyenne appartient à l'ensemble des valeurs atteintes par la fonction. »</t>
+        </is>
+      </c>
+      <c r="K567" s="9" t="n"/>
+      <c r="L567" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Intégration »</t>
+        </is>
+      </c>
+      <c r="M567" s="11" t="n"/>
+      <c r="N567" s="11" t="n"/>
+    </row>
+    <row r="568">
+      <c r="A568" s="9" t="inlineStr">
+        <is>
+          <t>M568</t>
+        </is>
+      </c>
+      <c r="B568" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C568" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D568" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 8 – Intégration sur un segment</t>
+        </is>
+      </c>
+      <c r="E568" s="9" t="inlineStr">
+        <is>
+          <t>Théorème</t>
+        </is>
+      </c>
+      <c r="F568" s="9" t="inlineStr">
+        <is>
+          <t>Aire entre deux courbes</t>
+        </is>
+      </c>
+      <c r="G568" s="9" t="inlineStr">
+        <is>
+          <t>Soient $a&lt;b$, $f$ et $g$ continues sur $[a,b]$ avec $f\le g$.</t>
+        </is>
+      </c>
+      <c r="H568" s="10" t="inlineStr">
+        <is>
+          <t>Quelle est l'aire (en u.a.) du domaine compris entre $\mathcal C_f$, $\mathcal C_g$ et les droites $x=a$, $x=b$ ?</t>
+        </is>
+      </c>
+      <c r="I568" s="9" t="inlineStr">
+        <is>
+          <t>$\mathcal A=\displaystyle\int_a^b\big(g(x)-f(x)\big)\,dx$ u.a. (l'unité d'aire est $\|\vec\imath\|\times\|\vec\jmath\|$).</t>
+        </is>
+      </c>
+      <c r="J568" s="9" t="inlineStr">
+        <is>
+          <t>Cours ; le programme définit l'intégrale comme une aire « intuitive » sans citer l'aire entre deux courbes.</t>
+        </is>
+      </c>
+      <c r="K568" s="9" t="n"/>
+      <c r="L568" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Intégration »</t>
+        </is>
+      </c>
+      <c r="M568" s="11" t="n"/>
+      <c r="N568" s="11" t="n"/>
+    </row>
+    <row r="569">
+      <c r="A569" s="9" t="inlineStr">
+        <is>
+          <t>M569</t>
+        </is>
+      </c>
+      <c r="B569" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C569" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D569" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 8 – Intégration sur un segment</t>
+        </is>
+      </c>
+      <c r="E569" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F569" s="9" t="inlineStr">
+        <is>
+          <t>Intégrale d’une fonction paire, impaire, périodique</t>
+        </is>
+      </c>
+      <c r="G569" s="9" t="inlineStr">
+        <is>
+          <t>Soient $a&gt;0$ et $f$ continue (sur $[-a,a]$, ou sur $\mathbb R$ et $T$-périodique).</t>
+        </is>
+      </c>
+      <c r="H569" s="10" t="inlineStr">
+        <is>
+          <t>Que vaut $\int_{-a}^af$ si $f$ est paire ? impaire ? Que dire des intégrales d'une fonction $T$-périodique sur une période ?</t>
+        </is>
+      </c>
+      <c r="I569" s="9" t="inlineStr">
+        <is>
+          <t>Paire : $\int_{-a}^af=2\int_0^af$. Impaire : $\int_{-a}^af=0$. $T$-périodique : $\int_{a+nT}^{b+nT}f=\int_a^bf$ ($n\in\mathbb Z$) et $\int_a^{a+T}f=\int_0^Tf$ pour tout $a$. (Conséquences du changement de variable.)</t>
+        </is>
+      </c>
+      <c r="J569" s="9" t="inlineStr">
+        <is>
+          <t>Corollaires du cours ; non cités par le programme.</t>
+        </is>
+      </c>
+      <c r="K569" s="9" t="n"/>
+      <c r="L569" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Intégration »</t>
+        </is>
+      </c>
+      <c r="M569" s="11" t="n"/>
+      <c r="N569" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M566" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M569" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -33867,7 +34047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M60"/>
+  <dimension ref="A1:M66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -37031,10 +37211,316 @@
       <c r="L60" s="14" t="n"/>
       <c r="M60" s="14" t="n"/>
     </row>
+    <row r="61">
+      <c r="A61" s="12" t="inlineStr">
+        <is>
+          <t>F060</t>
+        </is>
+      </c>
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C61" s="12" t="inlineStr">
+        <is>
+          <t>Primitives usuelles</t>
+        </is>
+      </c>
+      <c r="D61" s="12" t="inlineStr">
+        <is>
+          <t>Primitive de $u'e^u$</t>
+        </is>
+      </c>
+      <c r="E61" s="12" t="inlineStr">
+        <is>
+          <t>Soit $u$ une fonction de classe $\mathcal C^1$ sur un intervalle $I$.</t>
+        </is>
+      </c>
+      <c r="F61" s="13" t="inlineStr">
+        <is>
+          <t>Donner une primitive de $u'e^u$.</t>
+        </is>
+      </c>
+      <c r="G61" s="12" t="inlineStr">
+        <is>
+          <t>$e^u$</t>
+        </is>
+      </c>
+      <c r="H61" s="12" t="inlineStr">
+        <is>
+          <t>Analyse 3 : « Primitives de u′eᵘ, u′uⁿ, u′/u, u′/√u, u′ sin u, u′ cos u. »</t>
+        </is>
+      </c>
+      <c r="I61" s="12" t="n"/>
+      <c r="J61" s="12" t="n"/>
+      <c r="K61" s="12" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Intégration » (formes composées citées par le programme)</t>
+        </is>
+      </c>
+      <c r="L61" s="14" t="n"/>
+      <c r="M61" s="14" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="12" t="inlineStr">
+        <is>
+          <t>F061</t>
+        </is>
+      </c>
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C62" s="12" t="inlineStr">
+        <is>
+          <t>Primitives usuelles</t>
+        </is>
+      </c>
+      <c r="D62" s="12" t="inlineStr">
+        <is>
+          <t>Primitive de $u'u^n$ ($n\neq-1$)</t>
+        </is>
+      </c>
+      <c r="E62" s="12" t="inlineStr">
+        <is>
+          <t>Soit $u$ une fonction de classe $\mathcal C^1$ sur un intervalle $I$, et $n\in\mathbb Z\setminus\{-1\}$ ($u$ ne s'annule pas sur $I$ si $n&lt;0$).</t>
+        </is>
+      </c>
+      <c r="F62" s="13" t="inlineStr">
+        <is>
+          <t>Donner une primitive de $u'u^n$.</t>
+        </is>
+      </c>
+      <c r="G62" s="12" t="inlineStr">
+        <is>
+          <t>$\dfrac{u^{n+1}}{n+1}$</t>
+        </is>
+      </c>
+      <c r="H62" s="12" t="inlineStr">
+        <is>
+          <t>Analyse 3 : « Primitives de u′eᵘ, u′uⁿ, u′/u, u′/√u, u′ sin u, u′ cos u. »</t>
+        </is>
+      </c>
+      <c r="I62" s="12" t="n"/>
+      <c r="J62" s="12" t="n"/>
+      <c r="K62" s="12" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Intégration » (formes composées citées par le programme)</t>
+        </is>
+      </c>
+      <c r="L62" s="14" t="n"/>
+      <c r="M62" s="14" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="inlineStr">
+        <is>
+          <t>F062</t>
+        </is>
+      </c>
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C63" s="12" t="inlineStr">
+        <is>
+          <t>Primitives usuelles</t>
+        </is>
+      </c>
+      <c r="D63" s="12" t="inlineStr">
+        <is>
+          <t>Primitive de $\dfrac{u'}u$</t>
+        </is>
+      </c>
+      <c r="E63" s="12" t="inlineStr">
+        <is>
+          <t>Soit $u$ une fonction de classe $\mathcal C^1$ sur un intervalle $I$ ne s'annulant pas sur $I$.</t>
+        </is>
+      </c>
+      <c r="F63" s="13" t="inlineStr">
+        <is>
+          <t>Donner une primitive de $\dfrac{u'}u$.</t>
+        </is>
+      </c>
+      <c r="G63" s="12" t="inlineStr">
+        <is>
+          <t>$\ln|u|$</t>
+        </is>
+      </c>
+      <c r="H63" s="12" t="inlineStr">
+        <is>
+          <t>Analyse 3 : « Primitives de u′eᵘ, u′uⁿ, u′/u, u′/√u, u′ sin u, u′ cos u. »</t>
+        </is>
+      </c>
+      <c r="I63" s="12" t="n"/>
+      <c r="J63" s="12" t="n"/>
+      <c r="K63" s="12" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Intégration » (formes composées citées par le programme)</t>
+        </is>
+      </c>
+      <c r="L63" s="14" t="n"/>
+      <c r="M63" s="14" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="12" t="inlineStr">
+        <is>
+          <t>F063</t>
+        </is>
+      </c>
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C64" s="12" t="inlineStr">
+        <is>
+          <t>Primitives usuelles</t>
+        </is>
+      </c>
+      <c r="D64" s="12" t="inlineStr">
+        <is>
+          <t>Primitive de $\dfrac{u'}{\sqrt u}$</t>
+        </is>
+      </c>
+      <c r="E64" s="12" t="inlineStr">
+        <is>
+          <t>Soit $u$ une fonction de classe $\mathcal C^1$ sur un intervalle $I$, avec $u&gt;0$ sur $I$.</t>
+        </is>
+      </c>
+      <c r="F64" s="13" t="inlineStr">
+        <is>
+          <t>Donner une primitive de $\dfrac{u'}{\sqrt u}$.</t>
+        </is>
+      </c>
+      <c r="G64" s="12" t="inlineStr">
+        <is>
+          <t>$2\sqrt u$</t>
+        </is>
+      </c>
+      <c r="H64" s="12" t="inlineStr">
+        <is>
+          <t>Analyse 3 : « Primitives de u′eᵘ, u′uⁿ, u′/u, u′/√u, u′ sin u, u′ cos u. »</t>
+        </is>
+      </c>
+      <c r="I64" s="12" t="n"/>
+      <c r="J64" s="12" t="n"/>
+      <c r="K64" s="12" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Intégration » (formes composées citées par le programme)</t>
+        </is>
+      </c>
+      <c r="L64" s="14" t="n"/>
+      <c r="M64" s="14" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="inlineStr">
+        <is>
+          <t>F064</t>
+        </is>
+      </c>
+      <c r="B65" s="13" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C65" s="12" t="inlineStr">
+        <is>
+          <t>Primitives usuelles</t>
+        </is>
+      </c>
+      <c r="D65" s="12" t="inlineStr">
+        <is>
+          <t>Primitive de $u'\cos u$</t>
+        </is>
+      </c>
+      <c r="E65" s="12" t="inlineStr">
+        <is>
+          <t>Soit $u$ une fonction de classe $\mathcal C^1$ sur un intervalle $I$.</t>
+        </is>
+      </c>
+      <c r="F65" s="13" t="inlineStr">
+        <is>
+          <t>Donner une primitive de $u'\cos u$.</t>
+        </is>
+      </c>
+      <c r="G65" s="12" t="inlineStr">
+        <is>
+          <t>$\sin u$</t>
+        </is>
+      </c>
+      <c r="H65" s="12" t="inlineStr">
+        <is>
+          <t>Analyse 3 : « Primitives de u′eᵘ, u′uⁿ, u′/u, u′/√u, u′ sin u, u′ cos u. »</t>
+        </is>
+      </c>
+      <c r="I65" s="12" t="n"/>
+      <c r="J65" s="12" t="n"/>
+      <c r="K65" s="12" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Intégration » (formes composées citées par le programme)</t>
+        </is>
+      </c>
+      <c r="L65" s="14" t="n"/>
+      <c r="M65" s="14" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="12" t="inlineStr">
+        <is>
+          <t>F065</t>
+        </is>
+      </c>
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C66" s="12" t="inlineStr">
+        <is>
+          <t>Primitives usuelles</t>
+        </is>
+      </c>
+      <c r="D66" s="12" t="inlineStr">
+        <is>
+          <t>Primitive de $u'\sin u$</t>
+        </is>
+      </c>
+      <c r="E66" s="12" t="inlineStr">
+        <is>
+          <t>Soit $u$ une fonction de classe $\mathcal C^1$ sur un intervalle $I$.</t>
+        </is>
+      </c>
+      <c r="F66" s="13" t="inlineStr">
+        <is>
+          <t>Donner une primitive de $u'\sin u$.</t>
+        </is>
+      </c>
+      <c r="G66" s="12" t="inlineStr">
+        <is>
+          <t>$-\cos u$</t>
+        </is>
+      </c>
+      <c r="H66" s="12" t="inlineStr">
+        <is>
+          <t>Analyse 3 : « Primitives de u′eᵘ, u′uⁿ, u′/u, u′/√u, u′ sin u, u′ cos u. »</t>
+        </is>
+      </c>
+      <c r="I66" s="12" t="n"/>
+      <c r="J66" s="12" t="n"/>
+      <c r="K66" s="12" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Intégration » (formes composées citées par le programme)</t>
+        </is>
+      </c>
+      <c r="L66" s="14" t="n"/>
+      <c r="M66" s="14" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:M60"/>
   <dataValidations count="1">
-    <dataValidation sqref="L2:L60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -37090,7 +37576,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$566,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$569,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -37105,7 +37591,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$566,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$569,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -37120,7 +37606,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$566,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$569,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -37147,7 +37633,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$566)</f>
+        <f>COUNTA(Fiches!$M$2:$M$569)</f>
         <v/>
       </c>
     </row>
@@ -37193,15 +37679,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A13,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A13,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A13,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A13,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A13,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A13,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -37216,15 +37702,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A14,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A14,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A14,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A14,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A14,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A14,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -37239,15 +37725,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A15,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A15,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A15,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A15,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A15,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A15,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -37262,15 +37748,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A16,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A16,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A16,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A16,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A16,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A16,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -37285,15 +37771,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A17,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A17,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A17,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A17,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A17,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A17,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -37308,15 +37794,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A18,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A18,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A18,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A18,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A18,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A18,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -37331,15 +37817,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A19,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A19,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A19,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A19,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A19,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A19,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -37354,15 +37840,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A20,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A20,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A20,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A20,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A20,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A20,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -37377,15 +37863,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A21,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A21,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A21,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A21,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A21,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A21,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -37400,15 +37886,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A22,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A22,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A22,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A22,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A22,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A22,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -37423,15 +37909,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A23,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A23,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A23,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A23,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A23,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A23,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -37446,15 +37932,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A24,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A24,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A24,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A24,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A24,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A24,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -37469,15 +37955,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A25,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A25,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A25,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A25,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A25,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A25,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -37492,15 +37978,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A26,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A26,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A26,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A26,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A26,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A26,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -37515,15 +38001,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A27,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A27,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A27,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A27,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A27,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A27,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -37538,15 +38024,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A28,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A28,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A28,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A28,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A28,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A28,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -37561,15 +38047,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A29,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A29,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A29,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A29,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A29,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A29,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -37584,15 +38070,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A30,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A30,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A30,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A30,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A30,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A30,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -37607,15 +38093,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A31,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A31,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A31,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A31,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A31,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A31,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -37630,15 +38116,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A32,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A32,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A32,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A32,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A32,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A32,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -37653,15 +38139,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A33,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A33,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A33,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A33,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A33,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A33,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -37676,15 +38162,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A34,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A34,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A34,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A34,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A34,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A34,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -37699,15 +38185,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A35,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A35,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A35,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A35,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A35,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A35,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -37722,15 +38208,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A36,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A36,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A36,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A36,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A36,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A36,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -37745,15 +38231,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A37,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A37,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A37,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A37,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A37,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A37,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -37768,15 +38254,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A38,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A38,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A38,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A38,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A38,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A38,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -37791,15 +38277,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A39,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A39,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A39,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A39,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A39,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A39,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -37814,15 +38300,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A40,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A40,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A40,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A40,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A40,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A40,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -37837,15 +38323,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A41,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A41,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A41,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A41,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A41,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A41,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -37860,15 +38346,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A42,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A42,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A42,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A42,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A42,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A42,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -37883,15 +38369,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A43,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A43,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A43,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A43,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A43,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A43,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -37906,15 +38392,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A44,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A44,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A44,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A44,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A44,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A44,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -37929,15 +38415,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A45,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A45,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A45,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A45,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A45,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A45,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -37952,15 +38438,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A46,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A46,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A46,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A46,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A46,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A46,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -37975,15 +38461,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A47,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A47,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A47,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A47,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A47,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A47,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -37998,15 +38484,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A48,Fiches!$B$2:$B$566,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A48,Fiches!$B$2:$B$569,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A48,Fiches!$B$2:$B$566,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A48,Fiches!$B$2:$B$569,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$566,$A48,Fiches!$B$2:$B$566,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$569,$A48,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Logique et raisonnements : intégration du cours (connecteurs, implication, quantificateurs, récurrences)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N569"/>
+  <dimension ref="A1:N579"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -873,7 +873,7 @@
       </c>
       <c r="I2" s="9" t="inlineStr">
         <is>
-          <t>$A\subset B$ si et seulement si tout élément de $A$ appartient à $B$ : $\forall x,\ x\in A\Rightarrow x\in B$.</t>
+          <t>$A\subset B$ si et seulement si tout élément de $A$ appartient à $B$ : $\forall x,\ x\in A\Rightarrow x\in B$. On a $A=B\iff(A\subset B\text{ et }B\subset A)$ : on montre une égalité d'ensembles par double inclusion.</t>
         </is>
       </c>
       <c r="J2" s="9" t="inlineStr">
@@ -34030,10 +34030,610 @@
       <c r="M569" s="11" t="n"/>
       <c r="N569" s="11" t="n"/>
     </row>
+    <row r="570">
+      <c r="A570" s="9" t="inlineStr">
+        <is>
+          <t>M570</t>
+        </is>
+      </c>
+      <c r="B570" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C570" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D570" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 1 – Logique, ensembles</t>
+        </is>
+      </c>
+      <c r="E570" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F570" s="9" t="inlineStr">
+        <is>
+          <t>Négation de « et » et de « ou »</t>
+        </is>
+      </c>
+      <c r="G570" s="9" t="inlineStr">
+        <is>
+          <t>Soient $P$ et $Q$ deux assertions.</t>
+        </is>
+      </c>
+      <c r="H570" s="10" t="inlineStr">
+        <is>
+          <t>Écrire $\mathrm{non}(P\text{ et }Q)$ et $\mathrm{non}(P\text{ ou }Q)$. Le « ou » mathématique est-il inclusif ou exclusif ?</t>
+        </is>
+      </c>
+      <c r="I570" s="9" t="inlineStr">
+        <is>
+          <t>$\mathrm{non}(P\text{ et }Q)\iff(\mathrm{non}\,P)\text{ ou }(\mathrm{non}\,Q)$ ; $\mathrm{non}(P\text{ ou }Q)\iff(\mathrm{non}\,P)\text{ et }(\mathrm{non}\,Q)$. Le « ou » mathématique est inclusif : $P\text{ ou }Q$ est vraie dès qu'au moins l'une des deux l'est (éventuellement les deux).</t>
+        </is>
+      </c>
+      <c r="J570" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 1 : « Assertion, négation, « et », « ou » » ; « Négation d'un « et » et d'un « ou ». »</t>
+        </is>
+      </c>
+      <c r="K570" s="9" t="n"/>
+      <c r="L570" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Logique et raisonnements »</t>
+        </is>
+      </c>
+      <c r="M570" s="11" t="n"/>
+      <c r="N570" s="11" t="n"/>
+    </row>
+    <row r="571">
+      <c r="A571" s="9" t="inlineStr">
+        <is>
+          <t>M571</t>
+        </is>
+      </c>
+      <c r="B571" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C571" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D571" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 1 – Logique, ensembles</t>
+        </is>
+      </c>
+      <c r="E571" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F571" s="9" t="inlineStr">
+        <is>
+          <t>Distributivité de « et » et « ou »</t>
+        </is>
+      </c>
+      <c r="G571" s="9" t="inlineStr">
+        <is>
+          <t>Soient $A$, $B$, $C$ trois assertions.</t>
+        </is>
+      </c>
+      <c r="H571" s="10" t="inlineStr">
+        <is>
+          <t>Développer $A\text{ ou }(B\text{ et }C)$ et $A\text{ et }(B\text{ ou }C)$.</t>
+        </is>
+      </c>
+      <c r="I571" s="9" t="inlineStr">
+        <is>
+          <t>$A\text{ ou }(B\text{ et }C)\iff(A\text{ ou }B)\text{ et }(A\text{ ou }C)$ ; $A\text{ et }(B\text{ ou }C)\iff(A\text{ et }B)\text{ ou }(A\text{ et }C)$.</t>
+        </is>
+      </c>
+      <c r="J571" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 1 : « Distributivité du « ou » sur le « et » et du « et » sur le « ou ». »</t>
+        </is>
+      </c>
+      <c r="K571" s="9" t="n"/>
+      <c r="L571" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Logique et raisonnements »</t>
+        </is>
+      </c>
+      <c r="M571" s="11" t="n"/>
+      <c r="N571" s="11" t="n"/>
+    </row>
+    <row r="572">
+      <c r="A572" s="9" t="inlineStr">
+        <is>
+          <t>M572</t>
+        </is>
+      </c>
+      <c r="B572" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C572" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D572" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 1 – Logique, ensembles</t>
+        </is>
+      </c>
+      <c r="E572" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F572" s="9" t="inlineStr">
+        <is>
+          <t>Implication et sa négation</t>
+        </is>
+      </c>
+      <c r="G572" s="9" t="inlineStr">
+        <is>
+          <t>Soient $P$ et $Q$ deux assertions.</t>
+        </is>
+      </c>
+      <c r="H572" s="10" t="inlineStr">
+        <is>
+          <t>Que signifie $P\Rightarrow Q$ ? Quelle est sa négation ?</t>
+        </is>
+      </c>
+      <c r="I572" s="9" t="inlineStr">
+        <is>
+          <t>$P\Rightarrow Q$ est l'assertion « $Q$ ou $\mathrm{non}\,P$ » : si $P$ est vraie, $Q$ l'est (et si $P$ est fausse, l'implication est vraie). Négation : $P\text{ et }\mathrm{non}\,Q$ ; ce n'est pas une implication.</t>
+        </is>
+      </c>
+      <c r="J572" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 1 : « implication ».</t>
+        </is>
+      </c>
+      <c r="K572" s="9" t="n"/>
+      <c r="L572" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Logique et raisonnements »</t>
+        </is>
+      </c>
+      <c r="M572" s="11" t="n"/>
+      <c r="N572" s="11" t="n"/>
+    </row>
+    <row r="573">
+      <c r="A573" s="9" t="inlineStr">
+        <is>
+          <t>M573</t>
+        </is>
+      </c>
+      <c r="B573" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C573" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D573" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 1 – Logique, ensembles</t>
+        </is>
+      </c>
+      <c r="E573" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F573" s="9" t="inlineStr">
+        <is>
+          <t>Réciproque, contraposée, équivalence</t>
+        </is>
+      </c>
+      <c r="G573" s="9" t="inlineStr">
+        <is>
+          <t>Soient $P$ et $Q$ deux assertions.</t>
+        </is>
+      </c>
+      <c r="H573" s="10" t="inlineStr">
+        <is>
+          <t>Donner la réciproque et la contraposée de $P\Rightarrow Q$. Laquelle lui est équivalente ? Que signifie $P\iff Q$ ?</t>
+        </is>
+      </c>
+      <c r="I573" s="9" t="inlineStr">
+        <is>
+          <t>Réciproque : $Q\Rightarrow P$ (pas équivalente en général). Contraposée : $\mathrm{non}\,Q\Rightarrow\mathrm{non}\,P$, équivalente à $P\Rightarrow Q$ (principe de contraposition). $P\iff Q$ signifie $(P\Rightarrow Q)\text{ et }(Q\Rightarrow P)$ ; on la prouve par équivalences successives ou par double implication.</t>
+        </is>
+      </c>
+      <c r="J573" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 1 : « implication, équivalence » ; « Le principe de contraposition est rappelé. »</t>
+        </is>
+      </c>
+      <c r="K573" s="9" t="n"/>
+      <c r="L573" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Logique et raisonnements »</t>
+        </is>
+      </c>
+      <c r="M573" s="11" t="n"/>
+      <c r="N573" s="11" t="n"/>
+    </row>
+    <row r="574">
+      <c r="A574" s="9" t="inlineStr">
+        <is>
+          <t>M574</t>
+        </is>
+      </c>
+      <c r="B574" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C574" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D574" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 1 – Logique, ensembles</t>
+        </is>
+      </c>
+      <c r="E574" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F574" s="9" t="inlineStr">
+        <is>
+          <t>Condition nécessaire, condition suffisante</t>
+        </is>
+      </c>
+      <c r="G574" s="9" t="inlineStr">
+        <is>
+          <t>Soient $C$ une condition et $R$ un résultat.</t>
+        </is>
+      </c>
+      <c r="H574" s="10" t="inlineStr">
+        <is>
+          <t>Que signifient « $C$ est une condition suffisante pour $R$ » ? « nécessaire » ? « nécessaire et suffisante » ?</t>
+        </is>
+      </c>
+      <c r="I574" s="9" t="inlineStr">
+        <is>
+          <t>Suffisante : $C\Rightarrow R$. Nécessaire : $R\Rightarrow C$ (« pour avoir $R$, il faut $C$ »). Nécessaire et suffisante : $R\iff C$. Exemple : $x=-1$ est suffisante pour $x^2=1$, mais pas nécessaire.</t>
+        </is>
+      </c>
+      <c r="J574" s="9" t="inlineStr">
+        <is>
+          <t>Cours ; vocabulaire non cité par le programme.</t>
+        </is>
+      </c>
+      <c r="K574" s="9" t="n"/>
+      <c r="L574" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Logique et raisonnements »</t>
+        </is>
+      </c>
+      <c r="M574" s="11" t="n"/>
+      <c r="N574" s="11" t="n"/>
+    </row>
+    <row r="575">
+      <c r="A575" s="9" t="inlineStr">
+        <is>
+          <t>M575</t>
+        </is>
+      </c>
+      <c r="B575" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C575" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D575" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 1 – Logique, ensembles</t>
+        </is>
+      </c>
+      <c r="E575" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F575" s="9" t="inlineStr">
+        <is>
+          <t>Quantificateurs et négation</t>
+        </is>
+      </c>
+      <c r="G575" s="9" t="inlineStr">
+        <is>
+          <t>Soient $E$ un ensemble et $P(x)$ une assertion dépendant de $x\in E$.</t>
+        </is>
+      </c>
+      <c r="H575" s="10" t="inlineStr">
+        <is>
+          <t>Que signifient $\forall$, $\exists$, $\exists!$ ? Écrire la négation de $\forall x\in E,\ P(x)$ et de $\exists x\in E,\ P(x)$. L'ordre des quantificateurs compte-t-il ?</t>
+        </is>
+      </c>
+      <c r="I575" s="9" t="inlineStr">
+        <is>
+          <t>$\forall$ : pour tout ; $\exists$ : il existe au moins un ; $\exists!$ : il existe un unique. $\mathrm{non}(\forall x\in E,\ P(x))\iff\exists x\in E,\ \mathrm{non}\,P(x)$ ; $\mathrm{non}(\exists x\in E,\ P(x))\iff\forall x\in E,\ \mathrm{non}\,P(x)$ : on échange les quantificateurs et on nie l'assertion finale. Oui : $\forall x,\exists y$ et $\exists y,\forall x$ n'ont pas le même sens.</t>
+        </is>
+      </c>
+      <c r="J575" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 1 : « Quantificateurs universel et existentiel. Négation d'une assertion quantifiée. »</t>
+        </is>
+      </c>
+      <c r="K575" s="9" t="n"/>
+      <c r="L575" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Logique et raisonnements »</t>
+        </is>
+      </c>
+      <c r="M575" s="11" t="n"/>
+      <c r="N575" s="11" t="n"/>
+    </row>
+    <row r="576">
+      <c r="A576" s="9" t="inlineStr">
+        <is>
+          <t>M576</t>
+        </is>
+      </c>
+      <c r="B576" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C576" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D576" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 1 – Logique, ensembles</t>
+        </is>
+      </c>
+      <c r="E576" s="9" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+      <c r="F576" s="9" t="inlineStr">
+        <is>
+          <t>Raisonnement par l’absurde ou par contraposée</t>
+        </is>
+      </c>
+      <c r="G576" s="9" t="inlineStr">
+        <is>
+          <t>On veut prouver $P\Rightarrow Q$.</t>
+        </is>
+      </c>
+      <c r="H576" s="10" t="inlineStr">
+        <is>
+          <t>Décrire le raisonnement par contraposée et le raisonnement par l'absurde. En quoi diffèrent-ils ?</t>
+        </is>
+      </c>
+      <c r="I576" s="9" t="inlineStr">
+        <is>
+          <t>Contraposée : on suppose $\mathrm{non}\,Q$ et on démontre $\mathrm{non}\,P$. Absurde : on suppose $P$ et $\mathrm{non}\,Q$ et on aboutit à une contradiction (on montre que « $P$ et $\mathrm{non}\,Q$ » est fausse).</t>
+        </is>
+      </c>
+      <c r="J576" s="9" t="inlineStr">
+        <is>
+          <t>Cours ; le programme ne cite que la contraposition.</t>
+        </is>
+      </c>
+      <c r="K576" s="9" t="n"/>
+      <c r="L576" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Logique et raisonnements »</t>
+        </is>
+      </c>
+      <c r="M576" s="11" t="n"/>
+      <c r="N576" s="11" t="n"/>
+    </row>
+    <row r="577">
+      <c r="A577" s="9" t="inlineStr">
+        <is>
+          <t>M577</t>
+        </is>
+      </c>
+      <c r="B577" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C577" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D577" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 1 – Logique, ensembles</t>
+        </is>
+      </c>
+      <c r="E577" s="9" t="inlineStr">
+        <is>
+          <t>Théorème</t>
+        </is>
+      </c>
+      <c r="F577" s="9" t="inlineStr">
+        <is>
+          <t>Raisonnement par récurrence simple</t>
+        </is>
+      </c>
+      <c r="G577" s="9" t="inlineStr">
+        <is>
+          <t>Soient $n_0\in\mathbb N$ et $\mathcal P(n)$ une assertion définie pour $n\ge n_0$.</t>
+        </is>
+      </c>
+      <c r="H577" s="10" t="inlineStr">
+        <is>
+          <t>Énoncer le principe de récurrence (initialisation, hérédité).</t>
+        </is>
+      </c>
+      <c r="I577" s="9" t="inlineStr">
+        <is>
+          <t>Si $\mathcal P(n_0)$ est vraie (initialisation) et si, pour tout $n\ge n_0$, $\mathcal P(n)\Rightarrow\mathcal P(n+1)$ (hérédité), alors $\mathcal P(n)$ est vraie pour tout $n\ge n_0$.</t>
+        </is>
+      </c>
+      <c r="J577" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 1 : « Raisonnement par récurrence. »</t>
+        </is>
+      </c>
+      <c r="K577" s="9" t="n"/>
+      <c r="L577" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Logique et raisonnements »</t>
+        </is>
+      </c>
+      <c r="M577" s="11" t="n"/>
+      <c r="N577" s="11" t="n"/>
+    </row>
+    <row r="578">
+      <c r="A578" s="9" t="inlineStr">
+        <is>
+          <t>M578</t>
+        </is>
+      </c>
+      <c r="B578" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C578" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D578" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 1 – Logique, ensembles</t>
+        </is>
+      </c>
+      <c r="E578" s="9" t="inlineStr">
+        <is>
+          <t>Théorème</t>
+        </is>
+      </c>
+      <c r="F578" s="9" t="inlineStr">
+        <is>
+          <t>Récurrence double et récurrence forte</t>
+        </is>
+      </c>
+      <c r="G578" s="9" t="inlineStr">
+        <is>
+          <t>Soient $n_0\in\mathbb N$ et $\mathcal P(n)$ une assertion définie pour $n\ge n_0$.</t>
+        </is>
+      </c>
+      <c r="H578" s="10" t="inlineStr">
+        <is>
+          <t>Énoncer le principe de récurrence double, puis celui de récurrence forte.</t>
+        </is>
+      </c>
+      <c r="I578" s="9" t="inlineStr">
+        <is>
+          <t>Double : si $\mathcal P(n_0)$ et $\mathcal P(n_0+1)$ sont vraies et si, pour tout $n\ge n_0$, $(\mathcal P(n)\text{ et }\mathcal P(n+1))\Rightarrow\mathcal P(n+2)$, alors $\mathcal P(n)$ est vraie pour tout $n\ge n_0$. Forte : si $\mathcal P(n_0)$ est vraie et si, pour tout $n\ge n_0$, $(\mathcal P(n_0),\dots,\mathcal P(n))\Rightarrow\mathcal P(n+1)$, même conclusion.</t>
+        </is>
+      </c>
+      <c r="J578" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 1 : « Lorsqu'un raisonnement par récurrence nécessite une hypothèse dite « forte », la formulation de cette hypothèse devra être proposée. »</t>
+        </is>
+      </c>
+      <c r="K578" s="9" t="n"/>
+      <c r="L578" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Logique et raisonnements »</t>
+        </is>
+      </c>
+      <c r="M578" s="11" t="n"/>
+      <c r="N578" s="11" t="n"/>
+    </row>
+    <row r="579">
+      <c r="A579" s="9" t="inlineStr">
+        <is>
+          <t>M579</t>
+        </is>
+      </c>
+      <c r="B579" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C579" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D579" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 1 – Logique, ensembles</t>
+        </is>
+      </c>
+      <c r="E579" s="9" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+      <c r="F579" s="9" t="inlineStr">
+        <is>
+          <t>Raisonnement par analyse-synthèse</t>
+        </is>
+      </c>
+      <c r="G579" s="9" t="inlineStr">
+        <is>
+          <t>On cherche toutes les solutions d'un problème (par exemple une équation).</t>
+        </is>
+      </c>
+      <c r="H579" s="10" t="inlineStr">
+        <is>
+          <t>Décrire le raisonnement par analyse-synthèse.</t>
+        </is>
+      </c>
+      <c r="I579" s="9" t="inlineStr">
+        <is>
+          <t>Analyse : on suppose qu'une solution existe et on en déduit des conditions nécessaires, qui réduisent les candidats. Synthèse : on vérifie quels candidats sont effectivement solutions. Exemple : $\sqrt{x-3}+\sqrt x=3$.</t>
+        </is>
+      </c>
+      <c r="J579" s="9" t="inlineStr">
+        <is>
+          <t>Cours ; non cité par le programme.</t>
+        </is>
+      </c>
+      <c r="K579" s="9" t="n"/>
+      <c r="L579" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Logique et raisonnements »</t>
+        </is>
+      </c>
+      <c r="M579" s="11" t="n"/>
+      <c r="N579" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M569" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M579" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -37576,7 +38176,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$569,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$579,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -37591,7 +38191,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$569,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$579,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -37606,7 +38206,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$569,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$579,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -37633,7 +38233,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$569)</f>
+        <f>COUNTA(Fiches!$M$2:$M$579)</f>
         <v/>
       </c>
     </row>
@@ -37679,15 +38279,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A13,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A13,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A13,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A13,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A13,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A13,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -37702,15 +38302,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A14,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A14,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A14,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A14,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A14,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A14,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -37725,15 +38325,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A15,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A15,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A15,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A15,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A15,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A15,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -37748,15 +38348,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A16,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A16,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A16,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A16,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A16,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A16,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -37771,15 +38371,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A17,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A17,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A17,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A17,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A17,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A17,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -37794,15 +38394,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A18,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A18,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A18,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A18,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A18,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A18,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -37817,15 +38417,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A19,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A19,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A19,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A19,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A19,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A19,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -37840,15 +38440,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A20,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A20,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A20,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A20,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A20,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A20,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -37863,15 +38463,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A21,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A21,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A21,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A21,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A21,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A21,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -37886,15 +38486,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A22,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A22,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A22,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A22,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A22,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A22,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -37909,15 +38509,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A23,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A23,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A23,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A23,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A23,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A23,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -37932,15 +38532,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A24,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A24,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A24,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A24,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A24,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A24,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -37955,15 +38555,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A25,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A25,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A25,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A25,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A25,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A25,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -37978,15 +38578,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A26,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A26,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A26,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A26,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A26,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A26,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -38001,15 +38601,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A27,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A27,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A27,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A27,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A27,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A27,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -38024,15 +38624,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A28,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A28,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A28,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A28,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A28,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A28,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -38047,15 +38647,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A29,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A29,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A29,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A29,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A29,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A29,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -38070,15 +38670,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A30,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A30,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A30,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A30,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A30,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A30,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -38093,15 +38693,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A31,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A31,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A31,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A31,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A31,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A31,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -38116,15 +38716,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A32,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A32,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A32,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A32,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A32,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A32,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -38139,15 +38739,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A33,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A33,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A33,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A33,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A33,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A33,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -38162,15 +38762,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A34,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A34,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A34,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A34,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A34,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A34,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -38185,15 +38785,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A35,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A35,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A35,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A35,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A35,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A35,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -38208,15 +38808,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A36,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A36,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A36,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A36,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A36,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A36,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -38231,15 +38831,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A37,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A37,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A37,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A37,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A37,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A37,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -38254,15 +38854,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A38,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A38,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A38,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A38,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A38,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A38,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -38277,15 +38877,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A39,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A39,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A39,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A39,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A39,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A39,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -38300,15 +38900,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A40,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A40,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A40,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A40,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A40,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A40,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -38323,15 +38923,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A41,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A41,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A41,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A41,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A41,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A41,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -38346,15 +38946,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A42,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A42,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A42,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A42,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A42,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A42,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -38369,15 +38969,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A43,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A43,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A43,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A43,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A43,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A43,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -38392,15 +38992,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A44,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A44,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A44,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A44,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A44,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A44,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -38415,15 +39015,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A45,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A45,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A45,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A45,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A45,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A45,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -38438,15 +39038,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A46,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A46,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A46,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A46,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A46,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A46,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -38461,15 +39061,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A47,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A47,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A47,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A47,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A47,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A47,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -38484,15 +39084,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A48,Fiches!$B$2:$B$569,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A48,Fiches!$B$2:$B$579,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A48,Fiches!$B$2:$B$569,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A48,Fiches!$B$2:$B$579,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$569,$A48,Fiches!$B$2:$B$569,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$579,$A48,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Sommes et produits : intégration du cours (Σ/Π, changements d'indice, télescopage, sommes usuelles et doubles)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N579"/>
+  <dimension ref="A1:N587"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3014,7 +3014,7 @@
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>Combinaisons – Propriétés</t>
+          <t>Coefficients binomiaux – Propriétés</t>
         </is>
       </c>
       <c r="G40" s="9" t="inlineStr">
@@ -3024,17 +3024,17 @@
       </c>
       <c r="H40" s="10" t="inlineStr">
         <is>
-          <t>Donner la propriété de symétrie et la formule de Pascal pour les coefficients binomiaux.</t>
+          <t>Donner la propriété de symétrie, la formule de Pascal et la formule « sans factorielle » $k\binom nk$.</t>
         </is>
       </c>
       <c r="I40" s="9" t="inlineStr">
         <is>
-          <t>Symétrie : $\binom{n}{p}=\binom{n}{n-p}$. Formule de Pascal : $\binom{n}{p}+\binom{n}{p+1}=\binom{n+1}{p+1}$.</t>
+          <t>Symétrie : $\binom{n}{p}=\binom{n}{n-p}$. Formule de Pascal : $\binom{n}{p}+\binom{n}{p+1}=\binom{n+1}{p+1}$. Pour $k\ge1$ : $\binom nk=\dfrac nk\binom{n-1}{k-1}$, soit $k\binom nk=n\binom{n-1}{k-1}$.</t>
         </is>
       </c>
       <c r="J40" s="9" t="inlineStr">
         <is>
-          <t>« Triangle de Pascal. On met en valeur les formules (n k)=(n n−k) … (n k−1)+(n k)=(n+1 k) ».</t>
+          <t>Programme Outils 5 : « On met en valeur les formules : $\binom nk=\binom n{n-k}$, $\binom nk=\frac nk\binom{n-1}{k-1}$, $\binom n{k-1}+\binom nk=\binom{n+1}k$. »</t>
         </is>
       </c>
       <c r="K40" s="9" t="n">
@@ -34630,10 +34630,490 @@
       <c r="M579" s="11" t="n"/>
       <c r="N579" s="11" t="n"/>
     </row>
+    <row r="580">
+      <c r="A580" s="9" t="inlineStr">
+        <is>
+          <t>M580</t>
+        </is>
+      </c>
+      <c r="B580" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C580" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D580" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 5 – Méthodes de calcul</t>
+        </is>
+      </c>
+      <c r="E580" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F580" s="9" t="inlineStr">
+        <is>
+          <t>Symboles Σ et Π</t>
+        </is>
+      </c>
+      <c r="G580" s="9" t="inlineStr">
+        <is>
+          <t>Soient $n_0\le n$ deux entiers et $a_{n_0},\dots,a_n$ des nombres.</t>
+        </is>
+      </c>
+      <c r="H580" s="10" t="inlineStr">
+        <is>
+          <t>Que désignent $\sum_{k=n_0}^na_k$ et $\prod_{k=n_0}^na_k$ ? Combien de termes ? Que vaut une somme, un produit, sur un ensemble d'indices vide ?</t>
+        </is>
+      </c>
+      <c r="I580" s="9" t="inlineStr">
+        <is>
+          <t>$\sum_{k=n_0}^na_k=a_{n_0}+\dots+a_n$ et $\prod_{k=n_0}^na_k=a_{n_0}\times\dots\times a_n$ ; il y a $n-n_0+1$ termes ; $k$ est une variable muette. Une somme vide vaut $0$, un produit vide vaut $1$.</t>
+        </is>
+      </c>
+      <c r="J580" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 5 : « Notation Σ. On précise qu'une somme ayant un ensemble d'indices vide est nulle » ; « Notation Π … un produit ayant un ensemble d'indices vide vaut 1. »</t>
+        </is>
+      </c>
+      <c r="K580" s="9" t="n"/>
+      <c r="L580" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Sommes et produits »</t>
+        </is>
+      </c>
+      <c r="M580" s="11" t="n"/>
+      <c r="N580" s="11" t="n"/>
+    </row>
+    <row r="581">
+      <c r="A581" s="9" t="inlineStr">
+        <is>
+          <t>M581</t>
+        </is>
+      </c>
+      <c r="B581" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C581" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D581" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 5 – Méthodes de calcul</t>
+        </is>
+      </c>
+      <c r="E581" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F581" s="9" t="inlineStr">
+        <is>
+          <t>Règles de calcul sur Σ et Π</t>
+        </is>
+      </c>
+      <c r="G581" s="9" t="inlineStr">
+        <is>
+          <t>Soient $n_0\le p\le n$, $\lambda$ un nombre et $(a_k)$, $(b_k)$ des nombres.</t>
+        </is>
+      </c>
+      <c r="H581" s="10" t="inlineStr">
+        <is>
+          <t>Donner la linéarité de $\Sigma$, la relation de Chasles, et les règles correspondantes pour $\Pi$.</t>
+        </is>
+      </c>
+      <c r="I581" s="9" t="inlineStr">
+        <is>
+          <t>$\sum(a_k+b_k)=\sum a_k+\sum b_k$ ; $\sum\lambda a_k=\lambda\sum a_k$ ; $\sum_{k=n_0}^na_k=\sum_{k=n_0}^pa_k+\sum_{k=p+1}^na_k$. $\prod a_kb_k=\prod a_k\prod b_k$ ; $\prod_{k=n_0}^n\lambda a_k=\lambda^{n-n_0+1}\prod_{k=n_0}^na_k$ ; $\prod_{k=n_0}^na_k=\prod_{k=n_0}^pa_k\times\prod_{k=p+1}^na_k$.</t>
+        </is>
+      </c>
+      <c r="J581" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 5 : « Règles de calcul sur le symbole Σ : linéarité » ; « on se contente de mettre en valeur la multiplicativité du symbole Π. »</t>
+        </is>
+      </c>
+      <c r="K581" s="9" t="n"/>
+      <c r="L581" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Sommes et produits »</t>
+        </is>
+      </c>
+      <c r="M581" s="11" t="n"/>
+      <c r="N581" s="11" t="n"/>
+    </row>
+    <row r="582">
+      <c r="A582" s="9" t="inlineStr">
+        <is>
+          <t>M582</t>
+        </is>
+      </c>
+      <c r="B582" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C582" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D582" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 5 – Méthodes de calcul</t>
+        </is>
+      </c>
+      <c r="E582" s="9" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+      <c r="F582" s="9" t="inlineStr">
+        <is>
+          <t>Changements d’indice</t>
+        </is>
+      </c>
+      <c r="G582" s="9" t="inlineStr">
+        <is>
+          <t>Soient $n_0\le n$, $p\in\mathbb Z$ et $(a_k)$ des nombres.</t>
+        </is>
+      </c>
+      <c r="H582" s="10" t="inlineStr">
+        <is>
+          <t>Effectuer dans $\sum_{k=n_0}^na_k$ une translation $j=k+p$, puis une symétrie $j=n-k$ (pour $n_0=0$).</t>
+        </is>
+      </c>
+      <c r="I582" s="9" t="inlineStr">
+        <is>
+          <t>Translation : $\sum_{k=n_0}^na_k=\sum_{j=n_0+p}^{n+p}a_{j-p}$. Symétrie : $\sum_{k=0}^na_{n-k}=\sum_{j=0}^na_j$. On transforme les bornes en même temps que l'indice.</t>
+        </is>
+      </c>
+      <c r="J582" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 5 : « changements d'indices (translations et symétries) ».</t>
+        </is>
+      </c>
+      <c r="K582" s="9" t="n"/>
+      <c r="L582" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Sommes et produits »</t>
+        </is>
+      </c>
+      <c r="M582" s="11" t="n"/>
+      <c r="N582" s="11" t="n"/>
+    </row>
+    <row r="583">
+      <c r="A583" s="9" t="inlineStr">
+        <is>
+          <t>M583</t>
+        </is>
+      </c>
+      <c r="B583" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C583" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D583" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 5 – Méthodes de calcul</t>
+        </is>
+      </c>
+      <c r="E583" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F583" s="9" t="inlineStr">
+        <is>
+          <t>Télescopage</t>
+        </is>
+      </c>
+      <c r="G583" s="9" t="inlineStr">
+        <is>
+          <t>Soient $n_0\le n$ et $(a_k)$ des nombres (non nuls pour le produit).</t>
+        </is>
+      </c>
+      <c r="H583" s="10" t="inlineStr">
+        <is>
+          <t>Que valent $\sum_{k=n_0}^n(a_{k+1}-a_k)$ et $\prod_{k=n_0}^n\dfrac{a_{k+1}}{a_k}$ ?</t>
+        </is>
+      </c>
+      <c r="I583" s="9" t="inlineStr">
+        <is>
+          <t>$\sum_{k=n_0}^n(a_{k+1}-a_k)=a_{n+1}-a_{n_0}$ et $\prod_{k=n_0}^n\dfrac{a_{k+1}}{a_k}=\dfrac{a_{n+1}}{a_{n_0}}$. Exemple : $\sum_{k=1}^n\frac1{k(k+1)}=\sum_{k=1}^n\left(\frac1k-\frac1{k+1}\right)=1-\frac1{n+1}$.</t>
+        </is>
+      </c>
+      <c r="J583" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 5 : « télescopages ».</t>
+        </is>
+      </c>
+      <c r="K583" s="9" t="n"/>
+      <c r="L583" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Sommes et produits »</t>
+        </is>
+      </c>
+      <c r="M583" s="11" t="n"/>
+      <c r="N583" s="11" t="n"/>
+    </row>
+    <row r="584">
+      <c r="A584" s="9" t="inlineStr">
+        <is>
+          <t>M584</t>
+        </is>
+      </c>
+      <c r="B584" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C584" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D584" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 5 – Méthodes de calcul</t>
+        </is>
+      </c>
+      <c r="E584" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F584" s="9" t="inlineStr">
+        <is>
+          <t>Somme des n premiers carrés</t>
+        </is>
+      </c>
+      <c r="G584" s="9" t="inlineStr">
+        <is>
+          <t>Soit $n\in\mathbb N$.</t>
+        </is>
+      </c>
+      <c r="H584" s="10" t="inlineStr">
+        <is>
+          <t>Calculer $\sum_{k=1}^nk^2$.</t>
+        </is>
+      </c>
+      <c r="I584" s="9" t="inlineStr">
+        <is>
+          <t>$\sum_{k=1}^nk^2=\dfrac{n(n+1)(2n+1)}6$.</t>
+        </is>
+      </c>
+      <c r="J584" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 5 : « Sommes des n premiers entiers et des n premiers carrés. »</t>
+        </is>
+      </c>
+      <c r="K584" s="9" t="n"/>
+      <c r="L584" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Sommes et produits »</t>
+        </is>
+      </c>
+      <c r="M584" s="11" t="n"/>
+      <c r="N584" s="11" t="n"/>
+    </row>
+    <row r="585">
+      <c r="A585" s="9" t="inlineStr">
+        <is>
+          <t>M585</t>
+        </is>
+      </c>
+      <c r="B585" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C585" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D585" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 5 – Méthodes de calcul</t>
+        </is>
+      </c>
+      <c r="E585" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F585" s="9" t="inlineStr">
+        <is>
+          <t>Somme des n premiers cubes</t>
+        </is>
+      </c>
+      <c r="G585" s="9" t="inlineStr">
+        <is>
+          <t>Soit $n\in\mathbb N$.</t>
+        </is>
+      </c>
+      <c r="H585" s="10" t="inlineStr">
+        <is>
+          <t>Calculer $\sum_{k=1}^nk^3$.</t>
+        </is>
+      </c>
+      <c r="I585" s="9" t="inlineStr">
+        <is>
+          <t>$\sum_{k=1}^nk^3=\left(\dfrac{n(n+1)}2\right)^2$ (le carré de la somme des $n$ premiers entiers).</t>
+        </is>
+      </c>
+      <c r="J585" s="9" t="inlineStr">
+        <is>
+          <t>Cours (« à connaître par cœur ») ; le programme ne cite que les entiers et les carrés.</t>
+        </is>
+      </c>
+      <c r="K585" s="9" t="n"/>
+      <c r="L585" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Sommes et produits »</t>
+        </is>
+      </c>
+      <c r="M585" s="11" t="n"/>
+      <c r="N585" s="11" t="n"/>
+    </row>
+    <row r="586">
+      <c r="A586" s="9" t="inlineStr">
+        <is>
+          <t>M586</t>
+        </is>
+      </c>
+      <c r="B586" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C586" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D586" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 5 – Méthodes de calcul</t>
+        </is>
+      </c>
+      <c r="E586" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F586" s="9" t="inlineStr">
+        <is>
+          <t>Somme géométrique</t>
+        </is>
+      </c>
+      <c r="G586" s="9" t="inlineStr">
+        <is>
+          <t>Soient $q\in\mathbb C\setminus\{1\}$ et $n_0\le n$.</t>
+        </is>
+      </c>
+      <c r="H586" s="10" t="inlineStr">
+        <is>
+          <t>Calculer $\sum_{k=0}^nq^k$, puis la somme des termes $u_{n_0},\dots,u_n$ d'une suite géométrique de raison $q$.</t>
+        </is>
+      </c>
+      <c r="I586" s="9" t="inlineStr">
+        <is>
+          <t>$\sum_{k=0}^nq^k=\dfrac{q^{n+1}-1}{q-1}=\dfrac{1-q^{n+1}}{1-q}$ ; $\sum_{k=n_0}^nu_k=u_{n_0}\dfrac{1-q^{n-n_0+1}}{1-q}$ (premier terme × $\frac{1-q^{\text{nombre de termes}}}{1-q}$). Si $q=1$, la somme vaut $n+1$.</t>
+        </is>
+      </c>
+      <c r="J586" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 5 : « Somme de termes consécutifs d'une progression géométrique … La raison q est dans ℂ ∖ {1}. »</t>
+        </is>
+      </c>
+      <c r="K586" s="9" t="n"/>
+      <c r="L586" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Sommes et produits »</t>
+        </is>
+      </c>
+      <c r="M586" s="11" t="n"/>
+      <c r="N586" s="11" t="n"/>
+    </row>
+    <row r="587">
+      <c r="A587" s="9" t="inlineStr">
+        <is>
+          <t>M587</t>
+        </is>
+      </c>
+      <c r="B587" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C587" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D587" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 5 – Méthodes de calcul</t>
+        </is>
+      </c>
+      <c r="E587" s="9" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+      <c r="F587" s="9" t="inlineStr">
+        <is>
+          <t>Sommes doubles</t>
+        </is>
+      </c>
+      <c r="G587" s="9" t="inlineStr">
+        <is>
+          <t>Soient $n,m\in\mathbb N^*$ et $(a_{i,j})$ des nombres.</t>
+        </is>
+      </c>
+      <c r="H587" s="10" t="inlineStr">
+        <is>
+          <t>Écrire $\sum_{1\le i\le n,\,1\le j\le m}a_{i,j}$ et $\sum_{1\le i\le j\le n}a_{i,j}$ comme deux sommes simples successives.</t>
+        </is>
+      </c>
+      <c r="I587" s="9" t="inlineStr">
+        <is>
+          <t>$\sum_{\substack{1\le i\le n\\1\le j\le m}}a_{i,j}=\sum_{i=1}^n\sum_{j=1}^ma_{i,j}=\sum_{j=1}^m\sum_{i=1}^na_{i,j}$ ; $\sum_{1\le i\le j\le n}a_{i,j}=\sum_{i=1}^n\sum_{j=i}^na_{i,j}=\sum_{j=1}^n\sum_{i=1}^ja_{i,j}$.</t>
+        </is>
+      </c>
+      <c r="J587" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 5 : « Sommes doubles … mettre sous la forme de deux sommes simples successives. »</t>
+        </is>
+      </c>
+      <c r="K587" s="9" t="n"/>
+      <c r="L587" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Sommes et produits »</t>
+        </is>
+      </c>
+      <c r="M587" s="11" t="n"/>
+      <c r="N587" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M579" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M587" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -38176,7 +38656,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$579,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$587,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -38191,7 +38671,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$579,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$587,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -38206,7 +38686,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$579,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$587,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -38233,7 +38713,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$579)</f>
+        <f>COUNTA(Fiches!$M$2:$M$587)</f>
         <v/>
       </c>
     </row>
@@ -38279,15 +38759,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A13,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A13,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A13,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A13,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A13,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A13,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -38302,15 +38782,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A14,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A14,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A14,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A14,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A14,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A14,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -38325,15 +38805,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A15,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A15,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A15,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A15,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A15,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A15,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -38348,15 +38828,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A16,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A16,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A16,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A16,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A16,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A16,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -38371,15 +38851,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A17,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A17,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A17,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A17,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A17,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A17,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -38394,15 +38874,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A18,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A18,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A18,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A18,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A18,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A18,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -38417,15 +38897,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A19,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A19,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A19,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A19,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A19,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A19,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -38440,15 +38920,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A20,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A20,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A20,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A20,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A20,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A20,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -38463,15 +38943,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A21,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A21,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A21,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A21,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A21,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A21,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -38486,15 +38966,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A22,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A22,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A22,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A22,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A22,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A22,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -38509,15 +38989,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A23,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A23,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A23,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A23,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A23,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A23,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -38532,15 +39012,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A24,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A24,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A24,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A24,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A24,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A24,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -38555,15 +39035,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A25,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A25,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A25,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A25,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A25,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A25,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -38578,15 +39058,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A26,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A26,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A26,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A26,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A26,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A26,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -38601,15 +39081,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A27,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A27,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A27,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A27,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A27,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A27,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -38624,15 +39104,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A28,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A28,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A28,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A28,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A28,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A28,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -38647,15 +39127,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A29,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A29,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A29,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A29,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A29,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A29,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -38670,15 +39150,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A30,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A30,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A30,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A30,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A30,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A30,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -38693,15 +39173,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A31,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A31,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A31,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A31,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A31,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A31,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -38716,15 +39196,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A32,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A32,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A32,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A32,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A32,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A32,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -38739,15 +39219,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A33,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A33,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A33,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A33,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A33,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A33,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -38762,15 +39242,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A34,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A34,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A34,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A34,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A34,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A34,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -38785,15 +39265,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A35,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A35,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A35,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A35,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A35,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A35,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -38808,15 +39288,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A36,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A36,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A36,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A36,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A36,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A36,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -38831,15 +39311,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A37,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A37,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A37,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A37,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A37,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A37,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -38854,15 +39334,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A38,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A38,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A38,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A38,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A38,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A38,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -38877,15 +39357,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A39,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A39,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A39,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A39,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A39,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A39,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -38900,15 +39380,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A40,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A40,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A40,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A40,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A40,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A40,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -38923,15 +39403,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A41,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A41,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A41,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A41,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A41,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A41,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -38946,15 +39426,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A42,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A42,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A42,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A42,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A42,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A42,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -38969,15 +39449,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A43,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A43,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A43,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A43,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A43,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A43,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -38992,15 +39472,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A44,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A44,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A44,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A44,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A44,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A44,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -39015,15 +39495,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A45,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A45,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A45,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A45,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A45,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A45,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -39038,15 +39518,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A46,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A46,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A46,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A46,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A46,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A46,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -39061,15 +39541,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A47,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A47,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A47,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A47,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A47,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A47,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -39084,15 +39564,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A48,Fiches!$B$2:$B$579,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A48,Fiches!$B$2:$B$587,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A48,Fiches!$B$2:$B$579,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A48,Fiches!$B$2:$B$587,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$579,$A48,Fiches!$B$2:$B$579,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$587,$A48,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Suites récurrentes : arithmético-géométriques et récurrentes linéaires d'ordre 2
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N587"/>
+  <dimension ref="A1:N589"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -35110,10 +35110,130 @@
       <c r="M587" s="11" t="n"/>
       <c r="N587" s="11" t="n"/>
     </row>
+    <row r="588">
+      <c r="A588" s="9" t="inlineStr">
+        <is>
+          <t>M588</t>
+        </is>
+      </c>
+      <c r="B588" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C588" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D588" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 1 – Suites réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E588" s="9" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+      <c r="F588" s="9" t="inlineStr">
+        <is>
+          <t>Suites arithmético-géométriques</t>
+        </is>
+      </c>
+      <c r="G588" s="9" t="inlineStr">
+        <is>
+          <t>Soient $(a,b)\in\mathbb R^2$ et $(u_n)$ telle que $u_{n+1}=au_n+b$ pour tout $n$.</t>
+        </is>
+      </c>
+      <c r="H588" s="10" t="inlineStr">
+        <is>
+          <t>Comment obtenir l'expression de $u_n$ en fonction de $n$ ?</t>
+        </is>
+      </c>
+      <c r="I588" s="9" t="inlineStr">
+        <is>
+          <t>Si $a=1$, $(u_n)$ est arithmétique de raison $b$. Si $a\neq1$ : on cherche la suite constante solution, $L=aL+b$ (soit $L=\frac b{1-a}$) ; alors $v_n=u_n-L$ vérifie $v_{n+1}=av_n$, elle est géométrique de raison $a$ ; donc $u_n=L+a^n(u_0-L)$.</t>
+        </is>
+      </c>
+      <c r="J588" s="9" t="inlineStr">
+        <is>
+          <t>Programme Analyse 1 : « La formule donnant le terme général n'est pas au programme. On cherchera une suite constante solution pour déterminer toutes les solutions. »</t>
+        </is>
+      </c>
+      <c r="K588" s="9" t="n"/>
+      <c r="L588" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Suites récurrentes classiques »</t>
+        </is>
+      </c>
+      <c r="M588" s="11" t="n"/>
+      <c r="N588" s="11" t="n"/>
+    </row>
+    <row r="589">
+      <c r="A589" s="9" t="inlineStr">
+        <is>
+          <t>M589</t>
+        </is>
+      </c>
+      <c r="B589" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C589" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D589" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 1 – Suites réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E589" s="9" t="inlineStr">
+        <is>
+          <t>Théorème</t>
+        </is>
+      </c>
+      <c r="F589" s="9" t="inlineStr">
+        <is>
+          <t>Suites récurrentes linéaires d’ordre 2</t>
+        </is>
+      </c>
+      <c r="G589" s="9" t="inlineStr">
+        <is>
+          <t>Soient $a\in\mathbb R$, $b\in\mathbb R^*$ et $(u_n)$ réelle telle que $u_{n+2}=au_{n+1}+bu_n$ pour tout $n$.</t>
+        </is>
+      </c>
+      <c r="H589" s="10" t="inlineStr">
+        <is>
+          <t>Quelle est l'équation caractéristique ? Donner la forme de $u_n$ selon le signe de son discriminant $\Delta$.</t>
+        </is>
+      </c>
+      <c r="I589" s="9" t="inlineStr">
+        <is>
+          <t>Équation caractéristique : $x^2=ax+b$. Si $\Delta&gt;0$ (racines réelles $x_1\neq x_2$) : $u_n=\alpha x_1^n+\beta x_2^n$. Si $\Delta=0$ (racine double $x_0$) : $u_n=(\alpha n+\beta)x_0^n$. Si $\Delta&lt;0$ (racines $re^{\pm i\theta}$, $r&gt;0$) : $u_n=r^n(\alpha\cos n\theta+\beta\sin n\theta)$. Les réels $\alpha,\beta$ sont uniques, fixés par $u_0$ et $u_1$.</t>
+        </is>
+      </c>
+      <c r="J589" s="9" t="inlineStr">
+        <is>
+          <t>Programme Analyse 1 : « Suites vérifiant une relation du type $u_{n+2}=au_{n+1}+bu_n$. On se limite à la maitrise d'une méthode de calcul du n-ième terme à partir de l'équation caractéristique. Au besoin, on transite par ℂ. »</t>
+        </is>
+      </c>
+      <c r="K589" s="9" t="n"/>
+      <c r="L589" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Suites récurrentes classiques »</t>
+        </is>
+      </c>
+      <c r="M589" s="11" t="n"/>
+      <c r="N589" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M587" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M589" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -38656,7 +38776,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$587,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$589,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -38671,7 +38791,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$587,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$589,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -38686,7 +38806,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$587,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$589,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -38713,7 +38833,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$587)</f>
+        <f>COUNTA(Fiches!$M$2:$M$589)</f>
         <v/>
       </c>
     </row>
@@ -38759,15 +38879,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A13,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A13,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A13,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A13,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A13,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A13,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -38782,15 +38902,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A14,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A14,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A14,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A14,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A14,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A14,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -38805,15 +38925,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A15,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A15,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A15,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A15,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A15,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A15,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -38828,15 +38948,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A16,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A16,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A16,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A16,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A16,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A16,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -38851,15 +38971,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A17,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A17,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A17,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A17,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A17,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A17,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -38874,15 +38994,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A18,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A18,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A18,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A18,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A18,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A18,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -38897,15 +39017,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A19,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A19,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A19,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A19,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A19,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A19,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -38920,15 +39040,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A20,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A20,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A20,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A20,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A20,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A20,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -38943,15 +39063,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A21,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A21,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A21,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A21,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A21,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A21,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -38966,15 +39086,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A22,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A22,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A22,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A22,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A22,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A22,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -38989,15 +39109,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A23,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A23,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A23,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A23,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A23,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A23,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -39012,15 +39132,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A24,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A24,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A24,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A24,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A24,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A24,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -39035,15 +39155,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A25,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A25,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A25,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A25,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A25,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A25,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -39058,15 +39178,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A26,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A26,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A26,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A26,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A26,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A26,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -39081,15 +39201,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A27,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A27,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A27,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A27,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A27,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A27,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -39104,15 +39224,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A28,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A28,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A28,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A28,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A28,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A28,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -39127,15 +39247,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A29,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A29,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A29,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A29,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A29,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A29,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -39150,15 +39270,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A30,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A30,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A30,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A30,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A30,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A30,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -39173,15 +39293,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A31,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A31,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A31,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A31,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A31,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A31,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -39196,15 +39316,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A32,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A32,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A32,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A32,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A32,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A32,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -39219,15 +39339,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A33,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A33,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A33,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A33,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A33,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A33,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -39242,15 +39362,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A34,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A34,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A34,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A34,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A34,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A34,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -39265,15 +39385,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A35,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A35,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A35,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A35,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A35,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A35,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -39288,15 +39408,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A36,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A36,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A36,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A36,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A36,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A36,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -39311,15 +39431,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A37,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A37,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A37,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A37,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A37,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A37,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -39334,15 +39454,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A38,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A38,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A38,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A38,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A38,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A38,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -39357,15 +39477,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A39,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A39,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A39,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A39,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A39,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A39,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -39380,15 +39500,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A40,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A40,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A40,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A40,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A40,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A40,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -39403,15 +39523,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A41,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A41,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A41,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A41,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A41,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A41,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -39426,15 +39546,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A42,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A42,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A42,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A42,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A42,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A42,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -39449,15 +39569,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A43,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A43,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A43,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A43,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A43,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A43,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -39472,15 +39592,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A44,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A44,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A44,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A44,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A44,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A44,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -39495,15 +39615,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A45,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A45,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A45,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A45,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A45,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A45,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -39518,15 +39638,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A46,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A46,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A46,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A46,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A46,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A46,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -39541,15 +39661,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A47,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A47,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A47,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A47,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A47,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A47,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -39564,15 +39684,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A48,Fiches!$B$2:$B$587,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A48,Fiches!$B$2:$B$589,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A48,Fiches!$B$2:$B$587,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A48,Fiches!$B$2:$B$589,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$587,$A48,Fiches!$B$2:$B$587,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$589,$A48,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Applications linéaires : intégration du cours (opérations, Y=AX, rang, matrice canonique)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N589"/>
+  <dimension ref="A1:N592"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -20645,7 +20645,7 @@
       </c>
       <c r="I344" s="9" t="inlineStr">
         <is>
-          <t>$\forall(x,y)\in E^2,\ \forall\lambda\in\mathbb K,\ f(x+\lambda y)=f(x)+\lambda f(y)$. Ensemble noté $\mathcal L(E,F)$.</t>
+          <t>$\forall(x,y)\in E^2,\ \forall\lambda\in\mathbb K,\ f(x+\lambda y)=f(x)+\lambda f(y)$ (de façon équivalente, $f$ conserve les combinaisons linéaires : $f(\alpha x+\beta y)=\alpha f(x)+\beta f(y)$). Alors $f(0_E)=0_F$. Ensemble noté $\mathcal L(E,F)$.</t>
         </is>
       </c>
       <c r="J344" s="9" t="inlineStr">
@@ -20881,7 +20881,7 @@
       </c>
       <c r="I348" s="9" t="inlineStr">
         <is>
-          <t>$\mathrm{rg}f=\dim\mathrm{Im}f$.</t>
+          <t>$\mathrm{rg}f=\dim\mathrm{Im}f$. Si $(e_1,\dots,e_p)$ est une base de $E$ : $\mathrm{Im}f=\mathrm{Vect}(f(e_1),\dots,f(e_p))$, donc $\mathrm{rg}f=\mathrm{rg}(f(e_1),\dots,f(e_p))=\mathrm{rg}(\mathrm{Mat}f)$ (dans n'importe quelles bases).</t>
         </is>
       </c>
       <c r="J348" s="9" t="inlineStr">
@@ -21469,7 +21469,7 @@
       </c>
       <c r="I358" s="9" t="inlineStr">
         <is>
-          <t>Dans des bases fixées : $\mathrm{Mat}(\lambda f+g)=\lambda\mathrm{Mat}f+\mathrm{Mat}g$ ; $\mathrm{Mat}(g\circ f)=\mathrm{Mat}(g)\mathrm{Mat}(f)$ ; $f$ isomorphisme $\iff\mathrm{Mat}f$ inversible, et $\mathrm{Mat}(f^{-1})=(\mathrm{Mat}f)^{-1}$.</t>
+          <t>Dans des bases fixées : $\mathrm{Mat}(\lambda f+g)=\lambda\mathrm{Mat}f+\mathrm{Mat}g$ ; $\mathrm{Mat}(g\circ f)=\mathrm{Mat}(g)\mathrm{Mat}(f)$, d'où $\mathrm{Mat}(f^k)=(\mathrm{Mat}f)^k$ ; $f$ isomorphisme $\iff\mathrm{Mat}f$ inversible, et $\mathrm{Mat}(f^{-1})=(\mathrm{Mat}f)^{-1}$.</t>
         </is>
       </c>
       <c r="J358" s="9" t="inlineStr">
@@ -35230,10 +35230,190 @@
       <c r="M589" s="11" t="n"/>
       <c r="N589" s="11" t="n"/>
     </row>
+    <row r="590">
+      <c r="A590" s="9" t="inlineStr">
+        <is>
+          <t>M590</t>
+        </is>
+      </c>
+      <c r="B590" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C590" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2</t>
+        </is>
+      </c>
+      <c r="D590" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2 · Algèbre linéaire 2 – Applications linéaires et matrices</t>
+        </is>
+      </c>
+      <c r="E590" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F590" s="9" t="inlineStr">
+        <is>
+          <t>Propriétés des opérations sur les applications linéaires</t>
+        </is>
+      </c>
+      <c r="G590" s="9" t="inlineStr">
+        <is>
+          <t>Soient $f$, $g$, $h$ des applications linéaires (composables) et $\lambda\in\mathbb K$.</t>
+        </is>
+      </c>
+      <c r="H590" s="10" t="inlineStr">
+        <is>
+          <t>Comment la composition se comporte-t-elle avec la somme et le produit par un scalaire ? Est-elle commutative ?</t>
+        </is>
+      </c>
+      <c r="I590" s="9" t="inlineStr">
+        <is>
+          <t>$f\circ(g+h)=f\circ g+f\circ h$ ; $(f+g)\circ h=f\circ h+g\circ h$ ; $(\lambda f)\circ g=f\circ(\lambda g)=\lambda(f\circ g)$. La composition est associative mais pas commutative en général. Pour $f\in\mathcal L(E)$ : $f^0=\mathrm{id}_E$, $f^{n+1}=f\circ f^n$.</t>
+        </is>
+      </c>
+      <c r="J590" s="9" t="inlineStr">
+        <is>
+          <t>Programme : « Opérations sur les applications linéaires : addition, multiplication par un scalaire, composition, réciproque. Propriétés de ces opérations. » ; BCPST2 : « Notation $f^n$ ».</t>
+        </is>
+      </c>
+      <c r="K590" s="9" t="n"/>
+      <c r="L590" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Applications linéaires »</t>
+        </is>
+      </c>
+      <c r="M590" s="11" t="n"/>
+      <c r="N590" s="11" t="n"/>
+    </row>
+    <row r="591">
+      <c r="A591" s="9" t="inlineStr">
+        <is>
+          <t>M591</t>
+        </is>
+      </c>
+      <c r="B591" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C591" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2</t>
+        </is>
+      </c>
+      <c r="D591" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2 · Algèbre linéaire 2 – Applications linéaires et matrices</t>
+        </is>
+      </c>
+      <c r="E591" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F591" s="9" t="inlineStr">
+        <is>
+          <t>Image d’un vecteur : Y = AX</t>
+        </is>
+      </c>
+      <c r="G591" s="9" t="inlineStr">
+        <is>
+          <t>Soient $f\in\mathcal L(E,F)$, $\mathcal B$ et $\mathcal C$ des bases de $E$ et $F$, $A=\mathrm{Mat}_{\mathcal B,\mathcal C}(f)$ et $u\in E$.</t>
+        </is>
+      </c>
+      <c r="H591" s="10" t="inlineStr">
+        <is>
+          <t>Comment calculer les coordonnées de $f(u)$ à l'aide de $A$ ?</t>
+        </is>
+      </c>
+      <c r="I591" s="9" t="inlineStr">
+        <is>
+          <t>Si $X=\mathrm{Mat}_{\mathcal B}(u)$ et $Y=\mathrm{Mat}_{\mathcal C}(f(u))$, alors $Y=AX$, i.e. $\mathrm{Mat}_{\mathcal C}(f(u))=\mathrm{Mat}_{\mathcal B,\mathcal C}(f)\times\mathrm{Mat}_{\mathcal B}(u)$ : $y_i=\sum_{k=1}^pa_{ik}x_k$.</t>
+        </is>
+      </c>
+      <c r="J591" s="9" t="inlineStr">
+        <is>
+          <t>Programme : « Matrice d'une application linéaire dans des bases » ; lien noyau/image d'une matrice et de l'application qu'elle représente.</t>
+        </is>
+      </c>
+      <c r="K591" s="9" t="n"/>
+      <c r="L591" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Applications linéaires »</t>
+        </is>
+      </c>
+      <c r="M591" s="11" t="n"/>
+      <c r="N591" s="11" t="n"/>
+    </row>
+    <row r="592">
+      <c r="A592" s="9" t="inlineStr">
+        <is>
+          <t>M592</t>
+        </is>
+      </c>
+      <c r="B592" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C592" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2</t>
+        </is>
+      </c>
+      <c r="D592" s="9" t="inlineStr">
+        <is>
+          <t>BCPST2 · Algèbre linéaire 2 – Applications linéaires et matrices</t>
+        </is>
+      </c>
+      <c r="E592" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F592" s="9" t="inlineStr">
+        <is>
+          <t>Application linéaire canoniquement associée à une matrice</t>
+        </is>
+      </c>
+      <c r="G592" s="9" t="inlineStr">
+        <is>
+          <t>Soient $n,p\in\mathbb N^*$ et $A\in\mathcal M_{n,p}(\mathbb K)$.</t>
+        </is>
+      </c>
+      <c r="H592" s="10" t="inlineStr">
+        <is>
+          <t>Quelle application linéaire $A$ représente-t-elle dans les bases canoniques ? Quelle correspondance obtient-on ?</t>
+        </is>
+      </c>
+      <c r="I592" s="9" t="inlineStr">
+        <is>
+          <t>$f_A:\mathbb K^p\to\mathbb K^n$, l'unique application linéaire qui envoie le $j$-ème vecteur de la base canonique sur le vecteur dont les coordonnées forment la $j$-ème colonne $C_j$ de $A$ : $f_A(x_1,\dots,x_p)=\sum_jx_jC_j$. L'application $f\mapsto\mathrm{Mat}_{\mathrm{can}}(f)$ est une bijection de $\mathcal L(\mathbb K^p,\mathbb K^n)$ sur $\mathcal M_{n,p}(\mathbb K)$.</t>
+        </is>
+      </c>
+      <c r="J592" s="9" t="inlineStr">
+        <is>
+          <t>Cours ; le programme de 2ᵉ année demande d'éviter d'identifier un vecteur à sa matrice colonne.</t>
+        </is>
+      </c>
+      <c r="K592" s="9" t="n"/>
+      <c r="L592" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Applications linéaires »</t>
+        </is>
+      </c>
+      <c r="M592" s="11" t="n"/>
+      <c r="N592" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M589" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M592" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -38776,7 +38956,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$589,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$592,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -38791,7 +38971,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$589,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$592,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -38806,7 +38986,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$589,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$592,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -38833,7 +39013,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$589)</f>
+        <f>COUNTA(Fiches!$M$2:$M$592)</f>
         <v/>
       </c>
     </row>
@@ -38879,15 +39059,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A13,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A13,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A13,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A13,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A13,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A13,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -38902,15 +39082,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A14,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A14,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A14,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A14,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A14,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A14,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -38925,15 +39105,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A15,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A15,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A15,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A15,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A15,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A15,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -38948,15 +39128,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A16,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A16,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A16,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A16,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A16,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A16,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -38971,15 +39151,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A17,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A17,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A17,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A17,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A17,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A17,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -38994,15 +39174,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A18,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A18,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A18,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A18,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A18,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A18,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -39017,15 +39197,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A19,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A19,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A19,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A19,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A19,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A19,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -39040,15 +39220,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A20,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A20,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A20,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A20,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A20,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A20,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -39063,15 +39243,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A21,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A21,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A21,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A21,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A21,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A21,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -39086,15 +39266,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A22,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A22,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A22,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A22,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A22,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A22,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -39109,15 +39289,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A23,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A23,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A23,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A23,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A23,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A23,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -39132,15 +39312,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A24,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A24,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A24,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A24,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A24,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A24,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -39155,15 +39335,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A25,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A25,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A25,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A25,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A25,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A25,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -39178,15 +39358,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A26,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A26,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A26,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A26,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A26,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A26,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -39201,15 +39381,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A27,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A27,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A27,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A27,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A27,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A27,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -39224,15 +39404,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A28,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A28,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A28,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A28,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A28,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A28,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -39247,15 +39427,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A29,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A29,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A29,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A29,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A29,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A29,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -39270,15 +39450,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A30,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A30,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A30,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A30,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A30,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A30,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -39293,15 +39473,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A31,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A31,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A31,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A31,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A31,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A31,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -39316,15 +39496,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A32,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A32,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A32,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A32,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A32,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A32,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -39339,15 +39519,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A33,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A33,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A33,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A33,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A33,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A33,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -39362,15 +39542,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A34,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A34,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A34,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A34,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A34,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A34,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -39385,15 +39565,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A35,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A35,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A35,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A35,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A35,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A35,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -39408,15 +39588,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A36,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A36,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A36,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A36,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A36,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A36,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -39431,15 +39611,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A37,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A37,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A37,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A37,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A37,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A37,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -39454,15 +39634,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A38,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A38,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A38,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A38,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A38,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A38,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -39477,15 +39657,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A39,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A39,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A39,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A39,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A39,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A39,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -39500,15 +39680,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A40,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A40,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A40,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A40,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A40,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A40,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -39523,15 +39703,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A41,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A41,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A41,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A41,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A41,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A41,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -39546,15 +39726,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A42,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A42,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A42,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A42,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A42,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A42,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -39569,15 +39749,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A43,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A43,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A43,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A43,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A43,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A43,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -39592,15 +39772,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A44,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A44,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A44,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A44,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A44,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A44,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -39615,15 +39795,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A45,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A45,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A45,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A45,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A45,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A45,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -39638,15 +39818,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A46,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A46,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A46,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A46,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A46,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A46,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -39661,15 +39841,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A47,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A47,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A47,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A47,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A47,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A47,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -39684,15 +39864,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A48,Fiches!$B$2:$B$589,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A48,Fiches!$B$2:$B$592,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A48,Fiches!$B$2:$B$589,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A48,Fiches!$B$2:$B$592,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$589,$A48,Fiches!$B$2:$B$589,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$592,$A48,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Développements limités : position/tangente, parité, inverse et quotient
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N592"/>
+  <dimension ref="A1:N595"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -15535,7 +15535,7 @@
       </c>
       <c r="I255" s="9" t="inlineStr">
         <is>
-          <t>$g\circ f$ admet un $DL_n(a)$ de partie régulière $T_n(Q_n\circ P_n)$.</t>
+          <t>$g\circ f$ admet un $DL_n(a)$ de partie régulière $T_n(Q_n\circ P_n)$ (avec $Q_n$ écrit en puissances de $y-f(a)$). En pratique en $0$ : on compose $g(u)$ avec $u=f(x)$ qui doit tendre vers $0$ (sinon on se ramène en $0$, par exemple $e^{a+h}=e^ae^h$).</t>
         </is>
       </c>
       <c r="J255" s="9" t="inlineStr">
@@ -35410,10 +35410,190 @@
       <c r="M592" s="11" t="n"/>
       <c r="N592" s="11" t="n"/>
     </row>
+    <row r="593">
+      <c r="A593" s="9" t="inlineStr">
+        <is>
+          <t>M593</t>
+        </is>
+      </c>
+      <c r="B593" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C593" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D593" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 9 – Développements limités</t>
+        </is>
+      </c>
+      <c r="E593" s="9" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+      <c r="F593" s="9" t="inlineStr">
+        <is>
+          <t>Position de la courbe par rapport à sa tangente</t>
+        </is>
+      </c>
+      <c r="G593" s="9" t="inlineStr">
+        <is>
+          <t>Soit $f$ admettant en $a$ un DL $f(x)=f(a)+f'(a)(x-a)+c\,(x-a)^p+o\big((x-a)^p\big)$ avec $c\neq0$ et $p\ge2$.</t>
+        </is>
+      </c>
+      <c r="H593" s="10" t="inlineStr">
+        <is>
+          <t>Comment en déduire la position locale de la courbe de $f$ par rapport à sa tangente en $a$ ?</t>
+        </is>
+      </c>
+      <c r="I593" s="9" t="inlineStr">
+        <is>
+          <t>Au voisinage de $a$, $f(x)-[f(a)+f'(a)(x-a)]$ a le signe de $c\,(x-a)^p$. Si $p$ est pair : la courbe est au-dessus de la tangente si $c&gt;0$, au-dessous si $c&lt;0$. Si $p$ est impair : elle traverse sa tangente (point d'inflexion).</t>
+        </is>
+      </c>
+      <c r="J593" s="9" t="inlineStr">
+        <is>
+          <t>Programme Analyse 9 : « Étude locale d'une fonction : … tangente, position relative de la courbe et de la tangente. »</t>
+        </is>
+      </c>
+      <c r="K593" s="9" t="n"/>
+      <c r="L593" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Développements limités »</t>
+        </is>
+      </c>
+      <c r="M593" s="11" t="n"/>
+      <c r="N593" s="11" t="n"/>
+    </row>
+    <row r="594">
+      <c r="A594" s="9" t="inlineStr">
+        <is>
+          <t>M594</t>
+        </is>
+      </c>
+      <c r="B594" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C594" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D594" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 9 – Développements limités</t>
+        </is>
+      </c>
+      <c r="E594" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F594" s="9" t="inlineStr">
+        <is>
+          <t>DL d’une fonction paire ou impaire</t>
+        </is>
+      </c>
+      <c r="G594" s="9" t="inlineStr">
+        <is>
+          <t>Soit $f$ définie sur un intervalle symétrique et admettant un $DL_n(0)$.</t>
+        </is>
+      </c>
+      <c r="H594" s="10" t="inlineStr">
+        <is>
+          <t>Que dire de la partie régulière si $f$ est paire ? impaire ?</t>
+        </is>
+      </c>
+      <c r="I594" s="9" t="inlineStr">
+        <is>
+          <t>Si $f$ est paire, sa partie régulière ne contient que des puissances paires de $x$ ; si $f$ est impaire, que des puissances impaires (conséquence de l'unicité du DL). Exemples : $\cos$, $\sin$.</t>
+        </is>
+      </c>
+      <c r="J594" s="9" t="inlineStr">
+        <is>
+          <t>Exemple du cours ; non cité par le programme.</t>
+        </is>
+      </c>
+      <c r="K594" s="9" t="n"/>
+      <c r="L594" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Développements limités »</t>
+        </is>
+      </c>
+      <c r="M594" s="11" t="n"/>
+      <c r="N594" s="11" t="n"/>
+    </row>
+    <row r="595">
+      <c r="A595" s="9" t="inlineStr">
+        <is>
+          <t>M595</t>
+        </is>
+      </c>
+      <c r="B595" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C595" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D595" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 9 – Développements limités</t>
+        </is>
+      </c>
+      <c r="E595" s="9" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+      <c r="F595" s="9" t="inlineStr">
+        <is>
+          <t>DL d’un inverse, d’un quotient</t>
+        </is>
+      </c>
+      <c r="G595" s="9" t="inlineStr">
+        <is>
+          <t>Soient $f$, $g$ admettant un $DL_n(0)$ avec $g(0)=a\neq0$.</t>
+        </is>
+      </c>
+      <c r="H595" s="10" t="inlineStr">
+        <is>
+          <t>Comment obtenir le $DL_n(0)$ de $\dfrac1g$, puis de $\dfrac fg$ ? Comment traiter $\ln(a+h)$ et $e^{a+h}$ ?</t>
+        </is>
+      </c>
+      <c r="I595" s="9" t="inlineStr">
+        <is>
+          <t>$\dfrac1{g(x)}=\dfrac1a\times\dfrac1{1+u(x)}$ avec $u=\frac ga-1\to0$, puis on compose avec le DL de $\frac1{1+u}$ ; $\frac fg=f\times\frac1g$ (produit). De même $\ln(a+h)=\ln a+\ln\left(1+\frac ha\right)$ et $e^{a+h}=e^a\,e^h$.</t>
+        </is>
+      </c>
+      <c r="J595" s="9" t="inlineStr">
+        <is>
+          <t>Cours ; le programme ne cite que somme, produit et composée « sur des exemples simples ».</t>
+        </is>
+      </c>
+      <c r="K595" s="9" t="n"/>
+      <c r="L595" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Développements limités »</t>
+        </is>
+      </c>
+      <c r="M595" s="11" t="n"/>
+      <c r="N595" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M592" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M595" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -38956,7 +39136,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$592,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$595,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -38971,7 +39151,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$592,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$595,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -38986,7 +39166,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$592,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$595,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -39013,7 +39193,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$592)</f>
+        <f>COUNTA(Fiches!$M$2:$M$595)</f>
         <v/>
       </c>
     </row>
@@ -39059,15 +39239,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A13,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A13,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A13,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A13,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A13,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A13,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -39082,15 +39262,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A14,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A14,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A14,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A14,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A14,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A14,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -39105,15 +39285,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A15,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A15,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A15,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A15,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A15,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A15,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -39128,15 +39308,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A16,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A16,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A16,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A16,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A16,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A16,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -39151,15 +39331,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A17,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A17,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A17,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A17,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A17,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A17,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -39174,15 +39354,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A18,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A18,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A18,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A18,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A18,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A18,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -39197,15 +39377,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A19,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A19,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A19,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A19,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A19,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A19,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -39220,15 +39400,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A20,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A20,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A20,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A20,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A20,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A20,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -39243,15 +39423,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A21,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A21,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A21,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A21,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A21,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A21,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -39266,15 +39446,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A22,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A22,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A22,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A22,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A22,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A22,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -39289,15 +39469,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A23,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A23,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A23,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A23,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A23,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A23,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -39312,15 +39492,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A24,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A24,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A24,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A24,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A24,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A24,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -39335,15 +39515,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A25,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A25,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A25,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A25,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A25,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A25,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -39358,15 +39538,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A26,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A26,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A26,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A26,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A26,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A26,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -39381,15 +39561,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A27,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A27,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A27,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A27,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A27,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A27,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -39404,15 +39584,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A28,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A28,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A28,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A28,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A28,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A28,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -39427,15 +39607,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A29,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A29,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A29,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A29,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A29,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A29,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -39450,15 +39630,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A30,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A30,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A30,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A30,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A30,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A30,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -39473,15 +39653,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A31,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A31,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A31,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A31,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A31,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A31,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -39496,15 +39676,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A32,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A32,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A32,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A32,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A32,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A32,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -39519,15 +39699,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A33,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A33,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A33,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A33,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A33,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A33,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -39542,15 +39722,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A34,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A34,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A34,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A34,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A34,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A34,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -39565,15 +39745,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A35,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A35,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A35,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A35,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A35,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A35,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -39588,15 +39768,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A36,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A36,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A36,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A36,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A36,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A36,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -39611,15 +39791,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A37,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A37,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A37,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A37,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A37,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A37,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -39634,15 +39814,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A38,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A38,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A38,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A38,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A38,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A38,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -39657,15 +39837,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A39,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A39,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A39,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A39,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A39,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A39,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -39680,15 +39860,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A40,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A40,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A40,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A40,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A40,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A40,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -39703,15 +39883,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A41,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A41,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A41,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A41,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A41,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A41,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -39726,15 +39906,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A42,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A42,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A42,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A42,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A42,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A42,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -39749,15 +39929,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A43,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A43,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A43,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A43,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A43,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A43,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -39772,15 +39952,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A44,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A44,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A44,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A44,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A44,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A44,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -39795,15 +39975,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A45,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A45,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A45,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A45,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A45,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A45,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -39818,15 +39998,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A46,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A46,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A46,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A46,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A46,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A46,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -39841,15 +40021,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A47,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A47,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A47,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A47,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A47,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A47,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -39864,15 +40044,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A48,Fiches!$B$2:$B$592,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A48,Fiches!$B$2:$B$595,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A48,Fiches!$B$2:$B$592,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A48,Fiches!$B$2:$B$595,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$592,$A48,Fiches!$B$2:$B$592,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$595,$A48,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Étude de fonctions : réduction du domaine, plan d'étude, branches infinies
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N595"/>
+  <dimension ref="A1:N598"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -35590,10 +35590,190 @@
       <c r="M595" s="11" t="n"/>
       <c r="N595" s="11" t="n"/>
     </row>
+    <row r="596">
+      <c r="A596" s="9" t="inlineStr">
+        <is>
+          <t>M596</t>
+        </is>
+      </c>
+      <c r="B596" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C596" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D596" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E596" s="9" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+      <c r="F596" s="9" t="inlineStr">
+        <is>
+          <t>Réduction du domaine d’étude</t>
+        </is>
+      </c>
+      <c r="G596" s="9" t="inlineStr">
+        <is>
+          <t>Soient $f$ définie sur $D_f$, de courbe $\mathcal C_f$, et $a,b$ deux réels.</t>
+        </is>
+      </c>
+      <c r="H596" s="10" t="inlineStr">
+        <is>
+          <t>Comment réduire l'intervalle d'étude si $f$ est $T$-périodique ? paire ou impaire ? si $f(2a-x)=f(x)$ ? si $f(2a-x)=2b-f(x)$ ?</t>
+        </is>
+      </c>
+      <c r="I596" s="9" t="inlineStr">
+        <is>
+          <t>$T$-périodique : on étudie $f$ sur un intervalle de longueur $T$, puis on complète par translations de vecteur $T\vec\imath$. Paire (resp. impaire) : étude sur $D_f\cap\mathbb R_+$, puis symétrie par rapport à $(Oy)$ (resp. à $O$). Si $f(2a-x)=f(x)$ (avec $2a-x\in D_f$) : $\mathcal C_f$ est symétrique par rapport à la droite $x=a$. Si $f(2a-x)=2b-f(x)$ : symétrique par rapport au point $(a,b)$. Dans ces deux cas, étude sur $D_f\cap[a,+\infty[$.</t>
+        </is>
+      </c>
+      <c r="J596" s="9" t="inlineStr">
+        <is>
+          <t>Programme Analyse 2 : « Réduction du domaine d'étude selon les symétries et/ou les périodicités déterminées. On abordera uniquement des exemples simples. »</t>
+        </is>
+      </c>
+      <c r="K596" s="9" t="n"/>
+      <c r="L596" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Plan d’étude d’une fonction »</t>
+        </is>
+      </c>
+      <c r="M596" s="11" t="n"/>
+      <c r="N596" s="11" t="n"/>
+    </row>
+    <row r="597">
+      <c r="A597" s="9" t="inlineStr">
+        <is>
+          <t>M597</t>
+        </is>
+      </c>
+      <c r="B597" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C597" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D597" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E597" s="9" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+      <c r="F597" s="9" t="inlineStr">
+        <is>
+          <t>Plan d’étude d’une fonction</t>
+        </is>
+      </c>
+      <c r="G597" s="9" t="inlineStr">
+        <is>
+          <t>Soit $f$ une fonction réelle à étudier.</t>
+        </is>
+      </c>
+      <c r="H597" s="10" t="inlineStr">
+        <is>
+          <t>Quelles sont les étapes de l'étude de $f$ ?</t>
+        </is>
+      </c>
+      <c r="I597" s="9" t="inlineStr">
+        <is>
+          <t>1) Ensemble de définition et réduction du domaine (parité, périodicité, symétries). 2) Continuité (prolongement éventuel) et dérivabilité. 3) Signe de $f'$ et tableau de variations. 4) Limites aux bornes : asymptotes verticales, horizontales, obliques, branches paraboliques. 5) Tracé : symétries, tangentes remarquables (horizontales, verticales, aux bornes), asymptotes, points d'inflexion.</t>
+        </is>
+      </c>
+      <c r="J597" s="9" t="inlineStr">
+        <is>
+          <t>Programme Analyse 2 b) « Étude d'une fonction » : réduction du domaine, tableau de variations, tangente, asymptotes, tracé du graphe ; Analyse 9 : étude locale.</t>
+        </is>
+      </c>
+      <c r="K597" s="9" t="n"/>
+      <c r="L597" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Plan d’étude d’une fonction »</t>
+        </is>
+      </c>
+      <c r="M597" s="11" t="n"/>
+      <c r="N597" s="11" t="n"/>
+    </row>
+    <row r="598">
+      <c r="A598" s="9" t="inlineStr">
+        <is>
+          <t>M598</t>
+        </is>
+      </c>
+      <c r="B598" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C598" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D598" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 2 – Fonctions réelles usuelles</t>
+        </is>
+      </c>
+      <c r="E598" s="9" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+      <c r="F598" s="9" t="inlineStr">
+        <is>
+          <t>Branches infinies en +∞</t>
+        </is>
+      </c>
+      <c r="G598" s="9" t="inlineStr">
+        <is>
+          <t>Soit $f$ telle que $f(x)\to\pm\infty$ quand $x\to+\infty$.</t>
+        </is>
+      </c>
+      <c r="H598" s="10" t="inlineStr">
+        <is>
+          <t>Comment classer la branche infinie de $\mathcal C_f$ en $+\infty$ ?</t>
+        </is>
+      </c>
+      <c r="I598" s="9" t="inlineStr">
+        <is>
+          <t>On étudie $\lim\frac{f(x)}x$. Si elle vaut $\pm\infty$ : branche parabolique de direction $(Oy)$. Si elle vaut $0$ : branche parabolique de direction $(Ox)$. Si elle vaut $a\in\mathbb R^*$, on étudie $f(x)-ax$ : limite $b$ finie, la droite $y=ax+b$ est asymptote (position : signe de $f(x)-(ax+b)$) ; limite infinie, branche parabolique de direction $y=ax$.</t>
+        </is>
+      </c>
+      <c r="J598" s="9" t="inlineStr">
+        <is>
+          <t>Cours ; le programme cite les asymptotes (Analyse 2 et 9) mais pas les branches paraboliques.</t>
+        </is>
+      </c>
+      <c r="K598" s="9" t="n"/>
+      <c r="L598" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Plan d’étude d’une fonction »</t>
+        </is>
+      </c>
+      <c r="M598" s="11" t="n"/>
+      <c r="N598" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M595" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M598" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -39136,7 +39316,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$595,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$598,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -39151,7 +39331,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$595,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$598,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -39166,7 +39346,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$595,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$598,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -39193,7 +39373,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$595)</f>
+        <f>COUNTA(Fiches!$M$2:$M$598)</f>
         <v/>
       </c>
     </row>
@@ -39239,15 +39419,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A13,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A13,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A13,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A13,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A13,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A13,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -39262,15 +39442,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A14,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A14,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A14,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A14,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A14,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A14,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -39285,15 +39465,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A15,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A15,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A15,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A15,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A15,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A15,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -39308,15 +39488,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A16,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A16,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A16,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A16,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A16,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A16,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -39331,15 +39511,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A17,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A17,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A17,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A17,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A17,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A17,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -39354,15 +39534,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A18,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A18,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A18,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A18,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A18,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A18,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -39377,15 +39557,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A19,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A19,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A19,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A19,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A19,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A19,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -39400,15 +39580,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A20,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A20,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A20,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A20,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A20,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A20,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -39423,15 +39603,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A21,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A21,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A21,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A21,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A21,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A21,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -39446,15 +39626,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A22,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A22,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A22,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A22,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A22,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A22,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -39469,15 +39649,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A23,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A23,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A23,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A23,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A23,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A23,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -39492,15 +39672,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A24,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A24,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A24,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A24,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A24,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A24,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -39515,15 +39695,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A25,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A25,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A25,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A25,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A25,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A25,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -39538,15 +39718,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A26,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A26,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A26,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A26,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A26,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A26,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -39561,15 +39741,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A27,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A27,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A27,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A27,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A27,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A27,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -39584,15 +39764,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A28,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A28,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A28,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A28,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A28,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A28,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -39607,15 +39787,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A29,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A29,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A29,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A29,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A29,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A29,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -39630,15 +39810,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A30,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A30,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A30,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A30,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A30,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A30,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -39653,15 +39833,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A31,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A31,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A31,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A31,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A31,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A31,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -39676,15 +39856,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A32,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A32,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A32,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A32,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A32,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A32,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -39699,15 +39879,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A33,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A33,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A33,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A33,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A33,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A33,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -39722,15 +39902,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A34,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A34,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A34,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A34,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A34,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A34,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -39745,15 +39925,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A35,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A35,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A35,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A35,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A35,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A35,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -39768,15 +39948,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A36,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A36,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A36,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A36,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A36,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A36,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -39791,15 +39971,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A37,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A37,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A37,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A37,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A37,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A37,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -39814,15 +39994,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A38,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A38,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A38,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A38,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A38,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A38,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -39837,15 +40017,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A39,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A39,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A39,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A39,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A39,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A39,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -39860,15 +40040,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A40,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A40,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A40,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A40,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A40,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A40,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -39883,15 +40063,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A41,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A41,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A41,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A41,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A41,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A41,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -39906,15 +40086,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A42,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A42,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A42,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A42,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A42,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A42,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -39929,15 +40109,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A43,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A43,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A43,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A43,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A43,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A43,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -39952,15 +40132,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A44,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A44,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A44,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A44,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A44,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A44,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -39975,15 +40155,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A45,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A45,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A45,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A45,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A45,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A45,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -39998,15 +40178,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A46,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A46,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A46,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A46,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A46,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A46,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -40021,15 +40201,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A47,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A47,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A47,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A47,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A47,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A47,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -40044,15 +40224,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A48,Fiches!$B$2:$B$595,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A48,Fiches!$B$2:$B$598,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A48,Fiches!$B$2:$B$595,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A48,Fiches!$B$2:$B$598,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$595,$A48,Fiches!$B$2:$B$595,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$598,$A48,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Limites, continuité : croissances comparées, limites usuelles, prolongement, caractérisation séquentielle
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N598"/>
+  <dimension ref="A1:N602"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -11525,7 +11525,7 @@
       </c>
       <c r="I186" s="9" t="inlineStr">
         <is>
-          <t>$\forall\varepsilon&gt;0,\ \exists\eta&gt;0,\ \forall x\in I,\ |x-a|\le\eta\Rightarrow|f(x)-l|\le\varepsilon$. Variantes en $\pm\infty$ et pour les limites infinies (avec $A$, $B$ au lieu de $\varepsilon$, $\eta$).</t>
+          <t>$\forall\varepsilon&gt;0,\ \exists\eta&gt;0,\ \forall x\in I,\ |x-a|\le\eta\Rightarrow|f(x)-l|\le\varepsilon$. Variantes en $\pm\infty$ et pour les limites infinies (avec $A$, $B$ au lieu de $\varepsilon$, $\eta$). Si elle existe, la limite est unique.</t>
         </is>
       </c>
       <c r="J186" s="9" t="inlineStr">
@@ -12577,7 +12577,7 @@
       </c>
       <c r="I204" s="9" t="inlineStr">
         <is>
-          <t>$f+g$, $fg$, $\lambda f$ sont continues sur $I$ ; si $g$ ne s'annule pas sur $I$, $1/g$ et $f/g$ sont continues sur $I$.</t>
+          <t>$f+g$, $fg$, $\lambda f$ sont continues sur $I$ ; si $g$ ne s'annule pas sur $I$, $1/g$ et $f/g$ sont continues sur $I$. Les fonctions usuelles sont continues sur leur ensemble de définition.</t>
         </is>
       </c>
       <c r="J204" s="9" t="inlineStr">
@@ -12693,7 +12693,7 @@
       </c>
       <c r="I206" s="9" t="inlineStr">
         <is>
-          <t>Si $f$ est continue sur $[a,b]$, pour tout $y$ compris entre $f(a)$ et $f(b)$, il existe $c\in[a,b]$ tel que $f(c)=y$. L'image d'un intervalle par une fonction continue est un intervalle.</t>
+          <t>Si $f$ est continue sur $[a,b]$, pour tout $y$ compris entre $f(a)$ et $f(b)$, il existe $c\in[a,b]$ tel que $f(c)=y$. En particulier, si $f(a)f(b)\le0$, $f$ s'annule sur $[a,b]$. L'image d'un intervalle par une fonction continue est un intervalle.</t>
         </is>
       </c>
       <c r="J206" s="9" t="inlineStr">
@@ -35770,10 +35770,246 @@
       <c r="M598" s="11" t="n"/>
       <c r="N598" s="11" t="n"/>
     </row>
+    <row r="599">
+      <c r="A599" s="9" t="inlineStr">
+        <is>
+          <t>M599</t>
+        </is>
+      </c>
+      <c r="B599" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C599" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D599" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 6 – Limites, continuité</t>
+        </is>
+      </c>
+      <c r="E599" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F599" s="9" t="inlineStr">
+        <is>
+          <t>Croissances comparées (fonctions)</t>
+        </is>
+      </c>
+      <c r="G599" s="9" t="inlineStr">
+        <is>
+          <t>Soient $\alpha&gt;0$ et $\beta&gt;0$.</t>
+        </is>
+      </c>
+      <c r="H599" s="10" t="inlineStr">
+        <is>
+          <t>Donner les limites de croissances comparées entre puissances, exponentielle et logarithme (en $+\infty$, en $0^+$, en $-\infty$).</t>
+        </is>
+      </c>
+      <c r="I599" s="9" t="inlineStr">
+        <is>
+          <t>En $+\infty$ : $\dfrac{(\ln x)^\beta}{x^\alpha}\to0$ et $\dfrac{x^\alpha}{e^{\beta x}}\to0$ (en particulier $\frac{\ln x}x\to0$, $\frac{e^x}x\to+\infty$). En $0^+$ : $x^\alpha|\ln x|^\beta\to0$ (dont $x\ln x\to0^-$). En $-\infty$ : $|x|^\alpha e^x\to0$ (dont $xe^x\to0$).</t>
+        </is>
+      </c>
+      <c r="J599" s="9" t="inlineStr">
+        <is>
+          <t>Programme Analyse 6 : « Croissances comparées des fonctions exponentielles, puissances et logarithmes. Connaissance de $\lim_{x\to0}x^\alpha\ln^\beta(x)$, de $\lim_{x\to+\infty}x^\alpha\exp(-\beta x^\gamma)$. »</t>
+        </is>
+      </c>
+      <c r="K599" s="9" t="n"/>
+      <c r="L599" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Limites, continuité »</t>
+        </is>
+      </c>
+      <c r="M599" s="11" t="n"/>
+      <c r="N599" s="11" t="n"/>
+    </row>
+    <row r="600">
+      <c r="A600" s="9" t="inlineStr">
+        <is>
+          <t>M600</t>
+        </is>
+      </c>
+      <c r="B600" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C600" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D600" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 6 – Limites, continuité</t>
+        </is>
+      </c>
+      <c r="E600" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F600" s="9" t="inlineStr">
+        <is>
+          <t>Limites usuelles en 0</t>
+        </is>
+      </c>
+      <c r="G600" s="9" t="n"/>
+      <c r="H600" s="10" t="inlineStr">
+        <is>
+          <t>Donner les limites en $0$ de $\dfrac{\sin x}x$, $\dfrac{\tan x}x$, $\dfrac{1-\cos x}{x^2}$, $\dfrac{\ln(1+x)}x$, $\dfrac{e^x-1}x$.</t>
+        </is>
+      </c>
+      <c r="I600" s="9" t="inlineStr">
+        <is>
+          <t>$\dfrac{\sin x}x\to1$ ; $\dfrac{\tan x}x\to1$ ; $\dfrac{1-\cos x}{x^2}\to\dfrac12$ ; $\dfrac{\ln(1+x)}x\to1$ ; $\dfrac{e^x-1}x\to1$ (taux d'accroissement en $0$ de $\sin$, $\tan$, $\ln(1+\cdot)$, $\exp$).</t>
+        </is>
+      </c>
+      <c r="J600" s="9" t="inlineStr">
+        <is>
+          <t>Programme Analyse 6 : « Utilisation des équivalents pour la recherche de limites » ; ces limites traduisent les équivalents usuels en 0.</t>
+        </is>
+      </c>
+      <c r="K600" s="9" t="n"/>
+      <c r="L600" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Limites, continuité »</t>
+        </is>
+      </c>
+      <c r="M600" s="11" t="n"/>
+      <c r="N600" s="11" t="n"/>
+    </row>
+    <row r="601">
+      <c r="A601" s="9" t="inlineStr">
+        <is>
+          <t>M601</t>
+        </is>
+      </c>
+      <c r="B601" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C601" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D601" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 6 – Limites, continuité</t>
+        </is>
+      </c>
+      <c r="E601" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F601" s="9" t="inlineStr">
+        <is>
+          <t>Prolongement par continuité</t>
+        </is>
+      </c>
+      <c r="G601" s="9" t="inlineStr">
+        <is>
+          <t>Soient $I$ un intervalle, $a\in I$ et $f$ continue sur $I\setminus\{a\}$.</t>
+        </is>
+      </c>
+      <c r="H601" s="10" t="inlineStr">
+        <is>
+          <t>À quelle condition peut-on prolonger $f$ par continuité en $a$ ? Comment ?</t>
+        </is>
+      </c>
+      <c r="I601" s="9" t="inlineStr">
+        <is>
+          <t>Si $f$ admet une limite finie $l$ en $a$, la fonction $\tilde f$ égale à $f$ sur $I\setminus\{a\}$ et telle que $\tilde f(a)=l$ est continue sur $I$ : c'est le prolongement par continuité de $f$ en $a$. Exemple : $x\ln x$ se prolonge en $0$ par $0$.</t>
+        </is>
+      </c>
+      <c r="J601" s="9" t="inlineStr">
+        <is>
+          <t>Programme Analyse 6 : « Prolongement par continuité. »</t>
+        </is>
+      </c>
+      <c r="K601" s="9" t="n"/>
+      <c r="L601" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Limites, continuité »</t>
+        </is>
+      </c>
+      <c r="M601" s="11" t="n"/>
+      <c r="N601" s="11" t="n"/>
+    </row>
+    <row r="602">
+      <c r="A602" s="9" t="inlineStr">
+        <is>
+          <t>M602</t>
+        </is>
+      </c>
+      <c r="B602" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C602" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D602" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Analyse 6 – Limites, continuité</t>
+        </is>
+      </c>
+      <c r="E602" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F602" s="9" t="inlineStr">
+        <is>
+          <t>Caractérisation séquentielle de la limite</t>
+        </is>
+      </c>
+      <c r="G602" s="9" t="inlineStr">
+        <is>
+          <t>Soient $f$ définie sur $I$, $a$ un point ou une extrémité de $I$ et $l\in\mathbb R$.</t>
+        </is>
+      </c>
+      <c r="H602" s="10" t="inlineStr">
+        <is>
+          <t>Énoncer la caractérisation séquentielle de $\lim_af=l$. Comment l'utiliser pour montrer qu'une fonction n'a pas de limite en $a$ ?</t>
+        </is>
+      </c>
+      <c r="I602" s="9" t="inlineStr">
+        <is>
+          <t>$\lim_af=l$ ssi pour toute suite $(u_n)$ d'éléments de $I$ qui tend vers $a$, $f(u_n)\to l$. Pour montrer l'absence de limite : trouver deux suites $u_n\to a$ et $v_n\to a$ telles que $f(u_n)$ et $f(v_n)$ aient des limites différentes (ex. $\sin\frac1x$ en $0$).</t>
+        </is>
+      </c>
+      <c r="J602" s="9" t="inlineStr">
+        <is>
+          <t>Cours ; le programme ne demande que le sens direct (composition suite-fonction).</t>
+        </is>
+      </c>
+      <c r="K602" s="9" t="n"/>
+      <c r="L602" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Limites, continuité »</t>
+        </is>
+      </c>
+      <c r="M602" s="11" t="n"/>
+      <c r="N602" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M598" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M602" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -39316,7 +39552,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$598,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$602,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -39331,7 +39567,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$598,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$602,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -39346,7 +39582,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$598,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$602,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -39373,7 +39609,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$598)</f>
+        <f>COUNTA(Fiches!$M$2:$M$602)</f>
         <v/>
       </c>
     </row>
@@ -39419,15 +39655,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A13,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A13,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A13,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A13,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A13,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A13,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -39442,15 +39678,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A14,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A14,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A14,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A14,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A14,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A14,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -39465,15 +39701,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A15,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A15,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A15,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A15,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A15,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A15,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -39488,15 +39724,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A16,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A16,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A16,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A16,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A16,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A16,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -39511,15 +39747,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A17,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A17,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A17,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A17,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A17,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A17,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -39534,15 +39770,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A18,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A18,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A18,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A18,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A18,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A18,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -39557,15 +39793,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A19,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A19,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A19,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A19,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A19,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A19,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -39580,15 +39816,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A20,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A20,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A20,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A20,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A20,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A20,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -39603,15 +39839,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A21,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A21,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A21,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A21,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A21,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A21,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -39626,15 +39862,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A22,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A22,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A22,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A22,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A22,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A22,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -39649,15 +39885,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A23,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A23,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A23,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A23,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A23,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A23,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -39672,15 +39908,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A24,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A24,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A24,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A24,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A24,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A24,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -39695,15 +39931,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A25,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A25,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A25,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A25,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A25,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A25,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -39718,15 +39954,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A26,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A26,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A26,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A26,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A26,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A26,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -39741,15 +39977,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A27,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A27,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A27,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A27,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A27,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A27,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -39764,15 +40000,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A28,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A28,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A28,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A28,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A28,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A28,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -39787,15 +40023,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A29,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A29,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A29,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A29,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A29,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A29,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -39810,15 +40046,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A30,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A30,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A30,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A30,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A30,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A30,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -39833,15 +40069,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A31,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A31,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A31,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A31,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A31,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A31,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -39856,15 +40092,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A32,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A32,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A32,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A32,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A32,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A32,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -39879,15 +40115,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A33,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A33,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A33,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A33,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A33,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A33,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -39902,15 +40138,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A34,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A34,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A34,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A34,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A34,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A34,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -39925,15 +40161,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A35,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A35,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A35,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A35,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A35,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A35,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -39948,15 +40184,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A36,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A36,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A36,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A36,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A36,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A36,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -39971,15 +40207,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A37,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A37,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A37,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A37,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A37,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A37,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -39994,15 +40230,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A38,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A38,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A38,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A38,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A38,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A38,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -40017,15 +40253,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A39,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A39,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A39,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A39,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A39,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A39,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -40040,15 +40276,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A40,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A40,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A40,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A40,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A40,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A40,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -40063,15 +40299,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A41,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A41,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A41,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A41,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A41,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A41,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -40086,15 +40322,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A42,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A42,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A42,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A42,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A42,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A42,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -40109,15 +40345,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A43,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A43,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A43,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A43,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A43,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A43,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -40132,15 +40368,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A44,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A44,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A44,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A44,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A44,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A44,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -40155,15 +40391,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A45,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A45,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A45,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A45,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A45,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A45,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -40178,15 +40414,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A46,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A46,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A46,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A46,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A46,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A46,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -40201,15 +40437,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A47,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A47,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A47,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A47,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A47,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A47,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -40224,15 +40460,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A48,Fiches!$B$2:$B$598,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A48,Fiches!$B$2:$B$602,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A48,Fiches!$B$2:$B$598,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A48,Fiches!$B$2:$B$602,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$598,$A48,Fiches!$B$2:$B$598,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$602,$A48,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Nombres réels : bornes, inégalités, puissances, identités remarquables
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N602"/>
+  <dimension ref="A1:N607"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1217,7 +1217,7 @@
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>$E(x)=\lfloor x\rfloor$ est l'unique entier tel que $E(x)\le x&lt;E(x)+1$.</t>
+          <t>$E(x)=\lfloor x\rfloor$ est le plus grand entier inférieur ou égal à $x$ : l'unique entier tel que $\lfloor x\rfloor\le x&lt;\lfloor x\rfloor+1$, soit $x-1&lt;\lfloor x\rfloor\le x$. Ex. : $\lfloor\sqrt2\rfloor=1$, $\lfloor-3{,}1\rfloor=-4$.</t>
         </is>
       </c>
       <c r="J8" s="9" t="inlineStr">
@@ -30113,7 +30113,7 @@
       </c>
       <c r="I504" s="9" t="inlineStr">
         <is>
-          <t>$|x|=\max(x,-x)$ ; $|xy|=|x||y|$ ; $|x+y|\le|x|+|y|$ ; $|x-a|$ est la distance de $x$ à $a$, donc $|x-a|\le r\iff a-r\le x\le a+r$.</t>
+          <t>$|x|=\max(x,-x)$ ; $|x|=0\iff x=0$ ; $|x|=|y|\iff x=\pm y$ ; $\sqrt{x^2}=|x|$ ; $|xy|=|x||y|$ ; $|x+y|\le|x|+|y|$ (inégalité triangulaire). $|x-a|$ est la distance de $x$ à $a$, donc $|x-a|\le r\iff a-r\le x\le a+r$.</t>
         </is>
       </c>
       <c r="J504" s="9" t="inlineStr">
@@ -36005,11 +36005,311 @@
       </c>
       <c r="M602" s="11" t="n"/>
       <c r="N602" s="11" t="n"/>
+    </row>
+    <row r="603">
+      <c r="A603" s="9" t="inlineStr">
+        <is>
+          <t>M603</t>
+        </is>
+      </c>
+      <c r="B603" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C603" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D603" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 2 – Nombres réels</t>
+        </is>
+      </c>
+      <c r="E603" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F603" s="9" t="inlineStr">
+        <is>
+          <t>Majorant, maximum, borne supérieure</t>
+        </is>
+      </c>
+      <c r="G603" s="9" t="inlineStr">
+        <is>
+          <t>Soient $A$ une partie de $\mathbb R$ et $\alpha$ un réel.</t>
+        </is>
+      </c>
+      <c r="H603" s="10" t="inlineStr">
+        <is>
+          <t>Définir : $\alpha$ majorant (minorant) de $A$ ; $A$ majorée, minorée, bornée ; maximum (minimum) ; borne supérieure (inférieure). Quand existent-elles ?</t>
+        </is>
+      </c>
+      <c r="I603" s="9" t="inlineStr">
+        <is>
+          <t>Majorant : $\forall x\in A,\ x\le\alpha$ (minorant : $x\ge\alpha$). $A$ est majorée (minorée) si elle admet un majorant (minorant), bornée si les deux. Maximum : majorant de $A$ qui appartient à $A$ (minimum : minorant appartenant à $A$). $\sup A$ : le plus petit des majorants ; $\inf A$ : le plus grand des minorants. Toute partie non vide majorée (minorée) de $\mathbb R$ admet une borne supérieure (inférieure) ; si $A$ a un maximum, c'est $\sup A$.</t>
+        </is>
+      </c>
+      <c r="J603" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 2 : « Majorant, minorant, plus grand, plus petit élément d'une partie non vide de ℝ. Borne supérieure, borne inférieure. On admet l'existence de la borne supérieure d'une partie majorée non vide. »</t>
+        </is>
+      </c>
+      <c r="K603" s="9" t="n"/>
+      <c r="L603" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Les réels »</t>
+        </is>
+      </c>
+      <c r="M603" s="11" t="n"/>
+      <c r="N603" s="11" t="n"/>
+    </row>
+    <row r="604">
+      <c r="A604" s="9" t="inlineStr">
+        <is>
+          <t>M604</t>
+        </is>
+      </c>
+      <c r="B604" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C604" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D604" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 2 – Nombres réels</t>
+        </is>
+      </c>
+      <c r="E604" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F604" s="9" t="inlineStr">
+        <is>
+          <t>Parties de ℕ et de ℤ</t>
+        </is>
+      </c>
+      <c r="G604" s="9" t="inlineStr">
+        <is>
+          <t>Soit $A$ une partie non vide.</t>
+        </is>
+      </c>
+      <c r="H604" s="10" t="inlineStr">
+        <is>
+          <t>Que dire d'une partie non vide de $\mathbb N$ ? d'une partie non vide majorée de $\mathbb Z$ ? d'une partie finie non vide de $\mathbb R$ ?</t>
+        </is>
+      </c>
+      <c r="I604" s="9" t="inlineStr">
+        <is>
+          <t>Toute partie non vide de $\mathbb N$ admet un plus petit élément. Toute partie non vide majorée (minorée) de $\mathbb Z$ admet un plus grand (petit) élément. Toute partie finie non vide de $\mathbb R$ admet un maximum et un minimum.</t>
+        </is>
+      </c>
+      <c r="J604" s="9" t="inlineStr">
+        <is>
+          <t>Cours (admis) ; non cité par le programme.</t>
+        </is>
+      </c>
+      <c r="K604" s="9" t="n"/>
+      <c r="L604" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Les réels »</t>
+        </is>
+      </c>
+      <c r="M604" s="11" t="n"/>
+      <c r="N604" s="11" t="n"/>
+    </row>
+    <row r="605">
+      <c r="A605" s="9" t="inlineStr">
+        <is>
+          <t>M605</t>
+        </is>
+      </c>
+      <c r="B605" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C605" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D605" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 2 – Nombres réels</t>
+        </is>
+      </c>
+      <c r="E605" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F605" s="9" t="inlineStr">
+        <is>
+          <t>Manipulation des inégalités</t>
+        </is>
+      </c>
+      <c r="G605" s="9" t="inlineStr">
+        <is>
+          <t>Soient $x$, $y$, $z$, $t$ des réels.</t>
+        </is>
+      </c>
+      <c r="H605" s="10" t="inlineStr">
+        <is>
+          <t>Quelles opérations sur les inégalités sont permises ? Lesquelles sont interdites ?</t>
+        </is>
+      </c>
+      <c r="I605" s="9" t="inlineStr">
+        <is>
+          <t>Permis : ajouter un même réel ; additionner membre à membre ($x\le y$ et $z\le t\Rightarrow x+z\le y+t$) ; multiplier par $z\ge0$ (sens conservé) ou $z\le0$ (sens inversé) ; multiplier membre à membre des inégalités entre réels positifs ($0\le x\le y$ et $0\le z\le t\Rightarrow xz\le yt$) ; passer à l'inverse entre réels strictement positifs ($0&lt;x\le y\Rightarrow\frac1x\ge\frac1y$) ; appliquer une fonction croissante (sens conservé) ou décroissante (sens inversé). Interdit : soustraire ou diviser membre à membre (on ajoute l'opposé, on multiplie par l'inverse positif).</t>
+        </is>
+      </c>
+      <c r="J605" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 2 : « Manipulation des inégalités. Il s'agit d'une simple reprise des règles de calcul algébrique sur les inégalités. »</t>
+        </is>
+      </c>
+      <c r="K605" s="9" t="n"/>
+      <c r="L605" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Les réels »</t>
+        </is>
+      </c>
+      <c r="M605" s="11" t="n"/>
+      <c r="N605" s="11" t="n"/>
+    </row>
+    <row r="606">
+      <c r="A606" s="9" t="inlineStr">
+        <is>
+          <t>M606</t>
+        </is>
+      </c>
+      <c r="B606" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C606" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D606" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 2 – Nombres réels</t>
+        </is>
+      </c>
+      <c r="E606" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F606" s="9" t="inlineStr">
+        <is>
+          <t>Puissances entières et racine carrée</t>
+        </is>
+      </c>
+      <c r="G606" s="9" t="inlineStr">
+        <is>
+          <t>Soient $x,y\in\mathbb R^*$ et $n,m\in\mathbb Z$ (et $a,b\ge0$ pour les racines).</t>
+        </is>
+      </c>
+      <c r="H606" s="10" t="inlineStr">
+        <is>
+          <t>Donner les règles de calcul sur $x^n$ et sur $\sqrt a$.</t>
+        </is>
+      </c>
+      <c r="I606" s="9" t="inlineStr">
+        <is>
+          <t>$x^0=1$, $x^{-n}=\frac1{x^n}$ ; $x^nx^m=x^{n+m}$ ; $(x^n)^m=x^{nm}$ ; $(xy)^n=x^ny^n$ ; $\left(\frac xy\right)^n=\frac{x^n}{y^n}$. $\sqrt a$ est l'unique réel positif de carré $a$ ; $\sqrt{ab}=\sqrt a\sqrt b$ ; $\sqrt{a/b}=\sqrt a/\sqrt b$ ($b&gt;0$) ; pour tout réel $x$, $\sqrt{x^2}=|x|$.</t>
+        </is>
+      </c>
+      <c r="J606" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 2 : « Exposants, racine carrée … On attend une maitrise des formules $(xy)^n=x^ny^n$, $x^{n+m}=x^nx^m$, $(x^n)^m=x^{nm}$, $\sqrt{x^2}=|x|$, $\sqrt{xy}=\sqrt x\sqrt y$. »</t>
+        </is>
+      </c>
+      <c r="K606" s="9" t="n"/>
+      <c r="L606" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Les réels »</t>
+        </is>
+      </c>
+      <c r="M606" s="11" t="n"/>
+      <c r="N606" s="11" t="n"/>
+    </row>
+    <row r="607">
+      <c r="A607" s="9" t="inlineStr">
+        <is>
+          <t>M607</t>
+        </is>
+      </c>
+      <c r="B607" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C607" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D607" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 2 – Nombres réels</t>
+        </is>
+      </c>
+      <c r="E607" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F607" s="9" t="inlineStr">
+        <is>
+          <t>Identités remarquables</t>
+        </is>
+      </c>
+      <c r="G607" s="9" t="inlineStr">
+        <is>
+          <t>Soient $a$ et $b$ deux réels.</t>
+        </is>
+      </c>
+      <c r="H607" s="10" t="inlineStr">
+        <is>
+          <t>Donner les identités remarquables (carrés, différence de carrés, cubes).</t>
+        </is>
+      </c>
+      <c r="I607" s="9" t="inlineStr">
+        <is>
+          <t>$(a\pm b)^2=a^2\pm2ab+b^2$ ; $a^2-b^2=(a-b)(a+b)$. Cubes : $(a\pm b)^3=a^3\pm3a^2b+3ab^2\pm b^3$ (cas $n=3$ du binôme).</t>
+        </is>
+      </c>
+      <c r="J607" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 2 : « Les attendus se limitent aux formules $(a\pm b)^2$ et $a^2-b^2$ » ; les cubes sont dans le cours et découlent du binôme de Newton.</t>
+        </is>
+      </c>
+      <c r="K607" s="9" t="n"/>
+      <c r="L607" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Les réels »</t>
+        </is>
+      </c>
+      <c r="M607" s="11" t="n"/>
+      <c r="N607" s="11" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M602" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M607" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -39552,7 +39852,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$602,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$607,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -39567,7 +39867,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$602,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$607,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -39582,7 +39882,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$602,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$607,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -39609,7 +39909,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$602)</f>
+        <f>COUNTA(Fiches!$M$2:$M$607)</f>
         <v/>
       </c>
     </row>
@@ -39655,15 +39955,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A13,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A13,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A13,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A13,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A13,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A13,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -39678,15 +39978,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A14,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A14,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A14,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A14,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A14,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A14,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -39701,15 +40001,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A15,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A15,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A15,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A15,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A15,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A15,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -39724,15 +40024,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A16,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A16,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A16,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A16,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A16,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A16,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -39747,15 +40047,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A17,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A17,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A17,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A17,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A17,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A17,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -39770,15 +40070,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A18,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A18,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A18,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A18,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A18,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A18,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -39793,15 +40093,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A19,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A19,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A19,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A19,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A19,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A19,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -39816,15 +40116,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A20,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A20,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A20,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A20,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A20,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A20,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -39839,15 +40139,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A21,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A21,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A21,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A21,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A21,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A21,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -39862,15 +40162,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A22,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A22,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A22,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A22,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A22,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A22,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -39885,15 +40185,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A23,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A23,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A23,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A23,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A23,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A23,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -39908,15 +40208,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A24,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A24,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A24,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A24,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A24,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A24,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -39931,15 +40231,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A25,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A25,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A25,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A25,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A25,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A25,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -39954,15 +40254,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A26,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A26,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A26,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A26,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A26,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A26,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -39977,15 +40277,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A27,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A27,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A27,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A27,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A27,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A27,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -40000,15 +40300,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A28,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A28,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A28,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A28,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A28,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A28,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -40023,15 +40323,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A29,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A29,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A29,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A29,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A29,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A29,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -40046,15 +40346,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A30,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A30,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A30,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A30,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A30,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A30,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -40069,15 +40369,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A31,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A31,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A31,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A31,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A31,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A31,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -40092,15 +40392,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A32,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A32,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A32,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A32,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A32,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A32,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -40115,15 +40415,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A33,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A33,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A33,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A33,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A33,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A33,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -40138,15 +40438,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A34,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A34,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A34,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A34,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A34,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A34,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -40161,15 +40461,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A35,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A35,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A35,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A35,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A35,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A35,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -40184,15 +40484,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A36,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A36,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A36,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A36,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A36,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A36,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -40207,15 +40507,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A37,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A37,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A37,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A37,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A37,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A37,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -40230,15 +40530,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A38,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A38,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A38,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A38,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A38,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A38,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -40253,15 +40553,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A39,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A39,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A39,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A39,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A39,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A39,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -40276,15 +40576,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A40,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A40,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A40,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A40,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A40,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A40,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -40299,15 +40599,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A41,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A41,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A41,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A41,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A41,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A41,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -40322,15 +40622,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A42,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A42,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A42,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A42,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A42,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A42,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -40345,15 +40645,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A43,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A43,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A43,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A43,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A43,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A43,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -40368,15 +40668,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A44,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A44,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A44,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A44,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A44,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A44,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -40391,15 +40691,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A45,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A45,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A45,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A45,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A45,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A45,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -40414,15 +40714,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A46,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A46,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A46,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A46,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A46,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A46,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -40437,15 +40737,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A47,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A47,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A47,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A47,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A47,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A47,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -40460,15 +40760,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A48,Fiches!$B$2:$B$602,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A48,Fiches!$B$2:$B$607,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A48,Fiches!$B$2:$B$602,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A48,Fiches!$B$2:$B$607,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$602,$A48,Fiches!$B$2:$B$602,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$607,$A48,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Probabilités : vocabulaire des événements, conditionnement, indépendance
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N607"/>
+  <dimension ref="A1:N610"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -17375,7 +17375,7 @@
       </c>
       <c r="I287" s="9" t="inlineStr">
         <is>
-          <t>$P(B)=\sum_iP(B|A_i)P(A_i)$ (les termes où $P(A_i)=0$ sont comptés nuls).</t>
+          <t>$P(B)=\sum_{i=1}^nP(B\cap A_i)=\sum_{i=1}^nP(A_i)P_{A_i}(B)$ (on convient que $P(A_i)P_{A_i}(B)=0$ si $P(A_i)=0$). Cas particulier : $P(B)=P(A)P_A(B)+P(\bar A)P_{\bar A}(B)$.</t>
         </is>
       </c>
       <c r="J287" s="9" t="inlineStr">
@@ -17433,7 +17433,7 @@
       </c>
       <c r="I288" s="9" t="inlineStr">
         <is>
-          <t>$P(A_j|B)=\dfrac{P(B|A_j)P(A_j)}{\sum_iP(B|A_i)P(A_i)}$.</t>
+          <t>$P_B(A_j)=\dfrac{P_{A_j}(B)P(A_j)}{\sum_iP_{A_i}(B)P(A_i)}$. Version à deux événements ($P(A),P(B)\neq0$) : $P_B(A)=\dfrac{P_A(B)P(A)}{P(B)}$.</t>
         </is>
       </c>
       <c r="J288" s="9" t="inlineStr">
@@ -36306,10 +36306,190 @@
       <c r="M607" s="11" t="n"/>
       <c r="N607" s="11" t="n"/>
     </row>
+    <row r="608">
+      <c r="A608" s="9" t="inlineStr">
+        <is>
+          <t>M608</t>
+        </is>
+      </c>
+      <c r="B608" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C608" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D608" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Probabilités 1 – Concepts de base</t>
+        </is>
+      </c>
+      <c r="E608" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F608" s="9" t="inlineStr">
+        <is>
+          <t>Événements : vocabulaire ensembliste</t>
+        </is>
+      </c>
+      <c r="G608" s="9" t="inlineStr">
+        <is>
+          <t>Soient $\Omega$ un univers fini et $A$, $B$ deux événements.</t>
+        </is>
+      </c>
+      <c r="H608" s="10" t="inlineStr">
+        <is>
+          <t>Traduire en langage ensembliste : événement élémentaire, impossible, certain, « $A$ et $B$ », « $A$ ou $B$ », contraire de $A$, $A$ et $B$ incompatibles, « $A$ implique $B$ ».</t>
+        </is>
+      </c>
+      <c r="I608" s="9" t="inlineStr">
+        <is>
+          <t>Élémentaire : singleton $\{\omega\}$ ; impossible : $\varnothing$ ; certain : $\Omega$ ; « $A$ et $B$ » : $A\cap B$ ; « $A$ ou $B$ » : $A\cup B$ ; contraire : $\bar A=\Omega\setminus A$ ; incompatibles : $A\cap B=\varnothing$ ; « $A$ implique $B$ » : $A\subset B$.</t>
+        </is>
+      </c>
+      <c r="J608" s="9" t="inlineStr">
+        <is>
+          <t>Programme Probabilités 1 : « Événements. Événement certain, événement impossible, événements incompatibles. »</t>
+        </is>
+      </c>
+      <c r="K608" s="9" t="n"/>
+      <c r="L608" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Espaces probabilisés »</t>
+        </is>
+      </c>
+      <c r="M608" s="11" t="n"/>
+      <c r="N608" s="11" t="n"/>
+    </row>
+    <row r="609">
+      <c r="A609" s="9" t="inlineStr">
+        <is>
+          <t>M609</t>
+        </is>
+      </c>
+      <c r="B609" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C609" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D609" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Probabilités 1 – Concepts de base</t>
+        </is>
+      </c>
+      <c r="E609" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F609" s="9" t="inlineStr">
+        <is>
+          <t>Probabilité conditionnelle : P_A est une probabilité, conditionnement</t>
+        </is>
+      </c>
+      <c r="G609" s="9" t="inlineStr">
+        <is>
+          <t>Soient $A$ un événement avec $P(A)\neq0$ et $B$ un événement.</t>
+        </is>
+      </c>
+      <c r="H609" s="10" t="inlineStr">
+        <is>
+          <t>Quelle structure a $P_A$ ? Donner la formule de conditionnement.</t>
+        </is>
+      </c>
+      <c r="I609" s="9" t="inlineStr">
+        <is>
+          <t>$P_A:B\mapsto P_A(B)=\dfrac{P(A\cap B)}{P(A)}$ est une probabilité sur $\Omega$ (elle vérifie donc toutes les règles de calcul : $P_A(\bar B)=1-P_A(B)$, etc.). Formule de conditionnement : $P(A\cap B)=P(A)\,P_A(B)$.</t>
+        </is>
+      </c>
+      <c r="J609" s="9" t="inlineStr">
+        <is>
+          <t>Programme Probabilités 1 : « $P_A$ est une probabilité. Formule de conditionnement $P(A\cap B)=P(A)P_A(B)$. »</t>
+        </is>
+      </c>
+      <c r="K609" s="9" t="n"/>
+      <c r="L609" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Espaces probabilisés »</t>
+        </is>
+      </c>
+      <c r="M609" s="11" t="n"/>
+      <c r="N609" s="11" t="n"/>
+    </row>
+    <row r="610">
+      <c r="A610" s="9" t="inlineStr">
+        <is>
+          <t>M610</t>
+        </is>
+      </c>
+      <c r="B610" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C610" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D610" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Probabilités 1 – Concepts de base</t>
+        </is>
+      </c>
+      <c r="E610" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F610" s="9" t="inlineStr">
+        <is>
+          <t>Indépendance – propriétés</t>
+        </is>
+      </c>
+      <c r="G610" s="9" t="inlineStr">
+        <is>
+          <t>Soient $A$, $B$ deux événements (et $A_1,\dots,A_n$ des événements).</t>
+        </is>
+      </c>
+      <c r="H610" s="10" t="inlineStr">
+        <is>
+          <t>Caractériser l'indépendance de $A$ et $B$ par une probabilité conditionnelle. Que dire de $A$ et $\bar B$ ? de deux événements incompatibles ? Comment la mutuelle indépendance se transmet-elle aux contraires ?</t>
+        </is>
+      </c>
+      <c r="I610" s="9" t="inlineStr">
+        <is>
+          <t>Si $P(A)\neq0$ : $A$ et $B$ indépendants $\iff P_A(B)=P(B)$. Si $A$ et $B$ sont indépendants, alors $A$ et $\bar B$, $\bar A$ et $B$, $\bar A$ et $\bar B$ le sont aussi. $\varnothing$ et $\Omega$ sont indépendants de tout événement. Deux événements incompatibles de probabilités non nulles ne sont pas indépendants. Si $A_1,\dots,A_n$ sont mutuellement indépendants, en remplaçant certains $A_i$ par leur contraire on obtient encore des événements mutuellement indépendants.</t>
+        </is>
+      </c>
+      <c r="J610" s="9" t="inlineStr">
+        <is>
+          <t>Propriétés du cours ; le programme se limite aux définitions de l'indépendance.</t>
+        </is>
+      </c>
+      <c r="K610" s="9" t="n"/>
+      <c r="L610" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Espaces probabilisés »</t>
+        </is>
+      </c>
+      <c r="M610" s="11" t="n"/>
+      <c r="N610" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M607" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M610" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -39852,7 +40032,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$607,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$610,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -39867,7 +40047,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$607,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$610,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -39882,7 +40062,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$607,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$610,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -39909,7 +40089,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$607)</f>
+        <f>COUNTA(Fiches!$M$2:$M$610)</f>
         <v/>
       </c>
     </row>
@@ -39955,15 +40135,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A13,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A13,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A13,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A13,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A13,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A13,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -39978,15 +40158,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A14,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A14,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A14,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A14,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A14,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A14,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -40001,15 +40181,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A15,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A15,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A15,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A15,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A15,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A15,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -40024,15 +40204,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A16,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A16,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A16,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A16,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A16,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A16,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -40047,15 +40227,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A17,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A17,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A17,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A17,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A17,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A17,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -40070,15 +40250,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A18,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A18,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A18,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A18,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A18,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A18,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -40093,15 +40273,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A19,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A19,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A19,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A19,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A19,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A19,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -40116,15 +40296,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A20,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A20,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A20,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A20,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A20,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A20,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -40139,15 +40319,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A21,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A21,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A21,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A21,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A21,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A21,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -40162,15 +40342,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A22,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A22,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A22,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A22,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A22,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A22,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -40185,15 +40365,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A23,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A23,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A23,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A23,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A23,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A23,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -40208,15 +40388,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A24,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A24,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A24,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A24,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A24,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A24,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -40231,15 +40411,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A25,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A25,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A25,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A25,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A25,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A25,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -40254,15 +40434,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A26,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A26,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A26,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A26,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A26,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A26,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -40277,15 +40457,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A27,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A27,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A27,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A27,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A27,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A27,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -40300,15 +40480,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A28,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A28,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A28,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A28,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A28,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A28,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -40323,15 +40503,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A29,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A29,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A29,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A29,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A29,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A29,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -40346,15 +40526,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A30,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A30,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A30,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A30,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A30,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A30,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -40369,15 +40549,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A31,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A31,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A31,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A31,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A31,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A31,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -40392,15 +40572,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A32,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A32,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A32,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A32,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A32,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A32,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -40415,15 +40595,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A33,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A33,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A33,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A33,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A33,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A33,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -40438,15 +40618,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A34,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A34,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A34,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A34,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A34,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A34,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -40461,15 +40641,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A35,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A35,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A35,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A35,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A35,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A35,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -40484,15 +40664,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A36,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A36,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A36,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A36,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A36,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A36,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -40507,15 +40687,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A37,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A37,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A37,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A37,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A37,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A37,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -40530,15 +40710,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A38,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A38,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A38,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A38,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A38,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A38,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -40553,15 +40733,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A39,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A39,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A39,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A39,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A39,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A39,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -40576,15 +40756,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A40,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A40,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A40,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A40,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A40,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A40,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -40599,15 +40779,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A41,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A41,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A41,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A41,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A41,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A41,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -40622,15 +40802,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A42,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A42,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A42,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A42,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A42,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A42,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -40645,15 +40825,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A43,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A43,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A43,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A43,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A43,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A43,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -40668,15 +40848,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A44,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A44,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A44,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A44,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A44,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A44,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -40691,15 +40871,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A45,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A45,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A45,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A45,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A45,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A45,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -40714,15 +40894,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A46,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A46,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A46,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A46,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A46,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A46,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -40737,15 +40917,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A47,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A47,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A47,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A47,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A47,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A47,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -40760,15 +40940,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A48,Fiches!$B$2:$B$607,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A48,Fiches!$B$2:$B$610,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A48,Fiches!$B$2:$B$607,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A48,Fiches!$B$2:$B$610,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$607,$A48,Fiches!$B$2:$B$607,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$610,$A48,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Statistique descriptive : nouveau chapitre (10 cartes)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N610"/>
+  <dimension ref="A1:N620"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -36486,10 +36486,610 @@
       <c r="M610" s="11" t="n"/>
       <c r="N610" s="11" t="n"/>
     </row>
+    <row r="611">
+      <c r="A611" s="9" t="inlineStr">
+        <is>
+          <t>M611</t>
+        </is>
+      </c>
+      <c r="B611" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C611" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D611" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Statistique 1</t>
+        </is>
+      </c>
+      <c r="E611" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F611" s="9" t="inlineStr">
+        <is>
+          <t>Vocabulaire statistique</t>
+        </is>
+      </c>
+      <c r="G611" s="9" t="inlineStr">
+        <is>
+          <t>On étudie une population finie.</t>
+        </is>
+      </c>
+      <c r="H611" s="10" t="inlineStr">
+        <is>
+          <t>Définir : individu, taille, échantillon, caractère (qualitatif, quantitatif discret ou continu), modalités, série statistique.</t>
+        </is>
+      </c>
+      <c r="I611" s="9" t="inlineStr">
+        <is>
+          <t>Population : ensemble fini d'individus ; sa taille est son nombre d'individus ; un échantillon est une partie de la population. Un caractère (ou variable statistique) $x$ associe une donnée à chaque individu : quantitatif si elle est numérique (discret : valeurs isolées ; continu : valeurs dans un intervalle, souvent regroupées en classes), qualitatif sinon. Modalités : valeurs possibles du caractère. Série statistique de taille $n$ : le $n$-uplet $(x_1,\dots,x_n)$ des valeurs observées.</t>
+        </is>
+      </c>
+      <c r="J611" s="9" t="inlineStr">
+        <is>
+          <t>Programme Statistique 1 : « Caractère. Distinction entre caractères quantitatifs (discrets ou continus) et qualitatifs. Modalités d'un caractère, cas des regroupements par classes. »</t>
+        </is>
+      </c>
+      <c r="K611" s="9" t="n"/>
+      <c r="L611" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Statistiques »</t>
+        </is>
+      </c>
+      <c r="M611" s="11" t="n"/>
+      <c r="N611" s="11" t="n"/>
+    </row>
+    <row r="612">
+      <c r="A612" s="9" t="inlineStr">
+        <is>
+          <t>M612</t>
+        </is>
+      </c>
+      <c r="B612" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C612" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D612" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Statistique 1</t>
+        </is>
+      </c>
+      <c r="E612" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F612" s="9" t="inlineStr">
+        <is>
+          <t>Effectifs et fréquences</t>
+        </is>
+      </c>
+      <c r="G612" s="9" t="inlineStr">
+        <is>
+          <t>Soit une série $(x_1,\dots,x_n)$ de modalités $a_1&lt;\dots&lt;a_k$.</t>
+        </is>
+      </c>
+      <c r="H612" s="10" t="inlineStr">
+        <is>
+          <t>Définir l'effectif $n_j$ et la fréquence $f_j$ de $a_j$, ainsi que les effectifs et fréquences cumulés. Que valent $\sum n_j$ et $\sum f_j$ ?</t>
+        </is>
+      </c>
+      <c r="I612" s="9" t="inlineStr">
+        <is>
+          <t>$n_j$ : nombre d'individus $i$ tels que $x_i=a_j$ ; $f_j=\dfrac{n_j}n$. Effectif (fréquence) cumulé(e) de $a_j$ : nombre (proportion) d'individus tels que $x_i\le a_j$, soit $n_1+\dots+n_j$ ($f_1+\dots+f_j$). $\sum_{j=1}^kn_j=n$ et $\sum_{j=1}^kf_j=1$.</t>
+        </is>
+      </c>
+      <c r="J612" s="9" t="inlineStr">
+        <is>
+          <t>Programme Statistique 1 : « présentation dans un tableau : effectifs de chaque modalité. Effectifs cumulés, fréquences, fréquences cumulées. »</t>
+        </is>
+      </c>
+      <c r="K612" s="9" t="n"/>
+      <c r="L612" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Statistiques »</t>
+        </is>
+      </c>
+      <c r="M612" s="11" t="n"/>
+      <c r="N612" s="11" t="n"/>
+    </row>
+    <row r="613">
+      <c r="A613" s="9" t="inlineStr">
+        <is>
+          <t>M613</t>
+        </is>
+      </c>
+      <c r="B613" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C613" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D613" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Statistique 1</t>
+        </is>
+      </c>
+      <c r="E613" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F613" s="9" t="inlineStr">
+        <is>
+          <t>Représentations graphiques</t>
+        </is>
+      </c>
+      <c r="G613" s="9" t="inlineStr">
+        <is>
+          <t>Soit une série statistique d'un caractère quantitatif.</t>
+        </is>
+      </c>
+      <c r="H613" s="10" t="inlineStr">
+        <is>
+          <t>Quelles représentations graphiques utiliser (caractère discret, regroupé en classes, effectifs cumulés) ?</t>
+        </is>
+      </c>
+      <c r="I613" s="9" t="inlineStr">
+        <is>
+          <t>Diagramme en bâtons (caractère discret : un bâton de hauteur $n_j$ en chaque modalité $a_j$). Histogramme (classes : rectangles dont l'aire est proportionnelle à l'effectif, donc hauteur = effectif / amplitude). Polygone des effectifs (ou fréquences) cumulés croissants, qui permet de lire médiane, quartiles et déciles. Série double : nuage de points.</t>
+        </is>
+      </c>
+      <c r="J613" s="9" t="inlineStr">
+        <is>
+          <t>Programme Statistique 1 : « Représentations graphiques. Diagrammes en bâtons, histogrammes, polygones des effectifs cumulés (resp. fréquences cumulées). »</t>
+        </is>
+      </c>
+      <c r="K613" s="9" t="n"/>
+      <c r="L613" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Statistiques »</t>
+        </is>
+      </c>
+      <c r="M613" s="11" t="n"/>
+      <c r="N613" s="11" t="n"/>
+    </row>
+    <row r="614">
+      <c r="A614" s="9" t="inlineStr">
+        <is>
+          <t>M614</t>
+        </is>
+      </c>
+      <c r="B614" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C614" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D614" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Statistique 1</t>
+        </is>
+      </c>
+      <c r="E614" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F614" s="9" t="inlineStr">
+        <is>
+          <t>Mode et moyenne</t>
+        </is>
+      </c>
+      <c r="G614" s="9" t="inlineStr">
+        <is>
+          <t>Soit une série $(x_1,\dots,x_n)$ de modalités $a_1,\dots,a_k$, d'effectifs $n_j$ et de fréquences $f_j$.</t>
+        </is>
+      </c>
+      <c r="H614" s="10" t="inlineStr">
+        <is>
+          <t>Définir le mode et la moyenne $\bar x$ (à partir des observations, des effectifs, des fréquences, puis pour des classes $[b_j,c_j[$).</t>
+        </is>
+      </c>
+      <c r="I614" s="9" t="inlineStr">
+        <is>
+          <t>Mode : modalité d'effectif maximal (classe modale : effectif / amplitude maximal). $\bar x=\dfrac1n\sum_{i=1}^nx_i=\dfrac1n\sum_{j=1}^kn_ja_j=\sum_{j=1}^kf_ja_j$. Pour des classes, on remplace $a_j$ par le centre $\frac{b_j+c_j}2$ (valeur approchée).</t>
+        </is>
+      </c>
+      <c r="J614" s="9" t="inlineStr">
+        <is>
+          <t>Programme Statistique 1 : « Caractéristiques (empiriques) de position : mode, moyenne $\bar x$ (les calculs se font à partir des observations ou du tableau des effectifs). »</t>
+        </is>
+      </c>
+      <c r="K614" s="9" t="n"/>
+      <c r="L614" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Statistiques »</t>
+        </is>
+      </c>
+      <c r="M614" s="11" t="n"/>
+      <c r="N614" s="11" t="n"/>
+    </row>
+    <row r="615">
+      <c r="A615" s="9" t="inlineStr">
+        <is>
+          <t>M615</t>
+        </is>
+      </c>
+      <c r="B615" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C615" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D615" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Statistique 1</t>
+        </is>
+      </c>
+      <c r="E615" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F615" s="9" t="inlineStr">
+        <is>
+          <t>Médiane, quartiles, déciles</t>
+        </is>
+      </c>
+      <c r="G615" s="9" t="inlineStr">
+        <is>
+          <t>Soit une série de taille $n$ rangée par valeurs croissantes $x_{(1)}\le\dots\le x_{(n)}$.</t>
+        </is>
+      </c>
+      <c r="H615" s="10" t="inlineStr">
+        <is>
+          <t>Définir la médiane (selon la parité de $n$), puis les quartiles et déciles.</t>
+        </is>
+      </c>
+      <c r="I615" s="9" t="inlineStr">
+        <is>
+          <t>Médiane : valeur telle qu'au moins la moitié des individus ont une valeur inférieure ou égale et au moins la moitié une valeur supérieure ou égale. $n$ impair : $x_{((n+1)/2)}$ (individu médian) ; $n$ pair : $\frac12\big(x_{(n/2)}+x_{(n/2+1)}\big)$. Quartiles $Q_1$, $Q_3$ (déciles $D_1$, $D_9$) : valeurs où la fréquence cumulée atteint $25\,\%$, $75\,\%$ ($10\,\%$, $90\,\%$), lues sur le polygone des fréquences cumulées.</t>
+        </is>
+      </c>
+      <c r="J615" s="9" t="inlineStr">
+        <is>
+          <t>Programme Statistique 1 : « médiane … Modalité de l'individu médian ou moyenne des modalités des deux individus médians selon la parité de n » ; « quartiles, déciles (calculs à partir du polygone des effectifs cumulés ou des fréquences cumulées). »</t>
+        </is>
+      </c>
+      <c r="K615" s="9" t="n"/>
+      <c r="L615" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Statistiques »</t>
+        </is>
+      </c>
+      <c r="M615" s="11" t="n"/>
+      <c r="N615" s="11" t="n"/>
+    </row>
+    <row r="616">
+      <c r="A616" s="9" t="inlineStr">
+        <is>
+          <t>M616</t>
+        </is>
+      </c>
+      <c r="B616" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C616" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D616" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Statistique 1</t>
+        </is>
+      </c>
+      <c r="E616" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F616" s="9" t="inlineStr">
+        <is>
+          <t>Variance, écart-type, étendue</t>
+        </is>
+      </c>
+      <c r="G616" s="9" t="inlineStr">
+        <is>
+          <t>Soit une série $(x_1,\dots,x_n)$ de moyenne $\bar x$.</t>
+        </is>
+      </c>
+      <c r="H616" s="10" t="inlineStr">
+        <is>
+          <t>Définir l'étendue, la variance $s_x^2$ et l'écart-type $s_x$. Énoncer la formule de König-Huygens.</t>
+        </is>
+      </c>
+      <c r="I616" s="9" t="inlineStr">
+        <is>
+          <t>Étendue : $\max x_i-\min x_i$. $s_x^2=\dfrac1n\sum_{i=1}^n(x_i-\bar x)^2$ (moyenne des carrés des écarts à la moyenne) $=\dfrac1n\sum_jn_j(a_j-\bar x)^2$ ; $s_x=\sqrt{s_x^2}$. König-Huygens : $s_x^2=\overline{x^2}-\bar x^2=\dfrac1n\sum x_i^2-\bar x^2$.</t>
+        </is>
+      </c>
+      <c r="J616" s="9" t="inlineStr">
+        <is>
+          <t>Programme Statistique 1 : « Caractéristiques (empiriques) de dispersion : variance $s_x^2$ et écart-type $s_x$. La formule avec le facteur $\frac1{n-1}$ n'est pas un attendu du programme. »</t>
+        </is>
+      </c>
+      <c r="K616" s="9" t="n"/>
+      <c r="L616" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Statistiques »</t>
+        </is>
+      </c>
+      <c r="M616" s="11" t="n"/>
+      <c r="N616" s="11" t="n"/>
+    </row>
+    <row r="617">
+      <c r="A617" s="9" t="inlineStr">
+        <is>
+          <t>M617</t>
+        </is>
+      </c>
+      <c r="B617" s="10" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C617" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D617" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Statistique 1</t>
+        </is>
+      </c>
+      <c r="E617" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F617" s="9" t="inlineStr">
+        <is>
+          <t>Changement affine de caractère</t>
+        </is>
+      </c>
+      <c r="G617" s="9" t="inlineStr">
+        <is>
+          <t>Soient $(a,b)\in\mathbb R^2$ et $y_i=ax_i+b$ pour tout $i$.</t>
+        </is>
+      </c>
+      <c r="H617" s="10" t="inlineStr">
+        <is>
+          <t>Exprimer $\bar y$, $s_y^2$ et $s_y$ en fonction de ceux de $x$.</t>
+        </is>
+      </c>
+      <c r="I617" s="9" t="inlineStr">
+        <is>
+          <t>$\bar y=a\bar x+b$ ; $s_y^2=a^2s_x^2$ ; $s_y=|a|s_x$ (une translation ne change pas la dispersion).</t>
+        </is>
+      </c>
+      <c r="J617" s="9" t="inlineStr">
+        <is>
+          <t>Propriétés du cours ; non citées par le programme.</t>
+        </is>
+      </c>
+      <c r="K617" s="9" t="n"/>
+      <c r="L617" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Statistiques »</t>
+        </is>
+      </c>
+      <c r="M617" s="11" t="n"/>
+      <c r="N617" s="11" t="n"/>
+    </row>
+    <row r="618">
+      <c r="A618" s="9" t="inlineStr">
+        <is>
+          <t>M618</t>
+        </is>
+      </c>
+      <c r="B618" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C618" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D618" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Statistique 1</t>
+        </is>
+      </c>
+      <c r="E618" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F618" s="9" t="inlineStr">
+        <is>
+          <t>Série double : point moyen et covariance</t>
+        </is>
+      </c>
+      <c r="G618" s="9" t="inlineStr">
+        <is>
+          <t>Soit une série double $((x_1,y_1),\dots,(x_n,y_n))$.</t>
+        </is>
+      </c>
+      <c r="H618" s="10" t="inlineStr">
+        <is>
+          <t>Définir le point moyen du nuage et la covariance $s_{xy}$. Énoncer la formule de König-Huygens pour la covariance.</t>
+        </is>
+      </c>
+      <c r="I618" s="9" t="inlineStr">
+        <is>
+          <t>Point moyen : $G(\bar x,\bar y)$. $s_{xy}=\dfrac1n\sum_{i=1}^n(x_i-\bar x)(y_i-\bar y)$. König-Huygens : $s_{xy}=\overline{xy}-\bar x\,\bar y=\dfrac1n\sum x_iy_i-\bar x\bar y$ (moyenne du produit moins produit des moyennes). $s_{xx}=s_x^2$.</t>
+        </is>
+      </c>
+      <c r="J618" s="9" t="inlineStr">
+        <is>
+          <t>Programme Statistique 1 : « Représentation par un nuage de points de ℝ². Point moyen $(\bar x,\bar y)$ du nuage. Caractéristiques d'une série statistique double : covariance $s_{xy}$. »</t>
+        </is>
+      </c>
+      <c r="K618" s="9" t="n"/>
+      <c r="L618" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Statistiques »</t>
+        </is>
+      </c>
+      <c r="M618" s="11" t="n"/>
+      <c r="N618" s="11" t="n"/>
+    </row>
+    <row r="619">
+      <c r="A619" s="9" t="inlineStr">
+        <is>
+          <t>M619</t>
+        </is>
+      </c>
+      <c r="B619" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C619" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D619" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Statistique 1</t>
+        </is>
+      </c>
+      <c r="E619" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F619" s="9" t="inlineStr">
+        <is>
+          <t>Coefficient de corrélation linéaire</t>
+        </is>
+      </c>
+      <c r="G619" s="9" t="inlineStr">
+        <is>
+          <t>Soit une série double de caractères $x$, $y$ non constants.</t>
+        </is>
+      </c>
+      <c r="H619" s="10" t="inlineStr">
+        <is>
+          <t>Définir $r_{xy}$. Quelles sont ses valeurs possibles et son interprétation ?</t>
+        </is>
+      </c>
+      <c r="I619" s="9" t="inlineStr">
+        <is>
+          <t>$r_{xy}=\dfrac{s_{xy}}{s_xs_y}$, sans unité, avec $-1\le r_{xy}\le1$. $|r_{xy}|$ proche de $1$ : nuage presque aligné (relation presque affine), droite de pente du signe de $r_{xy}$ ; $r_{xy}$ proche de $0$ : pas de lien affine (il peut exister un lien non affine).</t>
+        </is>
+      </c>
+      <c r="J619" s="9" t="inlineStr">
+        <is>
+          <t>Programme Statistique 1 : « coefficient de corrélation $r_{xy}$ ».</t>
+        </is>
+      </c>
+      <c r="K619" s="9" t="n"/>
+      <c r="L619" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Statistiques »</t>
+        </is>
+      </c>
+      <c r="M619" s="11" t="n"/>
+      <c r="N619" s="11" t="n"/>
+    </row>
+    <row r="620">
+      <c r="A620" s="9" t="inlineStr">
+        <is>
+          <t>M620</t>
+        </is>
+      </c>
+      <c r="B620" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C620" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D620" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Statistique 1</t>
+        </is>
+      </c>
+      <c r="E620" s="9" t="inlineStr">
+        <is>
+          <t>Théorème</t>
+        </is>
+      </c>
+      <c r="F620" s="9" t="inlineStr">
+        <is>
+          <t>Ajustement affine par les moindres carrés</t>
+        </is>
+      </c>
+      <c r="G620" s="9" t="inlineStr">
+        <is>
+          <t>Soit une série double $(x_i,y_i)_{1\le i\le n}$ avec $x$ non constant.</t>
+        </is>
+      </c>
+      <c r="H620" s="10" t="inlineStr">
+        <is>
+          <t>Quelle est la droite de régression de $y$ en $x$ ? Que faire si le nuage n'est pas allongé selon une droite ?</t>
+        </is>
+      </c>
+      <c r="I620" s="9" t="inlineStr">
+        <is>
+          <t>La droite $y=ax+b$ qui minimise $\sum_{i=1}^n\big(y_i-(ax_i+b)\big)^2$ a pour coefficients $a=\dfrac{s_{xy}}{s_x^2}$ et $b=\bar y-a\bar x$ : elle passe par le point moyen $G(\bar x,\bar y)$. Si le nuage n'est pas « affine », on change de variable (par exemple $z=\ln y$ pour une croissance exponentielle) avant d'ajuster.</t>
+        </is>
+      </c>
+      <c r="J620" s="9" t="inlineStr">
+        <is>
+          <t>Programme Statistique 1 : « Approche descriptive de l'ajustement affine selon la méthode des moindres carrés. L'optimalité de l'ajustement est admise » ; « changements de variables ».</t>
+        </is>
+      </c>
+      <c r="K620" s="9" t="n"/>
+      <c r="L620" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Statistiques »</t>
+        </is>
+      </c>
+      <c r="M620" s="11" t="n"/>
+      <c r="N620" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M610" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M620" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -40032,7 +40632,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$610,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$620,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -40047,7 +40647,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$610,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$620,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -40062,7 +40662,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$610,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$620,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -40089,7 +40689,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$610)</f>
+        <f>COUNTA(Fiches!$M$2:$M$620)</f>
         <v/>
       </c>
     </row>
@@ -40135,15 +40735,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A13,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A13,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A13,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A13,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A13,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A13,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -40158,15 +40758,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A14,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A14,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A14,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A14,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A14,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A14,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -40181,15 +40781,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A15,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A15,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A15,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A15,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A15,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A15,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -40204,15 +40804,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A16,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A16,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A16,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A16,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A16,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A16,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -40227,15 +40827,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A17,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A17,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A17,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A17,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A17,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A17,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -40250,15 +40850,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A18,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A18,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A18,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A18,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A18,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A18,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -40273,15 +40873,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A19,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A19,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A19,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A19,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A19,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A19,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -40296,15 +40896,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A20,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A20,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A20,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A20,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A20,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A20,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -40319,15 +40919,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A21,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A21,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A21,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A21,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A21,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A21,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -40342,15 +40942,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A22,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A22,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A22,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A22,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A22,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A22,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -40365,15 +40965,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A23,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A23,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A23,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A23,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A23,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A23,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -40388,15 +40988,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A24,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A24,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A24,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A24,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A24,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A24,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -40411,15 +41011,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A25,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A25,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A25,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A25,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A25,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A25,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -40434,15 +41034,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A26,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A26,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A26,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A26,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A26,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A26,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -40457,15 +41057,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A27,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A27,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A27,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A27,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A27,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A27,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -40480,15 +41080,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A28,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A28,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A28,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A28,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A28,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A28,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -40503,15 +41103,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A29,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A29,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A29,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A29,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A29,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A29,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -40526,15 +41126,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A30,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A30,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A30,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A30,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A30,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A30,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -40549,15 +41149,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A31,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A31,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A31,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A31,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A31,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A31,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -40572,15 +41172,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A32,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A32,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A32,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A32,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A32,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A32,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -40595,15 +41195,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A33,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A33,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A33,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A33,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A33,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A33,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -40618,15 +41218,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A34,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A34,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A34,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A34,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A34,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A34,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -40641,15 +41241,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A35,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A35,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A35,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A35,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A35,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A35,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -40664,15 +41264,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A36,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A36,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A36,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A36,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A36,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A36,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -40687,15 +41287,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A37,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A37,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A37,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A37,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A37,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A37,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -40710,15 +41310,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A38,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A38,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A38,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A38,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A38,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A38,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -40733,15 +41333,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A39,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A39,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A39,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A39,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A39,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A39,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -40756,15 +41356,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A40,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A40,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A40,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A40,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A40,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A40,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -40779,15 +41379,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A41,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A41,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A41,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A41,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A41,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A41,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -40802,15 +41402,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A42,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A42,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A42,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A42,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A42,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A42,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -40825,15 +41425,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A43,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A43,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A43,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A43,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A43,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A43,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -40848,15 +41448,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A44,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A44,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A44,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A44,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A44,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A44,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -40871,15 +41471,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A45,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A45,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A45,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A45,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A45,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A45,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -40894,15 +41494,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A46,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A46,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A46,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A46,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A46,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A46,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -40917,15 +41517,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A47,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A47,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A47,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A47,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A47,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A47,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -40940,15 +41540,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A48,Fiches!$B$2:$B$610,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A48,Fiches!$B$2:$B$620,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A48,Fiches!$B$2:$B$610,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A48,Fiches!$B$2:$B$620,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$610,$A48,Fiches!$B$2:$B$610,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$620,$A48,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Trigonométrie : équations cos x = c, sin x = s, tan x = t
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N620"/>
+  <dimension ref="A1:N621"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -37086,10 +37086,70 @@
       <c r="M620" s="11" t="n"/>
       <c r="N620" s="11" t="n"/>
     </row>
+    <row r="621">
+      <c r="A621" s="9" t="inlineStr">
+        <is>
+          <t>M621</t>
+        </is>
+      </c>
+      <c r="B621" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C621" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D621" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Outils 3 – Trigonométrie</t>
+        </is>
+      </c>
+      <c r="E621" s="9" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+      <c r="F621" s="9" t="inlineStr">
+        <is>
+          <t>Équations trigonométriques cos x = c, sin x = s, tan x = t</t>
+        </is>
+      </c>
+      <c r="G621" s="9" t="inlineStr">
+        <is>
+          <t>Soient $a$ un réel et $x$ l'inconnue réelle.</t>
+        </is>
+      </c>
+      <c r="H621" s="10" t="inlineStr">
+        <is>
+          <t>Résoudre $\cos x=\cos a$, $\sin x=\sin a$, $\tan x=\tan a$. Comment exprimer une solution de $\cos x=c$, $\sin x=s$, $\tan x=t$ ?</t>
+        </is>
+      </c>
+      <c r="I621" s="9" t="inlineStr">
+        <is>
+          <t>$\cos x=\cos a\iff x\equiv a\ [2\pi]$ ou $x\equiv-a\ [2\pi]$ ; $\sin x=\sin a\iff x\equiv a\ [2\pi]$ ou $x\equiv\pi-a\ [2\pi]$ ; $\tan x=\tan a\iff x\equiv a\ [\pi]$ (avec $x,a\not\equiv\frac\pi2\ [\pi]$). Pour $c\in[-1,1]$, $\arccos c$ est l'unique solution de $\cos x=c$ dans $[0,\pi]$ ; pour $s\in[-1,1]$, $\arcsin s$ l'unique solution de $\sin x=s$ dans $[-\frac\pi2,\frac\pi2]$ ; pour $t\in\mathbb R$, $\arctan t$ l'unique solution de $\tan x=t$ dans $]-\frac\pi2,\frac\pi2[$.</t>
+        </is>
+      </c>
+      <c r="J621" s="9" t="inlineStr">
+        <is>
+          <t>Programme Outils 3 : « Résolution d'équations trigonométriques simples : cos(x) = c, sin(x) = s et tan(x) = t. Notations arccos, arcsin, arctan … définitions en termes de solutions d'équations dans certains intervalles. »</t>
+        </is>
+      </c>
+      <c r="K621" s="9" t="n"/>
+      <c r="L621" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le TD « Trigonométrie »</t>
+        </is>
+      </c>
+      <c r="M621" s="11" t="n"/>
+      <c r="N621" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M620" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M621" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -40632,7 +40692,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$620,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$621,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -40647,7 +40707,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$620,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$621,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -40662,7 +40722,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$620,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$621,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -40689,7 +40749,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$620)</f>
+        <f>COUNTA(Fiches!$M$2:$M$621)</f>
         <v/>
       </c>
     </row>
@@ -40735,15 +40795,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A13,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A13,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A13,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A13,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A13,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A13,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -40758,15 +40818,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A14,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A14,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A14,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A14,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A14,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A14,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -40781,15 +40841,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A15,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A15,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A15,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A15,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A15,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A15,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -40804,15 +40864,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A16,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A16,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A16,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A16,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A16,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A16,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -40827,15 +40887,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A17,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A17,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A17,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A17,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A17,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A17,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -40850,15 +40910,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A18,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A18,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A18,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A18,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A18,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A18,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -40873,15 +40933,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A19,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A19,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A19,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A19,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A19,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A19,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -40896,15 +40956,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A20,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A20,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A20,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A20,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A20,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A20,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -40919,15 +40979,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A21,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A21,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A21,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A21,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A21,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A21,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -40942,15 +41002,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A22,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A22,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A22,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A22,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A22,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A22,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -40965,15 +41025,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A23,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A23,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A23,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A23,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A23,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A23,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -40988,15 +41048,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A24,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A24,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A24,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A24,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A24,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A24,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -41011,15 +41071,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A25,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A25,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A25,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A25,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A25,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A25,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -41034,15 +41094,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A26,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A26,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A26,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A26,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A26,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A26,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -41057,15 +41117,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A27,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A27,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A27,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A27,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A27,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A27,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -41080,15 +41140,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A28,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A28,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A28,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A28,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A28,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A28,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -41103,15 +41163,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A29,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A29,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A29,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A29,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A29,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A29,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -41126,15 +41186,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A30,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A30,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A30,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A30,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A30,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A30,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -41149,15 +41209,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A31,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A31,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A31,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A31,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A31,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A31,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -41172,15 +41232,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A32,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A32,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A32,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A32,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A32,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A32,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -41195,15 +41255,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A33,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A33,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A33,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A33,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A33,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A33,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -41218,15 +41278,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A34,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A34,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A34,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A34,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A34,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A34,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -41241,15 +41301,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A35,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A35,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A35,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A35,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A35,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A35,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -41264,15 +41324,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A36,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A36,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A36,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A36,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A36,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A36,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -41287,15 +41347,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A37,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A37,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A37,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A37,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A37,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A37,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -41310,15 +41370,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A38,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A38,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A38,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A38,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A38,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A38,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -41333,15 +41393,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A39,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A39,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A39,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A39,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A39,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A39,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -41356,15 +41416,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A40,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A40,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A40,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A40,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A40,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A40,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -41379,15 +41439,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A41,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A41,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A41,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A41,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A41,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A41,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -41402,15 +41462,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A42,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A42,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A42,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A42,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A42,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A42,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -41425,15 +41485,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A43,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A43,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A43,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A43,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A43,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A43,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -41448,15 +41508,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A44,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A44,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A44,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A44,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A44,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A44,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -41471,15 +41531,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A45,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A45,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A45,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A45,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A45,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A45,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -41494,15 +41554,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A46,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A46,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A46,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A46,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A46,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A46,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -41517,15 +41577,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A47,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A47,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A47,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A47,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A47,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A47,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -41540,15 +41600,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A48,Fiches!$B$2:$B$620,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A48,Fiches!$B$2:$B$621,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A48,Fiches!$B$2:$B$620,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A48,Fiches!$B$2:$B$621,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$620,$A48,Fiches!$B$2:$B$620,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$621,$A48,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Variables aléatoires finies : loi, indicatrices, répartition, espérance, variance, indépendance
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N621"/>
+  <dimension ref="A1:N628"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -37146,10 +37146,430 @@
       <c r="M621" s="11" t="n"/>
       <c r="N621" s="11" t="n"/>
     </row>
+    <row r="622">
+      <c r="A622" s="9" t="inlineStr">
+        <is>
+          <t>M622</t>
+        </is>
+      </c>
+      <c r="B622" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C622" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D622" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Probabilités 2 – Variables sur un univers fini</t>
+        </is>
+      </c>
+      <c r="E622" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F622" s="9" t="inlineStr">
+        <is>
+          <t>Variable aléatoire finie et sa loi</t>
+        </is>
+      </c>
+      <c r="G622" s="9" t="inlineStr">
+        <is>
+          <t>Soit $(\Omega,P)$ un espace probabilisé fini.</t>
+        </is>
+      </c>
+      <c r="H622" s="10" t="inlineStr">
+        <is>
+          <t>Qu'est-ce qu'une variable aléatoire $X$ sur $\Omega$ ? Que désignent $(X\in I)$, $(X=x)$ ? Qu'est-ce que la loi de $X$ ?</t>
+        </is>
+      </c>
+      <c r="I622" s="9" t="inlineStr">
+        <is>
+          <t>Une application $X:\Omega\to\mathbb R$. $(X\in I)=\{\omega\in\Omega,\ X(\omega)\in I\}$, $(X=x)$, $(X\le x)$… sont des événements. La famille $(X=x)_{x\in X(\Omega)}$ est un système complet d'événements. Loi de $X$ : la donnée de $X(\Omega)$ et des $P(X=x)$, $x\in X(\Omega)$, avec $\sum_{x\in X(\Omega)}P(X=x)=1$.</t>
+        </is>
+      </c>
+      <c r="J622" s="9" t="inlineStr">
+        <is>
+          <t>Programme Probabilités 2 : « On nomme variable aléatoire sur un univers Ω (fini) toute application de Ω dans ℝ » ; « Système complet d'événements $(X=x)$ » ; « La loi … est l'application $x\mapsto P(X=x)$. »</t>
+        </is>
+      </c>
+      <c r="K622" s="9" t="n"/>
+      <c r="L622" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Variables aléatoires »</t>
+        </is>
+      </c>
+      <c r="M622" s="11" t="n"/>
+      <c r="N622" s="11" t="n"/>
+    </row>
+    <row r="623">
+      <c r="A623" s="9" t="inlineStr">
+        <is>
+          <t>M623</t>
+        </is>
+      </c>
+      <c r="B623" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C623" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D623" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Probabilités 2 – Variables sur un univers fini</t>
+        </is>
+      </c>
+      <c r="E623" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F623" s="9" t="inlineStr">
+        <is>
+          <t>Variables indicatrices</t>
+        </is>
+      </c>
+      <c r="G623" s="9" t="inlineStr">
+        <is>
+          <t>Soient $A$ et $B$ deux événements de $\Omega$.</t>
+        </is>
+      </c>
+      <c r="H623" s="10" t="inlineStr">
+        <is>
+          <t>Définir $\mathbb 1_A$. Exprimer $\mathbb 1_{A\cap B}$, $\mathbb 1_{\bar A}$, $\mathbb 1_{A\cup B}$. Quelle est la loi de $\mathbb 1_A$ et son espérance ?</t>
+        </is>
+      </c>
+      <c r="I623" s="9" t="inlineStr">
+        <is>
+          <t>$\mathbb 1_A(\omega)=1$ si $\omega\in A$, $0$ sinon. $\mathbb 1_{A\cap B}=\mathbb 1_A\mathbb 1_B=\min(\mathbb 1_A,\mathbb 1_B)$ ; $\mathbb 1_{\bar A}=1-\mathbb 1_A$ ; $\mathbb 1_{A\cup B}=\max(\mathbb 1_A,\mathbb 1_B)=\mathbb 1_A+\mathbb 1_B-\mathbb 1_A\mathbb 1_B$. $\mathbb 1_A\sim\mathcal B(P(A))$, donc $E(\mathbb 1_A)=P(A)$.</t>
+        </is>
+      </c>
+      <c r="J623" s="9" t="inlineStr">
+        <is>
+          <t>Programme Probabilités 2 : « Exemple des fonctions indicatrices. Notation $\mathbb 1_A$. Règles de calcul : intersection, union, complémentaire » ; « $E(\mathbb 1_A)=P(A)$ ».</t>
+        </is>
+      </c>
+      <c r="K623" s="9" t="n"/>
+      <c r="L623" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Variables aléatoires »</t>
+        </is>
+      </c>
+      <c r="M623" s="11" t="n"/>
+      <c r="N623" s="11" t="n"/>
+    </row>
+    <row r="624">
+      <c r="A624" s="9" t="inlineStr">
+        <is>
+          <t>M624</t>
+        </is>
+      </c>
+      <c r="B624" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C624" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D624" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Probabilités 2 – Variables sur un univers fini</t>
+        </is>
+      </c>
+      <c r="E624" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F624" s="9" t="inlineStr">
+        <is>
+          <t>Fonction de répartition d’une variable finie</t>
+        </is>
+      </c>
+      <c r="G624" s="9" t="inlineStr">
+        <is>
+          <t>Soit $X$ une variable aléatoire finie.</t>
+        </is>
+      </c>
+      <c r="H624" s="10" t="inlineStr">
+        <is>
+          <t>Définir $F_X$. Quelle est son allure ? Comment retrouver la loi de $X$ à partir de $F_X$ ?</t>
+        </is>
+      </c>
+      <c r="I624" s="9" t="inlineStr">
+        <is>
+          <t>$F_X(t)=P(X\le t)=\sum_{x\in X(\Omega),\,x\le t}P(X=x)$ pour $t\in\mathbb R$. C'est une fonction en escalier croissante, nulle avant la plus petite valeur, égale à $1$ après la plus grande ; elle saute en chaque $x\in X(\Omega)$ d'une hauteur $P(X=x)$. Si $x_1&lt;\dots&lt;x_n$ sont les valeurs : $P(X=x_1)=F_X(x_1)$, $P(X=x_i)=F_X(x_i)-F_X(x_{i-1})$ ; $P(a&lt;X\le b)=F_X(b)-F_X(a)$.</t>
+        </is>
+      </c>
+      <c r="J624" s="9" t="inlineStr">
+        <is>
+          <t>Programme Probabilités 2 : « La fonction de répartition de $X$ … $F_X(t)=P(X\le t)$ … représentation en escaliers. Les étudiants doivent savoir déterminer la loi d'une variable aléatoire à partir de sa fonction de répartition. »</t>
+        </is>
+      </c>
+      <c r="K624" s="9" t="n"/>
+      <c r="L624" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Variables aléatoires »</t>
+        </is>
+      </c>
+      <c r="M624" s="11" t="n"/>
+      <c r="N624" s="11" t="n"/>
+    </row>
+    <row r="625">
+      <c r="A625" s="9" t="inlineStr">
+        <is>
+          <t>M625</t>
+        </is>
+      </c>
+      <c r="B625" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C625" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D625" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Probabilités 2 – Variables sur un univers fini</t>
+        </is>
+      </c>
+      <c r="E625" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F625" s="9" t="inlineStr">
+        <is>
+          <t>Espérance : définition et propriétés</t>
+        </is>
+      </c>
+      <c r="G625" s="9" t="inlineStr">
+        <is>
+          <t>Soient $X$, $Y$ des variables aléatoires finies, $a,b\in\mathbb R$ et $u$ une fonction définie sur $X(\Omega)$.</t>
+        </is>
+      </c>
+      <c r="H625" s="10" t="inlineStr">
+        <is>
+          <t>Définir $E(X)$. Donner ses propriétés (linéarité, positivité, croissance) et le théorème de transfert.</t>
+        </is>
+      </c>
+      <c r="I625" s="9" t="inlineStr">
+        <is>
+          <t>$E(X)=\sum_{x\in X(\Omega)}xP(X=x)$ (moyenne des valeurs pondérée par leurs probabilités). Linéarité : $E(aX+bY)=aE(X)+bE(Y)$ ; positivité : $X\ge0\Rightarrow E(X)\ge0$ ; croissance : $X\le Y\Rightarrow E(X)\le E(Y)$. Transfert : $E(u(X))=\sum_{x\in X(\Omega)}u(x)P(X=x)$ (ex. $E(X^2)=\sum x^2P(X=x)$). $X$ est centrée si $E(X)=0$.</t>
+        </is>
+      </c>
+      <c r="J625" s="9" t="inlineStr">
+        <is>
+          <t>Programme Probabilités 2 : « Espérance … variable aléatoire centrée. On démontre que l'espérance est positive et croissante. La linéarité est énoncée » ; « Théorème de transfert. »</t>
+        </is>
+      </c>
+      <c r="K625" s="9" t="n"/>
+      <c r="L625" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Variables aléatoires »</t>
+        </is>
+      </c>
+      <c r="M625" s="11" t="n"/>
+      <c r="N625" s="11" t="n"/>
+    </row>
+    <row r="626">
+      <c r="A626" s="9" t="inlineStr">
+        <is>
+          <t>M626</t>
+        </is>
+      </c>
+      <c r="B626" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C626" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D626" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Probabilités 2 – Variables sur un univers fini</t>
+        </is>
+      </c>
+      <c r="E626" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F626" s="9" t="inlineStr">
+        <is>
+          <t>Variance, écart-type, variable centrée réduite</t>
+        </is>
+      </c>
+      <c r="G626" s="9" t="inlineStr">
+        <is>
+          <t>Soit $X$ une variable aléatoire finie.</t>
+        </is>
+      </c>
+      <c r="H626" s="10" t="inlineStr">
+        <is>
+          <t>Définir $V(X)$ et $\sigma(X)$. Énoncer la formule de König-Huygens. Qu'est-ce qu'une variable centrée réduite ?</t>
+        </is>
+      </c>
+      <c r="I626" s="9" t="inlineStr">
+        <is>
+          <t>$V(X)=E\big((X-E(X))^2\big)=\sum_x(x-E(X))^2P(X=x)\ge0$ ; $\sigma(X)=\sqrt{V(X)}$ (même unité que $X$). König-Huygens : $V(X)=E(X^2)-E(X)^2$. $V(aX+b)=a^2V(X)$. Centrée réduite : $E(X)=0$ et $V(X)=1$ ; si $\sigma(X)&gt;0$, $\dfrac{X-E(X)}{\sigma(X)}$ est centrée réduite.</t>
+        </is>
+      </c>
+      <c r="J626" s="9" t="inlineStr">
+        <is>
+          <t>Programme Probabilités 2 : « Moments. Variance V(X). Formule de König-Huygens. Écart-type σ(X). V(aX+b)=a²V(X). Variable centrée réduite. »</t>
+        </is>
+      </c>
+      <c r="K626" s="9" t="n"/>
+      <c r="L626" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Variables aléatoires »</t>
+        </is>
+      </c>
+      <c r="M626" s="11" t="n"/>
+      <c r="N626" s="11" t="n"/>
+    </row>
+    <row r="627">
+      <c r="A627" s="9" t="inlineStr">
+        <is>
+          <t>M627</t>
+        </is>
+      </c>
+      <c r="B627" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C627" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D627" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Probabilités 2 – Variables sur un univers fini</t>
+        </is>
+      </c>
+      <c r="E627" s="9" t="inlineStr">
+        <is>
+          <t>Définition</t>
+        </is>
+      </c>
+      <c r="F627" s="9" t="inlineStr">
+        <is>
+          <t>Indépendance de variables aléatoires finies</t>
+        </is>
+      </c>
+      <c r="G627" s="9" t="inlineStr">
+        <is>
+          <t>Soient $X$, $Y$ (et $X_1,\dots,X_n$) des variables aléatoires finies sur $\Omega$.</t>
+        </is>
+      </c>
+      <c r="H627" s="10" t="inlineStr">
+        <is>
+          <t>Définir l'indépendance de $X$ et $Y$, puis l'indépendance mutuelle de $X_1,\dots,X_n$. Que vaut alors $E(XY)$, $V(X+Y)$ ?</t>
+        </is>
+      </c>
+      <c r="I627" s="9" t="inlineStr">
+        <is>
+          <t>$X$ et $Y$ indépendantes : $\forall(x,y)\in X(\Omega)\times Y(\Omega)$, $P\big((X=x)\cap(Y=y)\big)=P(X=x)P(Y=y)$. Mutuellement indépendantes : $P\big(\bigcap_i(X_i=x_i)\big)=\prod_iP(X_i=x_i)$ pour tous $x_i\in X_i(\Omega)$. Si $X$, $Y$ indépendantes : $E(XY)=E(X)E(Y)$ et $V(X+Y)=V(X)+V(Y)$ ; plus généralement $V(X_1+\dots+X_n)=\sum V(X_i)$ si les $X_i$ sont indépendantes.</t>
+        </is>
+      </c>
+      <c r="J627" s="9" t="inlineStr">
+        <is>
+          <t>Programme Probabilités 2 : « Indépendance de deux variables aléatoires » ; « Généralisation : indépendance (mutuelle) de n variables aléatoires » ; « Si X et Y sont indépendantes, espérance de XY et variance de X+Y. Généralisation au cas de n variables. »</t>
+        </is>
+      </c>
+      <c r="K627" s="9" t="n"/>
+      <c r="L627" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Variables aléatoires »</t>
+        </is>
+      </c>
+      <c r="M627" s="11" t="n"/>
+      <c r="N627" s="11" t="n"/>
+    </row>
+    <row r="628">
+      <c r="A628" s="9" t="inlineStr">
+        <is>
+          <t>M628</t>
+        </is>
+      </c>
+      <c r="B628" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C628" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1</t>
+        </is>
+      </c>
+      <c r="D628" s="9" t="inlineStr">
+        <is>
+          <t>BCPST1 · Probabilités 2 – Variables sur un univers fini</t>
+        </is>
+      </c>
+      <c r="E628" s="9" t="inlineStr">
+        <is>
+          <t>Propriété</t>
+        </is>
+      </c>
+      <c r="F628" s="9" t="inlineStr">
+        <is>
+          <t>Sous-familles et lemme des coalitions</t>
+        </is>
+      </c>
+      <c r="G628" s="9" t="inlineStr">
+        <is>
+          <t>Soient $X_1,\dots,X_n,X_{n+1},\dots,X_{n+p}$ des variables aléatoires mutuellement indépendantes.</t>
+        </is>
+      </c>
+      <c r="H628" s="10" t="inlineStr">
+        <is>
+          <t>Que dire d'une sous-famille ? Énoncer le lemme des coalitions.</t>
+        </is>
+      </c>
+      <c r="I628" s="9" t="inlineStr">
+        <is>
+          <t>Toute sous-famille est formée de variables mutuellement indépendantes. Lemme des coalitions : $u(X_1,\dots,X_n)$ et $v(X_{n+1},\dots,X_{n+p})$ sont indépendantes ; plus généralement $u_1(X_1),\dots,u_n(X_n)$ sont mutuellement indépendantes.</t>
+        </is>
+      </c>
+      <c r="J628" s="9" t="inlineStr">
+        <is>
+          <t>Programme Probabilités 2 : « Propriétés de l'indépendance mutuelle (admises) : toute sous-famille … ; lemme des coalitions. »</t>
+        </is>
+      </c>
+      <c r="K628" s="9" t="n"/>
+      <c r="L628" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le cours « Variables aléatoires »</t>
+        </is>
+      </c>
+      <c r="M628" s="11" t="n"/>
+      <c r="N628" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N461"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M621" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M628" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -40692,7 +41112,7 @@
         </is>
       </c>
       <c r="B4" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$621,A4)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$628,A4)</f>
         <v/>
       </c>
       <c r="C4" s="22">
@@ -40707,7 +41127,7 @@
         </is>
       </c>
       <c r="B5" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$621,A5)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$628,A5)</f>
         <v/>
       </c>
       <c r="C5" s="22">
@@ -40722,7 +41142,7 @@
         </is>
       </c>
       <c r="B6" s="21">
-        <f>COUNTIF(Fiches!$B$2:$B$621,A6)</f>
+        <f>COUNTIF(Fiches!$B$2:$B$628,A6)</f>
         <v/>
       </c>
       <c r="C6" s="22">
@@ -40749,7 +41169,7 @@
         </is>
       </c>
       <c r="B9" s="21">
-        <f>COUNTA(Fiches!$M$2:$M$621)</f>
+        <f>COUNTA(Fiches!$M$2:$M$628)</f>
         <v/>
       </c>
     </row>
@@ -40795,15 +41215,15 @@
         </is>
       </c>
       <c r="B13" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A13,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A13,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C13" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A13,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A13,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D13" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A13,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A13,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E13" s="25">
@@ -40818,15 +41238,15 @@
         </is>
       </c>
       <c r="B14" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A14,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A14,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C14" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A14,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A14,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D14" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A14,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A14,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E14" s="25">
@@ -40841,15 +41261,15 @@
         </is>
       </c>
       <c r="B15" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A15,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A15,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C15" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A15,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A15,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D15" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A15,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A15,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E15" s="25">
@@ -40864,15 +41284,15 @@
         </is>
       </c>
       <c r="B16" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A16,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A16,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C16" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A16,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A16,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D16" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A16,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A16,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E16" s="25">
@@ -40887,15 +41307,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A17,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A17,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C17" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A17,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A17,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D17" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A17,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A17,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E17" s="25">
@@ -40910,15 +41330,15 @@
         </is>
       </c>
       <c r="B18" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A18,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A18,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C18" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A18,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A18,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D18" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A18,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A18,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E18" s="25">
@@ -40933,15 +41353,15 @@
         </is>
       </c>
       <c r="B19" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A19,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A19,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C19" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A19,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A19,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D19" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A19,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A19,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E19" s="25">
@@ -40956,15 +41376,15 @@
         </is>
       </c>
       <c r="B20" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A20,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A20,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C20" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A20,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A20,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D20" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A20,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A20,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E20" s="25">
@@ -40979,15 +41399,15 @@
         </is>
       </c>
       <c r="B21" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A21,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A21,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C21" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A21,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A21,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D21" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A21,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A21,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E21" s="25">
@@ -41002,15 +41422,15 @@
         </is>
       </c>
       <c r="B22" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A22,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A22,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C22" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A22,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A22,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D22" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A22,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A22,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E22" s="25">
@@ -41025,15 +41445,15 @@
         </is>
       </c>
       <c r="B23" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A23,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A23,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C23" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A23,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A23,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D23" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A23,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A23,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E23" s="25">
@@ -41048,15 +41468,15 @@
         </is>
       </c>
       <c r="B24" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A24,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A24,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C24" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A24,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A24,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D24" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A24,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A24,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E24" s="25">
@@ -41071,15 +41491,15 @@
         </is>
       </c>
       <c r="B25" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A25,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A25,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C25" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A25,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A25,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D25" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A25,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A25,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E25" s="25">
@@ -41094,15 +41514,15 @@
         </is>
       </c>
       <c r="B26" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A26,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A26,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C26" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A26,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A26,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D26" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A26,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A26,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E26" s="25">
@@ -41117,15 +41537,15 @@
         </is>
       </c>
       <c r="B27" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A27,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A27,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C27" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A27,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A27,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D27" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A27,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A27,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E27" s="25">
@@ -41140,15 +41560,15 @@
         </is>
       </c>
       <c r="B28" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A28,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A28,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C28" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A28,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A28,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D28" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A28,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A28,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E28" s="25">
@@ -41163,15 +41583,15 @@
         </is>
       </c>
       <c r="B29" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A29,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A29,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C29" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A29,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A29,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D29" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A29,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A29,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E29" s="25">
@@ -41186,15 +41606,15 @@
         </is>
       </c>
       <c r="B30" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A30,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A30,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C30" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A30,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A30,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D30" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A30,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A30,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E30" s="25">
@@ -41209,15 +41629,15 @@
         </is>
       </c>
       <c r="B31" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A31,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A31,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C31" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A31,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A31,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D31" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A31,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A31,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E31" s="25">
@@ -41232,15 +41652,15 @@
         </is>
       </c>
       <c r="B32" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A32,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A32,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C32" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A32,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A32,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D32" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A32,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A32,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E32" s="25">
@@ -41255,15 +41675,15 @@
         </is>
       </c>
       <c r="B33" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A33,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A33,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C33" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A33,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A33,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D33" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A33,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A33,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E33" s="25">
@@ -41278,15 +41698,15 @@
         </is>
       </c>
       <c r="B34" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A34,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A34,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C34" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A34,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A34,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D34" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A34,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A34,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E34" s="25">
@@ -41301,15 +41721,15 @@
         </is>
       </c>
       <c r="B35" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A35,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A35,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C35" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A35,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A35,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D35" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A35,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A35,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E35" s="25">
@@ -41324,15 +41744,15 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A36,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A36,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C36" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A36,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A36,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D36" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A36,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A36,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -41347,15 +41767,15 @@
         </is>
       </c>
       <c r="B37" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A37,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A37,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C37" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A37,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A37,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D37" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A37,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A37,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E37" s="25">
@@ -41370,15 +41790,15 @@
         </is>
       </c>
       <c r="B38" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A38,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A38,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C38" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A38,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A38,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D38" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A38,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A38,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E38" s="25">
@@ -41393,15 +41813,15 @@
         </is>
       </c>
       <c r="B39" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A39,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A39,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C39" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A39,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A39,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D39" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A39,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A39,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E39" s="25">
@@ -41416,15 +41836,15 @@
         </is>
       </c>
       <c r="B40" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A40,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A40,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C40" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A40,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A40,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D40" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A40,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A40,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E40" s="25">
@@ -41439,15 +41859,15 @@
         </is>
       </c>
       <c r="B41" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A41,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A41,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C41" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A41,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A41,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D41" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A41,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A41,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E41" s="25">
@@ -41462,15 +41882,15 @@
         </is>
       </c>
       <c r="B42" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A42,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A42,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C42" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A42,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A42,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D42" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A42,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A42,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E42" s="25">
@@ -41485,15 +41905,15 @@
         </is>
       </c>
       <c r="B43" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A43,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A43,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C43" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A43,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A43,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D43" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A43,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A43,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E43" s="25">
@@ -41508,15 +41928,15 @@
         </is>
       </c>
       <c r="B44" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A44,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A44,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C44" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A44,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A44,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D44" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A44,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A44,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E44" s="25">
@@ -41531,15 +41951,15 @@
         </is>
       </c>
       <c r="B45" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A45,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A45,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C45" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A45,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A45,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D45" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A45,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A45,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E45" s="25">
@@ -41554,15 +41974,15 @@
         </is>
       </c>
       <c r="B46" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A46,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A46,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C46" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A46,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A46,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D46" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A46,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A46,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E46" s="25">
@@ -41577,15 +41997,15 @@
         </is>
       </c>
       <c r="B47" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A47,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A47,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C47" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A47,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A47,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D47" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A47,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A47,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E47" s="25">
@@ -41600,15 +42020,15 @@
         </is>
       </c>
       <c r="B48" s="26">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A48,Fiches!$B$2:$B$621,"Noir – conforme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A48,Fiches!$B$2:$B$628,"Noir – conforme")</f>
         <v/>
       </c>
       <c r="C48" s="27">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A48,Fiches!$B$2:$B$621,"Orange – incertain")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A48,Fiches!$B$2:$B$628,"Orange – incertain")</f>
         <v/>
       </c>
       <c r="D48" s="28">
-        <f>COUNTIFS(Fiches!$D$2:$D$621,$A48,Fiches!$B$2:$B$621,"Rouge – hors programme")</f>
+        <f>COUNTIFS(Fiches!$D$2:$D$628,$A48,Fiches!$B$2:$B$628,"Rouge – hors programme")</f>
         <v/>
       </c>
       <c r="E48" s="25">

</xml_diff>

<commit_message>
Formulaire de trigonométrie : valeurs en π/2 et π, périodicité, tan(π/2−a), cos x = 0, sin x = 0
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -37583,7 +37583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M66"/>
+  <dimension ref="A1:M74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -41053,10 +41053,402 @@
       <c r="L66" s="14" t="n"/>
       <c r="M66" s="14" t="n"/>
     </row>
+    <row r="67">
+      <c r="A67" s="9" t="inlineStr">
+        <is>
+          <t>F066</t>
+        </is>
+      </c>
+      <c r="B67" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C67" s="9" t="inlineStr">
+        <is>
+          <t>Trigonométrie</t>
+        </is>
+      </c>
+      <c r="D67" s="9" t="inlineStr">
+        <is>
+          <t>$\cos\left(\frac\pi2\right)$</t>
+        </is>
+      </c>
+      <c r="E67" s="9" t="n"/>
+      <c r="F67" s="10" t="inlineStr">
+        <is>
+          <t>Donner la valeur exacte de $\cos\left(\frac\pi2\right)$.</t>
+        </is>
+      </c>
+      <c r="G67" s="9" t="inlineStr">
+        <is>
+          <t>$0$</t>
+        </is>
+      </c>
+      <c r="H67" s="9" t="inlineStr">
+        <is>
+          <t>Outils 3 : « Définition de cos(θ), sin(θ) et tan(θ). » Valeurs remarquables, prérequis du lycée.</t>
+        </is>
+      </c>
+      <c r="I67" s="9" t="n"/>
+      <c r="J67" s="9" t="n"/>
+      <c r="K67" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le formulaire de trigonométrie</t>
+        </is>
+      </c>
+      <c r="L67" s="11" t="n"/>
+      <c r="M67" s="11" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="9" t="inlineStr">
+        <is>
+          <t>F067</t>
+        </is>
+      </c>
+      <c r="B68" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C68" s="9" t="inlineStr">
+        <is>
+          <t>Trigonométrie</t>
+        </is>
+      </c>
+      <c r="D68" s="9" t="inlineStr">
+        <is>
+          <t>$\sin\left(\frac\pi2\right)$</t>
+        </is>
+      </c>
+      <c r="E68" s="9" t="n"/>
+      <c r="F68" s="10" t="inlineStr">
+        <is>
+          <t>Donner la valeur exacte de $\sin\left(\frac\pi2\right)$.</t>
+        </is>
+      </c>
+      <c r="G68" s="9" t="inlineStr">
+        <is>
+          <t>$1$</t>
+        </is>
+      </c>
+      <c r="H68" s="9" t="inlineStr">
+        <is>
+          <t>Outils 3 : « Définition de cos(θ), sin(θ) et tan(θ). » Valeurs remarquables, prérequis du lycée.</t>
+        </is>
+      </c>
+      <c r="I68" s="9" t="n"/>
+      <c r="J68" s="9" t="n"/>
+      <c r="K68" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le formulaire de trigonométrie</t>
+        </is>
+      </c>
+      <c r="L68" s="11" t="n"/>
+      <c r="M68" s="11" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="9" t="inlineStr">
+        <is>
+          <t>F068</t>
+        </is>
+      </c>
+      <c r="B69" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C69" s="9" t="inlineStr">
+        <is>
+          <t>Trigonométrie</t>
+        </is>
+      </c>
+      <c r="D69" s="9" t="inlineStr">
+        <is>
+          <t>$\cos\pi$</t>
+        </is>
+      </c>
+      <c r="E69" s="9" t="n"/>
+      <c r="F69" s="10" t="inlineStr">
+        <is>
+          <t>Donner la valeur exacte de $\cos\pi$.</t>
+        </is>
+      </c>
+      <c r="G69" s="9" t="inlineStr">
+        <is>
+          <t>$-1$</t>
+        </is>
+      </c>
+      <c r="H69" s="9" t="inlineStr">
+        <is>
+          <t>Outils 3 : « Définition de cos(θ), sin(θ) et tan(θ). » Valeurs remarquables, prérequis du lycée.</t>
+        </is>
+      </c>
+      <c r="I69" s="9" t="n"/>
+      <c r="J69" s="9" t="n"/>
+      <c r="K69" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le formulaire de trigonométrie</t>
+        </is>
+      </c>
+      <c r="L69" s="11" t="n"/>
+      <c r="M69" s="11" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="9" t="inlineStr">
+        <is>
+          <t>F069</t>
+        </is>
+      </c>
+      <c r="B70" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C70" s="9" t="inlineStr">
+        <is>
+          <t>Trigonométrie</t>
+        </is>
+      </c>
+      <c r="D70" s="9" t="inlineStr">
+        <is>
+          <t>$\sin\pi$</t>
+        </is>
+      </c>
+      <c r="E70" s="9" t="n"/>
+      <c r="F70" s="10" t="inlineStr">
+        <is>
+          <t>Donner la valeur exacte de $\sin\pi$.</t>
+        </is>
+      </c>
+      <c r="G70" s="9" t="inlineStr">
+        <is>
+          <t>$0$</t>
+        </is>
+      </c>
+      <c r="H70" s="9" t="inlineStr">
+        <is>
+          <t>Outils 3 : « Définition de cos(θ), sin(θ) et tan(θ). » Valeurs remarquables, prérequis du lycée.</t>
+        </is>
+      </c>
+      <c r="I70" s="9" t="n"/>
+      <c r="J70" s="9" t="n"/>
+      <c r="K70" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le formulaire de trigonométrie</t>
+        </is>
+      </c>
+      <c r="L70" s="11" t="n"/>
+      <c r="M70" s="11" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="9" t="inlineStr">
+        <is>
+          <t>F070</t>
+        </is>
+      </c>
+      <c r="B71" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C71" s="9" t="inlineStr">
+        <is>
+          <t>Trigonométrie</t>
+        </is>
+      </c>
+      <c r="D71" s="9" t="inlineStr">
+        <is>
+          <t>$\cos(a+2\pi)$</t>
+        </is>
+      </c>
+      <c r="E71" s="9" t="inlineStr">
+        <is>
+          <t>Soit $a$ un réel.</t>
+        </is>
+      </c>
+      <c r="F71" s="10" t="inlineStr">
+        <is>
+          <t>Compléter : $\cos(a+2\pi)$ $=\;\dots$</t>
+        </is>
+      </c>
+      <c r="G71" s="9" t="inlineStr">
+        <is>
+          <t>$\cos a$ ($\cos$ et $\sin$ sont $2\pi$-périodiques)</t>
+        </is>
+      </c>
+      <c r="H71" s="9" t="inlineStr">
+        <is>
+          <t>Outils 3 : « Formules découlant des symétries de cos, sin et tan » ; « Périodicité et symétries ».</t>
+        </is>
+      </c>
+      <c r="I71" s="9" t="n"/>
+      <c r="J71" s="9" t="n"/>
+      <c r="K71" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le formulaire de trigonométrie</t>
+        </is>
+      </c>
+      <c r="L71" s="11" t="n"/>
+      <c r="M71" s="11" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="9" t="inlineStr">
+        <is>
+          <t>F071</t>
+        </is>
+      </c>
+      <c r="B72" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C72" s="9" t="inlineStr">
+        <is>
+          <t>Trigonométrie</t>
+        </is>
+      </c>
+      <c r="D72" s="9" t="inlineStr">
+        <is>
+          <t>$\tan\left(\frac\pi2-a\right)$</t>
+        </is>
+      </c>
+      <c r="E72" s="9" t="inlineStr">
+        <is>
+          <t>Soit $a$ un réel tel que $\tan a$ et $\tan\left(\frac\pi2-a\right)$ soient définis et $\tan a\neq0$.</t>
+        </is>
+      </c>
+      <c r="F72" s="10" t="inlineStr">
+        <is>
+          <t>Compléter : $\tan\left(\frac\pi2-a\right)$ $=\;\dots$</t>
+        </is>
+      </c>
+      <c r="G72" s="9" t="inlineStr">
+        <is>
+          <t>$\dfrac1{\tan a}$</t>
+        </is>
+      </c>
+      <c r="H72" s="9" t="inlineStr">
+        <is>
+          <t>Outils 3 : « Formules découlant des symétries de cos, sin et tan » ; « Périodicité et symétries ».</t>
+        </is>
+      </c>
+      <c r="I72" s="9" t="n"/>
+      <c r="J72" s="9" t="n"/>
+      <c r="K72" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le formulaire de trigonométrie</t>
+        </is>
+      </c>
+      <c r="L72" s="11" t="n"/>
+      <c r="M72" s="11" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="9" t="inlineStr">
+        <is>
+          <t>F072</t>
+        </is>
+      </c>
+      <c r="B73" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C73" s="9" t="inlineStr">
+        <is>
+          <t>Trigonométrie</t>
+        </is>
+      </c>
+      <c r="D73" s="9" t="inlineStr">
+        <is>
+          <t>$\cos x=0$</t>
+        </is>
+      </c>
+      <c r="E73" s="9" t="inlineStr">
+        <is>
+          <t>Soit $x$ un réel.</t>
+        </is>
+      </c>
+      <c r="F73" s="10" t="inlineStr">
+        <is>
+          <t>Résoudre $\cos x=0$.</t>
+        </is>
+      </c>
+      <c r="G73" s="9" t="inlineStr">
+        <is>
+          <t>$x=\dfrac\pi2+k\pi$, $k\in\mathbb Z$</t>
+        </is>
+      </c>
+      <c r="H73" s="9" t="inlineStr">
+        <is>
+          <t>Outils 3 : « Résolution d'équations trigonométriques simples : cos(x) = c, sin(x) = s. »</t>
+        </is>
+      </c>
+      <c r="I73" s="9" t="n"/>
+      <c r="J73" s="9" t="n"/>
+      <c r="K73" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le formulaire de trigonométrie</t>
+        </is>
+      </c>
+      <c r="L73" s="11" t="n"/>
+      <c r="M73" s="11" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="9" t="inlineStr">
+        <is>
+          <t>F073</t>
+        </is>
+      </c>
+      <c r="B74" s="10" t="inlineStr">
+        <is>
+          <t>Noir – conforme</t>
+        </is>
+      </c>
+      <c r="C74" s="9" t="inlineStr">
+        <is>
+          <t>Trigonométrie</t>
+        </is>
+      </c>
+      <c r="D74" s="9" t="inlineStr">
+        <is>
+          <t>$\sin x=0$</t>
+        </is>
+      </c>
+      <c r="E74" s="9" t="inlineStr">
+        <is>
+          <t>Soit $x$ un réel.</t>
+        </is>
+      </c>
+      <c r="F74" s="10" t="inlineStr">
+        <is>
+          <t>Résoudre $\sin x=0$.</t>
+        </is>
+      </c>
+      <c r="G74" s="9" t="inlineStr">
+        <is>
+          <t>$x=k\pi$, $k\in\mathbb Z$</t>
+        </is>
+      </c>
+      <c r="H74" s="9" t="inlineStr">
+        <is>
+          <t>Outils 3 : « Résolution d'équations trigonométriques simples : cos(x) = c, sin(x) = s. »</t>
+        </is>
+      </c>
+      <c r="I74" s="9" t="n"/>
+      <c r="J74" s="9" t="n"/>
+      <c r="K74" s="9" t="inlineStr">
+        <is>
+          <t>Ajout d’après le formulaire de trigonométrie</t>
+        </is>
+      </c>
+      <c r="L74" s="11" t="n"/>
+      <c r="M74" s="11" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:M60"/>
   <dataValidations count="1">
-    <dataValidation sqref="L2:L66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>
@@ -41087,7 +41479,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
@@ -41161,7 +41552,6 @@
         <v/>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="25" t="inlineStr">
         <is>
@@ -41173,7 +41563,6 @@
         <v/>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Formulaire de trigonométrie : linéarisation de sin² et cos² (orange)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C3wC4vohcaqEtbhgDxU3AT
</commit_message>
<xml_diff>
--- a/source/fiches_maths.xlsx
+++ b/source/fiches_maths.xlsx
@@ -37583,7 +37583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M74"/>
+  <dimension ref="A1:M76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -41445,10 +41445,112 @@
       <c r="L74" s="11" t="n"/>
       <c r="M74" s="11" t="n"/>
     </row>
+    <row r="75">
+      <c r="A75" s="12" t="inlineStr">
+        <is>
+          <t>F074</t>
+        </is>
+      </c>
+      <c r="B75" s="13" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C75" s="12" t="inlineStr">
+        <is>
+          <t>Trigonométrie</t>
+        </is>
+      </c>
+      <c r="D75" s="12" t="inlineStr">
+        <is>
+          <t>$\sin^2a$ (linéarisation)</t>
+        </is>
+      </c>
+      <c r="E75" s="12" t="inlineStr">
+        <is>
+          <t>Soit $a$ un réel.</t>
+        </is>
+      </c>
+      <c r="F75" s="13" t="inlineStr">
+        <is>
+          <t>Exprimer $\sin^2a$ en fonction de $\cos 2a$.</t>
+        </is>
+      </c>
+      <c r="G75" s="12" t="inlineStr">
+        <is>
+          <t>$\dfrac{1-\cos 2a}2$</t>
+        </is>
+      </c>
+      <c r="H75" s="12" t="inlineStr">
+        <is>
+          <t>Outils 3 : formule non citée (« Les autres formules de trigonométrie ne sont pas des attendus du programme ») ; elle se déduit directement de $\cos 2a=1-2\sin^2a=2\cos^2a-1$.</t>
+        </is>
+      </c>
+      <c r="I75" s="12" t="n"/>
+      <c r="J75" s="12" t="n"/>
+      <c r="K75" s="12" t="inlineStr">
+        <is>
+          <t>Ajout d’après le formulaire de trigonométrie (choix de B)</t>
+        </is>
+      </c>
+      <c r="L75" s="14" t="n"/>
+      <c r="M75" s="14" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="12" t="inlineStr">
+        <is>
+          <t>F075</t>
+        </is>
+      </c>
+      <c r="B76" s="13" t="inlineStr">
+        <is>
+          <t>Orange – incertain</t>
+        </is>
+      </c>
+      <c r="C76" s="12" t="inlineStr">
+        <is>
+          <t>Trigonométrie</t>
+        </is>
+      </c>
+      <c r="D76" s="12" t="inlineStr">
+        <is>
+          <t>$\cos^2a$ (linéarisation)</t>
+        </is>
+      </c>
+      <c r="E76" s="12" t="inlineStr">
+        <is>
+          <t>Soit $a$ un réel.</t>
+        </is>
+      </c>
+      <c r="F76" s="13" t="inlineStr">
+        <is>
+          <t>Exprimer $\cos^2a$ en fonction de $\cos 2a$.</t>
+        </is>
+      </c>
+      <c r="G76" s="12" t="inlineStr">
+        <is>
+          <t>$\dfrac{1+\cos 2a}2$</t>
+        </is>
+      </c>
+      <c r="H76" s="12" t="inlineStr">
+        <is>
+          <t>Outils 3 : formule non citée (« Les autres formules de trigonométrie ne sont pas des attendus du programme ») ; elle se déduit directement de $\cos 2a=1-2\sin^2a=2\cos^2a-1$.</t>
+        </is>
+      </c>
+      <c r="I76" s="12" t="n"/>
+      <c r="J76" s="12" t="n"/>
+      <c r="K76" s="12" t="inlineStr">
+        <is>
+          <t>Ajout d’après le formulaire de trigonométrie (choix de B)</t>
+        </is>
+      </c>
+      <c r="L76" s="14" t="n"/>
+      <c r="M76" s="14" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:M60"/>
   <dataValidations count="1">
-    <dataValidation sqref="L2:L74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,Passer en noir,Passer en orange,Passer en rouge,Supprimer,Contenu à corriger"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>